<commit_message>
Atualizacao automatica 16/09/2026 11:05:59,41
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01BB175D-0DE1-4301-B8DE-5E90CDE07C1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EE76D23-1D9A-46DD-98F9-14E7E343F367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="101">
   <si>
     <t>Sel</t>
   </si>
@@ -154,118 +154,175 @@
     <t>Nº Série</t>
   </si>
   <si>
+    <t>10014979</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>90201</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>UN</t>
+  </si>
+  <si>
+    <t>FORNO ELETRICO NARDELLI TOP 40 40L BLACK - NARDELLI TOP 40 - 220 V</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>FORNOS</t>
+  </si>
+  <si>
+    <t>1858600041542</t>
+  </si>
+  <si>
+    <t>10016351</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>FORNO ELETRICO NARDELLI EMBUTIR INOX 60 LITROS - NARDELLI EMBUTIR INOX 60 LITROS - 127 V</t>
+  </si>
+  <si>
+    <t>FORNOE</t>
+  </si>
+  <si>
+    <t>1858400003510</t>
+  </si>
+  <si>
+    <t>1858400003511</t>
+  </si>
+  <si>
+    <t>1858400003512</t>
+  </si>
+  <si>
+    <t>1858400003513</t>
+  </si>
+  <si>
+    <t>1858400003514</t>
+  </si>
+  <si>
+    <t>1858400003515</t>
+  </si>
+  <si>
+    <t>1858400003516</t>
+  </si>
+  <si>
     <t>10018965</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>500</t>
-  </si>
-  <si>
-    <t>E</t>
-  </si>
-  <si>
-    <t>90201</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>UN</t>
-  </si>
-  <si>
     <t>FORNO ELETRICO NARDELLI E50 BLACK 50L - NARDELLI E50 BLACK 50 L - 220 V</t>
   </si>
   <si>
-    <t>100</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>FORNOE</t>
-  </si>
-  <si>
-    <t>1879900000415</t>
-  </si>
-  <si>
-    <t>1879900000416</t>
-  </si>
-  <si>
-    <t>1879900000417</t>
-  </si>
-  <si>
-    <t>1879900000418</t>
-  </si>
-  <si>
-    <t>1879900000419</t>
-  </si>
-  <si>
-    <t>1879900000420</t>
-  </si>
-  <si>
-    <t>1879900000421</t>
-  </si>
-  <si>
-    <t>1879900000422</t>
-  </si>
-  <si>
-    <t>10098965</t>
-  </si>
-  <si>
-    <t>FORNO ELETRICO TERIM E50 BLACK 50L - TERIM E50 BLACK 50 L - 220 V</t>
-  </si>
-  <si>
-    <t>1033300000101</t>
-  </si>
-  <si>
-    <t>1033300000102</t>
-  </si>
-  <si>
-    <t>1033300000103</t>
-  </si>
-  <si>
-    <t>1033300000104</t>
-  </si>
-  <si>
-    <t>1033300000105</t>
-  </si>
-  <si>
-    <t>1033300000106</t>
-  </si>
-  <si>
-    <t>1033300000107</t>
-  </si>
-  <si>
-    <t>1033300000108</t>
-  </si>
-  <si>
-    <t>1033300000109</t>
-  </si>
-  <si>
-    <t>1033300000110</t>
-  </si>
-  <si>
-    <t>1033300000111</t>
-  </si>
-  <si>
-    <t>1033300000112</t>
-  </si>
-  <si>
-    <t>1033300000113</t>
-  </si>
-  <si>
-    <t>1033300000114</t>
-  </si>
-  <si>
-    <t>1033300000115</t>
-  </si>
-  <si>
-    <t>1033300000116</t>
-  </si>
-  <si>
-    <t>1033300000117</t>
+    <t>1879900000465</t>
+  </si>
+  <si>
+    <t>1879900000466</t>
+  </si>
+  <si>
+    <t>1879900000467</t>
+  </si>
+  <si>
+    <t>1879900000468</t>
+  </si>
+  <si>
+    <t>1879900000469</t>
+  </si>
+  <si>
+    <t>1879900000470</t>
+  </si>
+  <si>
+    <t>1879900000471</t>
+  </si>
+  <si>
+    <t>1879900000472</t>
+  </si>
+  <si>
+    <t>1879900000473</t>
+  </si>
+  <si>
+    <t>1879900000474</t>
+  </si>
+  <si>
+    <t>10056354</t>
+  </si>
+  <si>
+    <t>FORNO ELETRICO FOGATTI EMBUTIR 60L BLACK - 127 V</t>
+  </si>
+  <si>
+    <t>1030900000070</t>
+  </si>
+  <si>
+    <t>1030900000071</t>
+  </si>
+  <si>
+    <t>1030900000072</t>
+  </si>
+  <si>
+    <t>1030900000073</t>
+  </si>
+  <si>
+    <t>1030900000074</t>
+  </si>
+  <si>
+    <t>1030900000075</t>
+  </si>
+  <si>
+    <t>1030900000076</t>
+  </si>
+  <si>
+    <t>1030900000077</t>
+  </si>
+  <si>
+    <t>1030900000078</t>
+  </si>
+  <si>
+    <t>1030900000079</t>
+  </si>
+  <si>
+    <t>1030900000080</t>
+  </si>
+  <si>
+    <t>1030900000081</t>
+  </si>
+  <si>
+    <t>1030900000082</t>
+  </si>
+  <si>
+    <t>1030900000083</t>
+  </si>
+  <si>
+    <t>1030900000084</t>
+  </si>
+  <si>
+    <t>1030900000085</t>
+  </si>
+  <si>
+    <t>1030900000086</t>
+  </si>
+  <si>
+    <t>1030900000087</t>
+  </si>
+  <si>
+    <t>1030900000088</t>
+  </si>
+  <si>
+    <t>1030900000089</t>
   </si>
 </sst>
 </file>
@@ -841,7 +898,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR26"/>
+  <dimension ref="A1:AR39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -995,10 +1052,10 @@
         <v>46</v>
       </c>
       <c r="F2" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G2" s="5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>47</v>
@@ -1013,10 +1070,10 @@
         <v>50</v>
       </c>
       <c r="L2" s="6">
-        <v>77</v>
+        <v>915</v>
       </c>
       <c r="M2" s="7">
-        <v>26766.79</v>
+        <v>171252.21</v>
       </c>
       <c r="N2" s="6">
         <v>1</v>
@@ -1025,7 +1082,7 @@
         <v>51</v>
       </c>
       <c r="P2" s="8">
-        <v>347.62</v>
+        <v>187.16</v>
       </c>
       <c r="Q2" s="6">
         <v>0</v>
@@ -1040,16 +1097,16 @@
         <v>52</v>
       </c>
       <c r="U2" s="10">
-        <v>67347</v>
+        <v>67407</v>
       </c>
       <c r="V2" s="11">
         <v>11</v>
       </c>
       <c r="W2" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X2" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.39027780000000001</v>
       </c>
       <c r="Y2" s="10">
         <v>0</v>
@@ -1120,19 +1177,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F3" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G3" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>47</v>
@@ -1147,19 +1204,19 @@
         <v>50</v>
       </c>
       <c r="L3" s="6">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="M3" s="7">
-        <v>27114.41</v>
+        <v>27544.42</v>
       </c>
       <c r="N3" s="6">
         <v>1</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P3" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q3" s="6">
         <v>0</v>
@@ -1174,16 +1231,16 @@
         <v>52</v>
       </c>
       <c r="U3" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V3" s="11">
         <v>11</v>
       </c>
       <c r="W3" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X3" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y3" s="10">
         <v>0</v>
@@ -1216,7 +1273,7 @@
         <v>53</v>
       </c>
       <c r="AI3" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ3" s="3" t="s">
         <v>52</v>
@@ -1243,7 +1300,7 @@
         <v>53</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1254,19 +1311,19 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F4" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G4" s="5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>47</v>
@@ -1281,19 +1338,19 @@
         <v>50</v>
       </c>
       <c r="L4" s="6">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="M4" s="7">
-        <v>27462.03</v>
+        <v>27921.74</v>
       </c>
       <c r="N4" s="6">
         <v>1</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P4" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q4" s="6">
         <v>0</v>
@@ -1308,16 +1365,16 @@
         <v>52</v>
       </c>
       <c r="U4" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V4" s="11">
         <v>11</v>
       </c>
       <c r="W4" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X4" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y4" s="10">
         <v>0</v>
@@ -1350,7 +1407,7 @@
         <v>53</v>
       </c>
       <c r="AI4" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ4" s="3" t="s">
         <v>52</v>
@@ -1377,7 +1434,7 @@
         <v>53</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1388,19 +1445,19 @@
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F5" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G5" s="5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>47</v>
@@ -1415,19 +1472,19 @@
         <v>50</v>
       </c>
       <c r="L5" s="6">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="M5" s="7">
-        <v>27809.65</v>
+        <v>28299.06</v>
       </c>
       <c r="N5" s="6">
         <v>1</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P5" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q5" s="6">
         <v>0</v>
@@ -1442,16 +1499,16 @@
         <v>52</v>
       </c>
       <c r="U5" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V5" s="11">
         <v>11</v>
       </c>
       <c r="W5" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X5" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y5" s="10">
         <v>0</v>
@@ -1484,7 +1541,7 @@
         <v>53</v>
       </c>
       <c r="AI5" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ5" s="3" t="s">
         <v>52</v>
@@ -1511,7 +1568,7 @@
         <v>53</v>
       </c>
       <c r="AR5" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1522,19 +1579,19 @@
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F6" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G6" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>47</v>
@@ -1549,19 +1606,19 @@
         <v>50</v>
       </c>
       <c r="L6" s="6">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="M6" s="7">
-        <v>28157.27</v>
+        <v>28676.39</v>
       </c>
       <c r="N6" s="6">
         <v>1</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P6" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q6" s="6">
         <v>0</v>
@@ -1576,16 +1633,16 @@
         <v>52</v>
       </c>
       <c r="U6" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V6" s="11">
         <v>11</v>
       </c>
       <c r="W6" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X6" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y6" s="10">
         <v>0</v>
@@ -1618,7 +1675,7 @@
         <v>53</v>
       </c>
       <c r="AI6" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ6" s="3" t="s">
         <v>52</v>
@@ -1645,7 +1702,7 @@
         <v>53</v>
       </c>
       <c r="AR6" s="3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1656,19 +1713,19 @@
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F7" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G7" s="5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>47</v>
@@ -1683,19 +1740,19 @@
         <v>50</v>
       </c>
       <c r="L7" s="6">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="M7" s="7">
-        <v>28504.89</v>
+        <v>29053.71</v>
       </c>
       <c r="N7" s="6">
         <v>1</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P7" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q7" s="6">
         <v>0</v>
@@ -1710,16 +1767,16 @@
         <v>52</v>
       </c>
       <c r="U7" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V7" s="11">
         <v>11</v>
       </c>
       <c r="W7" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X7" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y7" s="10">
         <v>0</v>
@@ -1752,7 +1809,7 @@
         <v>53</v>
       </c>
       <c r="AI7" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ7" s="3" t="s">
         <v>52</v>
@@ -1779,7 +1836,7 @@
         <v>53</v>
       </c>
       <c r="AR7" s="3" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
@@ -1790,19 +1847,19 @@
         <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F8" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G8" s="5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>47</v>
@@ -1817,19 +1874,19 @@
         <v>50</v>
       </c>
       <c r="L8" s="6">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="M8" s="7">
-        <v>28852.51</v>
+        <v>29431.03</v>
       </c>
       <c r="N8" s="6">
         <v>1</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P8" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q8" s="6">
         <v>0</v>
@@ -1844,16 +1901,16 @@
         <v>52</v>
       </c>
       <c r="U8" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V8" s="11">
         <v>11</v>
       </c>
       <c r="W8" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X8" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y8" s="10">
         <v>0</v>
@@ -1886,7 +1943,7 @@
         <v>53</v>
       </c>
       <c r="AI8" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ8" s="3" t="s">
         <v>52</v>
@@ -1913,7 +1970,7 @@
         <v>53</v>
       </c>
       <c r="AR8" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1924,19 +1981,19 @@
         <v>2</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F9" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G9" s="5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>47</v>
@@ -1951,19 +2008,19 @@
         <v>50</v>
       </c>
       <c r="L9" s="6">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="M9" s="7">
-        <v>29200.13</v>
+        <v>29808.35</v>
       </c>
       <c r="N9" s="6">
         <v>1</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="P9" s="8">
-        <v>347.62</v>
+        <v>377.32</v>
       </c>
       <c r="Q9" s="6">
         <v>0</v>
@@ -1978,16 +2035,16 @@
         <v>52</v>
       </c>
       <c r="U9" s="10">
-        <v>67347</v>
+        <v>66798</v>
       </c>
       <c r="V9" s="11">
         <v>11</v>
       </c>
       <c r="W9" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X9" s="12">
-        <v>0.43055559999999998</v>
+        <v>0.4583333</v>
       </c>
       <c r="Y9" s="10">
         <v>0</v>
@@ -2020,7 +2077,7 @@
         <v>53</v>
       </c>
       <c r="AI9" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ9" s="3" t="s">
         <v>52</v>
@@ -2047,7 +2104,7 @@
         <v>53</v>
       </c>
       <c r="AR9" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2058,7 +2115,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>45</v>
@@ -2067,10 +2124,10 @@
         <v>46</v>
       </c>
       <c r="F10" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G10" s="5">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>47</v>
@@ -2085,19 +2142,19 @@
         <v>50</v>
       </c>
       <c r="L10" s="6">
-        <v>3</v>
+        <v>127</v>
       </c>
       <c r="M10" s="7">
-        <v>1158.57</v>
+        <v>44105.13</v>
       </c>
       <c r="N10" s="6">
         <v>1</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P10" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q10" s="6">
         <v>0</v>
@@ -2112,16 +2169,16 @@
         <v>52</v>
       </c>
       <c r="U10" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V10" s="11">
         <v>11</v>
       </c>
       <c r="W10" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X10" s="12">
-        <v>0.30555559999999998</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y10" s="10">
         <v>0</v>
@@ -2154,7 +2211,7 @@
         <v>53</v>
       </c>
       <c r="AI10" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ10" s="3" t="s">
         <v>52</v>
@@ -2181,7 +2238,7 @@
         <v>53</v>
       </c>
       <c r="AR10" s="3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2192,7 +2249,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>45</v>
@@ -2201,10 +2258,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G11" s="5">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>47</v>
@@ -2219,19 +2276,19 @@
         <v>50</v>
       </c>
       <c r="L11" s="6">
-        <v>4</v>
+        <v>128</v>
       </c>
       <c r="M11" s="7">
-        <v>1544.76</v>
+        <v>44452.41</v>
       </c>
       <c r="N11" s="6">
         <v>1</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P11" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q11" s="6">
         <v>0</v>
@@ -2246,16 +2303,16 @@
         <v>52</v>
       </c>
       <c r="U11" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V11" s="11">
         <v>11</v>
       </c>
       <c r="W11" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X11" s="12">
-        <v>0.30555559999999998</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y11" s="10">
         <v>0</v>
@@ -2288,7 +2345,7 @@
         <v>53</v>
       </c>
       <c r="AI11" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ11" s="3" t="s">
         <v>52</v>
@@ -2315,7 +2372,7 @@
         <v>53</v>
       </c>
       <c r="AR11" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2326,7 +2383,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>45</v>
@@ -2335,10 +2392,10 @@
         <v>46</v>
       </c>
       <c r="F12" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G12" s="5">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>47</v>
@@ -2353,19 +2410,19 @@
         <v>50</v>
       </c>
       <c r="L12" s="6">
-        <v>5</v>
+        <v>129</v>
       </c>
       <c r="M12" s="7">
-        <v>1930.95</v>
+        <v>44799.7</v>
       </c>
       <c r="N12" s="6">
         <v>1</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P12" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q12" s="6">
         <v>0</v>
@@ -2380,16 +2437,16 @@
         <v>52</v>
       </c>
       <c r="U12" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V12" s="11">
         <v>11</v>
       </c>
       <c r="W12" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X12" s="12">
-        <v>0.30555559999999998</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y12" s="10">
         <v>0</v>
@@ -2422,7 +2479,7 @@
         <v>53</v>
       </c>
       <c r="AI12" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ12" s="3" t="s">
         <v>52</v>
@@ -2449,7 +2506,7 @@
         <v>53</v>
       </c>
       <c r="AR12" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2460,7 +2517,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>45</v>
@@ -2469,10 +2526,10 @@
         <v>46</v>
       </c>
       <c r="F13" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G13" s="5">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>47</v>
@@ -2487,19 +2544,19 @@
         <v>50</v>
       </c>
       <c r="L13" s="6">
-        <v>6</v>
+        <v>130</v>
       </c>
       <c r="M13" s="7">
-        <v>2317.14</v>
+        <v>45146.98</v>
       </c>
       <c r="N13" s="6">
         <v>1</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P13" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q13" s="6">
         <v>0</v>
@@ -2514,16 +2571,16 @@
         <v>52</v>
       </c>
       <c r="U13" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V13" s="11">
         <v>11</v>
       </c>
       <c r="W13" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X13" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y13" s="10">
         <v>0</v>
@@ -2556,7 +2613,7 @@
         <v>53</v>
       </c>
       <c r="AI13" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ13" s="3" t="s">
         <v>52</v>
@@ -2583,7 +2640,7 @@
         <v>53</v>
       </c>
       <c r="AR13" s="3" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2594,7 +2651,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>45</v>
@@ -2603,10 +2660,10 @@
         <v>46</v>
       </c>
       <c r="F14" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G14" s="5">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>47</v>
@@ -2621,19 +2678,19 @@
         <v>50</v>
       </c>
       <c r="L14" s="6">
-        <v>7</v>
+        <v>131</v>
       </c>
       <c r="M14" s="7">
-        <v>2703.33</v>
+        <v>45494.27</v>
       </c>
       <c r="N14" s="6">
         <v>1</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P14" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q14" s="6">
         <v>0</v>
@@ -2648,16 +2705,16 @@
         <v>52</v>
       </c>
       <c r="U14" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V14" s="11">
         <v>11</v>
       </c>
       <c r="W14" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X14" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y14" s="10">
         <v>0</v>
@@ -2690,7 +2747,7 @@
         <v>53</v>
       </c>
       <c r="AI14" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ14" s="3" t="s">
         <v>52</v>
@@ -2717,7 +2774,7 @@
         <v>53</v>
       </c>
       <c r="AR14" s="3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -2728,7 +2785,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>45</v>
@@ -2737,10 +2794,10 @@
         <v>46</v>
       </c>
       <c r="F15" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G15" s="5">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>47</v>
@@ -2755,19 +2812,19 @@
         <v>50</v>
       </c>
       <c r="L15" s="6">
-        <v>8</v>
+        <v>132</v>
       </c>
       <c r="M15" s="7">
-        <v>3089.52</v>
+        <v>45841.55</v>
       </c>
       <c r="N15" s="6">
         <v>1</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P15" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q15" s="6">
         <v>0</v>
@@ -2782,16 +2839,16 @@
         <v>52</v>
       </c>
       <c r="U15" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V15" s="11">
         <v>11</v>
       </c>
       <c r="W15" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X15" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y15" s="10">
         <v>0</v>
@@ -2824,7 +2881,7 @@
         <v>53</v>
       </c>
       <c r="AI15" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ15" s="3" t="s">
         <v>52</v>
@@ -2851,7 +2908,7 @@
         <v>53</v>
       </c>
       <c r="AR15" s="3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:44" x14ac:dyDescent="0.3">
@@ -2862,7 +2919,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>45</v>
@@ -2871,10 +2928,10 @@
         <v>46</v>
       </c>
       <c r="F16" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G16" s="5">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>47</v>
@@ -2889,19 +2946,19 @@
         <v>50</v>
       </c>
       <c r="L16" s="6">
-        <v>9</v>
+        <v>133</v>
       </c>
       <c r="M16" s="7">
-        <v>3475.71</v>
+        <v>46188.83</v>
       </c>
       <c r="N16" s="6">
         <v>1</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P16" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q16" s="6">
         <v>0</v>
@@ -2916,16 +2973,16 @@
         <v>52</v>
       </c>
       <c r="U16" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V16" s="11">
         <v>11</v>
       </c>
       <c r="W16" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X16" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y16" s="10">
         <v>0</v>
@@ -2958,7 +3015,7 @@
         <v>53</v>
       </c>
       <c r="AI16" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ16" s="3" t="s">
         <v>52</v>
@@ -2985,7 +3042,7 @@
         <v>53</v>
       </c>
       <c r="AR16" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:44" x14ac:dyDescent="0.3">
@@ -2996,7 +3053,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>45</v>
@@ -3005,10 +3062,10 @@
         <v>46</v>
       </c>
       <c r="F17" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G17" s="5">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>47</v>
@@ -3023,19 +3080,19 @@
         <v>50</v>
       </c>
       <c r="L17" s="6">
-        <v>10</v>
+        <v>134</v>
       </c>
       <c r="M17" s="7">
-        <v>3861.9</v>
+        <v>46536.12</v>
       </c>
       <c r="N17" s="6">
         <v>1</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P17" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q17" s="6">
         <v>0</v>
@@ -3050,16 +3107,16 @@
         <v>52</v>
       </c>
       <c r="U17" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V17" s="11">
         <v>11</v>
       </c>
       <c r="W17" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X17" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y17" s="10">
         <v>0</v>
@@ -3092,7 +3149,7 @@
         <v>53</v>
       </c>
       <c r="AI17" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ17" s="3" t="s">
         <v>52</v>
@@ -3119,7 +3176,7 @@
         <v>53</v>
       </c>
       <c r="AR17" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:44" x14ac:dyDescent="0.3">
@@ -3130,7 +3187,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>45</v>
@@ -3139,10 +3196,10 @@
         <v>46</v>
       </c>
       <c r="F18" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G18" s="5">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>47</v>
@@ -3157,19 +3214,19 @@
         <v>50</v>
       </c>
       <c r="L18" s="6">
-        <v>11</v>
+        <v>135</v>
       </c>
       <c r="M18" s="7">
-        <v>4248.09</v>
+        <v>46883.4</v>
       </c>
       <c r="N18" s="6">
         <v>1</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P18" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q18" s="6">
         <v>0</v>
@@ -3184,16 +3241,16 @@
         <v>52</v>
       </c>
       <c r="U18" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V18" s="11">
         <v>11</v>
       </c>
       <c r="W18" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X18" s="12">
-        <v>0.36111110000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y18" s="10">
         <v>0</v>
@@ -3226,7 +3283,7 @@
         <v>53</v>
       </c>
       <c r="AI18" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ18" s="3" t="s">
         <v>52</v>
@@ -3253,7 +3310,7 @@
         <v>53</v>
       </c>
       <c r="AR18" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:44" x14ac:dyDescent="0.3">
@@ -3264,7 +3321,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>45</v>
@@ -3273,10 +3330,10 @@
         <v>46</v>
       </c>
       <c r="F19" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G19" s="5">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>47</v>
@@ -3291,19 +3348,19 @@
         <v>50</v>
       </c>
       <c r="L19" s="6">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="M19" s="7">
-        <v>4634.28</v>
+        <v>47230.69</v>
       </c>
       <c r="N19" s="6">
         <v>1</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="P19" s="8">
-        <v>386.19</v>
+        <v>347.28</v>
       </c>
       <c r="Q19" s="6">
         <v>0</v>
@@ -3318,16 +3375,16 @@
         <v>52</v>
       </c>
       <c r="U19" s="10">
-        <v>67357</v>
+        <v>67347</v>
       </c>
       <c r="V19" s="11">
         <v>11</v>
       </c>
       <c r="W19" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X19" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.38958330000000002</v>
       </c>
       <c r="Y19" s="10">
         <v>0</v>
@@ -3360,7 +3417,7 @@
         <v>53</v>
       </c>
       <c r="AI19" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ19" s="3" t="s">
         <v>52</v>
@@ -3387,7 +3444,7 @@
         <v>53</v>
       </c>
       <c r="AR19" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:44" x14ac:dyDescent="0.3">
@@ -3398,19 +3455,19 @@
         <v>2</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F20" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G20" s="5">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>47</v>
@@ -3425,19 +3482,19 @@
         <v>50</v>
       </c>
       <c r="L20" s="6">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="M20" s="7">
-        <v>5020.47</v>
+        <v>650.74</v>
       </c>
       <c r="N20" s="6">
         <v>1</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P20" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q20" s="6">
         <v>0</v>
@@ -3452,16 +3509,16 @@
         <v>52</v>
       </c>
       <c r="U20" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V20" s="11">
         <v>11</v>
       </c>
       <c r="W20" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X20" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y20" s="10">
         <v>0</v>
@@ -3494,7 +3551,7 @@
         <v>53</v>
       </c>
       <c r="AI20" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ20" s="3" t="s">
         <v>52</v>
@@ -3521,7 +3578,7 @@
         <v>53</v>
       </c>
       <c r="AR20" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:44" x14ac:dyDescent="0.3">
@@ -3532,19 +3589,19 @@
         <v>2</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F21" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G21" s="5">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>47</v>
@@ -3559,19 +3616,19 @@
         <v>50</v>
       </c>
       <c r="L21" s="6">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="M21" s="7">
-        <v>5406.66</v>
+        <v>976.11</v>
       </c>
       <c r="N21" s="6">
         <v>1</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P21" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q21" s="6">
         <v>0</v>
@@ -3586,16 +3643,16 @@
         <v>52</v>
       </c>
       <c r="U21" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V21" s="11">
         <v>11</v>
       </c>
       <c r="W21" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X21" s="12">
-        <v>0.4034722</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y21" s="10">
         <v>0</v>
@@ -3628,7 +3685,7 @@
         <v>53</v>
       </c>
       <c r="AI21" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ21" s="3" t="s">
         <v>52</v>
@@ -3655,7 +3712,7 @@
         <v>53</v>
       </c>
       <c r="AR21" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:44" x14ac:dyDescent="0.3">
@@ -3666,19 +3723,19 @@
         <v>2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F22" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G22" s="5">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>47</v>
@@ -3693,19 +3750,19 @@
         <v>50</v>
       </c>
       <c r="L22" s="6">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="M22" s="7">
-        <v>5792.85</v>
+        <v>1301.48</v>
       </c>
       <c r="N22" s="6">
         <v>1</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P22" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q22" s="6">
         <v>0</v>
@@ -3720,16 +3777,16 @@
         <v>52</v>
       </c>
       <c r="U22" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V22" s="11">
         <v>11</v>
       </c>
       <c r="W22" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X22" s="12">
-        <v>0.4034722</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y22" s="10">
         <v>0</v>
@@ -3762,7 +3819,7 @@
         <v>53</v>
       </c>
       <c r="AI22" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ22" s="3" t="s">
         <v>52</v>
@@ -3789,7 +3846,7 @@
         <v>53</v>
       </c>
       <c r="AR22" s="3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:44" x14ac:dyDescent="0.3">
@@ -3800,19 +3857,19 @@
         <v>2</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F23" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G23" s="5">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>47</v>
@@ -3827,19 +3884,19 @@
         <v>50</v>
       </c>
       <c r="L23" s="6">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="M23" s="7">
-        <v>6179.04</v>
+        <v>1626.85</v>
       </c>
       <c r="N23" s="6">
         <v>1</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P23" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q23" s="6">
         <v>0</v>
@@ -3854,16 +3911,16 @@
         <v>52</v>
       </c>
       <c r="U23" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V23" s="11">
         <v>11</v>
       </c>
       <c r="W23" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X23" s="12">
-        <v>0.4034722</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y23" s="10">
         <v>0</v>
@@ -3896,7 +3953,7 @@
         <v>53</v>
       </c>
       <c r="AI23" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ23" s="3" t="s">
         <v>52</v>
@@ -3923,7 +3980,7 @@
         <v>53</v>
       </c>
       <c r="AR23" s="3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.3">
@@ -3934,19 +3991,19 @@
         <v>2</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F24" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G24" s="5">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>47</v>
@@ -3961,19 +4018,19 @@
         <v>50</v>
       </c>
       <c r="L24" s="6">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="M24" s="7">
-        <v>6565.23</v>
+        <v>1952.22</v>
       </c>
       <c r="N24" s="6">
         <v>1</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P24" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q24" s="6">
         <v>0</v>
@@ -3988,16 +4045,16 @@
         <v>52</v>
       </c>
       <c r="U24" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V24" s="11">
         <v>11</v>
       </c>
       <c r="W24" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X24" s="12">
-        <v>0.4034722</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y24" s="10">
         <v>0</v>
@@ -4030,7 +4087,7 @@
         <v>53</v>
       </c>
       <c r="AI24" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ24" s="3" t="s">
         <v>52</v>
@@ -4057,7 +4114,7 @@
         <v>53</v>
       </c>
       <c r="AR24" s="3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:44" x14ac:dyDescent="0.3">
@@ -4068,19 +4125,19 @@
         <v>2</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F25" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G25" s="5">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>47</v>
@@ -4095,19 +4152,19 @@
         <v>50</v>
       </c>
       <c r="L25" s="6">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="M25" s="7">
-        <v>6951.42</v>
+        <v>2277.59</v>
       </c>
       <c r="N25" s="6">
         <v>1</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P25" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q25" s="6">
         <v>0</v>
@@ -4122,16 +4179,16 @@
         <v>52</v>
       </c>
       <c r="U25" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V25" s="11">
         <v>11</v>
       </c>
       <c r="W25" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X25" s="12">
-        <v>0.4034722</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y25" s="10">
         <v>0</v>
@@ -4164,7 +4221,7 @@
         <v>53</v>
       </c>
       <c r="AI25" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ25" s="3" t="s">
         <v>52</v>
@@ -4191,7 +4248,7 @@
         <v>53</v>
       </c>
       <c r="AR25" s="3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:44" x14ac:dyDescent="0.3">
@@ -4202,19 +4259,19 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F26" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="G26" s="5">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>47</v>
@@ -4229,19 +4286,19 @@
         <v>50</v>
       </c>
       <c r="L26" s="6">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="M26" s="7">
-        <v>7337.61</v>
+        <v>2602.96</v>
       </c>
       <c r="N26" s="6">
         <v>1</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="P26" s="8">
-        <v>386.19</v>
+        <v>325.37</v>
       </c>
       <c r="Q26" s="6">
         <v>0</v>
@@ -4256,16 +4313,16 @@
         <v>52</v>
       </c>
       <c r="U26" s="10">
-        <v>67357</v>
+        <v>67488</v>
       </c>
       <c r="V26" s="11">
         <v>11</v>
       </c>
       <c r="W26" s="4">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="X26" s="12">
-        <v>0.4034722</v>
+        <v>0.44583329999999999</v>
       </c>
       <c r="Y26" s="10">
         <v>0</v>
@@ -4298,7 +4355,7 @@
         <v>53</v>
       </c>
       <c r="AI26" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="AJ26" s="3" t="s">
         <v>52</v>
@@ -4325,7 +4382,1749 @@
         <v>53</v>
       </c>
       <c r="AR26" s="3" t="s">
-        <v>81</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2">
+        <v>2</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G27" s="5">
+        <v>8</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L27" s="6">
+        <v>9</v>
+      </c>
+      <c r="M27" s="7">
+        <v>2928.33</v>
+      </c>
+      <c r="N27" s="6">
+        <v>1</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P27" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q27" s="6">
+        <v>0</v>
+      </c>
+      <c r="R27" s="7">
+        <v>0</v>
+      </c>
+      <c r="S27" s="9">
+        <v>0</v>
+      </c>
+      <c r="T27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U27" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V27" s="11">
+        <v>11</v>
+      </c>
+      <c r="W27" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X27" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y27" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG27" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR27" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2">
+        <v>2</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F28" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G28" s="5">
+        <v>9</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L28" s="6">
+        <v>10</v>
+      </c>
+      <c r="M28" s="7">
+        <v>3253.7</v>
+      </c>
+      <c r="N28" s="6">
+        <v>1</v>
+      </c>
+      <c r="O28" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P28" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="7">
+        <v>0</v>
+      </c>
+      <c r="S28" s="9">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U28" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V28" s="11">
+        <v>11</v>
+      </c>
+      <c r="W28" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X28" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y28" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG28" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK28" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM28" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR28" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>1</v>
+      </c>
+      <c r="B29" s="2">
+        <v>2</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G29" s="5">
+        <v>10</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L29" s="6">
+        <v>11</v>
+      </c>
+      <c r="M29" s="7">
+        <v>3579.07</v>
+      </c>
+      <c r="N29" s="6">
+        <v>1</v>
+      </c>
+      <c r="O29" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P29" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q29" s="6">
+        <v>0</v>
+      </c>
+      <c r="R29" s="7">
+        <v>0</v>
+      </c>
+      <c r="S29" s="9">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U29" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V29" s="11">
+        <v>11</v>
+      </c>
+      <c r="W29" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X29" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y29" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG29" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI29" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK29" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM29" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR29" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>1</v>
+      </c>
+      <c r="B30" s="2">
+        <v>2</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G30" s="5">
+        <v>11</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" s="6">
+        <v>12</v>
+      </c>
+      <c r="M30" s="7">
+        <v>3904.44</v>
+      </c>
+      <c r="N30" s="6">
+        <v>1</v>
+      </c>
+      <c r="O30" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P30" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="7">
+        <v>0</v>
+      </c>
+      <c r="S30" s="9">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U30" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V30" s="11">
+        <v>11</v>
+      </c>
+      <c r="W30" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X30" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y30" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG30" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI30" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK30" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM30" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR30" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2">
+        <v>2</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G31" s="5">
+        <v>12</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L31" s="6">
+        <v>13</v>
+      </c>
+      <c r="M31" s="7">
+        <v>4229.8100000000004</v>
+      </c>
+      <c r="N31" s="6">
+        <v>1</v>
+      </c>
+      <c r="O31" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P31" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q31" s="6">
+        <v>0</v>
+      </c>
+      <c r="R31" s="7">
+        <v>0</v>
+      </c>
+      <c r="S31" s="9">
+        <v>0</v>
+      </c>
+      <c r="T31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U31" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V31" s="11">
+        <v>11</v>
+      </c>
+      <c r="W31" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X31" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y31" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG31" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI31" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK31" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM31" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR31" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2">
+        <v>2</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G32" s="5">
+        <v>13</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L32" s="6">
+        <v>14</v>
+      </c>
+      <c r="M32" s="7">
+        <v>4555.18</v>
+      </c>
+      <c r="N32" s="6">
+        <v>1</v>
+      </c>
+      <c r="O32" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P32" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q32" s="6">
+        <v>0</v>
+      </c>
+      <c r="R32" s="7">
+        <v>0</v>
+      </c>
+      <c r="S32" s="9">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U32" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V32" s="11">
+        <v>11</v>
+      </c>
+      <c r="W32" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X32" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y32" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG32" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI32" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK32" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM32" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR32" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2">
+        <v>2</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G33" s="5">
+        <v>14</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L33" s="6">
+        <v>15</v>
+      </c>
+      <c r="M33" s="7">
+        <v>4880.55</v>
+      </c>
+      <c r="N33" s="6">
+        <v>1</v>
+      </c>
+      <c r="O33" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P33" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q33" s="6">
+        <v>0</v>
+      </c>
+      <c r="R33" s="7">
+        <v>0</v>
+      </c>
+      <c r="S33" s="9">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U33" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V33" s="11">
+        <v>11</v>
+      </c>
+      <c r="W33" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X33" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y33" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG33" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI33" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK33" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM33" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR33" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>1</v>
+      </c>
+      <c r="B34" s="2">
+        <v>2</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G34" s="5">
+        <v>15</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L34" s="6">
+        <v>16</v>
+      </c>
+      <c r="M34" s="7">
+        <v>5205.92</v>
+      </c>
+      <c r="N34" s="6">
+        <v>1</v>
+      </c>
+      <c r="O34" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P34" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q34" s="6">
+        <v>0</v>
+      </c>
+      <c r="R34" s="7">
+        <v>0</v>
+      </c>
+      <c r="S34" s="9">
+        <v>0</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U34" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V34" s="11">
+        <v>11</v>
+      </c>
+      <c r="W34" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X34" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y34" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG34" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI34" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK34" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM34" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR34" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2">
+        <v>2</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G35" s="5">
+        <v>16</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L35" s="6">
+        <v>17</v>
+      </c>
+      <c r="M35" s="7">
+        <v>5531.29</v>
+      </c>
+      <c r="N35" s="6">
+        <v>1</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P35" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q35" s="6">
+        <v>0</v>
+      </c>
+      <c r="R35" s="7">
+        <v>0</v>
+      </c>
+      <c r="S35" s="9">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U35" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V35" s="11">
+        <v>11</v>
+      </c>
+      <c r="W35" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X35" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y35" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI35" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR35" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>1</v>
+      </c>
+      <c r="B36" s="2">
+        <v>2</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F36" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G36" s="5">
+        <v>17</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L36" s="6">
+        <v>18</v>
+      </c>
+      <c r="M36" s="7">
+        <v>5856.66</v>
+      </c>
+      <c r="N36" s="6">
+        <v>1</v>
+      </c>
+      <c r="O36" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P36" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q36" s="6">
+        <v>0</v>
+      </c>
+      <c r="R36" s="7">
+        <v>0</v>
+      </c>
+      <c r="S36" s="9">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U36" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V36" s="11">
+        <v>11</v>
+      </c>
+      <c r="W36" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X36" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y36" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB36" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG36" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI36" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ36" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK36" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM36" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR36" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="37" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>1</v>
+      </c>
+      <c r="B37" s="2">
+        <v>2</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F37" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G37" s="5">
+        <v>18</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L37" s="6">
+        <v>19</v>
+      </c>
+      <c r="M37" s="7">
+        <v>6182.03</v>
+      </c>
+      <c r="N37" s="6">
+        <v>1</v>
+      </c>
+      <c r="O37" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P37" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q37" s="6">
+        <v>0</v>
+      </c>
+      <c r="R37" s="7">
+        <v>0</v>
+      </c>
+      <c r="S37" s="9">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U37" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V37" s="11">
+        <v>11</v>
+      </c>
+      <c r="W37" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X37" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y37" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG37" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI37" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK37" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM37" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR37" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>1</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F38" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G38" s="5">
+        <v>19</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L38" s="6">
+        <v>20</v>
+      </c>
+      <c r="M38" s="7">
+        <v>6507.4</v>
+      </c>
+      <c r="N38" s="6">
+        <v>1</v>
+      </c>
+      <c r="O38" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P38" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q38" s="6">
+        <v>0</v>
+      </c>
+      <c r="R38" s="7">
+        <v>0</v>
+      </c>
+      <c r="S38" s="9">
+        <v>0</v>
+      </c>
+      <c r="T38" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U38" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V38" s="11">
+        <v>11</v>
+      </c>
+      <c r="W38" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X38" s="12">
+        <v>0.44583329999999999</v>
+      </c>
+      <c r="Y38" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB38" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG38" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI38" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ38" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK38" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL38" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM38" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ38" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR38" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>1</v>
+      </c>
+      <c r="B39" s="2">
+        <v>2</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F39" s="4">
+        <v>46281</v>
+      </c>
+      <c r="G39" s="5">
+        <v>20</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L39" s="6">
+        <v>21</v>
+      </c>
+      <c r="M39" s="7">
+        <v>6832.77</v>
+      </c>
+      <c r="N39" s="6">
+        <v>1</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="P39" s="8">
+        <v>325.37</v>
+      </c>
+      <c r="Q39" s="6">
+        <v>0</v>
+      </c>
+      <c r="R39" s="7">
+        <v>0</v>
+      </c>
+      <c r="S39" s="9">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U39" s="10">
+        <v>67488</v>
+      </c>
+      <c r="V39" s="11">
+        <v>11</v>
+      </c>
+      <c r="W39" s="4">
+        <v>46281</v>
+      </c>
+      <c r="X39" s="12">
+        <v>0.4611111</v>
+      </c>
+      <c r="Y39" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG39" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI39" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AJ39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK39" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM39" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR39" s="3" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 17/09/2026 11:06:42,61
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EE76D23-1D9A-46DD-98F9-14E7E343F367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C4AA511D-7C10-4420-8CF1-6FF825804445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="91">
   <si>
     <t>Sel</t>
   </si>
@@ -154,10 +154,10 @@
     <t>Nº Série</t>
   </si>
   <si>
-    <t>10014979</t>
-  </si>
-  <si>
-    <t>2</t>
+    <t>10096354</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>500</t>
@@ -175,7 +175,7 @@
     <t>UN</t>
   </si>
   <si>
-    <t>FORNO ELETRICO NARDELLI TOP 40 40L BLACK - NARDELLI TOP 40 - 220 V</t>
+    <t>FORNO ELETRICO TERIM EMBUTIR 60L BLACK - 127 V</t>
   </si>
   <si>
     <t>100</t>
@@ -184,145 +184,115 @@
     <t/>
   </si>
   <si>
-    <t>FORNOS</t>
-  </si>
-  <si>
-    <t>1858600041542</t>
-  </si>
-  <si>
-    <t>10016351</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>FORNO ELETRICO NARDELLI EMBUTIR INOX 60 LITROS - NARDELLI EMBUTIR INOX 60 LITROS - 127 V</t>
-  </si>
-  <si>
     <t>FORNOE</t>
   </si>
   <si>
-    <t>1858400003510</t>
-  </si>
-  <si>
-    <t>1858400003511</t>
-  </si>
-  <si>
-    <t>1858400003512</t>
-  </si>
-  <si>
-    <t>1858400003513</t>
-  </si>
-  <si>
-    <t>1858400003514</t>
-  </si>
-  <si>
-    <t>1858400003515</t>
-  </si>
-  <si>
-    <t>1858400003516</t>
-  </si>
-  <si>
-    <t>10018965</t>
-  </si>
-  <si>
-    <t>FORNO ELETRICO NARDELLI E50 BLACK 50L - NARDELLI E50 BLACK 50 L - 220 V</t>
-  </si>
-  <si>
-    <t>1879900000465</t>
-  </si>
-  <si>
-    <t>1879900000466</t>
-  </si>
-  <si>
-    <t>1879900000467</t>
-  </si>
-  <si>
-    <t>1879900000468</t>
-  </si>
-  <si>
-    <t>1879900000469</t>
-  </si>
-  <si>
-    <t>1879900000470</t>
-  </si>
-  <si>
-    <t>1879900000471</t>
-  </si>
-  <si>
-    <t>1879900000472</t>
-  </si>
-  <si>
-    <t>1879900000473</t>
-  </si>
-  <si>
-    <t>1879900000474</t>
-  </si>
-  <si>
-    <t>10056354</t>
-  </si>
-  <si>
-    <t>FORNO ELETRICO FOGATTI EMBUTIR 60L BLACK - 127 V</t>
-  </si>
-  <si>
-    <t>1030900000070</t>
-  </si>
-  <si>
-    <t>1030900000071</t>
-  </si>
-  <si>
-    <t>1030900000072</t>
-  </si>
-  <si>
-    <t>1030900000073</t>
-  </si>
-  <si>
-    <t>1030900000074</t>
-  </si>
-  <si>
-    <t>1030900000075</t>
-  </si>
-  <si>
-    <t>1030900000076</t>
-  </si>
-  <si>
-    <t>1030900000077</t>
-  </si>
-  <si>
-    <t>1030900000078</t>
-  </si>
-  <si>
-    <t>1030900000079</t>
-  </si>
-  <si>
-    <t>1030900000080</t>
-  </si>
-  <si>
-    <t>1030900000081</t>
-  </si>
-  <si>
-    <t>1030900000082</t>
-  </si>
-  <si>
-    <t>1030900000083</t>
-  </si>
-  <si>
-    <t>1030900000084</t>
-  </si>
-  <si>
-    <t>1030900000085</t>
-  </si>
-  <si>
-    <t>1030900000086</t>
-  </si>
-  <si>
-    <t>1030900000087</t>
-  </si>
-  <si>
-    <t>1030900000088</t>
-  </si>
-  <si>
-    <t>1030900000089</t>
+    <t>1031100000267</t>
+  </si>
+  <si>
+    <t>1031100000268</t>
+  </si>
+  <si>
+    <t>1031100000269</t>
+  </si>
+  <si>
+    <t>1031100000270</t>
+  </si>
+  <si>
+    <t>1031100000271</t>
+  </si>
+  <si>
+    <t>1031100000272</t>
+  </si>
+  <si>
+    <t>1031100000273</t>
+  </si>
+  <si>
+    <t>1031100000274</t>
+  </si>
+  <si>
+    <t>1031100000275</t>
+  </si>
+  <si>
+    <t>1031100000276</t>
+  </si>
+  <si>
+    <t>1031100000277</t>
+  </si>
+  <si>
+    <t>1031100000278</t>
+  </si>
+  <si>
+    <t>1031100000279</t>
+  </si>
+  <si>
+    <t>1031100000280</t>
+  </si>
+  <si>
+    <t>1031100000281</t>
+  </si>
+  <si>
+    <t>1031100000282</t>
+  </si>
+  <si>
+    <t>1031100000283</t>
+  </si>
+  <si>
+    <t>1031100000284</t>
+  </si>
+  <si>
+    <t>1031100000285</t>
+  </si>
+  <si>
+    <t>1031100000286</t>
+  </si>
+  <si>
+    <t>1031100000287</t>
+  </si>
+  <si>
+    <t>1031100000288</t>
+  </si>
+  <si>
+    <t>1031100000289</t>
+  </si>
+  <si>
+    <t>1031100000290</t>
+  </si>
+  <si>
+    <t>1031100000291</t>
+  </si>
+  <si>
+    <t>1031100000292</t>
+  </si>
+  <si>
+    <t>1031100000293</t>
+  </si>
+  <si>
+    <t>1031100000294</t>
+  </si>
+  <si>
+    <t>1031100000295</t>
+  </si>
+  <si>
+    <t>1031100000296</t>
+  </si>
+  <si>
+    <t>1031100000297</t>
+  </si>
+  <si>
+    <t>1031100000298</t>
+  </si>
+  <si>
+    <t>1031100000299</t>
+  </si>
+  <si>
+    <t>1031100000300</t>
+  </si>
+  <si>
+    <t>1031100000301</t>
+  </si>
+  <si>
+    <t>1031100000302</t>
   </si>
 </sst>
 </file>
@@ -898,7 +868,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR39"/>
+  <dimension ref="A1:AR37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -1052,10 +1022,10 @@
         <v>46</v>
       </c>
       <c r="F2" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G2" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>47</v>
@@ -1070,10 +1040,10 @@
         <v>50</v>
       </c>
       <c r="L2" s="6">
-        <v>915</v>
+        <v>39</v>
       </c>
       <c r="M2" s="7">
-        <v>171252.21</v>
+        <v>14223.69</v>
       </c>
       <c r="N2" s="6">
         <v>1</v>
@@ -1082,7 +1052,7 @@
         <v>51</v>
       </c>
       <c r="P2" s="8">
-        <v>187.16</v>
+        <v>364.71</v>
       </c>
       <c r="Q2" s="6">
         <v>0</v>
@@ -1097,16 +1067,16 @@
         <v>52</v>
       </c>
       <c r="U2" s="10">
-        <v>67407</v>
+        <v>67518</v>
       </c>
       <c r="V2" s="11">
         <v>11</v>
       </c>
       <c r="W2" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X2" s="12">
-        <v>0.39027780000000001</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y2" s="10">
         <v>0</v>
@@ -1177,19 +1147,19 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F3" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G3" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>47</v>
@@ -1204,19 +1174,19 @@
         <v>50</v>
       </c>
       <c r="L3" s="6">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="M3" s="7">
-        <v>27544.42</v>
+        <v>14588.4</v>
       </c>
       <c r="N3" s="6">
         <v>1</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P3" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q3" s="6">
         <v>0</v>
@@ -1231,16 +1201,16 @@
         <v>52</v>
       </c>
       <c r="U3" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V3" s="11">
         <v>11</v>
       </c>
       <c r="W3" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X3" s="12">
-        <v>0.4583333</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y3" s="10">
         <v>0</v>
@@ -1273,7 +1243,7 @@
         <v>53</v>
       </c>
       <c r="AI3" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ3" s="3" t="s">
         <v>52</v>
@@ -1300,7 +1270,7 @@
         <v>53</v>
       </c>
       <c r="AR3" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1311,19 +1281,19 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F4" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G4" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>47</v>
@@ -1338,19 +1308,19 @@
         <v>50</v>
       </c>
       <c r="L4" s="6">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="M4" s="7">
-        <v>27921.74</v>
+        <v>14953.11</v>
       </c>
       <c r="N4" s="6">
         <v>1</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P4" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q4" s="6">
         <v>0</v>
@@ -1365,16 +1335,16 @@
         <v>52</v>
       </c>
       <c r="U4" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V4" s="11">
         <v>11</v>
       </c>
       <c r="W4" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X4" s="12">
-        <v>0.4583333</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y4" s="10">
         <v>0</v>
@@ -1407,7 +1377,7 @@
         <v>53</v>
       </c>
       <c r="AI4" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ4" s="3" t="s">
         <v>52</v>
@@ -1434,7 +1404,7 @@
         <v>53</v>
       </c>
       <c r="AR4" s="3" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1445,19 +1415,19 @@
         <v>2</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F5" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G5" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>47</v>
@@ -1472,19 +1442,19 @@
         <v>50</v>
       </c>
       <c r="L5" s="6">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="M5" s="7">
-        <v>28299.06</v>
+        <v>15317.82</v>
       </c>
       <c r="N5" s="6">
         <v>1</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P5" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q5" s="6">
         <v>0</v>
@@ -1499,16 +1469,16 @@
         <v>52</v>
       </c>
       <c r="U5" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V5" s="11">
         <v>11</v>
       </c>
       <c r="W5" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X5" s="12">
-        <v>0.4583333</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y5" s="10">
         <v>0</v>
@@ -1541,7 +1511,7 @@
         <v>53</v>
       </c>
       <c r="AI5" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ5" s="3" t="s">
         <v>52</v>
@@ -1568,7 +1538,7 @@
         <v>53</v>
       </c>
       <c r="AR5" s="3" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1579,19 +1549,19 @@
         <v>2</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F6" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G6" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>47</v>
@@ -1606,19 +1576,19 @@
         <v>50</v>
       </c>
       <c r="L6" s="6">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="M6" s="7">
-        <v>28676.39</v>
+        <v>15682.53</v>
       </c>
       <c r="N6" s="6">
         <v>1</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P6" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q6" s="6">
         <v>0</v>
@@ -1633,16 +1603,16 @@
         <v>52</v>
       </c>
       <c r="U6" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V6" s="11">
         <v>11</v>
       </c>
       <c r="W6" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X6" s="12">
-        <v>0.4583333</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y6" s="10">
         <v>0</v>
@@ -1675,34 +1645,34 @@
         <v>53</v>
       </c>
       <c r="AI6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK6" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL6" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM6" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ6" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR6" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="AJ6" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK6" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL6" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM6" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ6" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR6" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1713,19 +1683,19 @@
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F7" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G7" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>47</v>
@@ -1740,19 +1710,19 @@
         <v>50</v>
       </c>
       <c r="L7" s="6">
-        <v>77</v>
+        <v>44</v>
       </c>
       <c r="M7" s="7">
-        <v>29053.71</v>
+        <v>16047.24</v>
       </c>
       <c r="N7" s="6">
         <v>1</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P7" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q7" s="6">
         <v>0</v>
@@ -1767,16 +1737,16 @@
         <v>52</v>
       </c>
       <c r="U7" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V7" s="11">
         <v>11</v>
       </c>
       <c r="W7" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X7" s="12">
-        <v>0.4583333</v>
+        <v>0.32847219999999999</v>
       </c>
       <c r="Y7" s="10">
         <v>0</v>
@@ -1809,7 +1779,7 @@
         <v>53</v>
       </c>
       <c r="AI7" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ7" s="3" t="s">
         <v>52</v>
@@ -1836,7 +1806,7 @@
         <v>53</v>
       </c>
       <c r="AR7" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
@@ -1847,19 +1817,19 @@
         <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F8" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G8" s="5">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>47</v>
@@ -1874,19 +1844,19 @@
         <v>50</v>
       </c>
       <c r="L8" s="6">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="M8" s="7">
-        <v>29431.03</v>
+        <v>16411.95</v>
       </c>
       <c r="N8" s="6">
         <v>1</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P8" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q8" s="6">
         <v>0</v>
@@ -1901,16 +1871,16 @@
         <v>52</v>
       </c>
       <c r="U8" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V8" s="11">
         <v>11</v>
       </c>
       <c r="W8" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X8" s="12">
-        <v>0.4583333</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y8" s="10">
         <v>0</v>
@@ -1943,7 +1913,7 @@
         <v>53</v>
       </c>
       <c r="AI8" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ8" s="3" t="s">
         <v>52</v>
@@ -1970,7 +1940,7 @@
         <v>53</v>
       </c>
       <c r="AR8" s="3" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1981,19 +1951,19 @@
         <v>2</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F9" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G9" s="5">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>47</v>
@@ -2008,19 +1978,19 @@
         <v>50</v>
       </c>
       <c r="L9" s="6">
-        <v>79</v>
+        <v>46</v>
       </c>
       <c r="M9" s="7">
-        <v>29808.35</v>
+        <v>16776.66</v>
       </c>
       <c r="N9" s="6">
         <v>1</v>
       </c>
       <c r="O9" s="3" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="P9" s="8">
-        <v>377.32</v>
+        <v>364.71</v>
       </c>
       <c r="Q9" s="6">
         <v>0</v>
@@ -2035,16 +2005,16 @@
         <v>52</v>
       </c>
       <c r="U9" s="10">
-        <v>66798</v>
+        <v>67518</v>
       </c>
       <c r="V9" s="11">
         <v>11</v>
       </c>
       <c r="W9" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X9" s="12">
-        <v>0.4583333</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y9" s="10">
         <v>0</v>
@@ -2077,7 +2047,7 @@
         <v>53</v>
       </c>
       <c r="AI9" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ9" s="3" t="s">
         <v>52</v>
@@ -2104,7 +2074,7 @@
         <v>53</v>
       </c>
       <c r="AR9" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2115,7 +2085,7 @@
         <v>2</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>45</v>
@@ -2124,10 +2094,10 @@
         <v>46</v>
       </c>
       <c r="F10" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G10" s="5">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>47</v>
@@ -2142,19 +2112,19 @@
         <v>50</v>
       </c>
       <c r="L10" s="6">
-        <v>127</v>
+        <v>47</v>
       </c>
       <c r="M10" s="7">
-        <v>44105.13</v>
+        <v>17141.37</v>
       </c>
       <c r="N10" s="6">
         <v>1</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P10" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q10" s="6">
         <v>0</v>
@@ -2169,16 +2139,16 @@
         <v>52</v>
       </c>
       <c r="U10" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V10" s="11">
         <v>11</v>
       </c>
       <c r="W10" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X10" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y10" s="10">
         <v>0</v>
@@ -2211,7 +2181,7 @@
         <v>53</v>
       </c>
       <c r="AI10" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ10" s="3" t="s">
         <v>52</v>
@@ -2238,7 +2208,7 @@
         <v>53</v>
       </c>
       <c r="AR10" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2249,7 +2219,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>45</v>
@@ -2258,10 +2228,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G11" s="5">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>47</v>
@@ -2276,19 +2246,19 @@
         <v>50</v>
       </c>
       <c r="L11" s="6">
-        <v>128</v>
+        <v>48</v>
       </c>
       <c r="M11" s="7">
-        <v>44452.41</v>
+        <v>17506.080000000002</v>
       </c>
       <c r="N11" s="6">
         <v>1</v>
       </c>
       <c r="O11" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P11" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q11" s="6">
         <v>0</v>
@@ -2303,16 +2273,16 @@
         <v>52</v>
       </c>
       <c r="U11" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V11" s="11">
         <v>11</v>
       </c>
       <c r="W11" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X11" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y11" s="10">
         <v>0</v>
@@ -2345,7 +2315,7 @@
         <v>53</v>
       </c>
       <c r="AI11" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ11" s="3" t="s">
         <v>52</v>
@@ -2372,7 +2342,7 @@
         <v>53</v>
       </c>
       <c r="AR11" s="3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2383,7 +2353,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>45</v>
@@ -2392,10 +2362,10 @@
         <v>46</v>
       </c>
       <c r="F12" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G12" s="5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>47</v>
@@ -2410,19 +2380,19 @@
         <v>50</v>
       </c>
       <c r="L12" s="6">
-        <v>129</v>
+        <v>49</v>
       </c>
       <c r="M12" s="7">
-        <v>44799.7</v>
+        <v>17870.79</v>
       </c>
       <c r="N12" s="6">
         <v>1</v>
       </c>
       <c r="O12" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P12" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q12" s="6">
         <v>0</v>
@@ -2437,16 +2407,16 @@
         <v>52</v>
       </c>
       <c r="U12" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V12" s="11">
         <v>11</v>
       </c>
       <c r="W12" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X12" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y12" s="10">
         <v>0</v>
@@ -2479,7 +2449,7 @@
         <v>53</v>
       </c>
       <c r="AI12" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ12" s="3" t="s">
         <v>52</v>
@@ -2506,7 +2476,7 @@
         <v>53</v>
       </c>
       <c r="AR12" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2517,7 +2487,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>45</v>
@@ -2526,10 +2496,10 @@
         <v>46</v>
       </c>
       <c r="F13" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G13" s="5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>47</v>
@@ -2544,19 +2514,19 @@
         <v>50</v>
       </c>
       <c r="L13" s="6">
-        <v>130</v>
+        <v>50</v>
       </c>
       <c r="M13" s="7">
-        <v>45146.98</v>
+        <v>18235.5</v>
       </c>
       <c r="N13" s="6">
         <v>1</v>
       </c>
       <c r="O13" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P13" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q13" s="6">
         <v>0</v>
@@ -2571,16 +2541,16 @@
         <v>52</v>
       </c>
       <c r="U13" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V13" s="11">
         <v>11</v>
       </c>
       <c r="W13" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X13" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.37152780000000002</v>
       </c>
       <c r="Y13" s="10">
         <v>0</v>
@@ -2613,7 +2583,7 @@
         <v>53</v>
       </c>
       <c r="AI13" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ13" s="3" t="s">
         <v>52</v>
@@ -2640,7 +2610,7 @@
         <v>53</v>
       </c>
       <c r="AR13" s="3" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2651,7 +2621,7 @@
         <v>2</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>45</v>
@@ -2660,10 +2630,10 @@
         <v>46</v>
       </c>
       <c r="F14" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G14" s="5">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>47</v>
@@ -2678,19 +2648,19 @@
         <v>50</v>
       </c>
       <c r="L14" s="6">
-        <v>131</v>
+        <v>51</v>
       </c>
       <c r="M14" s="7">
-        <v>45494.27</v>
+        <v>18600.21</v>
       </c>
       <c r="N14" s="6">
         <v>1</v>
       </c>
       <c r="O14" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P14" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q14" s="6">
         <v>0</v>
@@ -2705,16 +2675,16 @@
         <v>52</v>
       </c>
       <c r="U14" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V14" s="11">
         <v>11</v>
       </c>
       <c r="W14" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X14" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y14" s="10">
         <v>0</v>
@@ -2747,7 +2717,7 @@
         <v>53</v>
       </c>
       <c r="AI14" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ14" s="3" t="s">
         <v>52</v>
@@ -2774,7 +2744,7 @@
         <v>53</v>
       </c>
       <c r="AR14" s="3" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -2785,7 +2755,7 @@
         <v>2</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>45</v>
@@ -2794,10 +2764,10 @@
         <v>46</v>
       </c>
       <c r="F15" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G15" s="5">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>47</v>
@@ -2812,19 +2782,19 @@
         <v>50</v>
       </c>
       <c r="L15" s="6">
-        <v>132</v>
+        <v>52</v>
       </c>
       <c r="M15" s="7">
-        <v>45841.55</v>
+        <v>18964.919999999998</v>
       </c>
       <c r="N15" s="6">
         <v>1</v>
       </c>
       <c r="O15" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P15" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q15" s="6">
         <v>0</v>
@@ -2839,16 +2809,16 @@
         <v>52</v>
       </c>
       <c r="U15" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V15" s="11">
         <v>11</v>
       </c>
       <c r="W15" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X15" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y15" s="10">
         <v>0</v>
@@ -2881,7 +2851,7 @@
         <v>53</v>
       </c>
       <c r="AI15" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ15" s="3" t="s">
         <v>52</v>
@@ -2908,7 +2878,7 @@
         <v>53</v>
       </c>
       <c r="AR15" s="3" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:44" x14ac:dyDescent="0.3">
@@ -2919,7 +2889,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>45</v>
@@ -2928,10 +2898,10 @@
         <v>46</v>
       </c>
       <c r="F16" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G16" s="5">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>47</v>
@@ -2946,19 +2916,19 @@
         <v>50</v>
       </c>
       <c r="L16" s="6">
-        <v>133</v>
+        <v>53</v>
       </c>
       <c r="M16" s="7">
-        <v>46188.83</v>
+        <v>19329.63</v>
       </c>
       <c r="N16" s="6">
         <v>1</v>
       </c>
       <c r="O16" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P16" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q16" s="6">
         <v>0</v>
@@ -2973,16 +2943,16 @@
         <v>52</v>
       </c>
       <c r="U16" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V16" s="11">
         <v>11</v>
       </c>
       <c r="W16" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X16" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y16" s="10">
         <v>0</v>
@@ -3015,7 +2985,7 @@
         <v>53</v>
       </c>
       <c r="AI16" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ16" s="3" t="s">
         <v>52</v>
@@ -3042,7 +3012,7 @@
         <v>53</v>
       </c>
       <c r="AR16" s="3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:44" x14ac:dyDescent="0.3">
@@ -3053,7 +3023,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>45</v>
@@ -3062,10 +3032,10 @@
         <v>46</v>
       </c>
       <c r="F17" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G17" s="5">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>47</v>
@@ -3080,19 +3050,19 @@
         <v>50</v>
       </c>
       <c r="L17" s="6">
-        <v>134</v>
+        <v>54</v>
       </c>
       <c r="M17" s="7">
-        <v>46536.12</v>
+        <v>19694.34</v>
       </c>
       <c r="N17" s="6">
         <v>1</v>
       </c>
       <c r="O17" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P17" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q17" s="6">
         <v>0</v>
@@ -3107,16 +3077,16 @@
         <v>52</v>
       </c>
       <c r="U17" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V17" s="11">
         <v>11</v>
       </c>
       <c r="W17" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X17" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y17" s="10">
         <v>0</v>
@@ -3149,7 +3119,7 @@
         <v>53</v>
       </c>
       <c r="AI17" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ17" s="3" t="s">
         <v>52</v>
@@ -3176,7 +3146,7 @@
         <v>53</v>
       </c>
       <c r="AR17" s="3" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:44" x14ac:dyDescent="0.3">
@@ -3187,7 +3157,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>45</v>
@@ -3196,10 +3166,10 @@
         <v>46</v>
       </c>
       <c r="F18" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G18" s="5">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>47</v>
@@ -3214,19 +3184,19 @@
         <v>50</v>
       </c>
       <c r="L18" s="6">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="M18" s="7">
-        <v>46883.4</v>
+        <v>20059.05</v>
       </c>
       <c r="N18" s="6">
         <v>1</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P18" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q18" s="6">
         <v>0</v>
@@ -3241,16 +3211,16 @@
         <v>52</v>
       </c>
       <c r="U18" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V18" s="11">
         <v>11</v>
       </c>
       <c r="W18" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X18" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y18" s="10">
         <v>0</v>
@@ -3283,7 +3253,7 @@
         <v>53</v>
       </c>
       <c r="AI18" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ18" s="3" t="s">
         <v>52</v>
@@ -3310,7 +3280,7 @@
         <v>53</v>
       </c>
       <c r="AR18" s="3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:44" x14ac:dyDescent="0.3">
@@ -3321,7 +3291,7 @@
         <v>2</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>45</v>
@@ -3330,10 +3300,10 @@
         <v>46</v>
       </c>
       <c r="F19" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G19" s="5">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>47</v>
@@ -3348,19 +3318,19 @@
         <v>50</v>
       </c>
       <c r="L19" s="6">
-        <v>136</v>
+        <v>56</v>
       </c>
       <c r="M19" s="7">
-        <v>47230.69</v>
+        <v>20423.759999999998</v>
       </c>
       <c r="N19" s="6">
         <v>1</v>
       </c>
       <c r="O19" s="3" t="s">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="P19" s="8">
-        <v>347.28</v>
+        <v>364.71</v>
       </c>
       <c r="Q19" s="6">
         <v>0</v>
@@ -3375,16 +3345,16 @@
         <v>52</v>
       </c>
       <c r="U19" s="10">
-        <v>67347</v>
+        <v>67518</v>
       </c>
       <c r="V19" s="11">
         <v>11</v>
       </c>
       <c r="W19" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X19" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y19" s="10">
         <v>0</v>
@@ -3417,7 +3387,7 @@
         <v>53</v>
       </c>
       <c r="AI19" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ19" s="3" t="s">
         <v>52</v>
@@ -3444,7 +3414,7 @@
         <v>53</v>
       </c>
       <c r="AR19" s="3" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:44" x14ac:dyDescent="0.3">
@@ -3455,19 +3425,19 @@
         <v>2</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F20" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G20" s="5">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>47</v>
@@ -3482,19 +3452,19 @@
         <v>50</v>
       </c>
       <c r="L20" s="6">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="M20" s="7">
-        <v>650.74</v>
+        <v>20788.47</v>
       </c>
       <c r="N20" s="6">
         <v>1</v>
       </c>
       <c r="O20" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P20" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q20" s="6">
         <v>0</v>
@@ -3509,16 +3479,16 @@
         <v>52</v>
       </c>
       <c r="U20" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V20" s="11">
         <v>11</v>
       </c>
       <c r="W20" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X20" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y20" s="10">
         <v>0</v>
@@ -3551,7 +3521,7 @@
         <v>53</v>
       </c>
       <c r="AI20" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ20" s="3" t="s">
         <v>52</v>
@@ -3578,7 +3548,7 @@
         <v>53</v>
       </c>
       <c r="AR20" s="3" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="21" spans="1:44" x14ac:dyDescent="0.3">
@@ -3589,19 +3559,19 @@
         <v>2</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F21" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G21" s="5">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>47</v>
@@ -3616,19 +3586,19 @@
         <v>50</v>
       </c>
       <c r="L21" s="6">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="M21" s="7">
-        <v>976.11</v>
+        <v>21153.18</v>
       </c>
       <c r="N21" s="6">
         <v>1</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P21" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q21" s="6">
         <v>0</v>
@@ -3643,16 +3613,16 @@
         <v>52</v>
       </c>
       <c r="U21" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V21" s="11">
         <v>11</v>
       </c>
       <c r="W21" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X21" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y21" s="10">
         <v>0</v>
@@ -3685,7 +3655,7 @@
         <v>53</v>
       </c>
       <c r="AI21" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ21" s="3" t="s">
         <v>52</v>
@@ -3712,7 +3682,7 @@
         <v>53</v>
       </c>
       <c r="AR21" s="3" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:44" x14ac:dyDescent="0.3">
@@ -3723,19 +3693,19 @@
         <v>2</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F22" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G22" s="5">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>47</v>
@@ -3750,19 +3720,19 @@
         <v>50</v>
       </c>
       <c r="L22" s="6">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="M22" s="7">
-        <v>1301.48</v>
+        <v>21517.89</v>
       </c>
       <c r="N22" s="6">
         <v>1</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P22" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q22" s="6">
         <v>0</v>
@@ -3777,16 +3747,16 @@
         <v>52</v>
       </c>
       <c r="U22" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V22" s="11">
         <v>11</v>
       </c>
       <c r="W22" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X22" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y22" s="10">
         <v>0</v>
@@ -3819,7 +3789,7 @@
         <v>53</v>
       </c>
       <c r="AI22" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ22" s="3" t="s">
         <v>52</v>
@@ -3846,7 +3816,7 @@
         <v>53</v>
       </c>
       <c r="AR22" s="3" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:44" x14ac:dyDescent="0.3">
@@ -3857,19 +3827,19 @@
         <v>2</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F23" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G23" s="5">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>47</v>
@@ -3884,19 +3854,19 @@
         <v>50</v>
       </c>
       <c r="L23" s="6">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="M23" s="7">
-        <v>1626.85</v>
+        <v>21882.6</v>
       </c>
       <c r="N23" s="6">
         <v>1</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P23" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q23" s="6">
         <v>0</v>
@@ -3911,16 +3881,16 @@
         <v>52</v>
       </c>
       <c r="U23" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V23" s="11">
         <v>11</v>
       </c>
       <c r="W23" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X23" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y23" s="10">
         <v>0</v>
@@ -3953,7 +3923,7 @@
         <v>53</v>
       </c>
       <c r="AI23" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ23" s="3" t="s">
         <v>52</v>
@@ -3980,7 +3950,7 @@
         <v>53</v>
       </c>
       <c r="AR23" s="3" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:44" x14ac:dyDescent="0.3">
@@ -3991,19 +3961,19 @@
         <v>2</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F24" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G24" s="5">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>47</v>
@@ -4018,19 +3988,19 @@
         <v>50</v>
       </c>
       <c r="L24" s="6">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="M24" s="7">
-        <v>1952.22</v>
+        <v>22247.31</v>
       </c>
       <c r="N24" s="6">
         <v>1</v>
       </c>
       <c r="O24" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P24" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q24" s="6">
         <v>0</v>
@@ -4045,16 +4015,16 @@
         <v>52</v>
       </c>
       <c r="U24" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V24" s="11">
         <v>11</v>
       </c>
       <c r="W24" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X24" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y24" s="10">
         <v>0</v>
@@ -4087,7 +4057,7 @@
         <v>53</v>
       </c>
       <c r="AI24" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ24" s="3" t="s">
         <v>52</v>
@@ -4114,7 +4084,7 @@
         <v>53</v>
       </c>
       <c r="AR24" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="25" spans="1:44" x14ac:dyDescent="0.3">
@@ -4125,19 +4095,19 @@
         <v>2</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F25" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G25" s="5">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>47</v>
@@ -4152,19 +4122,19 @@
         <v>50</v>
       </c>
       <c r="L25" s="6">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="M25" s="7">
-        <v>2277.59</v>
+        <v>22612.02</v>
       </c>
       <c r="N25" s="6">
         <v>1</v>
       </c>
       <c r="O25" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P25" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q25" s="6">
         <v>0</v>
@@ -4179,16 +4149,16 @@
         <v>52</v>
       </c>
       <c r="U25" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V25" s="11">
         <v>11</v>
       </c>
       <c r="W25" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X25" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.42152780000000001</v>
       </c>
       <c r="Y25" s="10">
         <v>0</v>
@@ -4221,7 +4191,7 @@
         <v>53</v>
       </c>
       <c r="AI25" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ25" s="3" t="s">
         <v>52</v>
@@ -4248,7 +4218,7 @@
         <v>53</v>
       </c>
       <c r="AR25" s="3" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:44" x14ac:dyDescent="0.3">
@@ -4259,19 +4229,19 @@
         <v>2</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F26" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G26" s="5">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>47</v>
@@ -4286,19 +4256,19 @@
         <v>50</v>
       </c>
       <c r="L26" s="6">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="M26" s="7">
-        <v>2602.96</v>
+        <v>22976.73</v>
       </c>
       <c r="N26" s="6">
         <v>1</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P26" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q26" s="6">
         <v>0</v>
@@ -4313,16 +4283,16 @@
         <v>52</v>
       </c>
       <c r="U26" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V26" s="11">
         <v>11</v>
       </c>
       <c r="W26" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X26" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y26" s="10">
         <v>0</v>
@@ -4355,7 +4325,7 @@
         <v>53</v>
       </c>
       <c r="AI26" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ26" s="3" t="s">
         <v>52</v>
@@ -4382,7 +4352,7 @@
         <v>53</v>
       </c>
       <c r="AR26" s="3" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:44" x14ac:dyDescent="0.3">
@@ -4393,19 +4363,19 @@
         <v>2</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F27" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G27" s="5">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>47</v>
@@ -4420,19 +4390,19 @@
         <v>50</v>
       </c>
       <c r="L27" s="6">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="M27" s="7">
-        <v>2928.33</v>
+        <v>23341.439999999999</v>
       </c>
       <c r="N27" s="6">
         <v>1</v>
       </c>
       <c r="O27" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P27" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q27" s="6">
         <v>0</v>
@@ -4447,16 +4417,16 @@
         <v>52</v>
       </c>
       <c r="U27" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V27" s="11">
         <v>11</v>
       </c>
       <c r="W27" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X27" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y27" s="10">
         <v>0</v>
@@ -4489,7 +4459,7 @@
         <v>53</v>
       </c>
       <c r="AI27" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ27" s="3" t="s">
         <v>52</v>
@@ -4516,7 +4486,7 @@
         <v>53</v>
       </c>
       <c r="AR27" s="3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:44" x14ac:dyDescent="0.3">
@@ -4527,19 +4497,19 @@
         <v>2</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F28" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G28" s="5">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>47</v>
@@ -4554,19 +4524,19 @@
         <v>50</v>
       </c>
       <c r="L28" s="6">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="M28" s="7">
-        <v>3253.7</v>
+        <v>23706.15</v>
       </c>
       <c r="N28" s="6">
         <v>1</v>
       </c>
       <c r="O28" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P28" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q28" s="6">
         <v>0</v>
@@ -4581,16 +4551,16 @@
         <v>52</v>
       </c>
       <c r="U28" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V28" s="11">
         <v>11</v>
       </c>
       <c r="W28" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X28" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y28" s="10">
         <v>0</v>
@@ -4623,7 +4593,7 @@
         <v>53</v>
       </c>
       <c r="AI28" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ28" s="3" t="s">
         <v>52</v>
@@ -4650,7 +4620,7 @@
         <v>53</v>
       </c>
       <c r="AR28" s="3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:44" x14ac:dyDescent="0.3">
@@ -4661,19 +4631,19 @@
         <v>2</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E29" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F29" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G29" s="5">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>47</v>
@@ -4688,19 +4658,19 @@
         <v>50</v>
       </c>
       <c r="L29" s="6">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="M29" s="7">
-        <v>3579.07</v>
+        <v>24070.86</v>
       </c>
       <c r="N29" s="6">
         <v>1</v>
       </c>
       <c r="O29" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P29" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q29" s="6">
         <v>0</v>
@@ -4715,16 +4685,16 @@
         <v>52</v>
       </c>
       <c r="U29" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V29" s="11">
         <v>11</v>
       </c>
       <c r="W29" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X29" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y29" s="10">
         <v>0</v>
@@ -4757,7 +4727,7 @@
         <v>53</v>
       </c>
       <c r="AI29" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ29" s="3" t="s">
         <v>52</v>
@@ -4784,7 +4754,7 @@
         <v>53</v>
       </c>
       <c r="AR29" s="3" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:44" x14ac:dyDescent="0.3">
@@ -4795,19 +4765,19 @@
         <v>2</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F30" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G30" s="5">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>47</v>
@@ -4822,19 +4792,19 @@
         <v>50</v>
       </c>
       <c r="L30" s="6">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="M30" s="7">
-        <v>3904.44</v>
+        <v>24435.57</v>
       </c>
       <c r="N30" s="6">
         <v>1</v>
       </c>
       <c r="O30" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P30" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q30" s="6">
         <v>0</v>
@@ -4849,16 +4819,16 @@
         <v>52</v>
       </c>
       <c r="U30" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V30" s="11">
         <v>11</v>
       </c>
       <c r="W30" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X30" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y30" s="10">
         <v>0</v>
@@ -4891,7 +4861,7 @@
         <v>53</v>
       </c>
       <c r="AI30" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ30" s="3" t="s">
         <v>52</v>
@@ -4918,7 +4888,7 @@
         <v>53</v>
       </c>
       <c r="AR30" s="3" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:44" x14ac:dyDescent="0.3">
@@ -4929,19 +4899,19 @@
         <v>2</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F31" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G31" s="5">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>47</v>
@@ -4956,19 +4926,19 @@
         <v>50</v>
       </c>
       <c r="L31" s="6">
-        <v>13</v>
+        <v>68</v>
       </c>
       <c r="M31" s="7">
-        <v>4229.8100000000004</v>
+        <v>24800.28</v>
       </c>
       <c r="N31" s="6">
         <v>1</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P31" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q31" s="6">
         <v>0</v>
@@ -4983,16 +4953,16 @@
         <v>52</v>
       </c>
       <c r="U31" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V31" s="11">
         <v>11</v>
       </c>
       <c r="W31" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X31" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y31" s="10">
         <v>0</v>
@@ -5025,7 +4995,7 @@
         <v>53</v>
       </c>
       <c r="AI31" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ31" s="3" t="s">
         <v>52</v>
@@ -5052,7 +5022,7 @@
         <v>53</v>
       </c>
       <c r="AR31" s="3" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:44" x14ac:dyDescent="0.3">
@@ -5063,19 +5033,19 @@
         <v>2</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F32" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G32" s="5">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>47</v>
@@ -5090,19 +5060,19 @@
         <v>50</v>
       </c>
       <c r="L32" s="6">
-        <v>14</v>
+        <v>69</v>
       </c>
       <c r="M32" s="7">
-        <v>4555.18</v>
+        <v>25164.99</v>
       </c>
       <c r="N32" s="6">
         <v>1</v>
       </c>
       <c r="O32" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P32" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q32" s="6">
         <v>0</v>
@@ -5117,16 +5087,16 @@
         <v>52</v>
       </c>
       <c r="U32" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V32" s="11">
         <v>11</v>
       </c>
       <c r="W32" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X32" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y32" s="10">
         <v>0</v>
@@ -5159,7 +5129,7 @@
         <v>53</v>
       </c>
       <c r="AI32" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ32" s="3" t="s">
         <v>52</v>
@@ -5186,7 +5156,7 @@
         <v>53</v>
       </c>
       <c r="AR32" s="3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="33" spans="1:44" x14ac:dyDescent="0.3">
@@ -5197,19 +5167,19 @@
         <v>2</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E33" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F33" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G33" s="5">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>47</v>
@@ -5224,19 +5194,19 @@
         <v>50</v>
       </c>
       <c r="L33" s="6">
-        <v>15</v>
+        <v>70</v>
       </c>
       <c r="M33" s="7">
-        <v>4880.55</v>
+        <v>25529.7</v>
       </c>
       <c r="N33" s="6">
         <v>1</v>
       </c>
       <c r="O33" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P33" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q33" s="6">
         <v>0</v>
@@ -5251,16 +5221,16 @@
         <v>52</v>
       </c>
       <c r="U33" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V33" s="11">
         <v>11</v>
       </c>
       <c r="W33" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X33" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y33" s="10">
         <v>0</v>
@@ -5293,7 +5263,7 @@
         <v>53</v>
       </c>
       <c r="AI33" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ33" s="3" t="s">
         <v>52</v>
@@ -5320,7 +5290,7 @@
         <v>53</v>
       </c>
       <c r="AR33" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:44" x14ac:dyDescent="0.3">
@@ -5331,19 +5301,19 @@
         <v>2</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F34" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G34" s="5">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>47</v>
@@ -5358,19 +5328,19 @@
         <v>50</v>
       </c>
       <c r="L34" s="6">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="M34" s="7">
-        <v>5205.92</v>
+        <v>25894.41</v>
       </c>
       <c r="N34" s="6">
         <v>1</v>
       </c>
       <c r="O34" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P34" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q34" s="6">
         <v>0</v>
@@ -5385,16 +5355,16 @@
         <v>52</v>
       </c>
       <c r="U34" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V34" s="11">
         <v>11</v>
       </c>
       <c r="W34" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X34" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y34" s="10">
         <v>0</v>
@@ -5427,7 +5397,7 @@
         <v>53</v>
       </c>
       <c r="AI34" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ34" s="3" t="s">
         <v>52</v>
@@ -5454,7 +5424,7 @@
         <v>53</v>
       </c>
       <c r="AR34" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="35" spans="1:44" x14ac:dyDescent="0.3">
@@ -5465,19 +5435,19 @@
         <v>2</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E35" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F35" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G35" s="5">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>47</v>
@@ -5492,19 +5462,19 @@
         <v>50</v>
       </c>
       <c r="L35" s="6">
-        <v>17</v>
+        <v>72</v>
       </c>
       <c r="M35" s="7">
-        <v>5531.29</v>
+        <v>26259.119999999999</v>
       </c>
       <c r="N35" s="6">
         <v>1</v>
       </c>
       <c r="O35" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P35" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q35" s="6">
         <v>0</v>
@@ -5519,16 +5489,16 @@
         <v>52</v>
       </c>
       <c r="U35" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V35" s="11">
         <v>11</v>
       </c>
       <c r="W35" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X35" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y35" s="10">
         <v>0</v>
@@ -5561,7 +5531,7 @@
         <v>53</v>
       </c>
       <c r="AI35" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ35" s="3" t="s">
         <v>52</v>
@@ -5588,7 +5558,7 @@
         <v>53</v>
       </c>
       <c r="AR35" s="3" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:44" x14ac:dyDescent="0.3">
@@ -5599,19 +5569,19 @@
         <v>2</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F36" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G36" s="5">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>47</v>
@@ -5626,19 +5596,19 @@
         <v>50</v>
       </c>
       <c r="L36" s="6">
-        <v>18</v>
+        <v>73</v>
       </c>
       <c r="M36" s="7">
-        <v>5856.66</v>
+        <v>26623.83</v>
       </c>
       <c r="N36" s="6">
         <v>1</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P36" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q36" s="6">
         <v>0</v>
@@ -5653,16 +5623,16 @@
         <v>52</v>
       </c>
       <c r="U36" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V36" s="11">
         <v>11</v>
       </c>
       <c r="W36" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X36" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y36" s="10">
         <v>0</v>
@@ -5695,7 +5665,7 @@
         <v>53</v>
       </c>
       <c r="AI36" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ36" s="3" t="s">
         <v>52</v>
@@ -5722,7 +5692,7 @@
         <v>53</v>
       </c>
       <c r="AR36" s="3" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.3">
@@ -5733,19 +5703,19 @@
         <v>2</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>79</v>
+        <v>44</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F37" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="G37" s="5">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>47</v>
@@ -5760,19 +5730,19 @@
         <v>50</v>
       </c>
       <c r="L37" s="6">
-        <v>19</v>
+        <v>74</v>
       </c>
       <c r="M37" s="7">
-        <v>6182.03</v>
+        <v>26988.54</v>
       </c>
       <c r="N37" s="6">
         <v>1</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="P37" s="8">
-        <v>325.37</v>
+        <v>364.71</v>
       </c>
       <c r="Q37" s="6">
         <v>0</v>
@@ -5787,16 +5757,16 @@
         <v>52</v>
       </c>
       <c r="U37" s="10">
-        <v>67488</v>
+        <v>67518</v>
       </c>
       <c r="V37" s="11">
         <v>11</v>
       </c>
       <c r="W37" s="4">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="X37" s="12">
-        <v>0.44583329999999999</v>
+        <v>0.46180559999999998</v>
       </c>
       <c r="Y37" s="10">
         <v>0</v>
@@ -5829,7 +5799,7 @@
         <v>53</v>
       </c>
       <c r="AI37" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="AJ37" s="3" t="s">
         <v>52</v>
@@ -5856,275 +5826,7 @@
         <v>53</v>
       </c>
       <c r="AR37" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
-        <v>1</v>
-      </c>
-      <c r="B38" s="2">
-        <v>2</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F38" s="4">
-        <v>46281</v>
-      </c>
-      <c r="G38" s="5">
-        <v>19</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K38" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L38" s="6">
-        <v>20</v>
-      </c>
-      <c r="M38" s="7">
-        <v>6507.4</v>
-      </c>
-      <c r="N38" s="6">
-        <v>1</v>
-      </c>
-      <c r="O38" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="P38" s="8">
-        <v>325.37</v>
-      </c>
-      <c r="Q38" s="6">
-        <v>0</v>
-      </c>
-      <c r="R38" s="7">
-        <v>0</v>
-      </c>
-      <c r="S38" s="9">
-        <v>0</v>
-      </c>
-      <c r="T38" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="U38" s="10">
-        <v>67488</v>
-      </c>
-      <c r="V38" s="11">
-        <v>11</v>
-      </c>
-      <c r="W38" s="4">
-        <v>46281</v>
-      </c>
-      <c r="X38" s="12">
-        <v>0.44583329999999999</v>
-      </c>
-      <c r="Y38" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB38" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG38" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI38" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AJ38" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK38" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL38" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM38" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ38" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR38" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="39" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
-        <v>1</v>
-      </c>
-      <c r="B39" s="2">
-        <v>2</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F39" s="4">
-        <v>46281</v>
-      </c>
-      <c r="G39" s="5">
-        <v>20</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K39" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L39" s="6">
-        <v>21</v>
-      </c>
-      <c r="M39" s="7">
-        <v>6832.77</v>
-      </c>
-      <c r="N39" s="6">
-        <v>1</v>
-      </c>
-      <c r="O39" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="P39" s="8">
-        <v>325.37</v>
-      </c>
-      <c r="Q39" s="6">
-        <v>0</v>
-      </c>
-      <c r="R39" s="7">
-        <v>0</v>
-      </c>
-      <c r="S39" s="9">
-        <v>0</v>
-      </c>
-      <c r="T39" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="U39" s="10">
-        <v>67488</v>
-      </c>
-      <c r="V39" s="11">
-        <v>11</v>
-      </c>
-      <c r="W39" s="4">
-        <v>46281</v>
-      </c>
-      <c r="X39" s="12">
-        <v>0.4611111</v>
-      </c>
-      <c r="Y39" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB39" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG39" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI39" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="AJ39" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK39" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL39" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM39" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ39" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR39" s="3" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 21/09/2026 13:49:51,39
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{47490F82-4881-428F-BFA1-9FB160A65523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E589B419-BF85-4E70-AAF1-541DC232E3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9494" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9638" uniqueCount="597">
   <si>
     <t>Sel</t>
   </si>
@@ -1723,6 +1723,30 @@
     <t>1883700000042</t>
   </si>
   <si>
+    <t>1883700000043</t>
+  </si>
+  <si>
+    <t>1883700000044</t>
+  </si>
+  <si>
+    <t>1883700000045</t>
+  </si>
+  <si>
+    <t>1883700000046</t>
+  </si>
+  <si>
+    <t>1883700000047</t>
+  </si>
+  <si>
+    <t>1883700000048</t>
+  </si>
+  <si>
+    <t>1883700000049</t>
+  </si>
+  <si>
+    <t>1883700000050</t>
+  </si>
+  <si>
     <t>10099364</t>
   </si>
   <si>
@@ -2362,7 +2386,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR526"/>
+  <dimension ref="A1:AR534"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -70177,7 +70201,7 @@
         <v>2</v>
       </c>
       <c r="C507" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D507" s="3" t="s">
         <v>151</v>
@@ -70189,7 +70213,7 @@
         <v>46286</v>
       </c>
       <c r="G507" s="5">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H507" s="3" t="s">
         <v>47</v>
@@ -70204,16 +70228,16 @@
         <v>50</v>
       </c>
       <c r="L507" s="6">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="M507" s="7">
-        <v>0</v>
+        <v>4310.3999999999996</v>
       </c>
       <c r="N507" s="6">
         <v>1</v>
       </c>
       <c r="O507" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P507" s="8">
         <v>179.6</v>
@@ -70231,7 +70255,7 @@
         <v>52</v>
       </c>
       <c r="U507" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V507" s="11">
         <v>11</v>
@@ -70240,7 +70264,7 @@
         <v>46286</v>
       </c>
       <c r="X507" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y507" s="10">
         <v>0</v>
@@ -70300,7 +70324,7 @@
         <v>53</v>
       </c>
       <c r="AR507" s="3" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="508" spans="1:44" x14ac:dyDescent="0.3">
@@ -70311,7 +70335,7 @@
         <v>2</v>
       </c>
       <c r="C508" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D508" s="3" t="s">
         <v>151</v>
@@ -70323,7 +70347,7 @@
         <v>46286</v>
       </c>
       <c r="G508" s="5">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="H508" s="3" t="s">
         <v>47</v>
@@ -70338,16 +70362,16 @@
         <v>50</v>
       </c>
       <c r="L508" s="6">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="M508" s="7">
-        <v>179.6</v>
+        <v>4490</v>
       </c>
       <c r="N508" s="6">
         <v>1</v>
       </c>
       <c r="O508" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P508" s="8">
         <v>179.6</v>
@@ -70365,7 +70389,7 @@
         <v>52</v>
       </c>
       <c r="U508" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V508" s="11">
         <v>11</v>
@@ -70374,7 +70398,7 @@
         <v>46286</v>
       </c>
       <c r="X508" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y508" s="10">
         <v>0</v>
@@ -70434,7 +70458,7 @@
         <v>53</v>
       </c>
       <c r="AR508" s="3" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
     </row>
     <row r="509" spans="1:44" x14ac:dyDescent="0.3">
@@ -70445,7 +70469,7 @@
         <v>2</v>
       </c>
       <c r="C509" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D509" s="3" t="s">
         <v>151</v>
@@ -70457,7 +70481,7 @@
         <v>46286</v>
       </c>
       <c r="G509" s="5">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="H509" s="3" t="s">
         <v>47</v>
@@ -70472,16 +70496,16 @@
         <v>50</v>
       </c>
       <c r="L509" s="6">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="M509" s="7">
-        <v>359.2</v>
+        <v>4669.6000000000004</v>
       </c>
       <c r="N509" s="6">
         <v>1</v>
       </c>
       <c r="O509" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P509" s="8">
         <v>179.6</v>
@@ -70499,7 +70523,7 @@
         <v>52</v>
       </c>
       <c r="U509" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V509" s="11">
         <v>11</v>
@@ -70508,7 +70532,7 @@
         <v>46286</v>
       </c>
       <c r="X509" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y509" s="10">
         <v>0</v>
@@ -70568,7 +70592,7 @@
         <v>53</v>
       </c>
       <c r="AR509" s="3" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="510" spans="1:44" x14ac:dyDescent="0.3">
@@ -70579,7 +70603,7 @@
         <v>2</v>
       </c>
       <c r="C510" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D510" s="3" t="s">
         <v>151</v>
@@ -70591,7 +70615,7 @@
         <v>46286</v>
       </c>
       <c r="G510" s="5">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="H510" s="3" t="s">
         <v>47</v>
@@ -70606,16 +70630,16 @@
         <v>50</v>
       </c>
       <c r="L510" s="6">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="M510" s="7">
-        <v>538.79999999999995</v>
+        <v>4849.2</v>
       </c>
       <c r="N510" s="6">
         <v>1</v>
       </c>
       <c r="O510" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P510" s="8">
         <v>179.6</v>
@@ -70633,7 +70657,7 @@
         <v>52</v>
       </c>
       <c r="U510" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V510" s="11">
         <v>11</v>
@@ -70642,7 +70666,7 @@
         <v>46286</v>
       </c>
       <c r="X510" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y510" s="10">
         <v>0</v>
@@ -70702,7 +70726,7 @@
         <v>53</v>
       </c>
       <c r="AR510" s="3" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
     </row>
     <row r="511" spans="1:44" x14ac:dyDescent="0.3">
@@ -70713,7 +70737,7 @@
         <v>2</v>
       </c>
       <c r="C511" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D511" s="3" t="s">
         <v>151</v>
@@ -70725,7 +70749,7 @@
         <v>46286</v>
       </c>
       <c r="G511" s="5">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="H511" s="3" t="s">
         <v>47</v>
@@ -70740,16 +70764,16 @@
         <v>50</v>
       </c>
       <c r="L511" s="6">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="M511" s="7">
-        <v>718.4</v>
+        <v>5028.8</v>
       </c>
       <c r="N511" s="6">
         <v>1</v>
       </c>
       <c r="O511" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P511" s="8">
         <v>179.6</v>
@@ -70767,7 +70791,7 @@
         <v>52</v>
       </c>
       <c r="U511" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V511" s="11">
         <v>11</v>
@@ -70776,7 +70800,7 @@
         <v>46286</v>
       </c>
       <c r="X511" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y511" s="10">
         <v>0</v>
@@ -70836,7 +70860,7 @@
         <v>53</v>
       </c>
       <c r="AR511" s="3" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="512" spans="1:44" x14ac:dyDescent="0.3">
@@ -70847,7 +70871,7 @@
         <v>2</v>
       </c>
       <c r="C512" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D512" s="3" t="s">
         <v>151</v>
@@ -70859,7 +70883,7 @@
         <v>46286</v>
       </c>
       <c r="G512" s="5">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="H512" s="3" t="s">
         <v>47</v>
@@ -70874,16 +70898,16 @@
         <v>50</v>
       </c>
       <c r="L512" s="6">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="M512" s="7">
-        <v>898</v>
+        <v>5208.3999999999996</v>
       </c>
       <c r="N512" s="6">
         <v>1</v>
       </c>
       <c r="O512" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P512" s="8">
         <v>179.6</v>
@@ -70901,7 +70925,7 @@
         <v>52</v>
       </c>
       <c r="U512" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V512" s="11">
         <v>11</v>
@@ -70910,7 +70934,7 @@
         <v>46286</v>
       </c>
       <c r="X512" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y512" s="10">
         <v>0</v>
@@ -70970,7 +70994,7 @@
         <v>53</v>
       </c>
       <c r="AR512" s="3" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="513" spans="1:44" x14ac:dyDescent="0.3">
@@ -70981,7 +71005,7 @@
         <v>2</v>
       </c>
       <c r="C513" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D513" s="3" t="s">
         <v>151</v>
@@ -70993,7 +71017,7 @@
         <v>46286</v>
       </c>
       <c r="G513" s="5">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="H513" s="3" t="s">
         <v>47</v>
@@ -71008,16 +71032,16 @@
         <v>50</v>
       </c>
       <c r="L513" s="6">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="M513" s="7">
-        <v>1077.5999999999999</v>
+        <v>5388</v>
       </c>
       <c r="N513" s="6">
         <v>1</v>
       </c>
       <c r="O513" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P513" s="8">
         <v>179.6</v>
@@ -71035,7 +71059,7 @@
         <v>52</v>
       </c>
       <c r="U513" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V513" s="11">
         <v>11</v>
@@ -71044,7 +71068,7 @@
         <v>46286</v>
       </c>
       <c r="X513" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y513" s="10">
         <v>0</v>
@@ -71104,7 +71128,7 @@
         <v>53</v>
       </c>
       <c r="AR513" s="3" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="514" spans="1:44" x14ac:dyDescent="0.3">
@@ -71115,7 +71139,7 @@
         <v>2</v>
       </c>
       <c r="C514" s="3" t="s">
-        <v>567</v>
+        <v>541</v>
       </c>
       <c r="D514" s="3" t="s">
         <v>151</v>
@@ -71127,7 +71151,7 @@
         <v>46286</v>
       </c>
       <c r="G514" s="5">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="H514" s="3" t="s">
         <v>47</v>
@@ -71142,16 +71166,16 @@
         <v>50</v>
       </c>
       <c r="L514" s="6">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="M514" s="7">
-        <v>1257.2</v>
+        <v>5567.6</v>
       </c>
       <c r="N514" s="6">
         <v>1</v>
       </c>
       <c r="O514" s="3" t="s">
-        <v>568</v>
+        <v>542</v>
       </c>
       <c r="P514" s="8">
         <v>179.6</v>
@@ -71169,7 +71193,7 @@
         <v>52</v>
       </c>
       <c r="U514" s="10">
-        <v>67522</v>
+        <v>67517</v>
       </c>
       <c r="V514" s="11">
         <v>11</v>
@@ -71178,7 +71202,7 @@
         <v>46286</v>
       </c>
       <c r="X514" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.54027780000000003</v>
       </c>
       <c r="Y514" s="10">
         <v>0</v>
@@ -71238,7 +71262,7 @@
         <v>53</v>
       </c>
       <c r="AR514" s="3" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
     </row>
     <row r="515" spans="1:44" x14ac:dyDescent="0.3">
@@ -71249,7 +71273,7 @@
         <v>2</v>
       </c>
       <c r="C515" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D515" s="3" t="s">
         <v>151</v>
@@ -71261,7 +71285,7 @@
         <v>46286</v>
       </c>
       <c r="G515" s="5">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H515" s="3" t="s">
         <v>47</v>
@@ -71276,16 +71300,16 @@
         <v>50</v>
       </c>
       <c r="L515" s="6">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M515" s="7">
-        <v>1436.8</v>
+        <v>0</v>
       </c>
       <c r="N515" s="6">
         <v>1</v>
       </c>
       <c r="O515" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P515" s="8">
         <v>179.6</v>
@@ -71312,7 +71336,7 @@
         <v>46286</v>
       </c>
       <c r="X515" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y515" s="10">
         <v>0</v>
@@ -71383,7 +71407,7 @@
         <v>2</v>
       </c>
       <c r="C516" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D516" s="3" t="s">
         <v>151</v>
@@ -71395,7 +71419,7 @@
         <v>46286</v>
       </c>
       <c r="G516" s="5">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H516" s="3" t="s">
         <v>47</v>
@@ -71410,16 +71434,16 @@
         <v>50</v>
       </c>
       <c r="L516" s="6">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="M516" s="7">
-        <v>1616.4</v>
+        <v>179.6</v>
       </c>
       <c r="N516" s="6">
         <v>1</v>
       </c>
       <c r="O516" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P516" s="8">
         <v>179.6</v>
@@ -71446,7 +71470,7 @@
         <v>46286</v>
       </c>
       <c r="X516" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y516" s="10">
         <v>0</v>
@@ -71517,7 +71541,7 @@
         <v>2</v>
       </c>
       <c r="C517" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D517" s="3" t="s">
         <v>151</v>
@@ -71529,7 +71553,7 @@
         <v>46286</v>
       </c>
       <c r="G517" s="5">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H517" s="3" t="s">
         <v>47</v>
@@ -71544,16 +71568,16 @@
         <v>50</v>
       </c>
       <c r="L517" s="6">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="M517" s="7">
-        <v>1796</v>
+        <v>359.2</v>
       </c>
       <c r="N517" s="6">
         <v>1</v>
       </c>
       <c r="O517" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P517" s="8">
         <v>179.6</v>
@@ -71580,7 +71604,7 @@
         <v>46286</v>
       </c>
       <c r="X517" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y517" s="10">
         <v>0</v>
@@ -71651,7 +71675,7 @@
         <v>2</v>
       </c>
       <c r="C518" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D518" s="3" t="s">
         <v>151</v>
@@ -71663,7 +71687,7 @@
         <v>46286</v>
       </c>
       <c r="G518" s="5">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H518" s="3" t="s">
         <v>47</v>
@@ -71678,16 +71702,16 @@
         <v>50</v>
       </c>
       <c r="L518" s="6">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="M518" s="7">
-        <v>1975.6</v>
+        <v>538.79999999999995</v>
       </c>
       <c r="N518" s="6">
         <v>1</v>
       </c>
       <c r="O518" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P518" s="8">
         <v>179.6</v>
@@ -71714,7 +71738,7 @@
         <v>46286</v>
       </c>
       <c r="X518" s="12">
-        <v>0.36805559999999998</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y518" s="10">
         <v>0</v>
@@ -71785,7 +71809,7 @@
         <v>2</v>
       </c>
       <c r="C519" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D519" s="3" t="s">
         <v>151</v>
@@ -71797,7 +71821,7 @@
         <v>46286</v>
       </c>
       <c r="G519" s="5">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H519" s="3" t="s">
         <v>47</v>
@@ -71812,16 +71836,16 @@
         <v>50</v>
       </c>
       <c r="L519" s="6">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="M519" s="7">
-        <v>2155.1999999999998</v>
+        <v>718.4</v>
       </c>
       <c r="N519" s="6">
         <v>1</v>
       </c>
       <c r="O519" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P519" s="8">
         <v>179.6</v>
@@ -71848,7 +71872,7 @@
         <v>46286</v>
       </c>
       <c r="X519" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y519" s="10">
         <v>0</v>
@@ -71919,7 +71943,7 @@
         <v>2</v>
       </c>
       <c r="C520" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D520" s="3" t="s">
         <v>151</v>
@@ -71931,7 +71955,7 @@
         <v>46286</v>
       </c>
       <c r="G520" s="5">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H520" s="3" t="s">
         <v>47</v>
@@ -71946,16 +71970,16 @@
         <v>50</v>
       </c>
       <c r="L520" s="6">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M520" s="7">
-        <v>2334.8000000000002</v>
+        <v>898</v>
       </c>
       <c r="N520" s="6">
         <v>1</v>
       </c>
       <c r="O520" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P520" s="8">
         <v>179.6</v>
@@ -71982,7 +72006,7 @@
         <v>46286</v>
       </c>
       <c r="X520" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y520" s="10">
         <v>0</v>
@@ -72053,7 +72077,7 @@
         <v>2</v>
       </c>
       <c r="C521" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D521" s="3" t="s">
         <v>151</v>
@@ -72065,7 +72089,7 @@
         <v>46286</v>
       </c>
       <c r="G521" s="5">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H521" s="3" t="s">
         <v>47</v>
@@ -72080,16 +72104,16 @@
         <v>50</v>
       </c>
       <c r="L521" s="6">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="M521" s="7">
-        <v>2514.4</v>
+        <v>1077.5999999999999</v>
       </c>
       <c r="N521" s="6">
         <v>1</v>
       </c>
       <c r="O521" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P521" s="8">
         <v>179.6</v>
@@ -72116,7 +72140,7 @@
         <v>46286</v>
       </c>
       <c r="X521" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y521" s="10">
         <v>0</v>
@@ -72187,7 +72211,7 @@
         <v>2</v>
       </c>
       <c r="C522" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D522" s="3" t="s">
         <v>151</v>
@@ -72199,7 +72223,7 @@
         <v>46286</v>
       </c>
       <c r="G522" s="5">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H522" s="3" t="s">
         <v>47</v>
@@ -72214,16 +72238,16 @@
         <v>50</v>
       </c>
       <c r="L522" s="6">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="M522" s="7">
-        <v>2694</v>
+        <v>1257.2</v>
       </c>
       <c r="N522" s="6">
         <v>1</v>
       </c>
       <c r="O522" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P522" s="8">
         <v>179.6</v>
@@ -72250,7 +72274,7 @@
         <v>46286</v>
       </c>
       <c r="X522" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y522" s="10">
         <v>0</v>
@@ -72321,7 +72345,7 @@
         <v>2</v>
       </c>
       <c r="C523" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D523" s="3" t="s">
         <v>151</v>
@@ -72333,7 +72357,7 @@
         <v>46286</v>
       </c>
       <c r="G523" s="5">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H523" s="3" t="s">
         <v>47</v>
@@ -72348,16 +72372,16 @@
         <v>50</v>
       </c>
       <c r="L523" s="6">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M523" s="7">
-        <v>2873.6</v>
+        <v>1436.8</v>
       </c>
       <c r="N523" s="6">
         <v>1</v>
       </c>
       <c r="O523" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P523" s="8">
         <v>179.6</v>
@@ -72384,7 +72408,7 @@
         <v>46286</v>
       </c>
       <c r="X523" s="12">
-        <v>0.40277780000000002</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y523" s="10">
         <v>0</v>
@@ -72455,7 +72479,7 @@
         <v>2</v>
       </c>
       <c r="C524" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D524" s="3" t="s">
         <v>151</v>
@@ -72467,7 +72491,7 @@
         <v>46286</v>
       </c>
       <c r="G524" s="5">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H524" s="3" t="s">
         <v>47</v>
@@ -72482,16 +72506,16 @@
         <v>50</v>
       </c>
       <c r="L524" s="6">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="M524" s="7">
-        <v>3053.2</v>
+        <v>1616.4</v>
       </c>
       <c r="N524" s="6">
         <v>1</v>
       </c>
       <c r="O524" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P524" s="8">
         <v>179.6</v>
@@ -72518,7 +72542,7 @@
         <v>46286</v>
       </c>
       <c r="X524" s="12">
-        <v>0.42361110000000002</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y524" s="10">
         <v>0</v>
@@ -72589,7 +72613,7 @@
         <v>2</v>
       </c>
       <c r="C525" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D525" s="3" t="s">
         <v>151</v>
@@ -72601,7 +72625,7 @@
         <v>46286</v>
       </c>
       <c r="G525" s="5">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H525" s="3" t="s">
         <v>47</v>
@@ -72616,16 +72640,16 @@
         <v>50</v>
       </c>
       <c r="L525" s="6">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="M525" s="7">
-        <v>3232.8</v>
+        <v>1796</v>
       </c>
       <c r="N525" s="6">
         <v>1</v>
       </c>
       <c r="O525" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P525" s="8">
         <v>179.6</v>
@@ -72652,7 +72676,7 @@
         <v>46286</v>
       </c>
       <c r="X525" s="12">
-        <v>0.42361110000000002</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y525" s="10">
         <v>0</v>
@@ -72723,7 +72747,7 @@
         <v>2</v>
       </c>
       <c r="C526" s="3" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="D526" s="3" t="s">
         <v>151</v>
@@ -72735,7 +72759,7 @@
         <v>46286</v>
       </c>
       <c r="G526" s="5">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H526" s="3" t="s">
         <v>47</v>
@@ -72750,16 +72774,16 @@
         <v>50</v>
       </c>
       <c r="L526" s="6">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="M526" s="7">
-        <v>3412.4</v>
+        <v>1975.6</v>
       </c>
       <c r="N526" s="6">
         <v>1</v>
       </c>
       <c r="O526" s="3" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="P526" s="8">
         <v>179.6</v>
@@ -72786,7 +72810,7 @@
         <v>46286</v>
       </c>
       <c r="X526" s="12">
-        <v>0.48472219999999999</v>
+        <v>0.36805559999999998</v>
       </c>
       <c r="Y526" s="10">
         <v>0</v>
@@ -72847,6 +72871,1078 @@
       </c>
       <c r="AR526" s="3" t="s">
         <v>588</v>
+      </c>
+    </row>
+    <row r="527" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A527" s="1">
+        <v>1</v>
+      </c>
+      <c r="B527" s="2">
+        <v>2</v>
+      </c>
+      <c r="C527" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D527" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E527" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F527" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G527" s="5">
+        <v>19</v>
+      </c>
+      <c r="H527" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I527" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J527" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K527" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L527" s="6">
+        <v>12</v>
+      </c>
+      <c r="M527" s="7">
+        <v>2155.1999999999998</v>
+      </c>
+      <c r="N527" s="6">
+        <v>1</v>
+      </c>
+      <c r="O527" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P527" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q527" s="6">
+        <v>0</v>
+      </c>
+      <c r="R527" s="7">
+        <v>0</v>
+      </c>
+      <c r="S527" s="9">
+        <v>0</v>
+      </c>
+      <c r="T527" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U527" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V527" s="11">
+        <v>11</v>
+      </c>
+      <c r="W527" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X527" s="12">
+        <v>0.40277780000000002</v>
+      </c>
+      <c r="Y527" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB527" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG527" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI527" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ527" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK527" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL527" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM527" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ527" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR527" s="3" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="528" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A528" s="1">
+        <v>1</v>
+      </c>
+      <c r="B528" s="2">
+        <v>2</v>
+      </c>
+      <c r="C528" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D528" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E528" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F528" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G528" s="5">
+        <v>20</v>
+      </c>
+      <c r="H528" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I528" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J528" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K528" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L528" s="6">
+        <v>13</v>
+      </c>
+      <c r="M528" s="7">
+        <v>2334.8000000000002</v>
+      </c>
+      <c r="N528" s="6">
+        <v>1</v>
+      </c>
+      <c r="O528" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P528" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q528" s="6">
+        <v>0</v>
+      </c>
+      <c r="R528" s="7">
+        <v>0</v>
+      </c>
+      <c r="S528" s="9">
+        <v>0</v>
+      </c>
+      <c r="T528" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U528" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V528" s="11">
+        <v>11</v>
+      </c>
+      <c r="W528" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X528" s="12">
+        <v>0.40277780000000002</v>
+      </c>
+      <c r="Y528" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB528" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG528" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI528" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ528" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK528" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL528" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM528" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ528" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR528" s="3" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="529" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A529" s="1">
+        <v>1</v>
+      </c>
+      <c r="B529" s="2">
+        <v>2</v>
+      </c>
+      <c r="C529" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D529" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E529" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F529" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G529" s="5">
+        <v>21</v>
+      </c>
+      <c r="H529" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I529" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J529" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K529" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L529" s="6">
+        <v>14</v>
+      </c>
+      <c r="M529" s="7">
+        <v>2514.4</v>
+      </c>
+      <c r="N529" s="6">
+        <v>1</v>
+      </c>
+      <c r="O529" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P529" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q529" s="6">
+        <v>0</v>
+      </c>
+      <c r="R529" s="7">
+        <v>0</v>
+      </c>
+      <c r="S529" s="9">
+        <v>0</v>
+      </c>
+      <c r="T529" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U529" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V529" s="11">
+        <v>11</v>
+      </c>
+      <c r="W529" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X529" s="12">
+        <v>0.40277780000000002</v>
+      </c>
+      <c r="Y529" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB529" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG529" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI529" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ529" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK529" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL529" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM529" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ529" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR529" s="3" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="530" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A530" s="1">
+        <v>1</v>
+      </c>
+      <c r="B530" s="2">
+        <v>2</v>
+      </c>
+      <c r="C530" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D530" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E530" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F530" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G530" s="5">
+        <v>22</v>
+      </c>
+      <c r="H530" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I530" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J530" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K530" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L530" s="6">
+        <v>15</v>
+      </c>
+      <c r="M530" s="7">
+        <v>2694</v>
+      </c>
+      <c r="N530" s="6">
+        <v>1</v>
+      </c>
+      <c r="O530" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P530" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q530" s="6">
+        <v>0</v>
+      </c>
+      <c r="R530" s="7">
+        <v>0</v>
+      </c>
+      <c r="S530" s="9">
+        <v>0</v>
+      </c>
+      <c r="T530" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U530" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V530" s="11">
+        <v>11</v>
+      </c>
+      <c r="W530" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X530" s="12">
+        <v>0.40277780000000002</v>
+      </c>
+      <c r="Y530" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB530" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG530" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI530" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ530" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK530" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL530" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM530" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ530" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR530" s="3" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="531" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A531" s="1">
+        <v>1</v>
+      </c>
+      <c r="B531" s="2">
+        <v>2</v>
+      </c>
+      <c r="C531" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D531" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E531" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F531" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G531" s="5">
+        <v>23</v>
+      </c>
+      <c r="H531" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I531" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J531" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K531" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L531" s="6">
+        <v>16</v>
+      </c>
+      <c r="M531" s="7">
+        <v>2873.6</v>
+      </c>
+      <c r="N531" s="6">
+        <v>1</v>
+      </c>
+      <c r="O531" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P531" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q531" s="6">
+        <v>0</v>
+      </c>
+      <c r="R531" s="7">
+        <v>0</v>
+      </c>
+      <c r="S531" s="9">
+        <v>0</v>
+      </c>
+      <c r="T531" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U531" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V531" s="11">
+        <v>11</v>
+      </c>
+      <c r="W531" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X531" s="12">
+        <v>0.40277780000000002</v>
+      </c>
+      <c r="Y531" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB531" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG531" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI531" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ531" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK531" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL531" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM531" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ531" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR531" s="3" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="532" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A532" s="1">
+        <v>1</v>
+      </c>
+      <c r="B532" s="2">
+        <v>2</v>
+      </c>
+      <c r="C532" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D532" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E532" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F532" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G532" s="5">
+        <v>24</v>
+      </c>
+      <c r="H532" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I532" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J532" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K532" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L532" s="6">
+        <v>17</v>
+      </c>
+      <c r="M532" s="7">
+        <v>3053.2</v>
+      </c>
+      <c r="N532" s="6">
+        <v>1</v>
+      </c>
+      <c r="O532" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P532" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q532" s="6">
+        <v>0</v>
+      </c>
+      <c r="R532" s="7">
+        <v>0</v>
+      </c>
+      <c r="S532" s="9">
+        <v>0</v>
+      </c>
+      <c r="T532" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U532" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V532" s="11">
+        <v>11</v>
+      </c>
+      <c r="W532" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X532" s="12">
+        <v>0.42361110000000002</v>
+      </c>
+      <c r="Y532" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB532" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG532" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI532" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ532" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK532" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL532" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM532" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ532" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR532" s="3" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="533" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A533" s="1">
+        <v>1</v>
+      </c>
+      <c r="B533" s="2">
+        <v>2</v>
+      </c>
+      <c r="C533" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D533" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E533" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F533" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G533" s="5">
+        <v>25</v>
+      </c>
+      <c r="H533" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I533" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J533" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K533" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L533" s="6">
+        <v>18</v>
+      </c>
+      <c r="M533" s="7">
+        <v>3232.8</v>
+      </c>
+      <c r="N533" s="6">
+        <v>1</v>
+      </c>
+      <c r="O533" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P533" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q533" s="6">
+        <v>0</v>
+      </c>
+      <c r="R533" s="7">
+        <v>0</v>
+      </c>
+      <c r="S533" s="9">
+        <v>0</v>
+      </c>
+      <c r="T533" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U533" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V533" s="11">
+        <v>11</v>
+      </c>
+      <c r="W533" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X533" s="12">
+        <v>0.42361110000000002</v>
+      </c>
+      <c r="Y533" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB533" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG533" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI533" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ533" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK533" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL533" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM533" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ533" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR533" s="3" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="534" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A534" s="1">
+        <v>1</v>
+      </c>
+      <c r="B534" s="2">
+        <v>2</v>
+      </c>
+      <c r="C534" s="3" t="s">
+        <v>575</v>
+      </c>
+      <c r="D534" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E534" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F534" s="4">
+        <v>46286</v>
+      </c>
+      <c r="G534" s="5">
+        <v>28</v>
+      </c>
+      <c r="H534" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I534" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J534" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K534" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L534" s="6">
+        <v>19</v>
+      </c>
+      <c r="M534" s="7">
+        <v>3412.4</v>
+      </c>
+      <c r="N534" s="6">
+        <v>1</v>
+      </c>
+      <c r="O534" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="P534" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q534" s="6">
+        <v>0</v>
+      </c>
+      <c r="R534" s="7">
+        <v>0</v>
+      </c>
+      <c r="S534" s="9">
+        <v>0</v>
+      </c>
+      <c r="T534" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U534" s="10">
+        <v>67522</v>
+      </c>
+      <c r="V534" s="11">
+        <v>11</v>
+      </c>
+      <c r="W534" s="4">
+        <v>46286</v>
+      </c>
+      <c r="X534" s="12">
+        <v>0.48472219999999999</v>
+      </c>
+      <c r="Y534" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB534" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG534" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI534" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ534" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK534" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL534" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM534" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ534" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR534" s="3" t="s">
+        <v>596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 29/09/2026 10:51:43,91
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{066C9073-3BBA-4FB3-B322-5F38662DDB57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1988AABC-3E81-423C-B2BD-2BB38A6CAA82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="122">
   <si>
     <t>Sel</t>
   </si>
@@ -305,6 +305,87 @@
   </si>
   <si>
     <t>1883500000069</t>
+  </si>
+  <si>
+    <t>1883500000070</t>
+  </si>
+  <si>
+    <t>1883500000071</t>
+  </si>
+  <si>
+    <t>1883500000072</t>
+  </si>
+  <si>
+    <t>1883500000073</t>
+  </si>
+  <si>
+    <t>1883500000074</t>
+  </si>
+  <si>
+    <t>1883500000075</t>
+  </si>
+  <si>
+    <t>1883500000076</t>
+  </si>
+  <si>
+    <t>1883500000077</t>
+  </si>
+  <si>
+    <t>1883500000078</t>
+  </si>
+  <si>
+    <t>1883500000079</t>
+  </si>
+  <si>
+    <t>1883500000080</t>
+  </si>
+  <si>
+    <t>1883500000081</t>
+  </si>
+  <si>
+    <t>1883500000082</t>
+  </si>
+  <si>
+    <t>1883500000083</t>
+  </si>
+  <si>
+    <t>1883500000084</t>
+  </si>
+  <si>
+    <t>1883500000085</t>
+  </si>
+  <si>
+    <t>1883500000086</t>
+  </si>
+  <si>
+    <t>1883500000087</t>
+  </si>
+  <si>
+    <t>1883500000088</t>
+  </si>
+  <si>
+    <t>1883500000089</t>
+  </si>
+  <si>
+    <t>1883500000090</t>
+  </si>
+  <si>
+    <t>1883500000091</t>
+  </si>
+  <si>
+    <t>1883500000092</t>
+  </si>
+  <si>
+    <t>1883500000093</t>
+  </si>
+  <si>
+    <t>1883500000094</t>
+  </si>
+  <si>
+    <t>1883500000095</t>
+  </si>
+  <si>
+    <t>1883500000096</t>
   </si>
 </sst>
 </file>
@@ -880,7 +961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR38"/>
+  <dimension ref="A1:AR65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -5973,6 +6054,3624 @@
       </c>
       <c r="AR38" s="3" t="s">
         <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>1</v>
+      </c>
+      <c r="B39" s="2">
+        <v>2</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F39" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G39" s="5">
+        <v>131</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L39" s="6">
+        <v>4</v>
+      </c>
+      <c r="M39" s="7">
+        <v>718.4</v>
+      </c>
+      <c r="N39" s="6">
+        <v>1</v>
+      </c>
+      <c r="O39" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P39" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q39" s="6">
+        <v>0</v>
+      </c>
+      <c r="R39" s="7">
+        <v>0</v>
+      </c>
+      <c r="S39" s="9">
+        <v>0</v>
+      </c>
+      <c r="T39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U39" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V39" s="11">
+        <v>11</v>
+      </c>
+      <c r="W39" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X39" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y39" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG39" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI39" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ39" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK39" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL39" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM39" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR39" s="3" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>1</v>
+      </c>
+      <c r="B40" s="2">
+        <v>2</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F40" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G40" s="5">
+        <v>132</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L40" s="6">
+        <v>5</v>
+      </c>
+      <c r="M40" s="7">
+        <v>898</v>
+      </c>
+      <c r="N40" s="6">
+        <v>1</v>
+      </c>
+      <c r="O40" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P40" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q40" s="6">
+        <v>0</v>
+      </c>
+      <c r="R40" s="7">
+        <v>0</v>
+      </c>
+      <c r="S40" s="9">
+        <v>0</v>
+      </c>
+      <c r="T40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U40" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V40" s="11">
+        <v>11</v>
+      </c>
+      <c r="W40" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X40" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y40" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB40" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG40" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI40" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ40" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK40" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL40" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM40" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR40" s="3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>1</v>
+      </c>
+      <c r="B41" s="2">
+        <v>2</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F41" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G41" s="5">
+        <v>133</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L41" s="6">
+        <v>6</v>
+      </c>
+      <c r="M41" s="7">
+        <v>1077.5999999999999</v>
+      </c>
+      <c r="N41" s="6">
+        <v>1</v>
+      </c>
+      <c r="O41" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P41" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q41" s="6">
+        <v>0</v>
+      </c>
+      <c r="R41" s="7">
+        <v>0</v>
+      </c>
+      <c r="S41" s="9">
+        <v>0</v>
+      </c>
+      <c r="T41" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U41" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V41" s="11">
+        <v>11</v>
+      </c>
+      <c r="W41" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X41" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y41" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB41" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG41" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI41" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ41" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK41" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL41" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM41" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR41" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>1</v>
+      </c>
+      <c r="B42" s="2">
+        <v>2</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F42" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G42" s="5">
+        <v>134</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L42" s="6">
+        <v>7</v>
+      </c>
+      <c r="M42" s="7">
+        <v>1257.2</v>
+      </c>
+      <c r="N42" s="6">
+        <v>1</v>
+      </c>
+      <c r="O42" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P42" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q42" s="6">
+        <v>0</v>
+      </c>
+      <c r="R42" s="7">
+        <v>0</v>
+      </c>
+      <c r="S42" s="9">
+        <v>0</v>
+      </c>
+      <c r="T42" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U42" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V42" s="11">
+        <v>11</v>
+      </c>
+      <c r="W42" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X42" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y42" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB42" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG42" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI42" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ42" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK42" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL42" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM42" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ42" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR42" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="43" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>1</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F43" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G43" s="5">
+        <v>135</v>
+      </c>
+      <c r="H43" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I43" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L43" s="6">
+        <v>8</v>
+      </c>
+      <c r="M43" s="7">
+        <v>1436.8</v>
+      </c>
+      <c r="N43" s="6">
+        <v>1</v>
+      </c>
+      <c r="O43" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P43" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q43" s="6">
+        <v>0</v>
+      </c>
+      <c r="R43" s="7">
+        <v>0</v>
+      </c>
+      <c r="S43" s="9">
+        <v>0</v>
+      </c>
+      <c r="T43" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U43" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V43" s="11">
+        <v>11</v>
+      </c>
+      <c r="W43" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X43" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y43" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB43" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG43" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI43" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ43" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK43" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL43" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM43" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ43" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR43" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="44" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>1</v>
+      </c>
+      <c r="B44" s="2">
+        <v>2</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F44" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G44" s="5">
+        <v>136</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L44" s="6">
+        <v>9</v>
+      </c>
+      <c r="M44" s="7">
+        <v>1616.4</v>
+      </c>
+      <c r="N44" s="6">
+        <v>1</v>
+      </c>
+      <c r="O44" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P44" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q44" s="6">
+        <v>0</v>
+      </c>
+      <c r="R44" s="7">
+        <v>0</v>
+      </c>
+      <c r="S44" s="9">
+        <v>0</v>
+      </c>
+      <c r="T44" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U44" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V44" s="11">
+        <v>11</v>
+      </c>
+      <c r="W44" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X44" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y44" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB44" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG44" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI44" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ44" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK44" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL44" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM44" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ44" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR44" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>1</v>
+      </c>
+      <c r="B45" s="2">
+        <v>2</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F45" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G45" s="5">
+        <v>137</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K45" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L45" s="6">
+        <v>10</v>
+      </c>
+      <c r="M45" s="7">
+        <v>1796</v>
+      </c>
+      <c r="N45" s="6">
+        <v>1</v>
+      </c>
+      <c r="O45" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P45" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q45" s="6">
+        <v>0</v>
+      </c>
+      <c r="R45" s="7">
+        <v>0</v>
+      </c>
+      <c r="S45" s="9">
+        <v>0</v>
+      </c>
+      <c r="T45" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U45" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V45" s="11">
+        <v>11</v>
+      </c>
+      <c r="W45" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X45" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y45" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB45" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG45" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI45" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ45" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK45" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL45" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM45" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ45" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR45" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>1</v>
+      </c>
+      <c r="B46" s="2">
+        <v>2</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F46" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G46" s="5">
+        <v>138</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L46" s="6">
+        <v>11</v>
+      </c>
+      <c r="M46" s="7">
+        <v>1975.6</v>
+      </c>
+      <c r="N46" s="6">
+        <v>1</v>
+      </c>
+      <c r="O46" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P46" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q46" s="6">
+        <v>0</v>
+      </c>
+      <c r="R46" s="7">
+        <v>0</v>
+      </c>
+      <c r="S46" s="9">
+        <v>0</v>
+      </c>
+      <c r="T46" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U46" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V46" s="11">
+        <v>11</v>
+      </c>
+      <c r="W46" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X46" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y46" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB46" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG46" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI46" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ46" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK46" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL46" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM46" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ46" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR46" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="47" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>1</v>
+      </c>
+      <c r="B47" s="2">
+        <v>2</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F47" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G47" s="5">
+        <v>139</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L47" s="6">
+        <v>12</v>
+      </c>
+      <c r="M47" s="7">
+        <v>2155.1999999999998</v>
+      </c>
+      <c r="N47" s="6">
+        <v>1</v>
+      </c>
+      <c r="O47" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P47" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q47" s="6">
+        <v>0</v>
+      </c>
+      <c r="R47" s="7">
+        <v>0</v>
+      </c>
+      <c r="S47" s="9">
+        <v>0</v>
+      </c>
+      <c r="T47" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U47" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V47" s="11">
+        <v>11</v>
+      </c>
+      <c r="W47" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X47" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y47" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB47" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG47" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI47" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ47" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK47" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL47" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM47" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR47" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="48" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>1</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F48" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G48" s="5">
+        <v>140</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L48" s="6">
+        <v>13</v>
+      </c>
+      <c r="M48" s="7">
+        <v>2334.8000000000002</v>
+      </c>
+      <c r="N48" s="6">
+        <v>1</v>
+      </c>
+      <c r="O48" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P48" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q48" s="6">
+        <v>0</v>
+      </c>
+      <c r="R48" s="7">
+        <v>0</v>
+      </c>
+      <c r="S48" s="9">
+        <v>0</v>
+      </c>
+      <c r="T48" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U48" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V48" s="11">
+        <v>11</v>
+      </c>
+      <c r="W48" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X48" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y48" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB48" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG48" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI48" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ48" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK48" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL48" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM48" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ48" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR48" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>1</v>
+      </c>
+      <c r="B49" s="2">
+        <v>2</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F49" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G49" s="5">
+        <v>141</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L49" s="6">
+        <v>14</v>
+      </c>
+      <c r="M49" s="7">
+        <v>2514.4</v>
+      </c>
+      <c r="N49" s="6">
+        <v>1</v>
+      </c>
+      <c r="O49" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P49" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q49" s="6">
+        <v>0</v>
+      </c>
+      <c r="R49" s="7">
+        <v>0</v>
+      </c>
+      <c r="S49" s="9">
+        <v>0</v>
+      </c>
+      <c r="T49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U49" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V49" s="11">
+        <v>11</v>
+      </c>
+      <c r="W49" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X49" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y49" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB49" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG49" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI49" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ49" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK49" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL49" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM49" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ49" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR49" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="50" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>1</v>
+      </c>
+      <c r="B50" s="2">
+        <v>2</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F50" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G50" s="5">
+        <v>142</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K50" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L50" s="6">
+        <v>15</v>
+      </c>
+      <c r="M50" s="7">
+        <v>2694</v>
+      </c>
+      <c r="N50" s="6">
+        <v>1</v>
+      </c>
+      <c r="O50" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P50" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q50" s="6">
+        <v>0</v>
+      </c>
+      <c r="R50" s="7">
+        <v>0</v>
+      </c>
+      <c r="S50" s="9">
+        <v>0</v>
+      </c>
+      <c r="T50" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U50" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V50" s="11">
+        <v>11</v>
+      </c>
+      <c r="W50" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X50" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y50" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB50" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG50" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI50" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ50" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK50" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL50" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM50" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ50" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR50" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="51" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>1</v>
+      </c>
+      <c r="B51" s="2">
+        <v>2</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F51" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G51" s="5">
+        <v>143</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K51" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L51" s="6">
+        <v>16</v>
+      </c>
+      <c r="M51" s="7">
+        <v>2873.6</v>
+      </c>
+      <c r="N51" s="6">
+        <v>1</v>
+      </c>
+      <c r="O51" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P51" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q51" s="6">
+        <v>0</v>
+      </c>
+      <c r="R51" s="7">
+        <v>0</v>
+      </c>
+      <c r="S51" s="9">
+        <v>0</v>
+      </c>
+      <c r="T51" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U51" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V51" s="11">
+        <v>11</v>
+      </c>
+      <c r="W51" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X51" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y51" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB51" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG51" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI51" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ51" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK51" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL51" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM51" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ51" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR51" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="52" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>1</v>
+      </c>
+      <c r="B52" s="2">
+        <v>2</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F52" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G52" s="5">
+        <v>144</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K52" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L52" s="6">
+        <v>17</v>
+      </c>
+      <c r="M52" s="7">
+        <v>3053.2</v>
+      </c>
+      <c r="N52" s="6">
+        <v>1</v>
+      </c>
+      <c r="O52" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P52" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q52" s="6">
+        <v>0</v>
+      </c>
+      <c r="R52" s="7">
+        <v>0</v>
+      </c>
+      <c r="S52" s="9">
+        <v>0</v>
+      </c>
+      <c r="T52" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U52" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V52" s="11">
+        <v>11</v>
+      </c>
+      <c r="W52" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X52" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y52" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB52" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG52" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI52" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ52" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK52" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL52" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM52" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ52" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR52" s="3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A53" s="1">
+        <v>1</v>
+      </c>
+      <c r="B53" s="2">
+        <v>2</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F53" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G53" s="5">
+        <v>145</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K53" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L53" s="6">
+        <v>18</v>
+      </c>
+      <c r="M53" s="7">
+        <v>3232.8</v>
+      </c>
+      <c r="N53" s="6">
+        <v>1</v>
+      </c>
+      <c r="O53" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P53" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q53" s="6">
+        <v>0</v>
+      </c>
+      <c r="R53" s="7">
+        <v>0</v>
+      </c>
+      <c r="S53" s="9">
+        <v>0</v>
+      </c>
+      <c r="T53" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U53" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V53" s="11">
+        <v>11</v>
+      </c>
+      <c r="W53" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X53" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y53" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB53" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG53" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI53" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ53" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK53" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL53" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM53" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ53" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR53" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A54" s="1">
+        <v>1</v>
+      </c>
+      <c r="B54" s="2">
+        <v>2</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G54" s="5">
+        <v>146</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J54" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K54" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L54" s="6">
+        <v>19</v>
+      </c>
+      <c r="M54" s="7">
+        <v>3412.4</v>
+      </c>
+      <c r="N54" s="6">
+        <v>1</v>
+      </c>
+      <c r="O54" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P54" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q54" s="6">
+        <v>0</v>
+      </c>
+      <c r="R54" s="7">
+        <v>0</v>
+      </c>
+      <c r="S54" s="9">
+        <v>0</v>
+      </c>
+      <c r="T54" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U54" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V54" s="11">
+        <v>11</v>
+      </c>
+      <c r="W54" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X54" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y54" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB54" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG54" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI54" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ54" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK54" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL54" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM54" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ54" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR54" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A55" s="1">
+        <v>1</v>
+      </c>
+      <c r="B55" s="2">
+        <v>2</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F55" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G55" s="5">
+        <v>147</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J55" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K55" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L55" s="6">
+        <v>20</v>
+      </c>
+      <c r="M55" s="7">
+        <v>3592</v>
+      </c>
+      <c r="N55" s="6">
+        <v>1</v>
+      </c>
+      <c r="O55" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P55" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q55" s="6">
+        <v>0</v>
+      </c>
+      <c r="R55" s="7">
+        <v>0</v>
+      </c>
+      <c r="S55" s="9">
+        <v>0</v>
+      </c>
+      <c r="T55" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U55" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V55" s="11">
+        <v>11</v>
+      </c>
+      <c r="W55" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X55" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y55" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB55" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG55" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI55" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ55" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK55" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL55" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM55" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ55" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR55" s="3" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A56" s="1">
+        <v>1</v>
+      </c>
+      <c r="B56" s="2">
+        <v>2</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F56" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G56" s="5">
+        <v>148</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L56" s="6">
+        <v>21</v>
+      </c>
+      <c r="M56" s="7">
+        <v>3771.6</v>
+      </c>
+      <c r="N56" s="6">
+        <v>1</v>
+      </c>
+      <c r="O56" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P56" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q56" s="6">
+        <v>0</v>
+      </c>
+      <c r="R56" s="7">
+        <v>0</v>
+      </c>
+      <c r="S56" s="9">
+        <v>0</v>
+      </c>
+      <c r="T56" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U56" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V56" s="11">
+        <v>11</v>
+      </c>
+      <c r="W56" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X56" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y56" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB56" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG56" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI56" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ56" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK56" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL56" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM56" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ56" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR56" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A57" s="1">
+        <v>1</v>
+      </c>
+      <c r="B57" s="2">
+        <v>2</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F57" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G57" s="5">
+        <v>149</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L57" s="6">
+        <v>22</v>
+      </c>
+      <c r="M57" s="7">
+        <v>3951.2</v>
+      </c>
+      <c r="N57" s="6">
+        <v>1</v>
+      </c>
+      <c r="O57" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P57" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q57" s="6">
+        <v>0</v>
+      </c>
+      <c r="R57" s="7">
+        <v>0</v>
+      </c>
+      <c r="S57" s="9">
+        <v>0</v>
+      </c>
+      <c r="T57" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U57" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V57" s="11">
+        <v>11</v>
+      </c>
+      <c r="W57" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X57" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y57" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB57" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG57" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI57" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ57" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK57" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL57" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM57" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ57" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR57" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A58" s="1">
+        <v>1</v>
+      </c>
+      <c r="B58" s="2">
+        <v>2</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F58" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G58" s="5">
+        <v>150</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J58" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K58" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L58" s="6">
+        <v>23</v>
+      </c>
+      <c r="M58" s="7">
+        <v>4130.8</v>
+      </c>
+      <c r="N58" s="6">
+        <v>1</v>
+      </c>
+      <c r="O58" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P58" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q58" s="6">
+        <v>0</v>
+      </c>
+      <c r="R58" s="7">
+        <v>0</v>
+      </c>
+      <c r="S58" s="9">
+        <v>0</v>
+      </c>
+      <c r="T58" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U58" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V58" s="11">
+        <v>11</v>
+      </c>
+      <c r="W58" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X58" s="12">
+        <v>0.4243056</v>
+      </c>
+      <c r="Y58" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB58" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG58" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI58" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ58" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK58" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL58" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM58" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ58" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR58" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>1</v>
+      </c>
+      <c r="B59" s="2">
+        <v>2</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F59" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G59" s="5">
+        <v>151</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J59" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K59" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L59" s="6">
+        <v>24</v>
+      </c>
+      <c r="M59" s="7">
+        <v>4310.3999999999996</v>
+      </c>
+      <c r="N59" s="6">
+        <v>1</v>
+      </c>
+      <c r="O59" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P59" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q59" s="6">
+        <v>0</v>
+      </c>
+      <c r="R59" s="7">
+        <v>0</v>
+      </c>
+      <c r="S59" s="9">
+        <v>0</v>
+      </c>
+      <c r="T59" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U59" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V59" s="11">
+        <v>11</v>
+      </c>
+      <c r="W59" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X59" s="12">
+        <v>0.43125000000000002</v>
+      </c>
+      <c r="Y59" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB59" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG59" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI59" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ59" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK59" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL59" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM59" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ59" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR59" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="60" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>1</v>
+      </c>
+      <c r="B60" s="2">
+        <v>2</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F60" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G60" s="5">
+        <v>152</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J60" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K60" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L60" s="6">
+        <v>25</v>
+      </c>
+      <c r="M60" s="7">
+        <v>4490</v>
+      </c>
+      <c r="N60" s="6">
+        <v>1</v>
+      </c>
+      <c r="O60" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P60" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q60" s="6">
+        <v>0</v>
+      </c>
+      <c r="R60" s="7">
+        <v>0</v>
+      </c>
+      <c r="S60" s="9">
+        <v>0</v>
+      </c>
+      <c r="T60" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U60" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V60" s="11">
+        <v>11</v>
+      </c>
+      <c r="W60" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X60" s="12">
+        <v>0.43125000000000002</v>
+      </c>
+      <c r="Y60" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB60" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG60" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI60" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ60" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK60" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL60" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM60" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ60" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR60" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>1</v>
+      </c>
+      <c r="B61" s="2">
+        <v>2</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F61" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G61" s="5">
+        <v>153</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J61" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K61" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L61" s="6">
+        <v>26</v>
+      </c>
+      <c r="M61" s="7">
+        <v>4669.6000000000004</v>
+      </c>
+      <c r="N61" s="6">
+        <v>1</v>
+      </c>
+      <c r="O61" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P61" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q61" s="6">
+        <v>0</v>
+      </c>
+      <c r="R61" s="7">
+        <v>0</v>
+      </c>
+      <c r="S61" s="9">
+        <v>0</v>
+      </c>
+      <c r="T61" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U61" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V61" s="11">
+        <v>11</v>
+      </c>
+      <c r="W61" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X61" s="12">
+        <v>0.4451389</v>
+      </c>
+      <c r="Y61" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB61" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG61" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI61" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ61" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK61" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL61" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM61" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ61" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR61" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>1</v>
+      </c>
+      <c r="B62" s="2">
+        <v>2</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F62" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G62" s="5">
+        <v>154</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L62" s="6">
+        <v>27</v>
+      </c>
+      <c r="M62" s="7">
+        <v>4849.2</v>
+      </c>
+      <c r="N62" s="6">
+        <v>1</v>
+      </c>
+      <c r="O62" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P62" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q62" s="6">
+        <v>0</v>
+      </c>
+      <c r="R62" s="7">
+        <v>0</v>
+      </c>
+      <c r="S62" s="9">
+        <v>0</v>
+      </c>
+      <c r="T62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U62" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V62" s="11">
+        <v>11</v>
+      </c>
+      <c r="W62" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X62" s="12">
+        <v>0.4451389</v>
+      </c>
+      <c r="Y62" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG62" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI62" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR62" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>1</v>
+      </c>
+      <c r="B63" s="2">
+        <v>2</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F63" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G63" s="5">
+        <v>155</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L63" s="6">
+        <v>28</v>
+      </c>
+      <c r="M63" s="7">
+        <v>5028.8</v>
+      </c>
+      <c r="N63" s="6">
+        <v>1</v>
+      </c>
+      <c r="O63" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P63" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q63" s="6">
+        <v>0</v>
+      </c>
+      <c r="R63" s="7">
+        <v>0</v>
+      </c>
+      <c r="S63" s="9">
+        <v>0</v>
+      </c>
+      <c r="T63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U63" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V63" s="11">
+        <v>11</v>
+      </c>
+      <c r="W63" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X63" s="12">
+        <v>0.4451389</v>
+      </c>
+      <c r="Y63" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB63" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG63" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI63" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR63" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="64" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>1</v>
+      </c>
+      <c r="B64" s="2">
+        <v>2</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F64" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G64" s="5">
+        <v>156</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K64" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L64" s="6">
+        <v>29</v>
+      </c>
+      <c r="M64" s="7">
+        <v>5208.3999999999996</v>
+      </c>
+      <c r="N64" s="6">
+        <v>1</v>
+      </c>
+      <c r="O64" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P64" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q64" s="6">
+        <v>0</v>
+      </c>
+      <c r="R64" s="7">
+        <v>0</v>
+      </c>
+      <c r="S64" s="9">
+        <v>0</v>
+      </c>
+      <c r="T64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U64" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V64" s="11">
+        <v>11</v>
+      </c>
+      <c r="W64" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X64" s="12">
+        <v>0.4451389</v>
+      </c>
+      <c r="Y64" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG64" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI64" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR64" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="65" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>1</v>
+      </c>
+      <c r="B65" s="2">
+        <v>2</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F65" s="4">
+        <v>46294</v>
+      </c>
+      <c r="G65" s="5">
+        <v>157</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K65" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L65" s="6">
+        <v>30</v>
+      </c>
+      <c r="M65" s="7">
+        <v>5388</v>
+      </c>
+      <c r="N65" s="6">
+        <v>1</v>
+      </c>
+      <c r="O65" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="P65" s="8">
+        <v>179.6</v>
+      </c>
+      <c r="Q65" s="6">
+        <v>0</v>
+      </c>
+      <c r="R65" s="7">
+        <v>0</v>
+      </c>
+      <c r="S65" s="9">
+        <v>0</v>
+      </c>
+      <c r="T65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U65" s="10">
+        <v>67757</v>
+      </c>
+      <c r="V65" s="11">
+        <v>11</v>
+      </c>
+      <c r="W65" s="4">
+        <v>46294</v>
+      </c>
+      <c r="X65" s="12">
+        <v>0.4451389</v>
+      </c>
+      <c r="Y65" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG65" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI65" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR65" s="3" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 05/10/2026 10:51:39,74
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DC00DC7-3BD8-4046-89DE-C90AC9EE9402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5159EF4-79E1-4A3A-BC2E-86054DE6C167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="96">
   <si>
     <t>Sel</t>
   </si>
@@ -154,10 +154,10 @@
     <t>Nº Série</t>
   </si>
   <si>
-    <t>10016354</t>
-  </si>
-  <si>
-    <t>1</t>
+    <t>10016351</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
   <si>
     <t>500</t>
@@ -175,7 +175,7 @@
     <t>UN</t>
   </si>
   <si>
-    <t>FORNO ELETRICO NARDELLI EMBUTIR 60L BLACK - NARDELLI EMBUTIR 60L BLACK - 127 V</t>
+    <t>FORNO ELETRICO NARDELLI EMBUTIR INOX 60 LITROS - NARDELLI EMBUTIR INOX 60 LITROS - 220 V</t>
   </si>
   <si>
     <t>100</t>
@@ -187,142 +187,127 @@
     <t>FORNOE</t>
   </si>
   <si>
-    <t>1871400013047</t>
-  </si>
-  <si>
-    <t>1871400013048</t>
-  </si>
-  <si>
-    <t>1871400013049</t>
-  </si>
-  <si>
-    <t>1871400013050</t>
-  </si>
-  <si>
-    <t>1871400013051</t>
-  </si>
-  <si>
-    <t>1871400013052</t>
-  </si>
-  <si>
-    <t>1871400013053</t>
-  </si>
-  <si>
-    <t>1871400013054</t>
-  </si>
-  <si>
-    <t>1871400013055</t>
-  </si>
-  <si>
-    <t>1871400013056</t>
-  </si>
-  <si>
-    <t>1871400013057</t>
-  </si>
-  <si>
-    <t>1871400013058</t>
-  </si>
-  <si>
-    <t>1871400013059</t>
-  </si>
-  <si>
-    <t>1871400013060</t>
-  </si>
-  <si>
-    <t>1871400013061</t>
-  </si>
-  <si>
-    <t>1871400013062</t>
-  </si>
-  <si>
-    <t>1871400013063</t>
-  </si>
-  <si>
-    <t>1871400013064</t>
-  </si>
-  <si>
-    <t>1871400013065</t>
-  </si>
-  <si>
-    <t>1871400013066</t>
-  </si>
-  <si>
-    <t>1871400013067</t>
-  </si>
-  <si>
-    <t>1871400013068</t>
-  </si>
-  <si>
-    <t>1871400013069</t>
-  </si>
-  <si>
-    <t>1871400013070</t>
-  </si>
-  <si>
-    <t>1871400013071</t>
-  </si>
-  <si>
-    <t>1871400013072</t>
-  </si>
-  <si>
-    <t>1871400013073</t>
-  </si>
-  <si>
-    <t>1871400013074</t>
-  </si>
-  <si>
-    <t>1871400013075</t>
-  </si>
-  <si>
-    <t>1871400013076</t>
-  </si>
-  <si>
-    <t>1871400013077</t>
-  </si>
-  <si>
-    <t>1871400013078</t>
-  </si>
-  <si>
-    <t>1871400013079</t>
-  </si>
-  <si>
-    <t>1871400013080</t>
-  </si>
-  <si>
-    <t>10056354</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>FORNO ELETRICO FOGATTI EMBUTIR 60L BLACK - 220 V</t>
-  </si>
-  <si>
-    <t>1031000000104</t>
-  </si>
-  <si>
-    <t>1031000000105</t>
-  </si>
-  <si>
-    <t>1031000000106</t>
-  </si>
-  <si>
-    <t>1031000000107</t>
-  </si>
-  <si>
-    <t>1031000000108</t>
-  </si>
-  <si>
-    <t>1031000000109</t>
-  </si>
-  <si>
-    <t>1031000000110</t>
-  </si>
-  <si>
-    <t>1031000000111</t>
-  </si>
-  <si>
-    <t>1031000000112</t>
+    <t>1875400003126</t>
+  </si>
+  <si>
+    <t>1875400003127</t>
+  </si>
+  <si>
+    <t>1875400003128</t>
+  </si>
+  <si>
+    <t>1875400003129</t>
+  </si>
+  <si>
+    <t>1875400003130</t>
+  </si>
+  <si>
+    <t>1875400003131</t>
+  </si>
+  <si>
+    <t>1875400003132</t>
+  </si>
+  <si>
+    <t>1875400003133</t>
+  </si>
+  <si>
+    <t>1875400003134</t>
+  </si>
+  <si>
+    <t>1875400003135</t>
+  </si>
+  <si>
+    <t>1875400003136</t>
+  </si>
+  <si>
+    <t>1875400003137</t>
+  </si>
+  <si>
+    <t>1875400003138</t>
+  </si>
+  <si>
+    <t>1875400003139</t>
+  </si>
+  <si>
+    <t>1875400003140</t>
+  </si>
+  <si>
+    <t>1875400003141</t>
+  </si>
+  <si>
+    <t>1875400003142</t>
+  </si>
+  <si>
+    <t>1875400003143</t>
+  </si>
+  <si>
+    <t>1875400003144</t>
+  </si>
+  <si>
+    <t>1875400003145</t>
+  </si>
+  <si>
+    <t>1875400003146</t>
+  </si>
+  <si>
+    <t>1875400003147</t>
+  </si>
+  <si>
+    <t>1875400003148</t>
+  </si>
+  <si>
+    <t>1875400003149</t>
+  </si>
+  <si>
+    <t>1875400003150</t>
+  </si>
+  <si>
+    <t>1875400003151</t>
+  </si>
+  <si>
+    <t>1875400003152</t>
+  </si>
+  <si>
+    <t>1875400003153</t>
+  </si>
+  <si>
+    <t>1875400003154</t>
+  </si>
+  <si>
+    <t>1875400003155</t>
+  </si>
+  <si>
+    <t>1875400003156</t>
+  </si>
+  <si>
+    <t>1875400003157</t>
+  </si>
+  <si>
+    <t>1875400003158</t>
+  </si>
+  <si>
+    <t>1875400003159</t>
+  </si>
+  <si>
+    <t>1875400003160</t>
+  </si>
+  <si>
+    <t>1875400003161</t>
+  </si>
+  <si>
+    <t>1875400003162</t>
+  </si>
+  <si>
+    <t>1875400003163</t>
+  </si>
+  <si>
+    <t>1875400003164</t>
+  </si>
+  <si>
+    <t>1875400003165</t>
+  </si>
+  <si>
+    <t>1875400003166</t>
   </si>
 </sst>
 </file>
@@ -898,7 +883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR44"/>
+  <dimension ref="A1:AR42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -1052,10 +1037,10 @@
         <v>46</v>
       </c>
       <c r="F2" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G2" s="5">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>47</v>
@@ -1070,10 +1055,10 @@
         <v>50</v>
       </c>
       <c r="L2" s="6">
-        <v>571</v>
+        <v>77</v>
       </c>
       <c r="M2" s="7">
-        <v>191724.92</v>
+        <v>28797.17</v>
       </c>
       <c r="N2" s="6">
         <v>1</v>
@@ -1082,7 +1067,7 @@
         <v>51</v>
       </c>
       <c r="P2" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q2" s="6">
         <v>0</v>
@@ -1097,16 +1082,16 @@
         <v>52</v>
       </c>
       <c r="U2" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V2" s="11">
         <v>11</v>
       </c>
       <c r="W2" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X2" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y2" s="10">
         <v>0</v>
@@ -1186,10 +1171,10 @@
         <v>46</v>
       </c>
       <c r="F3" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G3" s="5">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>47</v>
@@ -1204,10 +1189,10 @@
         <v>50</v>
       </c>
       <c r="L3" s="6">
-        <v>572</v>
+        <v>78</v>
       </c>
       <c r="M3" s="7">
-        <v>192060.69</v>
+        <v>29171.16</v>
       </c>
       <c r="N3" s="6">
         <v>1</v>
@@ -1216,7 +1201,7 @@
         <v>51</v>
       </c>
       <c r="P3" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q3" s="6">
         <v>0</v>
@@ -1231,16 +1216,16 @@
         <v>52</v>
       </c>
       <c r="U3" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V3" s="11">
         <v>11</v>
       </c>
       <c r="W3" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X3" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y3" s="10">
         <v>0</v>
@@ -1320,10 +1305,10 @@
         <v>46</v>
       </c>
       <c r="F4" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G4" s="5">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>47</v>
@@ -1338,10 +1323,10 @@
         <v>50</v>
       </c>
       <c r="L4" s="6">
-        <v>573</v>
+        <v>79</v>
       </c>
       <c r="M4" s="7">
-        <v>192396.46</v>
+        <v>29545.15</v>
       </c>
       <c r="N4" s="6">
         <v>1</v>
@@ -1350,7 +1335,7 @@
         <v>51</v>
       </c>
       <c r="P4" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q4" s="6">
         <v>0</v>
@@ -1365,16 +1350,16 @@
         <v>52</v>
       </c>
       <c r="U4" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V4" s="11">
         <v>11</v>
       </c>
       <c r="W4" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X4" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y4" s="10">
         <v>0</v>
@@ -1454,10 +1439,10 @@
         <v>46</v>
       </c>
       <c r="F5" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G5" s="5">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>47</v>
@@ -1472,10 +1457,10 @@
         <v>50</v>
       </c>
       <c r="L5" s="6">
-        <v>574</v>
+        <v>80</v>
       </c>
       <c r="M5" s="7">
-        <v>192732.23</v>
+        <v>29919.14</v>
       </c>
       <c r="N5" s="6">
         <v>1</v>
@@ -1484,7 +1469,7 @@
         <v>51</v>
       </c>
       <c r="P5" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q5" s="6">
         <v>0</v>
@@ -1499,16 +1484,16 @@
         <v>52</v>
       </c>
       <c r="U5" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V5" s="11">
         <v>11</v>
       </c>
       <c r="W5" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X5" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y5" s="10">
         <v>0</v>
@@ -1588,10 +1573,10 @@
         <v>46</v>
       </c>
       <c r="F6" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G6" s="5">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>47</v>
@@ -1606,10 +1591,10 @@
         <v>50</v>
       </c>
       <c r="L6" s="6">
-        <v>575</v>
+        <v>81</v>
       </c>
       <c r="M6" s="7">
-        <v>193068</v>
+        <v>30293.13</v>
       </c>
       <c r="N6" s="6">
         <v>1</v>
@@ -1618,7 +1603,7 @@
         <v>51</v>
       </c>
       <c r="P6" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q6" s="6">
         <v>0</v>
@@ -1633,16 +1618,16 @@
         <v>52</v>
       </c>
       <c r="U6" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V6" s="11">
         <v>11</v>
       </c>
       <c r="W6" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X6" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y6" s="10">
         <v>0</v>
@@ -1722,10 +1707,10 @@
         <v>46</v>
       </c>
       <c r="F7" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G7" s="5">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>47</v>
@@ -1740,10 +1725,10 @@
         <v>50</v>
       </c>
       <c r="L7" s="6">
-        <v>576</v>
+        <v>82</v>
       </c>
       <c r="M7" s="7">
-        <v>193403.77</v>
+        <v>30667.119999999999</v>
       </c>
       <c r="N7" s="6">
         <v>1</v>
@@ -1752,7 +1737,7 @@
         <v>51</v>
       </c>
       <c r="P7" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q7" s="6">
         <v>0</v>
@@ -1767,16 +1752,16 @@
         <v>52</v>
       </c>
       <c r="U7" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V7" s="11">
         <v>11</v>
       </c>
       <c r="W7" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X7" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y7" s="10">
         <v>0</v>
@@ -1856,10 +1841,10 @@
         <v>46</v>
       </c>
       <c r="F8" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G8" s="5">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>47</v>
@@ -1874,10 +1859,10 @@
         <v>50</v>
       </c>
       <c r="L8" s="6">
-        <v>577</v>
+        <v>83</v>
       </c>
       <c r="M8" s="7">
-        <v>193739.54</v>
+        <v>31041.11</v>
       </c>
       <c r="N8" s="6">
         <v>1</v>
@@ -1886,7 +1871,7 @@
         <v>51</v>
       </c>
       <c r="P8" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q8" s="6">
         <v>0</v>
@@ -1901,16 +1886,16 @@
         <v>52</v>
       </c>
       <c r="U8" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V8" s="11">
         <v>11</v>
       </c>
       <c r="W8" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X8" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y8" s="10">
         <v>0</v>
@@ -1990,10 +1975,10 @@
         <v>46</v>
       </c>
       <c r="F9" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G9" s="5">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>47</v>
@@ -2008,10 +1993,10 @@
         <v>50</v>
       </c>
       <c r="L9" s="6">
-        <v>578</v>
+        <v>84</v>
       </c>
       <c r="M9" s="7">
-        <v>194075.31</v>
+        <v>31415.1</v>
       </c>
       <c r="N9" s="6">
         <v>1</v>
@@ -2020,7 +2005,7 @@
         <v>51</v>
       </c>
       <c r="P9" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q9" s="6">
         <v>0</v>
@@ -2035,16 +2020,16 @@
         <v>52</v>
       </c>
       <c r="U9" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V9" s="11">
         <v>11</v>
       </c>
       <c r="W9" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X9" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y9" s="10">
         <v>0</v>
@@ -2124,10 +2109,10 @@
         <v>46</v>
       </c>
       <c r="F10" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G10" s="5">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>47</v>
@@ -2142,10 +2127,10 @@
         <v>50</v>
       </c>
       <c r="L10" s="6">
-        <v>579</v>
+        <v>85</v>
       </c>
       <c r="M10" s="7">
-        <v>194411.08</v>
+        <v>31789.09</v>
       </c>
       <c r="N10" s="6">
         <v>1</v>
@@ -2154,7 +2139,7 @@
         <v>51</v>
       </c>
       <c r="P10" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q10" s="6">
         <v>0</v>
@@ -2169,16 +2154,16 @@
         <v>52</v>
       </c>
       <c r="U10" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V10" s="11">
         <v>11</v>
       </c>
       <c r="W10" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X10" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y10" s="10">
         <v>0</v>
@@ -2258,10 +2243,10 @@
         <v>46</v>
       </c>
       <c r="F11" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G11" s="5">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>47</v>
@@ -2276,10 +2261,10 @@
         <v>50</v>
       </c>
       <c r="L11" s="6">
-        <v>580</v>
+        <v>86</v>
       </c>
       <c r="M11" s="7">
-        <v>194746.85</v>
+        <v>32163.08</v>
       </c>
       <c r="N11" s="6">
         <v>1</v>
@@ -2288,7 +2273,7 @@
         <v>51</v>
       </c>
       <c r="P11" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q11" s="6">
         <v>0</v>
@@ -2303,16 +2288,16 @@
         <v>52</v>
       </c>
       <c r="U11" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V11" s="11">
         <v>11</v>
       </c>
       <c r="W11" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X11" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y11" s="10">
         <v>0</v>
@@ -2392,10 +2377,10 @@
         <v>46</v>
       </c>
       <c r="F12" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G12" s="5">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>47</v>
@@ -2410,10 +2395,10 @@
         <v>50</v>
       </c>
       <c r="L12" s="6">
-        <v>581</v>
+        <v>87</v>
       </c>
       <c r="M12" s="7">
-        <v>195082.62</v>
+        <v>32537.07</v>
       </c>
       <c r="N12" s="6">
         <v>1</v>
@@ -2422,7 +2407,7 @@
         <v>51</v>
       </c>
       <c r="P12" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q12" s="6">
         <v>0</v>
@@ -2437,16 +2422,16 @@
         <v>52</v>
       </c>
       <c r="U12" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V12" s="11">
         <v>11</v>
       </c>
       <c r="W12" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X12" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y12" s="10">
         <v>0</v>
@@ -2526,10 +2511,10 @@
         <v>46</v>
       </c>
       <c r="F13" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G13" s="5">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>47</v>
@@ -2544,10 +2529,10 @@
         <v>50</v>
       </c>
       <c r="L13" s="6">
-        <v>582</v>
+        <v>88</v>
       </c>
       <c r="M13" s="7">
-        <v>195418.39</v>
+        <v>32911.06</v>
       </c>
       <c r="N13" s="6">
         <v>1</v>
@@ -2556,7 +2541,7 @@
         <v>51</v>
       </c>
       <c r="P13" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q13" s="6">
         <v>0</v>
@@ -2571,16 +2556,16 @@
         <v>52</v>
       </c>
       <c r="U13" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V13" s="11">
         <v>11</v>
       </c>
       <c r="W13" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X13" s="12">
-        <v>0.35486109999999998</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y13" s="10">
         <v>0</v>
@@ -2660,10 +2645,10 @@
         <v>46</v>
       </c>
       <c r="F14" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G14" s="5">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>47</v>
@@ -2678,10 +2663,10 @@
         <v>50</v>
       </c>
       <c r="L14" s="6">
-        <v>583</v>
+        <v>89</v>
       </c>
       <c r="M14" s="7">
-        <v>195754.17</v>
+        <v>33285.050000000003</v>
       </c>
       <c r="N14" s="6">
         <v>1</v>
@@ -2690,7 +2675,7 @@
         <v>51</v>
       </c>
       <c r="P14" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q14" s="6">
         <v>0</v>
@@ -2705,16 +2690,16 @@
         <v>52</v>
       </c>
       <c r="U14" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V14" s="11">
         <v>11</v>
       </c>
       <c r="W14" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X14" s="12">
-        <v>0.3618056</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y14" s="10">
         <v>0</v>
@@ -2794,10 +2779,10 @@
         <v>46</v>
       </c>
       <c r="F15" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G15" s="5">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>47</v>
@@ -2812,10 +2797,10 @@
         <v>50</v>
       </c>
       <c r="L15" s="6">
-        <v>584</v>
+        <v>90</v>
       </c>
       <c r="M15" s="7">
-        <v>196089.94</v>
+        <v>33659.03</v>
       </c>
       <c r="N15" s="6">
         <v>1</v>
@@ -2824,7 +2809,7 @@
         <v>51</v>
       </c>
       <c r="P15" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q15" s="6">
         <v>0</v>
@@ -2839,16 +2824,16 @@
         <v>52</v>
       </c>
       <c r="U15" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V15" s="11">
         <v>11</v>
       </c>
       <c r="W15" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X15" s="12">
-        <v>0.3618056</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y15" s="10">
         <v>0</v>
@@ -2928,10 +2913,10 @@
         <v>46</v>
       </c>
       <c r="F16" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G16" s="5">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>47</v>
@@ -2946,10 +2931,10 @@
         <v>50</v>
       </c>
       <c r="L16" s="6">
-        <v>585</v>
+        <v>91</v>
       </c>
       <c r="M16" s="7">
-        <v>196425.71</v>
+        <v>34033.019999999997</v>
       </c>
       <c r="N16" s="6">
         <v>1</v>
@@ -2958,7 +2943,7 @@
         <v>51</v>
       </c>
       <c r="P16" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q16" s="6">
         <v>0</v>
@@ -2973,16 +2958,16 @@
         <v>52</v>
       </c>
       <c r="U16" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V16" s="11">
         <v>11</v>
       </c>
       <c r="W16" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X16" s="12">
-        <v>0.3618056</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y16" s="10">
         <v>0</v>
@@ -3062,10 +3047,10 @@
         <v>46</v>
       </c>
       <c r="F17" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G17" s="5">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>47</v>
@@ -3080,10 +3065,10 @@
         <v>50</v>
       </c>
       <c r="L17" s="6">
-        <v>586</v>
+        <v>92</v>
       </c>
       <c r="M17" s="7">
-        <v>196761.48</v>
+        <v>34407.01</v>
       </c>
       <c r="N17" s="6">
         <v>1</v>
@@ -3092,7 +3077,7 @@
         <v>51</v>
       </c>
       <c r="P17" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q17" s="6">
         <v>0</v>
@@ -3107,16 +3092,16 @@
         <v>52</v>
       </c>
       <c r="U17" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V17" s="11">
         <v>11</v>
       </c>
       <c r="W17" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X17" s="12">
-        <v>0.3826389</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y17" s="10">
         <v>0</v>
@@ -3196,10 +3181,10 @@
         <v>46</v>
       </c>
       <c r="F18" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G18" s="5">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>47</v>
@@ -3214,10 +3199,10 @@
         <v>50</v>
       </c>
       <c r="L18" s="6">
-        <v>587</v>
+        <v>93</v>
       </c>
       <c r="M18" s="7">
-        <v>197097.25</v>
+        <v>34781</v>
       </c>
       <c r="N18" s="6">
         <v>1</v>
@@ -3226,7 +3211,7 @@
         <v>51</v>
       </c>
       <c r="P18" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q18" s="6">
         <v>0</v>
@@ -3241,16 +3226,16 @@
         <v>52</v>
       </c>
       <c r="U18" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V18" s="11">
         <v>11</v>
       </c>
       <c r="W18" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X18" s="12">
-        <v>0.3826389</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y18" s="10">
         <v>0</v>
@@ -3330,10 +3315,10 @@
         <v>46</v>
       </c>
       <c r="F19" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G19" s="5">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>47</v>
@@ -3348,10 +3333,10 @@
         <v>50</v>
       </c>
       <c r="L19" s="6">
-        <v>588</v>
+        <v>94</v>
       </c>
       <c r="M19" s="7">
-        <v>197433.02</v>
+        <v>35154.99</v>
       </c>
       <c r="N19" s="6">
         <v>1</v>
@@ -3360,7 +3345,7 @@
         <v>51</v>
       </c>
       <c r="P19" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q19" s="6">
         <v>0</v>
@@ -3375,16 +3360,16 @@
         <v>52</v>
       </c>
       <c r="U19" s="10">
-        <v>67391</v>
+        <v>67750</v>
       </c>
       <c r="V19" s="11">
         <v>11</v>
       </c>
       <c r="W19" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X19" s="12">
-        <v>0.3826389</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y19" s="10">
         <v>0</v>
@@ -3464,10 +3449,10 @@
         <v>46</v>
       </c>
       <c r="F20" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G20" s="5">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>47</v>
@@ -3482,10 +3467,10 @@
         <v>50</v>
       </c>
       <c r="L20" s="6">
-        <v>589</v>
+        <v>95</v>
       </c>
       <c r="M20" s="7">
-        <v>197768.79</v>
+        <v>35528.980000000003</v>
       </c>
       <c r="N20" s="6">
         <v>1</v>
@@ -3494,7 +3479,7 @@
         <v>51</v>
       </c>
       <c r="P20" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q20" s="6">
         <v>0</v>
@@ -3509,16 +3494,16 @@
         <v>52</v>
       </c>
       <c r="U20" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V20" s="11">
         <v>11</v>
       </c>
       <c r="W20" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X20" s="12">
-        <v>0.38958330000000002</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y20" s="10">
         <v>0</v>
@@ -3598,10 +3583,10 @@
         <v>46</v>
       </c>
       <c r="F21" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G21" s="5">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>47</v>
@@ -3616,10 +3601,10 @@
         <v>50</v>
       </c>
       <c r="L21" s="6">
-        <v>590</v>
+        <v>96</v>
       </c>
       <c r="M21" s="7">
-        <v>198104.56</v>
+        <v>35902.97</v>
       </c>
       <c r="N21" s="6">
         <v>1</v>
@@ -3628,7 +3613,7 @@
         <v>51</v>
       </c>
       <c r="P21" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q21" s="6">
         <v>0</v>
@@ -3643,16 +3628,16 @@
         <v>52</v>
       </c>
       <c r="U21" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V21" s="11">
         <v>11</v>
       </c>
       <c r="W21" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X21" s="12">
-        <v>0.4034722</v>
+        <v>0.37708330000000001</v>
       </c>
       <c r="Y21" s="10">
         <v>0</v>
@@ -3732,10 +3717,10 @@
         <v>46</v>
       </c>
       <c r="F22" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G22" s="5">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>47</v>
@@ -3750,10 +3735,10 @@
         <v>50</v>
       </c>
       <c r="L22" s="6">
-        <v>591</v>
+        <v>97</v>
       </c>
       <c r="M22" s="7">
-        <v>198440.33</v>
+        <v>36276.959999999999</v>
       </c>
       <c r="N22" s="6">
         <v>1</v>
@@ -3762,7 +3747,7 @@
         <v>51</v>
       </c>
       <c r="P22" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q22" s="6">
         <v>0</v>
@@ -3777,16 +3762,16 @@
         <v>52</v>
       </c>
       <c r="U22" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V22" s="11">
         <v>11</v>
       </c>
       <c r="W22" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X22" s="12">
-        <v>0.4034722</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y22" s="10">
         <v>0</v>
@@ -3866,10 +3851,10 @@
         <v>46</v>
       </c>
       <c r="F23" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G23" s="5">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>47</v>
@@ -3884,10 +3869,10 @@
         <v>50</v>
       </c>
       <c r="L23" s="6">
-        <v>592</v>
+        <v>98</v>
       </c>
       <c r="M23" s="7">
-        <v>198776.1</v>
+        <v>36650.949999999997</v>
       </c>
       <c r="N23" s="6">
         <v>1</v>
@@ -3896,7 +3881,7 @@
         <v>51</v>
       </c>
       <c r="P23" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q23" s="6">
         <v>0</v>
@@ -3911,16 +3896,16 @@
         <v>52</v>
       </c>
       <c r="U23" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V23" s="11">
         <v>11</v>
       </c>
       <c r="W23" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X23" s="12">
-        <v>0.4034722</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y23" s="10">
         <v>0</v>
@@ -4000,10 +3985,10 @@
         <v>46</v>
       </c>
       <c r="F24" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G24" s="5">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>47</v>
@@ -4018,10 +4003,10 @@
         <v>50</v>
       </c>
       <c r="L24" s="6">
-        <v>593</v>
+        <v>99</v>
       </c>
       <c r="M24" s="7">
-        <v>199111.87</v>
+        <v>37024.94</v>
       </c>
       <c r="N24" s="6">
         <v>1</v>
@@ -4030,7 +4015,7 @@
         <v>51</v>
       </c>
       <c r="P24" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q24" s="6">
         <v>0</v>
@@ -4045,16 +4030,16 @@
         <v>52</v>
       </c>
       <c r="U24" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V24" s="11">
         <v>11</v>
       </c>
       <c r="W24" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X24" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y24" s="10">
         <v>0</v>
@@ -4134,10 +4119,10 @@
         <v>46</v>
       </c>
       <c r="F25" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G25" s="5">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>47</v>
@@ -4152,10 +4137,10 @@
         <v>50</v>
       </c>
       <c r="L25" s="6">
-        <v>594</v>
+        <v>100</v>
       </c>
       <c r="M25" s="7">
-        <v>199447.64</v>
+        <v>37398.93</v>
       </c>
       <c r="N25" s="6">
         <v>1</v>
@@ -4164,7 +4149,7 @@
         <v>51</v>
       </c>
       <c r="P25" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q25" s="6">
         <v>0</v>
@@ -4179,16 +4164,16 @@
         <v>52</v>
       </c>
       <c r="U25" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V25" s="11">
         <v>11</v>
       </c>
       <c r="W25" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X25" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y25" s="10">
         <v>0</v>
@@ -4268,10 +4253,10 @@
         <v>46</v>
       </c>
       <c r="F26" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G26" s="5">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>47</v>
@@ -4286,10 +4271,10 @@
         <v>50</v>
       </c>
       <c r="L26" s="6">
-        <v>595</v>
+        <v>101</v>
       </c>
       <c r="M26" s="7">
-        <v>199783.41</v>
+        <v>37772.92</v>
       </c>
       <c r="N26" s="6">
         <v>1</v>
@@ -4298,7 +4283,7 @@
         <v>51</v>
       </c>
       <c r="P26" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q26" s="6">
         <v>0</v>
@@ -4313,16 +4298,16 @@
         <v>52</v>
       </c>
       <c r="U26" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V26" s="11">
         <v>11</v>
       </c>
       <c r="W26" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X26" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y26" s="10">
         <v>0</v>
@@ -4402,10 +4387,10 @@
         <v>46</v>
       </c>
       <c r="F27" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G27" s="5">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>47</v>
@@ -4420,10 +4405,10 @@
         <v>50</v>
       </c>
       <c r="L27" s="6">
-        <v>596</v>
+        <v>102</v>
       </c>
       <c r="M27" s="7">
-        <v>200119.18</v>
+        <v>38146.910000000003</v>
       </c>
       <c r="N27" s="6">
         <v>1</v>
@@ -4432,7 +4417,7 @@
         <v>51</v>
       </c>
       <c r="P27" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q27" s="6">
         <v>0</v>
@@ -4447,16 +4432,16 @@
         <v>52</v>
       </c>
       <c r="U27" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V27" s="11">
         <v>11</v>
       </c>
       <c r="W27" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X27" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y27" s="10">
         <v>0</v>
@@ -4536,10 +4521,10 @@
         <v>46</v>
       </c>
       <c r="F28" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G28" s="5">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>47</v>
@@ -4554,10 +4539,10 @@
         <v>50</v>
       </c>
       <c r="L28" s="6">
-        <v>597</v>
+        <v>103</v>
       </c>
       <c r="M28" s="7">
-        <v>200454.95</v>
+        <v>38520.9</v>
       </c>
       <c r="N28" s="6">
         <v>1</v>
@@ -4566,7 +4551,7 @@
         <v>51</v>
       </c>
       <c r="P28" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q28" s="6">
         <v>0</v>
@@ -4581,16 +4566,16 @@
         <v>52</v>
       </c>
       <c r="U28" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V28" s="11">
         <v>11</v>
       </c>
       <c r="W28" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X28" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y28" s="10">
         <v>0</v>
@@ -4670,10 +4655,10 @@
         <v>46</v>
       </c>
       <c r="F29" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G29" s="5">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>47</v>
@@ -4688,10 +4673,10 @@
         <v>50</v>
       </c>
       <c r="L29" s="6">
-        <v>598</v>
+        <v>104</v>
       </c>
       <c r="M29" s="7">
-        <v>200790.72</v>
+        <v>38894.879999999997</v>
       </c>
       <c r="N29" s="6">
         <v>1</v>
@@ -4700,7 +4685,7 @@
         <v>51</v>
       </c>
       <c r="P29" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q29" s="6">
         <v>0</v>
@@ -4715,16 +4700,16 @@
         <v>52</v>
       </c>
       <c r="U29" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V29" s="11">
         <v>11</v>
       </c>
       <c r="W29" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X29" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y29" s="10">
         <v>0</v>
@@ -4804,10 +4789,10 @@
         <v>46</v>
       </c>
       <c r="F30" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G30" s="5">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>47</v>
@@ -4822,10 +4807,10 @@
         <v>50</v>
       </c>
       <c r="L30" s="6">
-        <v>599</v>
+        <v>105</v>
       </c>
       <c r="M30" s="7">
-        <v>201126.49</v>
+        <v>39268.870000000003</v>
       </c>
       <c r="N30" s="6">
         <v>1</v>
@@ -4834,7 +4819,7 @@
         <v>51</v>
       </c>
       <c r="P30" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q30" s="6">
         <v>0</v>
@@ -4849,16 +4834,16 @@
         <v>52</v>
       </c>
       <c r="U30" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V30" s="11">
         <v>11</v>
       </c>
       <c r="W30" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X30" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y30" s="10">
         <v>0</v>
@@ -4938,10 +4923,10 @@
         <v>46</v>
       </c>
       <c r="F31" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G31" s="5">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>47</v>
@@ -4956,10 +4941,10 @@
         <v>50</v>
       </c>
       <c r="L31" s="6">
-        <v>600</v>
+        <v>106</v>
       </c>
       <c r="M31" s="7">
-        <v>201462.26</v>
+        <v>39642.86</v>
       </c>
       <c r="N31" s="6">
         <v>1</v>
@@ -4968,7 +4953,7 @@
         <v>51</v>
       </c>
       <c r="P31" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q31" s="6">
         <v>0</v>
@@ -4983,16 +4968,16 @@
         <v>52</v>
       </c>
       <c r="U31" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V31" s="11">
         <v>11</v>
       </c>
       <c r="W31" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X31" s="12">
-        <v>0.4243056</v>
+        <v>0.39791670000000001</v>
       </c>
       <c r="Y31" s="10">
         <v>0</v>
@@ -5072,10 +5057,10 @@
         <v>46</v>
       </c>
       <c r="F32" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G32" s="5">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>47</v>
@@ -5090,10 +5075,10 @@
         <v>50</v>
       </c>
       <c r="L32" s="6">
-        <v>601</v>
+        <v>107</v>
       </c>
       <c r="M32" s="7">
-        <v>201798.03</v>
+        <v>40016.85</v>
       </c>
       <c r="N32" s="6">
         <v>1</v>
@@ -5102,7 +5087,7 @@
         <v>51</v>
       </c>
       <c r="P32" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q32" s="6">
         <v>0</v>
@@ -5117,16 +5102,16 @@
         <v>52</v>
       </c>
       <c r="U32" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V32" s="11">
         <v>11</v>
       </c>
       <c r="W32" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X32" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.41875000000000001</v>
       </c>
       <c r="Y32" s="10">
         <v>0</v>
@@ -5206,10 +5191,10 @@
         <v>46</v>
       </c>
       <c r="F33" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G33" s="5">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>47</v>
@@ -5224,10 +5209,10 @@
         <v>50</v>
       </c>
       <c r="L33" s="6">
-        <v>602</v>
+        <v>108</v>
       </c>
       <c r="M33" s="7">
-        <v>202133.8</v>
+        <v>40390.839999999997</v>
       </c>
       <c r="N33" s="6">
         <v>1</v>
@@ -5236,7 +5221,7 @@
         <v>51</v>
       </c>
       <c r="P33" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q33" s="6">
         <v>0</v>
@@ -5251,16 +5236,16 @@
         <v>52</v>
       </c>
       <c r="U33" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V33" s="11">
         <v>11</v>
       </c>
       <c r="W33" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X33" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.41875000000000001</v>
       </c>
       <c r="Y33" s="10">
         <v>0</v>
@@ -5340,10 +5325,10 @@
         <v>46</v>
       </c>
       <c r="F34" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G34" s="5">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>47</v>
@@ -5358,10 +5343,10 @@
         <v>50</v>
       </c>
       <c r="L34" s="6">
-        <v>603</v>
+        <v>109</v>
       </c>
       <c r="M34" s="7">
-        <v>202469.57</v>
+        <v>40764.83</v>
       </c>
       <c r="N34" s="6">
         <v>1</v>
@@ -5370,7 +5355,7 @@
         <v>51</v>
       </c>
       <c r="P34" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q34" s="6">
         <v>0</v>
@@ -5385,16 +5370,16 @@
         <v>52</v>
       </c>
       <c r="U34" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V34" s="11">
         <v>11</v>
       </c>
       <c r="W34" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X34" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.41875000000000001</v>
       </c>
       <c r="Y34" s="10">
         <v>0</v>
@@ -5474,10 +5459,10 @@
         <v>46</v>
       </c>
       <c r="F35" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G35" s="5">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>47</v>
@@ -5492,10 +5477,10 @@
         <v>50</v>
       </c>
       <c r="L35" s="6">
-        <v>604</v>
+        <v>110</v>
       </c>
       <c r="M35" s="7">
-        <v>202805.34</v>
+        <v>41138.82</v>
       </c>
       <c r="N35" s="6">
         <v>1</v>
@@ -5504,7 +5489,7 @@
         <v>51</v>
       </c>
       <c r="P35" s="8">
-        <v>335.77</v>
+        <v>373.99</v>
       </c>
       <c r="Q35" s="6">
         <v>0</v>
@@ -5519,16 +5504,16 @@
         <v>52</v>
       </c>
       <c r="U35" s="10">
-        <v>67506</v>
+        <v>67750</v>
       </c>
       <c r="V35" s="11">
         <v>11</v>
       </c>
       <c r="W35" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X35" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y35" s="10">
         <v>0</v>
@@ -5599,19 +5584,19 @@
         <v>2</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F36" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G36" s="5">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>47</v>
@@ -5626,19 +5611,19 @@
         <v>50</v>
       </c>
       <c r="L36" s="6">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="M36" s="7">
-        <v>5115.3599999999997</v>
+        <v>41512.81</v>
       </c>
       <c r="N36" s="6">
         <v>1</v>
       </c>
       <c r="O36" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P36" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q36" s="6">
         <v>0</v>
@@ -5653,16 +5638,16 @@
         <v>52</v>
       </c>
       <c r="U36" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V36" s="11">
         <v>11</v>
       </c>
       <c r="W36" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X36" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y36" s="10">
         <v>0</v>
@@ -5722,7 +5707,7 @@
         <v>53</v>
       </c>
       <c r="AR36" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:44" x14ac:dyDescent="0.3">
@@ -5733,19 +5718,19 @@
         <v>2</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F37" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G37" s="5">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>47</v>
@@ -5760,19 +5745,19 @@
         <v>50</v>
       </c>
       <c r="L37" s="6">
-        <v>17</v>
+        <v>112</v>
       </c>
       <c r="M37" s="7">
-        <v>5435.07</v>
+        <v>41886.800000000003</v>
       </c>
       <c r="N37" s="6">
         <v>1</v>
       </c>
       <c r="O37" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P37" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q37" s="6">
         <v>0</v>
@@ -5787,16 +5772,16 @@
         <v>52</v>
       </c>
       <c r="U37" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V37" s="11">
         <v>11</v>
       </c>
       <c r="W37" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X37" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y37" s="10">
         <v>0</v>
@@ -5856,7 +5841,7 @@
         <v>53</v>
       </c>
       <c r="AR37" s="3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:44" x14ac:dyDescent="0.3">
@@ -5867,19 +5852,19 @@
         <v>2</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E38" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F38" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G38" s="5">
-        <v>4</v>
+        <v>63</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>47</v>
@@ -5894,19 +5879,19 @@
         <v>50</v>
       </c>
       <c r="L38" s="6">
-        <v>18</v>
+        <v>113</v>
       </c>
       <c r="M38" s="7">
-        <v>5754.78</v>
+        <v>42260.79</v>
       </c>
       <c r="N38" s="6">
         <v>1</v>
       </c>
       <c r="O38" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P38" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q38" s="6">
         <v>0</v>
@@ -5921,16 +5906,16 @@
         <v>52</v>
       </c>
       <c r="U38" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V38" s="11">
         <v>11</v>
       </c>
       <c r="W38" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X38" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y38" s="10">
         <v>0</v>
@@ -5990,7 +5975,7 @@
         <v>53</v>
       </c>
       <c r="AR38" s="3" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:44" x14ac:dyDescent="0.3">
@@ -6001,19 +5986,19 @@
         <v>2</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E39" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F39" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G39" s="5">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>47</v>
@@ -6028,19 +6013,19 @@
         <v>50</v>
       </c>
       <c r="L39" s="6">
-        <v>19</v>
+        <v>114</v>
       </c>
       <c r="M39" s="7">
-        <v>6074.49</v>
+        <v>42634.78</v>
       </c>
       <c r="N39" s="6">
         <v>1</v>
       </c>
       <c r="O39" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P39" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q39" s="6">
         <v>0</v>
@@ -6055,16 +6040,16 @@
         <v>52</v>
       </c>
       <c r="U39" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V39" s="11">
         <v>11</v>
       </c>
       <c r="W39" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X39" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y39" s="10">
         <v>0</v>
@@ -6124,7 +6109,7 @@
         <v>53</v>
       </c>
       <c r="AR39" s="3" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:44" x14ac:dyDescent="0.3">
@@ -6135,19 +6120,19 @@
         <v>2</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F40" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G40" s="5">
-        <v>6</v>
+        <v>65</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>47</v>
@@ -6162,19 +6147,19 @@
         <v>50</v>
       </c>
       <c r="L40" s="6">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="M40" s="7">
-        <v>6394.2</v>
+        <v>43008.77</v>
       </c>
       <c r="N40" s="6">
         <v>1</v>
       </c>
       <c r="O40" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P40" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q40" s="6">
         <v>0</v>
@@ -6189,16 +6174,16 @@
         <v>52</v>
       </c>
       <c r="U40" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V40" s="11">
         <v>11</v>
       </c>
       <c r="W40" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X40" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43888890000000003</v>
       </c>
       <c r="Y40" s="10">
         <v>0</v>
@@ -6258,7 +6243,7 @@
         <v>53</v>
       </c>
       <c r="AR40" s="3" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:44" x14ac:dyDescent="0.3">
@@ -6269,19 +6254,19 @@
         <v>2</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F41" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G41" s="5">
-        <v>7</v>
+        <v>66</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>47</v>
@@ -6296,19 +6281,19 @@
         <v>50</v>
       </c>
       <c r="L41" s="6">
-        <v>21</v>
+        <v>116</v>
       </c>
       <c r="M41" s="7">
-        <v>6713.91</v>
+        <v>43382.76</v>
       </c>
       <c r="N41" s="6">
         <v>1</v>
       </c>
       <c r="O41" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P41" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q41" s="6">
         <v>0</v>
@@ -6323,16 +6308,16 @@
         <v>52</v>
       </c>
       <c r="U41" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V41" s="11">
         <v>11</v>
       </c>
       <c r="W41" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X41" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43958330000000001</v>
       </c>
       <c r="Y41" s="10">
         <v>0</v>
@@ -6392,7 +6377,7 @@
         <v>53</v>
       </c>
       <c r="AR41" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:44" x14ac:dyDescent="0.3">
@@ -6403,19 +6388,19 @@
         <v>2</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>89</v>
+        <v>44</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>46</v>
       </c>
       <c r="F42" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="G42" s="5">
-        <v>8</v>
+        <v>67</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>47</v>
@@ -6430,19 +6415,19 @@
         <v>50</v>
       </c>
       <c r="L42" s="6">
-        <v>22</v>
+        <v>117</v>
       </c>
       <c r="M42" s="7">
-        <v>7033.62</v>
+        <v>43756.74</v>
       </c>
       <c r="N42" s="6">
         <v>1</v>
       </c>
       <c r="O42" s="3" t="s">
-        <v>91</v>
+        <v>51</v>
       </c>
       <c r="P42" s="8">
-        <v>319.70999999999998</v>
+        <v>373.99</v>
       </c>
       <c r="Q42" s="6">
         <v>0</v>
@@ -6457,16 +6442,16 @@
         <v>52</v>
       </c>
       <c r="U42" s="10">
-        <v>68001</v>
+        <v>67750</v>
       </c>
       <c r="V42" s="11">
         <v>11</v>
       </c>
       <c r="W42" s="4">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="X42" s="12">
-        <v>0.46458329999999998</v>
+        <v>0.43958330000000001</v>
       </c>
       <c r="Y42" s="10">
         <v>0</v>
@@ -6526,275 +6511,7 @@
         <v>53</v>
       </c>
       <c r="AR42" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="43" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
-        <v>1</v>
-      </c>
-      <c r="B43" s="2">
-        <v>2</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F43" s="4">
-        <v>46296</v>
-      </c>
-      <c r="G43" s="5">
-        <v>9</v>
-      </c>
-      <c r="H43" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I43" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J43" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K43" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L43" s="6">
-        <v>23</v>
-      </c>
-      <c r="M43" s="7">
-        <v>7353.33</v>
-      </c>
-      <c r="N43" s="6">
-        <v>1</v>
-      </c>
-      <c r="O43" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="P43" s="8">
-        <v>319.70999999999998</v>
-      </c>
-      <c r="Q43" s="6">
-        <v>0</v>
-      </c>
-      <c r="R43" s="7">
-        <v>0</v>
-      </c>
-      <c r="S43" s="9">
-        <v>0</v>
-      </c>
-      <c r="T43" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="U43" s="10">
-        <v>68001</v>
-      </c>
-      <c r="V43" s="11">
-        <v>11</v>
-      </c>
-      <c r="W43" s="4">
-        <v>46296</v>
-      </c>
-      <c r="X43" s="12">
-        <v>0.46458329999999998</v>
-      </c>
-      <c r="Y43" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB43" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG43" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI43" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AJ43" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK43" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL43" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM43" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ43" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR43" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="44" spans="1:44" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
-        <v>1</v>
-      </c>
-      <c r="B44" s="2">
-        <v>2</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F44" s="4">
-        <v>46296</v>
-      </c>
-      <c r="G44" s="5">
-        <v>10</v>
-      </c>
-      <c r="H44" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I44" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J44" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K44" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L44" s="6">
-        <v>24</v>
-      </c>
-      <c r="M44" s="7">
-        <v>7673.04</v>
-      </c>
-      <c r="N44" s="6">
-        <v>1</v>
-      </c>
-      <c r="O44" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="P44" s="8">
-        <v>319.70999999999998</v>
-      </c>
-      <c r="Q44" s="6">
-        <v>0</v>
-      </c>
-      <c r="R44" s="7">
-        <v>0</v>
-      </c>
-      <c r="S44" s="9">
-        <v>0</v>
-      </c>
-      <c r="T44" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="U44" s="10">
-        <v>68001</v>
-      </c>
-      <c r="V44" s="11">
-        <v>11</v>
-      </c>
-      <c r="W44" s="4">
-        <v>46296</v>
-      </c>
-      <c r="X44" s="12">
-        <v>0.46458329999999998</v>
-      </c>
-      <c r="Y44" s="10">
-        <v>0</v>
-      </c>
-      <c r="Z44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AA44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AB44" s="13">
-        <v>0</v>
-      </c>
-      <c r="AC44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AD44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AE44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AF44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AG44" s="5">
-        <v>0</v>
-      </c>
-      <c r="AH44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AI44" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AJ44" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK44" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL44" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM44" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ44" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR44" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 14/10/2026 12:29:41,21
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5065AE5E-4ACF-47D6-9DC9-F70C82E33F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FDE10212-F98F-43BC-80EA-26185F1B8912}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8036" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8072" uniqueCount="506">
   <si>
     <t>Sel</t>
   </si>
@@ -1306,6 +1306,12 @@
     <t>1871400013178</t>
   </si>
   <si>
+    <t>1871400013179</t>
+  </si>
+  <si>
+    <t>1871400013180</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -2107,7 +2113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR445"/>
+  <dimension ref="A1:AR447"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -51835,7 +51841,7 @@
         <v>411</v>
       </c>
       <c r="D372" s="3" t="s">
-        <v>428</v>
+        <v>45</v>
       </c>
       <c r="E372" s="3" t="s">
         <v>46</v>
@@ -51844,7 +51850,7 @@
         <v>46309</v>
       </c>
       <c r="G372" s="5">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="H372" s="3" t="s">
         <v>47</v>
@@ -51859,19 +51865,19 @@
         <v>50</v>
       </c>
       <c r="L372" s="6">
-        <v>662</v>
+        <v>485</v>
       </c>
       <c r="M372" s="7">
-        <v>215971.5</v>
+        <v>161790.49</v>
       </c>
       <c r="N372" s="6">
         <v>1</v>
       </c>
       <c r="O372" s="3" t="s">
-        <v>429</v>
+        <v>412</v>
       </c>
       <c r="P372" s="8">
-        <v>326.24</v>
+        <v>333.59</v>
       </c>
       <c r="Q372" s="6">
         <v>0</v>
@@ -51886,7 +51892,7 @@
         <v>52</v>
       </c>
       <c r="U372" s="10">
-        <v>68241</v>
+        <v>68286</v>
       </c>
       <c r="V372" s="11">
         <v>11</v>
@@ -51895,7 +51901,7 @@
         <v>46309</v>
       </c>
       <c r="X372" s="12">
-        <v>0.3125</v>
+        <v>0.49305559999999998</v>
       </c>
       <c r="Y372" s="10">
         <v>0</v>
@@ -51955,7 +51961,7 @@
         <v>53</v>
       </c>
       <c r="AR372" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="373" spans="1:44" x14ac:dyDescent="0.3">
@@ -51969,7 +51975,7 @@
         <v>411</v>
       </c>
       <c r="D373" s="3" t="s">
-        <v>428</v>
+        <v>45</v>
       </c>
       <c r="E373" s="3" t="s">
         <v>46</v>
@@ -51978,7 +51984,7 @@
         <v>46309</v>
       </c>
       <c r="G373" s="5">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="H373" s="3" t="s">
         <v>47</v>
@@ -51993,19 +51999,19 @@
         <v>50</v>
       </c>
       <c r="L373" s="6">
-        <v>663</v>
+        <v>486</v>
       </c>
       <c r="M373" s="7">
-        <v>216297.75</v>
+        <v>162124.07</v>
       </c>
       <c r="N373" s="6">
         <v>1</v>
       </c>
       <c r="O373" s="3" t="s">
-        <v>429</v>
+        <v>412</v>
       </c>
       <c r="P373" s="8">
-        <v>326.24</v>
+        <v>333.59</v>
       </c>
       <c r="Q373" s="6">
         <v>0</v>
@@ -52020,7 +52026,7 @@
         <v>52</v>
       </c>
       <c r="U373" s="10">
-        <v>68241</v>
+        <v>68286</v>
       </c>
       <c r="V373" s="11">
         <v>11</v>
@@ -52029,7 +52035,7 @@
         <v>46309</v>
       </c>
       <c r="X373" s="12">
-        <v>0.3125</v>
+        <v>0.49305559999999998</v>
       </c>
       <c r="Y373" s="10">
         <v>0</v>
@@ -52089,7 +52095,7 @@
         <v>53</v>
       </c>
       <c r="AR373" s="3" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="374" spans="1:44" x14ac:dyDescent="0.3">
@@ -52103,7 +52109,7 @@
         <v>411</v>
       </c>
       <c r="D374" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E374" s="3" t="s">
         <v>46</v>
@@ -52112,7 +52118,7 @@
         <v>46309</v>
       </c>
       <c r="G374" s="5">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H374" s="3" t="s">
         <v>47</v>
@@ -52127,16 +52133,16 @@
         <v>50</v>
       </c>
       <c r="L374" s="6">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="M374" s="7">
-        <v>216623.99</v>
+        <v>215971.5</v>
       </c>
       <c r="N374" s="6">
         <v>1</v>
       </c>
       <c r="O374" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P374" s="8">
         <v>326.24</v>
@@ -52237,7 +52243,7 @@
         <v>411</v>
       </c>
       <c r="D375" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E375" s="3" t="s">
         <v>46</v>
@@ -52246,7 +52252,7 @@
         <v>46309</v>
       </c>
       <c r="G375" s="5">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H375" s="3" t="s">
         <v>47</v>
@@ -52261,16 +52267,16 @@
         <v>50</v>
       </c>
       <c r="L375" s="6">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="M375" s="7">
-        <v>216950.23</v>
+        <v>216297.75</v>
       </c>
       <c r="N375" s="6">
         <v>1</v>
       </c>
       <c r="O375" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P375" s="8">
         <v>326.24</v>
@@ -52371,7 +52377,7 @@
         <v>411</v>
       </c>
       <c r="D376" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E376" s="3" t="s">
         <v>46</v>
@@ -52380,7 +52386,7 @@
         <v>46309</v>
       </c>
       <c r="G376" s="5">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H376" s="3" t="s">
         <v>47</v>
@@ -52395,16 +52401,16 @@
         <v>50</v>
       </c>
       <c r="L376" s="6">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="M376" s="7">
-        <v>217276.47</v>
+        <v>216623.99</v>
       </c>
       <c r="N376" s="6">
         <v>1</v>
       </c>
       <c r="O376" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P376" s="8">
         <v>326.24</v>
@@ -52505,7 +52511,7 @@
         <v>411</v>
       </c>
       <c r="D377" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E377" s="3" t="s">
         <v>46</v>
@@ -52514,7 +52520,7 @@
         <v>46309</v>
       </c>
       <c r="G377" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H377" s="3" t="s">
         <v>47</v>
@@ -52529,16 +52535,16 @@
         <v>50</v>
       </c>
       <c r="L377" s="6">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="M377" s="7">
-        <v>217602.71</v>
+        <v>216950.23</v>
       </c>
       <c r="N377" s="6">
         <v>1</v>
       </c>
       <c r="O377" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P377" s="8">
         <v>326.24</v>
@@ -52639,7 +52645,7 @@
         <v>411</v>
       </c>
       <c r="D378" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E378" s="3" t="s">
         <v>46</v>
@@ -52648,7 +52654,7 @@
         <v>46309</v>
       </c>
       <c r="G378" s="5">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H378" s="3" t="s">
         <v>47</v>
@@ -52663,16 +52669,16 @@
         <v>50</v>
       </c>
       <c r="L378" s="6">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="M378" s="7">
-        <v>217928.95</v>
+        <v>217276.47</v>
       </c>
       <c r="N378" s="6">
         <v>1</v>
       </c>
       <c r="O378" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P378" s="8">
         <v>326.24</v>
@@ -52773,7 +52779,7 @@
         <v>411</v>
       </c>
       <c r="D379" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E379" s="3" t="s">
         <v>46</v>
@@ -52782,7 +52788,7 @@
         <v>46309</v>
       </c>
       <c r="G379" s="5">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H379" s="3" t="s">
         <v>47</v>
@@ -52797,16 +52803,16 @@
         <v>50</v>
       </c>
       <c r="L379" s="6">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="M379" s="7">
-        <v>218255.19</v>
+        <v>217602.71</v>
       </c>
       <c r="N379" s="6">
         <v>1</v>
       </c>
       <c r="O379" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P379" s="8">
         <v>326.24</v>
@@ -52833,7 +52839,7 @@
         <v>46309</v>
       </c>
       <c r="X379" s="12">
-        <v>0.32708330000000002</v>
+        <v>0.3125</v>
       </c>
       <c r="Y379" s="10">
         <v>0</v>
@@ -52907,7 +52913,7 @@
         <v>411</v>
       </c>
       <c r="D380" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E380" s="3" t="s">
         <v>46</v>
@@ -52916,7 +52922,7 @@
         <v>46309</v>
       </c>
       <c r="G380" s="5">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H380" s="3" t="s">
         <v>47</v>
@@ -52931,16 +52937,16 @@
         <v>50</v>
       </c>
       <c r="L380" s="6">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="M380" s="7">
-        <v>218581.43</v>
+        <v>217928.95</v>
       </c>
       <c r="N380" s="6">
         <v>1</v>
       </c>
       <c r="O380" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P380" s="8">
         <v>326.24</v>
@@ -52967,7 +52973,7 @@
         <v>46309</v>
       </c>
       <c r="X380" s="12">
-        <v>0.32708330000000002</v>
+        <v>0.3125</v>
       </c>
       <c r="Y380" s="10">
         <v>0</v>
@@ -53041,7 +53047,7 @@
         <v>411</v>
       </c>
       <c r="D381" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E381" s="3" t="s">
         <v>46</v>
@@ -53050,7 +53056,7 @@
         <v>46309</v>
       </c>
       <c r="G381" s="5">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H381" s="3" t="s">
         <v>47</v>
@@ -53065,16 +53071,16 @@
         <v>50</v>
       </c>
       <c r="L381" s="6">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="M381" s="7">
-        <v>218907.67</v>
+        <v>218255.19</v>
       </c>
       <c r="N381" s="6">
         <v>1</v>
       </c>
       <c r="O381" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P381" s="8">
         <v>326.24</v>
@@ -53175,7 +53181,7 @@
         <v>411</v>
       </c>
       <c r="D382" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E382" s="3" t="s">
         <v>46</v>
@@ -53184,7 +53190,7 @@
         <v>46309</v>
       </c>
       <c r="G382" s="5">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H382" s="3" t="s">
         <v>47</v>
@@ -53199,16 +53205,16 @@
         <v>50</v>
       </c>
       <c r="L382" s="6">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="M382" s="7">
-        <v>219233.91</v>
+        <v>218581.43</v>
       </c>
       <c r="N382" s="6">
         <v>1</v>
       </c>
       <c r="O382" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P382" s="8">
         <v>326.24</v>
@@ -53309,7 +53315,7 @@
         <v>411</v>
       </c>
       <c r="D383" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E383" s="3" t="s">
         <v>46</v>
@@ -53318,7 +53324,7 @@
         <v>46309</v>
       </c>
       <c r="G383" s="5">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H383" s="3" t="s">
         <v>47</v>
@@ -53333,16 +53339,16 @@
         <v>50</v>
       </c>
       <c r="L383" s="6">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="M383" s="7">
-        <v>219560.15</v>
+        <v>218907.67</v>
       </c>
       <c r="N383" s="6">
         <v>1</v>
       </c>
       <c r="O383" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P383" s="8">
         <v>326.24</v>
@@ -53443,7 +53449,7 @@
         <v>411</v>
       </c>
       <c r="D384" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E384" s="3" t="s">
         <v>46</v>
@@ -53452,7 +53458,7 @@
         <v>46309</v>
       </c>
       <c r="G384" s="5">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H384" s="3" t="s">
         <v>47</v>
@@ -53467,16 +53473,16 @@
         <v>50</v>
       </c>
       <c r="L384" s="6">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="M384" s="7">
-        <v>219886.4</v>
+        <v>219233.91</v>
       </c>
       <c r="N384" s="6">
         <v>1</v>
       </c>
       <c r="O384" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P384" s="8">
         <v>326.24</v>
@@ -53577,7 +53583,7 @@
         <v>411</v>
       </c>
       <c r="D385" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E385" s="3" t="s">
         <v>46</v>
@@ -53586,7 +53592,7 @@
         <v>46309</v>
       </c>
       <c r="G385" s="5">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H385" s="3" t="s">
         <v>47</v>
@@ -53601,16 +53607,16 @@
         <v>50</v>
       </c>
       <c r="L385" s="6">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="M385" s="7">
-        <v>220212.64</v>
+        <v>219560.15</v>
       </c>
       <c r="N385" s="6">
         <v>1</v>
       </c>
       <c r="O385" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P385" s="8">
         <v>326.24</v>
@@ -53637,7 +53643,7 @@
         <v>46309</v>
       </c>
       <c r="X385" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.32708330000000002</v>
       </c>
       <c r="Y385" s="10">
         <v>0</v>
@@ -53711,7 +53717,7 @@
         <v>411</v>
       </c>
       <c r="D386" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E386" s="3" t="s">
         <v>46</v>
@@ -53720,7 +53726,7 @@
         <v>46309</v>
       </c>
       <c r="G386" s="5">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H386" s="3" t="s">
         <v>47</v>
@@ -53735,16 +53741,16 @@
         <v>50</v>
       </c>
       <c r="L386" s="6">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="M386" s="7">
-        <v>220538.88</v>
+        <v>219886.4</v>
       </c>
       <c r="N386" s="6">
         <v>1</v>
       </c>
       <c r="O386" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P386" s="8">
         <v>326.24</v>
@@ -53771,7 +53777,7 @@
         <v>46309</v>
       </c>
       <c r="X386" s="12">
-        <v>0.34027780000000002</v>
+        <v>0.32708330000000002</v>
       </c>
       <c r="Y386" s="10">
         <v>0</v>
@@ -53845,7 +53851,7 @@
         <v>411</v>
       </c>
       <c r="D387" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E387" s="3" t="s">
         <v>46</v>
@@ -53854,7 +53860,7 @@
         <v>46309</v>
       </c>
       <c r="G387" s="5">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H387" s="3" t="s">
         <v>47</v>
@@ -53869,16 +53875,16 @@
         <v>50</v>
       </c>
       <c r="L387" s="6">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="M387" s="7">
-        <v>220865.12</v>
+        <v>220212.64</v>
       </c>
       <c r="N387" s="6">
         <v>1</v>
       </c>
       <c r="O387" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P387" s="8">
         <v>326.24</v>
@@ -53979,7 +53985,7 @@
         <v>411</v>
       </c>
       <c r="D388" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E388" s="3" t="s">
         <v>46</v>
@@ -53988,7 +53994,7 @@
         <v>46309</v>
       </c>
       <c r="G388" s="5">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H388" s="3" t="s">
         <v>47</v>
@@ -54003,16 +54009,16 @@
         <v>50</v>
       </c>
       <c r="L388" s="6">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="M388" s="7">
-        <v>221191.36</v>
+        <v>220538.88</v>
       </c>
       <c r="N388" s="6">
         <v>1</v>
       </c>
       <c r="O388" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P388" s="8">
         <v>326.24</v>
@@ -54113,7 +54119,7 @@
         <v>411</v>
       </c>
       <c r="D389" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E389" s="3" t="s">
         <v>46</v>
@@ -54122,7 +54128,7 @@
         <v>46309</v>
       </c>
       <c r="G389" s="5">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H389" s="3" t="s">
         <v>47</v>
@@ -54137,16 +54143,16 @@
         <v>50</v>
       </c>
       <c r="L389" s="6">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="M389" s="7">
-        <v>221517.6</v>
+        <v>220865.12</v>
       </c>
       <c r="N389" s="6">
         <v>1</v>
       </c>
       <c r="O389" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P389" s="8">
         <v>326.24</v>
@@ -54247,7 +54253,7 @@
         <v>411</v>
       </c>
       <c r="D390" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E390" s="3" t="s">
         <v>46</v>
@@ -54256,7 +54262,7 @@
         <v>46309</v>
       </c>
       <c r="G390" s="5">
-        <v>310</v>
+        <v>21</v>
       </c>
       <c r="H390" s="3" t="s">
         <v>47</v>
@@ -54271,16 +54277,16 @@
         <v>50</v>
       </c>
       <c r="L390" s="6">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="M390" s="7">
-        <v>221843.84</v>
+        <v>221191.36</v>
       </c>
       <c r="N390" s="6">
         <v>1</v>
       </c>
       <c r="O390" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P390" s="8">
         <v>326.24</v>
@@ -54307,7 +54313,7 @@
         <v>46309</v>
       </c>
       <c r="X390" s="12">
-        <v>0.4819444</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y390" s="10">
         <v>0</v>
@@ -54381,7 +54387,7 @@
         <v>411</v>
       </c>
       <c r="D391" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E391" s="3" t="s">
         <v>46</v>
@@ -54390,7 +54396,7 @@
         <v>46309</v>
       </c>
       <c r="G391" s="5">
-        <v>311</v>
+        <v>22</v>
       </c>
       <c r="H391" s="3" t="s">
         <v>47</v>
@@ -54405,16 +54411,16 @@
         <v>50</v>
       </c>
       <c r="L391" s="6">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="M391" s="7">
-        <v>222170.08</v>
+        <v>221517.6</v>
       </c>
       <c r="N391" s="6">
         <v>1</v>
       </c>
       <c r="O391" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P391" s="8">
         <v>326.24</v>
@@ -54441,7 +54447,7 @@
         <v>46309</v>
       </c>
       <c r="X391" s="12">
-        <v>0.4819444</v>
+        <v>0.34027780000000002</v>
       </c>
       <c r="Y391" s="10">
         <v>0</v>
@@ -54515,7 +54521,7 @@
         <v>411</v>
       </c>
       <c r="D392" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E392" s="3" t="s">
         <v>46</v>
@@ -54524,7 +54530,7 @@
         <v>46309</v>
       </c>
       <c r="G392" s="5">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="H392" s="3" t="s">
         <v>47</v>
@@ -54539,16 +54545,16 @@
         <v>50</v>
       </c>
       <c r="L392" s="6">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="M392" s="7">
-        <v>222496.32</v>
+        <v>221843.84</v>
       </c>
       <c r="N392" s="6">
         <v>1</v>
       </c>
       <c r="O392" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P392" s="8">
         <v>326.24</v>
@@ -54649,7 +54655,7 @@
         <v>411</v>
       </c>
       <c r="D393" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E393" s="3" t="s">
         <v>46</v>
@@ -54658,7 +54664,7 @@
         <v>46309</v>
       </c>
       <c r="G393" s="5">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H393" s="3" t="s">
         <v>47</v>
@@ -54673,16 +54679,16 @@
         <v>50</v>
       </c>
       <c r="L393" s="6">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="M393" s="7">
-        <v>222822.56</v>
+        <v>222170.08</v>
       </c>
       <c r="N393" s="6">
         <v>1</v>
       </c>
       <c r="O393" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P393" s="8">
         <v>326.24</v>
@@ -54783,7 +54789,7 @@
         <v>411</v>
       </c>
       <c r="D394" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E394" s="3" t="s">
         <v>46</v>
@@ -54792,7 +54798,7 @@
         <v>46309</v>
       </c>
       <c r="G394" s="5">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H394" s="3" t="s">
         <v>47</v>
@@ -54807,16 +54813,16 @@
         <v>50</v>
       </c>
       <c r="L394" s="6">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="M394" s="7">
-        <v>223148.81</v>
+        <v>222496.32</v>
       </c>
       <c r="N394" s="6">
         <v>1</v>
       </c>
       <c r="O394" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P394" s="8">
         <v>326.24</v>
@@ -54917,7 +54923,7 @@
         <v>411</v>
       </c>
       <c r="D395" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E395" s="3" t="s">
         <v>46</v>
@@ -54926,7 +54932,7 @@
         <v>46309</v>
       </c>
       <c r="G395" s="5">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H395" s="3" t="s">
         <v>47</v>
@@ -54941,16 +54947,16 @@
         <v>50</v>
       </c>
       <c r="L395" s="6">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="M395" s="7">
-        <v>223475.05</v>
+        <v>222822.56</v>
       </c>
       <c r="N395" s="6">
         <v>1</v>
       </c>
       <c r="O395" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P395" s="8">
         <v>326.24</v>
@@ -55051,7 +55057,7 @@
         <v>411</v>
       </c>
       <c r="D396" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E396" s="3" t="s">
         <v>46</v>
@@ -55060,7 +55066,7 @@
         <v>46309</v>
       </c>
       <c r="G396" s="5">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H396" s="3" t="s">
         <v>47</v>
@@ -55075,16 +55081,16 @@
         <v>50</v>
       </c>
       <c r="L396" s="6">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="M396" s="7">
-        <v>223801.29</v>
+        <v>223148.81</v>
       </c>
       <c r="N396" s="6">
         <v>1</v>
       </c>
       <c r="O396" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P396" s="8">
         <v>326.24</v>
@@ -55185,7 +55191,7 @@
         <v>411</v>
       </c>
       <c r="D397" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E397" s="3" t="s">
         <v>46</v>
@@ -55194,7 +55200,7 @@
         <v>46309</v>
       </c>
       <c r="G397" s="5">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="H397" s="3" t="s">
         <v>47</v>
@@ -55209,16 +55215,16 @@
         <v>50</v>
       </c>
       <c r="L397" s="6">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="M397" s="7">
-        <v>224127.53</v>
+        <v>223475.05</v>
       </c>
       <c r="N397" s="6">
         <v>1</v>
       </c>
       <c r="O397" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P397" s="8">
         <v>326.24</v>
@@ -55319,7 +55325,7 @@
         <v>411</v>
       </c>
       <c r="D398" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E398" s="3" t="s">
         <v>46</v>
@@ -55328,7 +55334,7 @@
         <v>46309</v>
       </c>
       <c r="G398" s="5">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="H398" s="3" t="s">
         <v>47</v>
@@ -55343,16 +55349,16 @@
         <v>50</v>
       </c>
       <c r="L398" s="6">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="M398" s="7">
-        <v>224453.77</v>
+        <v>223801.29</v>
       </c>
       <c r="N398" s="6">
         <v>1</v>
       </c>
       <c r="O398" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P398" s="8">
         <v>326.24</v>
@@ -55453,7 +55459,7 @@
         <v>411</v>
       </c>
       <c r="D399" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E399" s="3" t="s">
         <v>46</v>
@@ -55462,7 +55468,7 @@
         <v>46309</v>
       </c>
       <c r="G399" s="5">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="H399" s="3" t="s">
         <v>47</v>
@@ -55477,16 +55483,16 @@
         <v>50</v>
       </c>
       <c r="L399" s="6">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="M399" s="7">
-        <v>224780.01</v>
+        <v>224127.53</v>
       </c>
       <c r="N399" s="6">
         <v>1</v>
       </c>
       <c r="O399" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P399" s="8">
         <v>326.24</v>
@@ -55587,7 +55593,7 @@
         <v>411</v>
       </c>
       <c r="D400" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E400" s="3" t="s">
         <v>46</v>
@@ -55596,7 +55602,7 @@
         <v>46309</v>
       </c>
       <c r="G400" s="5">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H400" s="3" t="s">
         <v>47</v>
@@ -55611,16 +55617,16 @@
         <v>50</v>
       </c>
       <c r="L400" s="6">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="M400" s="7">
-        <v>225106.25</v>
+        <v>224453.77</v>
       </c>
       <c r="N400" s="6">
         <v>1</v>
       </c>
       <c r="O400" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P400" s="8">
         <v>326.24</v>
@@ -55721,7 +55727,7 @@
         <v>411</v>
       </c>
       <c r="D401" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E401" s="3" t="s">
         <v>46</v>
@@ -55730,7 +55736,7 @@
         <v>46309</v>
       </c>
       <c r="G401" s="5">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="H401" s="3" t="s">
         <v>47</v>
@@ -55745,16 +55751,16 @@
         <v>50</v>
       </c>
       <c r="L401" s="6">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="M401" s="7">
-        <v>225432.49</v>
+        <v>224780.01</v>
       </c>
       <c r="N401" s="6">
         <v>1</v>
       </c>
       <c r="O401" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P401" s="8">
         <v>326.24</v>
@@ -55855,7 +55861,7 @@
         <v>411</v>
       </c>
       <c r="D402" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E402" s="3" t="s">
         <v>46</v>
@@ -55864,7 +55870,7 @@
         <v>46309</v>
       </c>
       <c r="G402" s="5">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H402" s="3" t="s">
         <v>47</v>
@@ -55879,16 +55885,16 @@
         <v>50</v>
       </c>
       <c r="L402" s="6">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="M402" s="7">
-        <v>225758.73</v>
+        <v>225106.25</v>
       </c>
       <c r="N402" s="6">
         <v>1</v>
       </c>
       <c r="O402" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P402" s="8">
         <v>326.24</v>
@@ -55989,7 +55995,7 @@
         <v>411</v>
       </c>
       <c r="D403" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E403" s="3" t="s">
         <v>46</v>
@@ -55998,7 +56004,7 @@
         <v>46309</v>
       </c>
       <c r="G403" s="5">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H403" s="3" t="s">
         <v>47</v>
@@ -56013,16 +56019,16 @@
         <v>50</v>
       </c>
       <c r="L403" s="6">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="M403" s="7">
-        <v>226084.97</v>
+        <v>225432.49</v>
       </c>
       <c r="N403" s="6">
         <v>1</v>
       </c>
       <c r="O403" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P403" s="8">
         <v>326.24</v>
@@ -56123,7 +56129,7 @@
         <v>411</v>
       </c>
       <c r="D404" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E404" s="3" t="s">
         <v>46</v>
@@ -56132,7 +56138,7 @@
         <v>46309</v>
       </c>
       <c r="G404" s="5">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="H404" s="3" t="s">
         <v>47</v>
@@ -56147,16 +56153,16 @@
         <v>50</v>
       </c>
       <c r="L404" s="6">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="M404" s="7">
-        <v>226411.21</v>
+        <v>225758.73</v>
       </c>
       <c r="N404" s="6">
         <v>1</v>
       </c>
       <c r="O404" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P404" s="8">
         <v>326.24</v>
@@ -56257,7 +56263,7 @@
         <v>411</v>
       </c>
       <c r="D405" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E405" s="3" t="s">
         <v>46</v>
@@ -56266,7 +56272,7 @@
         <v>46309</v>
       </c>
       <c r="G405" s="5">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H405" s="3" t="s">
         <v>47</v>
@@ -56281,16 +56287,16 @@
         <v>50</v>
       </c>
       <c r="L405" s="6">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="M405" s="7">
-        <v>226737.46</v>
+        <v>226084.97</v>
       </c>
       <c r="N405" s="6">
         <v>1</v>
       </c>
       <c r="O405" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P405" s="8">
         <v>326.24</v>
@@ -56391,7 +56397,7 @@
         <v>411</v>
       </c>
       <c r="D406" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E406" s="3" t="s">
         <v>46</v>
@@ -56400,7 +56406,7 @@
         <v>46309</v>
       </c>
       <c r="G406" s="5">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H406" s="3" t="s">
         <v>47</v>
@@ -56415,16 +56421,16 @@
         <v>50</v>
       </c>
       <c r="L406" s="6">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="M406" s="7">
-        <v>227063.7</v>
+        <v>226411.21</v>
       </c>
       <c r="N406" s="6">
         <v>1</v>
       </c>
       <c r="O406" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P406" s="8">
         <v>326.24</v>
@@ -56525,7 +56531,7 @@
         <v>411</v>
       </c>
       <c r="D407" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E407" s="3" t="s">
         <v>46</v>
@@ -56534,7 +56540,7 @@
         <v>46309</v>
       </c>
       <c r="G407" s="5">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H407" s="3" t="s">
         <v>47</v>
@@ -56549,16 +56555,16 @@
         <v>50</v>
       </c>
       <c r="L407" s="6">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="M407" s="7">
-        <v>227389.94</v>
+        <v>226737.46</v>
       </c>
       <c r="N407" s="6">
         <v>1</v>
       </c>
       <c r="O407" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P407" s="8">
         <v>326.24</v>
@@ -56659,7 +56665,7 @@
         <v>411</v>
       </c>
       <c r="D408" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E408" s="3" t="s">
         <v>46</v>
@@ -56668,7 +56674,7 @@
         <v>46309</v>
       </c>
       <c r="G408" s="5">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H408" s="3" t="s">
         <v>47</v>
@@ -56683,16 +56689,16 @@
         <v>50</v>
       </c>
       <c r="L408" s="6">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="M408" s="7">
-        <v>227716.18</v>
+        <v>227063.7</v>
       </c>
       <c r="N408" s="6">
         <v>1</v>
       </c>
       <c r="O408" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P408" s="8">
         <v>326.24</v>
@@ -56793,7 +56799,7 @@
         <v>411</v>
       </c>
       <c r="D409" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E409" s="3" t="s">
         <v>46</v>
@@ -56802,7 +56808,7 @@
         <v>46309</v>
       </c>
       <c r="G409" s="5">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="H409" s="3" t="s">
         <v>47</v>
@@ -56817,16 +56823,16 @@
         <v>50</v>
       </c>
       <c r="L409" s="6">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="M409" s="7">
-        <v>228042.42</v>
+        <v>227389.94</v>
       </c>
       <c r="N409" s="6">
         <v>1</v>
       </c>
       <c r="O409" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P409" s="8">
         <v>326.24</v>
@@ -56927,7 +56933,7 @@
         <v>411</v>
       </c>
       <c r="D410" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E410" s="3" t="s">
         <v>46</v>
@@ -56936,7 +56942,7 @@
         <v>46309</v>
       </c>
       <c r="G410" s="5">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="H410" s="3" t="s">
         <v>47</v>
@@ -56951,16 +56957,16 @@
         <v>50</v>
       </c>
       <c r="L410" s="6">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="M410" s="7">
-        <v>228368.66</v>
+        <v>227716.18</v>
       </c>
       <c r="N410" s="6">
         <v>1</v>
       </c>
       <c r="O410" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P410" s="8">
         <v>326.24</v>
@@ -57061,7 +57067,7 @@
         <v>411</v>
       </c>
       <c r="D411" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E411" s="3" t="s">
         <v>46</v>
@@ -57070,7 +57076,7 @@
         <v>46309</v>
       </c>
       <c r="G411" s="5">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="H411" s="3" t="s">
         <v>47</v>
@@ -57085,16 +57091,16 @@
         <v>50</v>
       </c>
       <c r="L411" s="6">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="M411" s="7">
-        <v>228694.9</v>
+        <v>228042.42</v>
       </c>
       <c r="N411" s="6">
         <v>1</v>
       </c>
       <c r="O411" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P411" s="8">
         <v>326.24</v>
@@ -57195,7 +57201,7 @@
         <v>411</v>
       </c>
       <c r="D412" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E412" s="3" t="s">
         <v>46</v>
@@ -57204,7 +57210,7 @@
         <v>46309</v>
       </c>
       <c r="G412" s="5">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H412" s="3" t="s">
         <v>47</v>
@@ -57219,16 +57225,16 @@
         <v>50</v>
       </c>
       <c r="L412" s="6">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="M412" s="7">
-        <v>229021.14</v>
+        <v>228368.66</v>
       </c>
       <c r="N412" s="6">
         <v>1</v>
       </c>
       <c r="O412" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P412" s="8">
         <v>326.24</v>
@@ -57329,7 +57335,7 @@
         <v>411</v>
       </c>
       <c r="D413" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E413" s="3" t="s">
         <v>46</v>
@@ -57338,7 +57344,7 @@
         <v>46309</v>
       </c>
       <c r="G413" s="5">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="H413" s="3" t="s">
         <v>47</v>
@@ -57353,16 +57359,16 @@
         <v>50</v>
       </c>
       <c r="L413" s="6">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="M413" s="7">
-        <v>229347.38</v>
+        <v>228694.9</v>
       </c>
       <c r="N413" s="6">
         <v>1</v>
       </c>
       <c r="O413" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P413" s="8">
         <v>326.24</v>
@@ -57463,7 +57469,7 @@
         <v>411</v>
       </c>
       <c r="D414" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E414" s="3" t="s">
         <v>46</v>
@@ -57472,7 +57478,7 @@
         <v>46309</v>
       </c>
       <c r="G414" s="5">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H414" s="3" t="s">
         <v>47</v>
@@ -57487,16 +57493,16 @@
         <v>50</v>
       </c>
       <c r="L414" s="6">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="M414" s="7">
-        <v>229673.62</v>
+        <v>229021.14</v>
       </c>
       <c r="N414" s="6">
         <v>1</v>
       </c>
       <c r="O414" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P414" s="8">
         <v>326.24</v>
@@ -57597,7 +57603,7 @@
         <v>411</v>
       </c>
       <c r="D415" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E415" s="3" t="s">
         <v>46</v>
@@ -57606,7 +57612,7 @@
         <v>46309</v>
       </c>
       <c r="G415" s="5">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="H415" s="3" t="s">
         <v>47</v>
@@ -57621,16 +57627,16 @@
         <v>50</v>
       </c>
       <c r="L415" s="6">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="M415" s="7">
-        <v>229999.86</v>
+        <v>229347.38</v>
       </c>
       <c r="N415" s="6">
         <v>1</v>
       </c>
       <c r="O415" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P415" s="8">
         <v>326.24</v>
@@ -57731,7 +57737,7 @@
         <v>411</v>
       </c>
       <c r="D416" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E416" s="3" t="s">
         <v>46</v>
@@ -57740,7 +57746,7 @@
         <v>46309</v>
       </c>
       <c r="G416" s="5">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="H416" s="3" t="s">
         <v>47</v>
@@ -57755,16 +57761,16 @@
         <v>50</v>
       </c>
       <c r="L416" s="6">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="M416" s="7">
-        <v>230326.11</v>
+        <v>229673.62</v>
       </c>
       <c r="N416" s="6">
         <v>1</v>
       </c>
       <c r="O416" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P416" s="8">
         <v>326.24</v>
@@ -57865,7 +57871,7 @@
         <v>411</v>
       </c>
       <c r="D417" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E417" s="3" t="s">
         <v>46</v>
@@ -57874,7 +57880,7 @@
         <v>46309</v>
       </c>
       <c r="G417" s="5">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="H417" s="3" t="s">
         <v>47</v>
@@ -57889,16 +57895,16 @@
         <v>50</v>
       </c>
       <c r="L417" s="6">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="M417" s="7">
-        <v>230652.35</v>
+        <v>229999.86</v>
       </c>
       <c r="N417" s="6">
         <v>1</v>
       </c>
       <c r="O417" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P417" s="8">
         <v>326.24</v>
@@ -57999,7 +58005,7 @@
         <v>411</v>
       </c>
       <c r="D418" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E418" s="3" t="s">
         <v>46</v>
@@ -58008,7 +58014,7 @@
         <v>46309</v>
       </c>
       <c r="G418" s="5">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H418" s="3" t="s">
         <v>47</v>
@@ -58023,16 +58029,16 @@
         <v>50</v>
       </c>
       <c r="L418" s="6">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="M418" s="7">
-        <v>230978.59</v>
+        <v>230326.11</v>
       </c>
       <c r="N418" s="6">
         <v>1</v>
       </c>
       <c r="O418" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P418" s="8">
         <v>326.24</v>
@@ -58133,7 +58139,7 @@
         <v>411</v>
       </c>
       <c r="D419" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E419" s="3" t="s">
         <v>46</v>
@@ -58142,7 +58148,7 @@
         <v>46309</v>
       </c>
       <c r="G419" s="5">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="H419" s="3" t="s">
         <v>47</v>
@@ -58157,16 +58163,16 @@
         <v>50</v>
       </c>
       <c r="L419" s="6">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="M419" s="7">
-        <v>231304.83</v>
+        <v>230652.35</v>
       </c>
       <c r="N419" s="6">
         <v>1</v>
       </c>
       <c r="O419" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P419" s="8">
         <v>326.24</v>
@@ -58193,7 +58199,7 @@
         <v>46309</v>
       </c>
       <c r="X419" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.4819444</v>
       </c>
       <c r="Y419" s="10">
         <v>0</v>
@@ -58267,7 +58273,7 @@
         <v>411</v>
       </c>
       <c r="D420" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E420" s="3" t="s">
         <v>46</v>
@@ -58276,7 +58282,7 @@
         <v>46309</v>
       </c>
       <c r="G420" s="5">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H420" s="3" t="s">
         <v>47</v>
@@ -58291,16 +58297,16 @@
         <v>50</v>
       </c>
       <c r="L420" s="6">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="M420" s="7">
-        <v>231631.07</v>
+        <v>230978.59</v>
       </c>
       <c r="N420" s="6">
         <v>1</v>
       </c>
       <c r="O420" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P420" s="8">
         <v>326.24</v>
@@ -58327,7 +58333,7 @@
         <v>46309</v>
       </c>
       <c r="X420" s="12">
-        <v>0.48263889999999998</v>
+        <v>0.4819444</v>
       </c>
       <c r="Y420" s="10">
         <v>0</v>
@@ -58401,7 +58407,7 @@
         <v>411</v>
       </c>
       <c r="D421" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E421" s="3" t="s">
         <v>46</v>
@@ -58410,7 +58416,7 @@
         <v>46309</v>
       </c>
       <c r="G421" s="5">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="H421" s="3" t="s">
         <v>47</v>
@@ -58425,16 +58431,16 @@
         <v>50</v>
       </c>
       <c r="L421" s="6">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="M421" s="7">
-        <v>231957.31</v>
+        <v>231304.83</v>
       </c>
       <c r="N421" s="6">
         <v>1</v>
       </c>
       <c r="O421" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P421" s="8">
         <v>326.24</v>
@@ -58535,7 +58541,7 @@
         <v>411</v>
       </c>
       <c r="D422" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E422" s="3" t="s">
         <v>46</v>
@@ -58544,7 +58550,7 @@
         <v>46309</v>
       </c>
       <c r="G422" s="5">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H422" s="3" t="s">
         <v>47</v>
@@ -58559,16 +58565,16 @@
         <v>50</v>
       </c>
       <c r="L422" s="6">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="M422" s="7">
-        <v>232283.55</v>
+        <v>231631.07</v>
       </c>
       <c r="N422" s="6">
         <v>1</v>
       </c>
       <c r="O422" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P422" s="8">
         <v>326.24</v>
@@ -58669,7 +58675,7 @@
         <v>411</v>
       </c>
       <c r="D423" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E423" s="3" t="s">
         <v>46</v>
@@ -58678,7 +58684,7 @@
         <v>46309</v>
       </c>
       <c r="G423" s="5">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H423" s="3" t="s">
         <v>47</v>
@@ -58693,16 +58699,16 @@
         <v>50</v>
       </c>
       <c r="L423" s="6">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="M423" s="7">
-        <v>232609.79</v>
+        <v>231957.31</v>
       </c>
       <c r="N423" s="6">
         <v>1</v>
       </c>
       <c r="O423" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P423" s="8">
         <v>326.24</v>
@@ -58803,7 +58809,7 @@
         <v>411</v>
       </c>
       <c r="D424" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E424" s="3" t="s">
         <v>46</v>
@@ -58812,7 +58818,7 @@
         <v>46309</v>
       </c>
       <c r="G424" s="5">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H424" s="3" t="s">
         <v>47</v>
@@ -58827,16 +58833,16 @@
         <v>50</v>
       </c>
       <c r="L424" s="6">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="M424" s="7">
-        <v>232936.03</v>
+        <v>232283.55</v>
       </c>
       <c r="N424" s="6">
         <v>1</v>
       </c>
       <c r="O424" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P424" s="8">
         <v>326.24</v>
@@ -58937,7 +58943,7 @@
         <v>411</v>
       </c>
       <c r="D425" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E425" s="3" t="s">
         <v>46</v>
@@ -58946,7 +58952,7 @@
         <v>46309</v>
       </c>
       <c r="G425" s="5">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="H425" s="3" t="s">
         <v>47</v>
@@ -58961,16 +58967,16 @@
         <v>50</v>
       </c>
       <c r="L425" s="6">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="M425" s="7">
-        <v>233262.27</v>
+        <v>232609.79</v>
       </c>
       <c r="N425" s="6">
         <v>1</v>
       </c>
       <c r="O425" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P425" s="8">
         <v>326.24</v>
@@ -59071,7 +59077,7 @@
         <v>411</v>
       </c>
       <c r="D426" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E426" s="3" t="s">
         <v>46</v>
@@ -59080,7 +59086,7 @@
         <v>46309</v>
       </c>
       <c r="G426" s="5">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="H426" s="3" t="s">
         <v>47</v>
@@ -59095,16 +59101,16 @@
         <v>50</v>
       </c>
       <c r="L426" s="6">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="M426" s="7">
-        <v>233588.52</v>
+        <v>232936.03</v>
       </c>
       <c r="N426" s="6">
         <v>1</v>
       </c>
       <c r="O426" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P426" s="8">
         <v>326.24</v>
@@ -59205,7 +59211,7 @@
         <v>411</v>
       </c>
       <c r="D427" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E427" s="3" t="s">
         <v>46</v>
@@ -59214,7 +59220,7 @@
         <v>46309</v>
       </c>
       <c r="G427" s="5">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="H427" s="3" t="s">
         <v>47</v>
@@ -59229,16 +59235,16 @@
         <v>50</v>
       </c>
       <c r="L427" s="6">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="M427" s="7">
-        <v>233914.76</v>
+        <v>233262.27</v>
       </c>
       <c r="N427" s="6">
         <v>1</v>
       </c>
       <c r="O427" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P427" s="8">
         <v>326.24</v>
@@ -59339,7 +59345,7 @@
         <v>411</v>
       </c>
       <c r="D428" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E428" s="3" t="s">
         <v>46</v>
@@ -59348,7 +59354,7 @@
         <v>46309</v>
       </c>
       <c r="G428" s="5">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H428" s="3" t="s">
         <v>47</v>
@@ -59363,16 +59369,16 @@
         <v>50</v>
       </c>
       <c r="L428" s="6">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="M428" s="7">
-        <v>234241</v>
+        <v>233588.52</v>
       </c>
       <c r="N428" s="6">
         <v>1</v>
       </c>
       <c r="O428" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P428" s="8">
         <v>326.24</v>
@@ -59473,7 +59479,7 @@
         <v>411</v>
       </c>
       <c r="D429" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E429" s="3" t="s">
         <v>46</v>
@@ -59482,7 +59488,7 @@
         <v>46309</v>
       </c>
       <c r="G429" s="5">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="H429" s="3" t="s">
         <v>47</v>
@@ -59497,16 +59503,16 @@
         <v>50</v>
       </c>
       <c r="L429" s="6">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="M429" s="7">
-        <v>234567.24</v>
+        <v>233914.76</v>
       </c>
       <c r="N429" s="6">
         <v>1</v>
       </c>
       <c r="O429" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P429" s="8">
         <v>326.24</v>
@@ -59607,7 +59613,7 @@
         <v>411</v>
       </c>
       <c r="D430" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E430" s="3" t="s">
         <v>46</v>
@@ -59616,7 +59622,7 @@
         <v>46309</v>
       </c>
       <c r="G430" s="5">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H430" s="3" t="s">
         <v>47</v>
@@ -59631,16 +59637,16 @@
         <v>50</v>
       </c>
       <c r="L430" s="6">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="M430" s="7">
-        <v>234893.48</v>
+        <v>234241</v>
       </c>
       <c r="N430" s="6">
         <v>1</v>
       </c>
       <c r="O430" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P430" s="8">
         <v>326.24</v>
@@ -59741,7 +59747,7 @@
         <v>411</v>
       </c>
       <c r="D431" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E431" s="3" t="s">
         <v>46</v>
@@ -59750,7 +59756,7 @@
         <v>46309</v>
       </c>
       <c r="G431" s="5">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="H431" s="3" t="s">
         <v>47</v>
@@ -59765,16 +59771,16 @@
         <v>50</v>
       </c>
       <c r="L431" s="6">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="M431" s="7">
-        <v>235219.72</v>
+        <v>234567.24</v>
       </c>
       <c r="N431" s="6">
         <v>1</v>
       </c>
       <c r="O431" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P431" s="8">
         <v>326.24</v>
@@ -59875,7 +59881,7 @@
         <v>411</v>
       </c>
       <c r="D432" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E432" s="3" t="s">
         <v>46</v>
@@ -59884,7 +59890,7 @@
         <v>46309</v>
       </c>
       <c r="G432" s="5">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H432" s="3" t="s">
         <v>47</v>
@@ -59899,16 +59905,16 @@
         <v>50</v>
       </c>
       <c r="L432" s="6">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="M432" s="7">
-        <v>235545.96</v>
+        <v>234893.48</v>
       </c>
       <c r="N432" s="6">
         <v>1</v>
       </c>
       <c r="O432" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P432" s="8">
         <v>326.24</v>
@@ -60009,7 +60015,7 @@
         <v>411</v>
       </c>
       <c r="D433" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E433" s="3" t="s">
         <v>46</v>
@@ -60018,7 +60024,7 @@
         <v>46309</v>
       </c>
       <c r="G433" s="5">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="H433" s="3" t="s">
         <v>47</v>
@@ -60033,16 +60039,16 @@
         <v>50</v>
       </c>
       <c r="L433" s="6">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="M433" s="7">
-        <v>235872.2</v>
+        <v>235219.72</v>
       </c>
       <c r="N433" s="6">
         <v>1</v>
       </c>
       <c r="O433" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P433" s="8">
         <v>326.24</v>
@@ -60143,7 +60149,7 @@
         <v>411</v>
       </c>
       <c r="D434" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E434" s="3" t="s">
         <v>46</v>
@@ -60152,7 +60158,7 @@
         <v>46309</v>
       </c>
       <c r="G434" s="5">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="H434" s="3" t="s">
         <v>47</v>
@@ -60167,16 +60173,16 @@
         <v>50</v>
       </c>
       <c r="L434" s="6">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="M434" s="7">
-        <v>236198.44</v>
+        <v>235545.96</v>
       </c>
       <c r="N434" s="6">
         <v>1</v>
       </c>
       <c r="O434" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P434" s="8">
         <v>326.24</v>
@@ -60277,7 +60283,7 @@
         <v>411</v>
       </c>
       <c r="D435" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E435" s="3" t="s">
         <v>46</v>
@@ -60286,7 +60292,7 @@
         <v>46309</v>
       </c>
       <c r="G435" s="5">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="H435" s="3" t="s">
         <v>47</v>
@@ -60301,16 +60307,16 @@
         <v>50</v>
       </c>
       <c r="L435" s="6">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="M435" s="7">
-        <v>236524.68</v>
+        <v>235872.2</v>
       </c>
       <c r="N435" s="6">
         <v>1</v>
       </c>
       <c r="O435" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P435" s="8">
         <v>326.24</v>
@@ -60411,7 +60417,7 @@
         <v>411</v>
       </c>
       <c r="D436" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E436" s="3" t="s">
         <v>46</v>
@@ -60420,7 +60426,7 @@
         <v>46309</v>
       </c>
       <c r="G436" s="5">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H436" s="3" t="s">
         <v>47</v>
@@ -60435,16 +60441,16 @@
         <v>50</v>
       </c>
       <c r="L436" s="6">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="M436" s="7">
-        <v>236850.92</v>
+        <v>236198.44</v>
       </c>
       <c r="N436" s="6">
         <v>1</v>
       </c>
       <c r="O436" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P436" s="8">
         <v>326.24</v>
@@ -60545,7 +60551,7 @@
         <v>411</v>
       </c>
       <c r="D437" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E437" s="3" t="s">
         <v>46</v>
@@ -60554,7 +60560,7 @@
         <v>46309</v>
       </c>
       <c r="G437" s="5">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="H437" s="3" t="s">
         <v>47</v>
@@ -60569,16 +60575,16 @@
         <v>50</v>
       </c>
       <c r="L437" s="6">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="M437" s="7">
-        <v>237177.17</v>
+        <v>236524.68</v>
       </c>
       <c r="N437" s="6">
         <v>1</v>
       </c>
       <c r="O437" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P437" s="8">
         <v>326.24</v>
@@ -60679,7 +60685,7 @@
         <v>411</v>
       </c>
       <c r="D438" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E438" s="3" t="s">
         <v>46</v>
@@ -60688,7 +60694,7 @@
         <v>46309</v>
       </c>
       <c r="G438" s="5">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="H438" s="3" t="s">
         <v>47</v>
@@ -60703,16 +60709,16 @@
         <v>50</v>
       </c>
       <c r="L438" s="6">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="M438" s="7">
-        <v>237503.41</v>
+        <v>236850.92</v>
       </c>
       <c r="N438" s="6">
         <v>1</v>
       </c>
       <c r="O438" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P438" s="8">
         <v>326.24</v>
@@ -60813,7 +60819,7 @@
         <v>411</v>
       </c>
       <c r="D439" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E439" s="3" t="s">
         <v>46</v>
@@ -60822,7 +60828,7 @@
         <v>46309</v>
       </c>
       <c r="G439" s="5">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H439" s="3" t="s">
         <v>47</v>
@@ -60837,16 +60843,16 @@
         <v>50</v>
       </c>
       <c r="L439" s="6">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="M439" s="7">
-        <v>237829.65</v>
+        <v>237177.17</v>
       </c>
       <c r="N439" s="6">
         <v>1</v>
       </c>
       <c r="O439" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P439" s="8">
         <v>326.24</v>
@@ -60947,7 +60953,7 @@
         <v>411</v>
       </c>
       <c r="D440" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E440" s="3" t="s">
         <v>46</v>
@@ -60956,7 +60962,7 @@
         <v>46309</v>
       </c>
       <c r="G440" s="5">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="H440" s="3" t="s">
         <v>47</v>
@@ -60971,16 +60977,16 @@
         <v>50</v>
       </c>
       <c r="L440" s="6">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="M440" s="7">
-        <v>238155.89</v>
+        <v>237503.41</v>
       </c>
       <c r="N440" s="6">
         <v>1</v>
       </c>
       <c r="O440" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P440" s="8">
         <v>326.24</v>
@@ -61081,7 +61087,7 @@
         <v>411</v>
       </c>
       <c r="D441" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E441" s="3" t="s">
         <v>46</v>
@@ -61090,7 +61096,7 @@
         <v>46309</v>
       </c>
       <c r="G441" s="5">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="H441" s="3" t="s">
         <v>47</v>
@@ -61105,16 +61111,16 @@
         <v>50</v>
       </c>
       <c r="L441" s="6">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="M441" s="7">
-        <v>238482.13</v>
+        <v>237829.65</v>
       </c>
       <c r="N441" s="6">
         <v>1</v>
       </c>
       <c r="O441" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P441" s="8">
         <v>326.24</v>
@@ -61215,7 +61221,7 @@
         <v>411</v>
       </c>
       <c r="D442" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E442" s="3" t="s">
         <v>46</v>
@@ -61224,7 +61230,7 @@
         <v>46309</v>
       </c>
       <c r="G442" s="5">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="H442" s="3" t="s">
         <v>47</v>
@@ -61239,16 +61245,16 @@
         <v>50</v>
       </c>
       <c r="L442" s="6">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="M442" s="7">
-        <v>238808.37</v>
+        <v>238155.89</v>
       </c>
       <c r="N442" s="6">
         <v>1</v>
       </c>
       <c r="O442" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P442" s="8">
         <v>326.24</v>
@@ -61349,7 +61355,7 @@
         <v>411</v>
       </c>
       <c r="D443" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E443" s="3" t="s">
         <v>46</v>
@@ -61358,7 +61364,7 @@
         <v>46309</v>
       </c>
       <c r="G443" s="5">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="H443" s="3" t="s">
         <v>47</v>
@@ -61373,16 +61379,16 @@
         <v>50</v>
       </c>
       <c r="L443" s="6">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="M443" s="7">
-        <v>239134.61</v>
+        <v>238482.13</v>
       </c>
       <c r="N443" s="6">
         <v>1</v>
       </c>
       <c r="O443" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P443" s="8">
         <v>326.24</v>
@@ -61483,7 +61489,7 @@
         <v>411</v>
       </c>
       <c r="D444" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E444" s="3" t="s">
         <v>46</v>
@@ -61492,7 +61498,7 @@
         <v>46309</v>
       </c>
       <c r="G444" s="5">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="H444" s="3" t="s">
         <v>47</v>
@@ -61507,16 +61513,16 @@
         <v>50</v>
       </c>
       <c r="L444" s="6">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="M444" s="7">
-        <v>239460.85</v>
+        <v>238808.37</v>
       </c>
       <c r="N444" s="6">
         <v>1</v>
       </c>
       <c r="O444" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P444" s="8">
         <v>326.24</v>
@@ -61617,7 +61623,7 @@
         <v>411</v>
       </c>
       <c r="D445" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E445" s="3" t="s">
         <v>46</v>
@@ -61626,7 +61632,7 @@
         <v>46309</v>
       </c>
       <c r="G445" s="5">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H445" s="3" t="s">
         <v>47</v>
@@ -61641,16 +61647,16 @@
         <v>50</v>
       </c>
       <c r="L445" s="6">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="M445" s="7">
-        <v>239787.09</v>
+        <v>239134.61</v>
       </c>
       <c r="N445" s="6">
         <v>1</v>
       </c>
       <c r="O445" s="3" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="P445" s="8">
         <v>326.24</v>
@@ -61738,6 +61744,274 @@
       </c>
       <c r="AR445" s="3" t="s">
         <v>503</v>
+      </c>
+    </row>
+    <row r="446" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A446" s="1">
+        <v>1</v>
+      </c>
+      <c r="B446" s="2">
+        <v>2</v>
+      </c>
+      <c r="C446" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D446" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="E446" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F446" s="4">
+        <v>46309</v>
+      </c>
+      <c r="G446" s="5">
+        <v>364</v>
+      </c>
+      <c r="H446" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I446" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J446" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K446" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L446" s="6">
+        <v>734</v>
+      </c>
+      <c r="M446" s="7">
+        <v>239460.85</v>
+      </c>
+      <c r="N446" s="6">
+        <v>1</v>
+      </c>
+      <c r="O446" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="P446" s="8">
+        <v>326.24</v>
+      </c>
+      <c r="Q446" s="6">
+        <v>0</v>
+      </c>
+      <c r="R446" s="7">
+        <v>0</v>
+      </c>
+      <c r="S446" s="9">
+        <v>0</v>
+      </c>
+      <c r="T446" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U446" s="10">
+        <v>68241</v>
+      </c>
+      <c r="V446" s="11">
+        <v>11</v>
+      </c>
+      <c r="W446" s="4">
+        <v>46309</v>
+      </c>
+      <c r="X446" s="12">
+        <v>0.48263889999999998</v>
+      </c>
+      <c r="Y446" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB446" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG446" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI446" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="AJ446" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK446" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL446" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM446" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ446" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR446" s="3" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="447" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A447" s="1">
+        <v>1</v>
+      </c>
+      <c r="B447" s="2">
+        <v>2</v>
+      </c>
+      <c r="C447" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D447" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="E447" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F447" s="4">
+        <v>46309</v>
+      </c>
+      <c r="G447" s="5">
+        <v>365</v>
+      </c>
+      <c r="H447" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I447" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J447" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K447" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L447" s="6">
+        <v>735</v>
+      </c>
+      <c r="M447" s="7">
+        <v>239787.09</v>
+      </c>
+      <c r="N447" s="6">
+        <v>1</v>
+      </c>
+      <c r="O447" s="3" t="s">
+        <v>431</v>
+      </c>
+      <c r="P447" s="8">
+        <v>326.24</v>
+      </c>
+      <c r="Q447" s="6">
+        <v>0</v>
+      </c>
+      <c r="R447" s="7">
+        <v>0</v>
+      </c>
+      <c r="S447" s="9">
+        <v>0</v>
+      </c>
+      <c r="T447" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U447" s="10">
+        <v>68241</v>
+      </c>
+      <c r="V447" s="11">
+        <v>11</v>
+      </c>
+      <c r="W447" s="4">
+        <v>46309</v>
+      </c>
+      <c r="X447" s="12">
+        <v>0.48263889999999998</v>
+      </c>
+      <c r="Y447" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB447" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG447" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI447" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="AJ447" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK447" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL447" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM447" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ447" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR447" s="3" t="s">
+        <v>505</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 15/10/2026 11:49:59,84
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5D6A882B-F241-46A0-AECF-52FC6496C1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BDB3656D-40FD-45C7-B998-DA5DF92238CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6326" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6578" uniqueCount="420">
   <si>
     <t>Sel</t>
   </si>
@@ -1239,6 +1239,48 @@
   <si>
     <t>1883500000331</t>
   </si>
+  <si>
+    <t>1883500000332</t>
+  </si>
+  <si>
+    <t>1883500000333</t>
+  </si>
+  <si>
+    <t>1883500000334</t>
+  </si>
+  <si>
+    <t>1883500000335</t>
+  </si>
+  <si>
+    <t>1883500000336</t>
+  </si>
+  <si>
+    <t>1883500000337</t>
+  </si>
+  <si>
+    <t>1883500000338</t>
+  </si>
+  <si>
+    <t>1883500000339</t>
+  </si>
+  <si>
+    <t>1883500000340</t>
+  </si>
+  <si>
+    <t>1883500000341</t>
+  </si>
+  <si>
+    <t>1883500000342</t>
+  </si>
+  <si>
+    <t>1883500000343</t>
+  </si>
+  <si>
+    <t>1883500000344</t>
+  </si>
+  <si>
+    <t>1883500000345</t>
+  </si>
 </sst>
 </file>
 
@@ -1813,7 +1855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR350"/>
+  <dimension ref="A1:AR364"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -48714,6 +48756,1882 @@
       </c>
       <c r="AR350" s="3" t="s">
         <v>405</v>
+      </c>
+    </row>
+    <row r="351" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A351" s="1">
+        <v>1</v>
+      </c>
+      <c r="B351" s="2">
+        <v>2</v>
+      </c>
+      <c r="C351" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D351" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E351" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F351" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G351" s="5">
+        <v>69</v>
+      </c>
+      <c r="H351" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I351" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J351" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K351" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L351" s="6">
+        <v>109</v>
+      </c>
+      <c r="M351" s="7">
+        <v>19334.419999999998</v>
+      </c>
+      <c r="N351" s="6">
+        <v>1</v>
+      </c>
+      <c r="O351" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P351" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q351" s="6">
+        <v>0</v>
+      </c>
+      <c r="R351" s="7">
+        <v>0</v>
+      </c>
+      <c r="S351" s="9">
+        <v>0</v>
+      </c>
+      <c r="T351" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U351" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V351" s="11">
+        <v>11</v>
+      </c>
+      <c r="W351" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X351" s="12">
+        <v>0.45624999999999999</v>
+      </c>
+      <c r="Y351" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB351" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG351" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI351" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ351" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK351" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL351" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM351" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ351" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR351" s="3" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="352" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A352" s="1">
+        <v>1</v>
+      </c>
+      <c r="B352" s="2">
+        <v>2</v>
+      </c>
+      <c r="C352" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D352" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E352" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F352" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G352" s="5">
+        <v>70</v>
+      </c>
+      <c r="H352" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I352" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J352" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K352" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L352" s="6">
+        <v>110</v>
+      </c>
+      <c r="M352" s="7">
+        <v>19511.8</v>
+      </c>
+      <c r="N352" s="6">
+        <v>1</v>
+      </c>
+      <c r="O352" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P352" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q352" s="6">
+        <v>0</v>
+      </c>
+      <c r="R352" s="7">
+        <v>0</v>
+      </c>
+      <c r="S352" s="9">
+        <v>0</v>
+      </c>
+      <c r="T352" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U352" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V352" s="11">
+        <v>11</v>
+      </c>
+      <c r="W352" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X352" s="12">
+        <v>0.45624999999999999</v>
+      </c>
+      <c r="Y352" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB352" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG352" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI352" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ352" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK352" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL352" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM352" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ352" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR352" s="3" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="353" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A353" s="1">
+        <v>1</v>
+      </c>
+      <c r="B353" s="2">
+        <v>2</v>
+      </c>
+      <c r="C353" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D353" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E353" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F353" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G353" s="5">
+        <v>71</v>
+      </c>
+      <c r="H353" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I353" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J353" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K353" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L353" s="6">
+        <v>111</v>
+      </c>
+      <c r="M353" s="7">
+        <v>19689.18</v>
+      </c>
+      <c r="N353" s="6">
+        <v>1</v>
+      </c>
+      <c r="O353" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P353" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q353" s="6">
+        <v>0</v>
+      </c>
+      <c r="R353" s="7">
+        <v>0</v>
+      </c>
+      <c r="S353" s="9">
+        <v>0</v>
+      </c>
+      <c r="T353" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U353" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V353" s="11">
+        <v>11</v>
+      </c>
+      <c r="W353" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X353" s="12">
+        <v>0.45624999999999999</v>
+      </c>
+      <c r="Y353" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB353" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG353" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI353" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ353" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK353" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM353" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR353" s="3" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="354" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A354" s="1">
+        <v>1</v>
+      </c>
+      <c r="B354" s="2">
+        <v>2</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E354" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F354" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G354" s="5">
+        <v>72</v>
+      </c>
+      <c r="H354" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I354" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J354" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K354" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L354" s="6">
+        <v>112</v>
+      </c>
+      <c r="M354" s="7">
+        <v>19866.560000000001</v>
+      </c>
+      <c r="N354" s="6">
+        <v>1</v>
+      </c>
+      <c r="O354" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P354" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q354" s="6">
+        <v>0</v>
+      </c>
+      <c r="R354" s="7">
+        <v>0</v>
+      </c>
+      <c r="S354" s="9">
+        <v>0</v>
+      </c>
+      <c r="T354" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U354" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V354" s="11">
+        <v>11</v>
+      </c>
+      <c r="W354" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X354" s="12">
+        <v>0.46388889999999999</v>
+      </c>
+      <c r="Y354" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB354" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG354" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI354" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ354" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK354" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM354" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR354" s="3" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="355" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A355" s="1">
+        <v>1</v>
+      </c>
+      <c r="B355" s="2">
+        <v>2</v>
+      </c>
+      <c r="C355" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D355" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E355" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F355" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G355" s="5">
+        <v>73</v>
+      </c>
+      <c r="H355" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I355" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J355" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K355" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L355" s="6">
+        <v>113</v>
+      </c>
+      <c r="M355" s="7">
+        <v>20043.939999999999</v>
+      </c>
+      <c r="N355" s="6">
+        <v>1</v>
+      </c>
+      <c r="O355" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P355" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q355" s="6">
+        <v>0</v>
+      </c>
+      <c r="R355" s="7">
+        <v>0</v>
+      </c>
+      <c r="S355" s="9">
+        <v>0</v>
+      </c>
+      <c r="T355" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U355" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V355" s="11">
+        <v>11</v>
+      </c>
+      <c r="W355" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X355" s="12">
+        <v>0.46388889999999999</v>
+      </c>
+      <c r="Y355" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB355" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG355" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI355" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ355" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK355" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM355" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR355" s="3" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="356" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A356" s="1">
+        <v>1</v>
+      </c>
+      <c r="B356" s="2">
+        <v>2</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E356" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F356" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G356" s="5">
+        <v>74</v>
+      </c>
+      <c r="H356" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I356" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J356" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K356" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L356" s="6">
+        <v>114</v>
+      </c>
+      <c r="M356" s="7">
+        <v>20221.32</v>
+      </c>
+      <c r="N356" s="6">
+        <v>1</v>
+      </c>
+      <c r="O356" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P356" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q356" s="6">
+        <v>0</v>
+      </c>
+      <c r="R356" s="7">
+        <v>0</v>
+      </c>
+      <c r="S356" s="9">
+        <v>0</v>
+      </c>
+      <c r="T356" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U356" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V356" s="11">
+        <v>11</v>
+      </c>
+      <c r="W356" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X356" s="12">
+        <v>0.46388889999999999</v>
+      </c>
+      <c r="Y356" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB356" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG356" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI356" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ356" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR356" s="3" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="357" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A357" s="1">
+        <v>1</v>
+      </c>
+      <c r="B357" s="2">
+        <v>2</v>
+      </c>
+      <c r="C357" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D357" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E357" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F357" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G357" s="5">
+        <v>75</v>
+      </c>
+      <c r="H357" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I357" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J357" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K357" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L357" s="6">
+        <v>115</v>
+      </c>
+      <c r="M357" s="7">
+        <v>20398.7</v>
+      </c>
+      <c r="N357" s="6">
+        <v>1</v>
+      </c>
+      <c r="O357" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P357" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q357" s="6">
+        <v>0</v>
+      </c>
+      <c r="R357" s="7">
+        <v>0</v>
+      </c>
+      <c r="S357" s="9">
+        <v>0</v>
+      </c>
+      <c r="T357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U357" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V357" s="11">
+        <v>11</v>
+      </c>
+      <c r="W357" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X357" s="12">
+        <v>0.47013890000000003</v>
+      </c>
+      <c r="Y357" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB357" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG357" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI357" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR357" s="3" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="358" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A358" s="1">
+        <v>1</v>
+      </c>
+      <c r="B358" s="2">
+        <v>2</v>
+      </c>
+      <c r="C358" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D358" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E358" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F358" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G358" s="5">
+        <v>76</v>
+      </c>
+      <c r="H358" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I358" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J358" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K358" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L358" s="6">
+        <v>116</v>
+      </c>
+      <c r="M358" s="7">
+        <v>20576.080000000002</v>
+      </c>
+      <c r="N358" s="6">
+        <v>1</v>
+      </c>
+      <c r="O358" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P358" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q358" s="6">
+        <v>0</v>
+      </c>
+      <c r="R358" s="7">
+        <v>0</v>
+      </c>
+      <c r="S358" s="9">
+        <v>0</v>
+      </c>
+      <c r="T358" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U358" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V358" s="11">
+        <v>11</v>
+      </c>
+      <c r="W358" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X358" s="12">
+        <v>0.47013890000000003</v>
+      </c>
+      <c r="Y358" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB358" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG358" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI358" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ358" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK358" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL358" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM358" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ358" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR358" s="3" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="359" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A359" s="1">
+        <v>1</v>
+      </c>
+      <c r="B359" s="2">
+        <v>2</v>
+      </c>
+      <c r="C359" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D359" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E359" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F359" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G359" s="5">
+        <v>77</v>
+      </c>
+      <c r="H359" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I359" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J359" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K359" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L359" s="6">
+        <v>117</v>
+      </c>
+      <c r="M359" s="7">
+        <v>20753.46</v>
+      </c>
+      <c r="N359" s="6">
+        <v>1</v>
+      </c>
+      <c r="O359" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P359" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q359" s="6">
+        <v>0</v>
+      </c>
+      <c r="R359" s="7">
+        <v>0</v>
+      </c>
+      <c r="S359" s="9">
+        <v>0</v>
+      </c>
+      <c r="T359" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U359" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V359" s="11">
+        <v>11</v>
+      </c>
+      <c r="W359" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X359" s="12">
+        <v>0.47013890000000003</v>
+      </c>
+      <c r="Y359" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB359" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG359" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI359" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ359" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK359" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL359" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM359" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ359" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR359" s="3" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="360" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A360" s="1">
+        <v>1</v>
+      </c>
+      <c r="B360" s="2">
+        <v>2</v>
+      </c>
+      <c r="C360" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D360" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E360" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F360" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G360" s="5">
+        <v>78</v>
+      </c>
+      <c r="H360" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I360" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J360" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K360" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L360" s="6">
+        <v>118</v>
+      </c>
+      <c r="M360" s="7">
+        <v>20930.84</v>
+      </c>
+      <c r="N360" s="6">
+        <v>1</v>
+      </c>
+      <c r="O360" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P360" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q360" s="6">
+        <v>0</v>
+      </c>
+      <c r="R360" s="7">
+        <v>0</v>
+      </c>
+      <c r="S360" s="9">
+        <v>0</v>
+      </c>
+      <c r="T360" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U360" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V360" s="11">
+        <v>11</v>
+      </c>
+      <c r="W360" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X360" s="12">
+        <v>0.47013890000000003</v>
+      </c>
+      <c r="Y360" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB360" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG360" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI360" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ360" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK360" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL360" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM360" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ360" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR360" s="3" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="361" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A361" s="1">
+        <v>1</v>
+      </c>
+      <c r="B361" s="2">
+        <v>2</v>
+      </c>
+      <c r="C361" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D361" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E361" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F361" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G361" s="5">
+        <v>79</v>
+      </c>
+      <c r="H361" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I361" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J361" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K361" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L361" s="6">
+        <v>119</v>
+      </c>
+      <c r="M361" s="7">
+        <v>21108.22</v>
+      </c>
+      <c r="N361" s="6">
+        <v>1</v>
+      </c>
+      <c r="O361" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P361" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q361" s="6">
+        <v>0</v>
+      </c>
+      <c r="R361" s="7">
+        <v>0</v>
+      </c>
+      <c r="S361" s="9">
+        <v>0</v>
+      </c>
+      <c r="T361" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U361" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V361" s="11">
+        <v>11</v>
+      </c>
+      <c r="W361" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X361" s="12">
+        <v>0.48472219999999999</v>
+      </c>
+      <c r="Y361" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB361" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG361" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI361" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ361" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK361" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL361" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM361" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ361" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR361" s="3" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="362" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A362" s="1">
+        <v>1</v>
+      </c>
+      <c r="B362" s="2">
+        <v>2</v>
+      </c>
+      <c r="C362" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D362" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E362" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F362" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G362" s="5">
+        <v>80</v>
+      </c>
+      <c r="H362" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I362" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J362" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K362" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L362" s="6">
+        <v>120</v>
+      </c>
+      <c r="M362" s="7">
+        <v>21285.599999999999</v>
+      </c>
+      <c r="N362" s="6">
+        <v>1</v>
+      </c>
+      <c r="O362" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P362" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q362" s="6">
+        <v>0</v>
+      </c>
+      <c r="R362" s="7">
+        <v>0</v>
+      </c>
+      <c r="S362" s="9">
+        <v>0</v>
+      </c>
+      <c r="T362" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U362" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V362" s="11">
+        <v>11</v>
+      </c>
+      <c r="W362" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X362" s="12">
+        <v>0.48472219999999999</v>
+      </c>
+      <c r="Y362" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB362" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG362" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI362" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ362" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK362" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL362" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM362" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ362" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR362" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="363" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A363" s="1">
+        <v>1</v>
+      </c>
+      <c r="B363" s="2">
+        <v>2</v>
+      </c>
+      <c r="C363" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D363" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E363" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F363" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G363" s="5">
+        <v>81</v>
+      </c>
+      <c r="H363" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I363" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J363" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K363" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L363" s="6">
+        <v>121</v>
+      </c>
+      <c r="M363" s="7">
+        <v>21462.98</v>
+      </c>
+      <c r="N363" s="6">
+        <v>1</v>
+      </c>
+      <c r="O363" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P363" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q363" s="6">
+        <v>0</v>
+      </c>
+      <c r="R363" s="7">
+        <v>0</v>
+      </c>
+      <c r="S363" s="9">
+        <v>0</v>
+      </c>
+      <c r="T363" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U363" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V363" s="11">
+        <v>11</v>
+      </c>
+      <c r="W363" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X363" s="12">
+        <v>0.48472219999999999</v>
+      </c>
+      <c r="Y363" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB363" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG363" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI363" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ363" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK363" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL363" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM363" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ363" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR363" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="364" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A364" s="1">
+        <v>1</v>
+      </c>
+      <c r="B364" s="2">
+        <v>2</v>
+      </c>
+      <c r="C364" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="D364" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E364" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F364" s="4">
+        <v>46310</v>
+      </c>
+      <c r="G364" s="5">
+        <v>82</v>
+      </c>
+      <c r="H364" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I364" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J364" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K364" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L364" s="6">
+        <v>122</v>
+      </c>
+      <c r="M364" s="7">
+        <v>21640.36</v>
+      </c>
+      <c r="N364" s="6">
+        <v>1</v>
+      </c>
+      <c r="O364" s="3" t="s">
+        <v>339</v>
+      </c>
+      <c r="P364" s="8">
+        <v>177.38</v>
+      </c>
+      <c r="Q364" s="6">
+        <v>0</v>
+      </c>
+      <c r="R364" s="7">
+        <v>0</v>
+      </c>
+      <c r="S364" s="9">
+        <v>0</v>
+      </c>
+      <c r="T364" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U364" s="10">
+        <v>68297</v>
+      </c>
+      <c r="V364" s="11">
+        <v>11</v>
+      </c>
+      <c r="W364" s="4">
+        <v>46310</v>
+      </c>
+      <c r="X364" s="12">
+        <v>0.48472219999999999</v>
+      </c>
+      <c r="Y364" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB364" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG364" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI364" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ364" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK364" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL364" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM364" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ364" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR364" s="3" t="s">
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 19/10/2026  9:52:32,24
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0B86848-D91F-41EF-A757-FE548C0FF71F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9467281-37A1-492B-813F-256A2F3EF1D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="692" uniqueCount="93">
   <si>
     <t>Sel</t>
   </si>
@@ -236,6 +236,69 @@
   </si>
   <si>
     <t>1858400003830</t>
+  </si>
+  <si>
+    <t>1858400003831</t>
+  </si>
+  <si>
+    <t>1858400003832</t>
+  </si>
+  <si>
+    <t>1858400003833</t>
+  </si>
+  <si>
+    <t>1858400003834</t>
+  </si>
+  <si>
+    <t>1858400003835</t>
+  </si>
+  <si>
+    <t>1858400003836</t>
+  </si>
+  <si>
+    <t>1858400003837</t>
+  </si>
+  <si>
+    <t>1858400003838</t>
+  </si>
+  <si>
+    <t>1858400003839</t>
+  </si>
+  <si>
+    <t>1858400003840</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>FORNO ELETRICO NARDELLI EMBUTIR INOX 60 LITROS - NARDELLI EMBUTIR INOX 60 LITROS - 220 V</t>
+  </si>
+  <si>
+    <t>1875400003196</t>
+  </si>
+  <si>
+    <t>1875400003197</t>
+  </si>
+  <si>
+    <t>1875400003198</t>
+  </si>
+  <si>
+    <t>1875400003199</t>
+  </si>
+  <si>
+    <t>1875400003200</t>
+  </si>
+  <si>
+    <t>1875400003201</t>
+  </si>
+  <si>
+    <t>1875400003202</t>
+  </si>
+  <si>
+    <t>1875400003203</t>
+  </si>
+  <si>
+    <t>1875400003204</t>
   </si>
 </sst>
 </file>
@@ -811,7 +874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR18"/>
+  <dimension ref="A1:AR37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -3224,6 +3287,2552 @@
       </c>
       <c r="AR18" s="3" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2">
+        <v>2</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F19" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G19" s="5">
+        <v>18</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L19" s="6">
+        <v>186</v>
+      </c>
+      <c r="M19" s="7">
+        <v>71029.3</v>
+      </c>
+      <c r="N19" s="6">
+        <v>1</v>
+      </c>
+      <c r="O19" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P19" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>0</v>
+      </c>
+      <c r="R19" s="7">
+        <v>0</v>
+      </c>
+      <c r="S19" s="9">
+        <v>0</v>
+      </c>
+      <c r="T19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U19" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V19" s="11">
+        <v>11</v>
+      </c>
+      <c r="W19" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X19" s="12">
+        <v>0.35</v>
+      </c>
+      <c r="Y19" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB19" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG19" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK19" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL19" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM19" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR19" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2">
+        <v>2</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G20" s="5">
+        <v>19</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L20" s="6">
+        <v>187</v>
+      </c>
+      <c r="M20" s="7">
+        <v>71411.179999999993</v>
+      </c>
+      <c r="N20" s="6">
+        <v>1</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P20" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q20" s="6">
+        <v>0</v>
+      </c>
+      <c r="R20" s="7">
+        <v>0</v>
+      </c>
+      <c r="S20" s="9">
+        <v>0</v>
+      </c>
+      <c r="T20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U20" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V20" s="11">
+        <v>11</v>
+      </c>
+      <c r="W20" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X20" s="12">
+        <v>0.35</v>
+      </c>
+      <c r="Y20" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB20" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG20" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ20" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK20" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL20" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM20" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ20" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR20" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2">
+        <v>2</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G21" s="5">
+        <v>20</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I21" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K21" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L21" s="6">
+        <v>188</v>
+      </c>
+      <c r="M21" s="7">
+        <v>71793.06</v>
+      </c>
+      <c r="N21" s="6">
+        <v>1</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P21" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q21" s="6">
+        <v>0</v>
+      </c>
+      <c r="R21" s="7">
+        <v>0</v>
+      </c>
+      <c r="S21" s="9">
+        <v>0</v>
+      </c>
+      <c r="T21" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U21" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V21" s="11">
+        <v>11</v>
+      </c>
+      <c r="W21" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X21" s="12">
+        <v>0.35</v>
+      </c>
+      <c r="Y21" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB21" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG21" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ21" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK21" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL21" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM21" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ21" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR21" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>1</v>
+      </c>
+      <c r="B22" s="2">
+        <v>2</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F22" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G22" s="5">
+        <v>21</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L22" s="6">
+        <v>189</v>
+      </c>
+      <c r="M22" s="7">
+        <v>72174.929999999993</v>
+      </c>
+      <c r="N22" s="6">
+        <v>1</v>
+      </c>
+      <c r="O22" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P22" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>0</v>
+      </c>
+      <c r="R22" s="7">
+        <v>0</v>
+      </c>
+      <c r="S22" s="9">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U22" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V22" s="11">
+        <v>11</v>
+      </c>
+      <c r="W22" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X22" s="12">
+        <v>0.35625000000000001</v>
+      </c>
+      <c r="Y22" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB22" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG22" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI22" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ22" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL22" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM22" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ22" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR22" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2">
+        <v>2</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G23" s="5">
+        <v>22</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L23" s="6">
+        <v>190</v>
+      </c>
+      <c r="M23" s="7">
+        <v>72556.81</v>
+      </c>
+      <c r="N23" s="6">
+        <v>1</v>
+      </c>
+      <c r="O23" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P23" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>0</v>
+      </c>
+      <c r="R23" s="7">
+        <v>0</v>
+      </c>
+      <c r="S23" s="9">
+        <v>0</v>
+      </c>
+      <c r="T23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U23" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V23" s="11">
+        <v>11</v>
+      </c>
+      <c r="W23" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X23" s="12">
+        <v>0.35625000000000001</v>
+      </c>
+      <c r="Y23" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB23" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG23" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK23" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL23" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM23" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ23" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR23" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>1</v>
+      </c>
+      <c r="B24" s="2">
+        <v>2</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F24" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G24" s="5">
+        <v>23</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L24" s="6">
+        <v>191</v>
+      </c>
+      <c r="M24" s="7">
+        <v>72938.69</v>
+      </c>
+      <c r="N24" s="6">
+        <v>1</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P24" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q24" s="6">
+        <v>0</v>
+      </c>
+      <c r="R24" s="7">
+        <v>0</v>
+      </c>
+      <c r="S24" s="9">
+        <v>0</v>
+      </c>
+      <c r="T24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U24" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V24" s="11">
+        <v>11</v>
+      </c>
+      <c r="W24" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X24" s="12">
+        <v>0.35625000000000001</v>
+      </c>
+      <c r="Y24" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB24" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG24" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL24" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM24" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR24" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>1</v>
+      </c>
+      <c r="B25" s="2">
+        <v>2</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F25" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G25" s="5">
+        <v>24</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K25" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L25" s="6">
+        <v>192</v>
+      </c>
+      <c r="M25" s="7">
+        <v>73320.570000000007</v>
+      </c>
+      <c r="N25" s="6">
+        <v>1</v>
+      </c>
+      <c r="O25" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P25" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>0</v>
+      </c>
+      <c r="R25" s="7">
+        <v>0</v>
+      </c>
+      <c r="S25" s="9">
+        <v>0</v>
+      </c>
+      <c r="T25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U25" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V25" s="11">
+        <v>11</v>
+      </c>
+      <c r="W25" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X25" s="12">
+        <v>0.35625000000000001</v>
+      </c>
+      <c r="Y25" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB25" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG25" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ25" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK25" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL25" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM25" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR25" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>1</v>
+      </c>
+      <c r="B26" s="2">
+        <v>2</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F26" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G26" s="5">
+        <v>25</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K26" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L26" s="6">
+        <v>193</v>
+      </c>
+      <c r="M26" s="7">
+        <v>73702.45</v>
+      </c>
+      <c r="N26" s="6">
+        <v>1</v>
+      </c>
+      <c r="O26" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P26" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q26" s="6">
+        <v>0</v>
+      </c>
+      <c r="R26" s="7">
+        <v>0</v>
+      </c>
+      <c r="S26" s="9">
+        <v>0</v>
+      </c>
+      <c r="T26" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U26" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V26" s="11">
+        <v>11</v>
+      </c>
+      <c r="W26" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X26" s="12">
+        <v>0.36388890000000002</v>
+      </c>
+      <c r="Y26" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB26" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG26" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ26" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK26" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL26" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM26" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ26" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR26" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" s="2">
+        <v>2</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F27" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G27" s="5">
+        <v>26</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I27" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K27" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L27" s="6">
+        <v>194</v>
+      </c>
+      <c r="M27" s="7">
+        <v>74084.320000000007</v>
+      </c>
+      <c r="N27" s="6">
+        <v>1</v>
+      </c>
+      <c r="O27" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P27" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q27" s="6">
+        <v>0</v>
+      </c>
+      <c r="R27" s="7">
+        <v>0</v>
+      </c>
+      <c r="S27" s="9">
+        <v>0</v>
+      </c>
+      <c r="T27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U27" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V27" s="11">
+        <v>11</v>
+      </c>
+      <c r="W27" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X27" s="12">
+        <v>0.36388890000000002</v>
+      </c>
+      <c r="Y27" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB27" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG27" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI27" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ27" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL27" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM27" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ27" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR27" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" s="2">
+        <v>2</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F28" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G28" s="5">
+        <v>27</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I28" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L28" s="6">
+        <v>195</v>
+      </c>
+      <c r="M28" s="7">
+        <v>74466.2</v>
+      </c>
+      <c r="N28" s="6">
+        <v>1</v>
+      </c>
+      <c r="O28" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P28" s="8">
+        <v>381.88</v>
+      </c>
+      <c r="Q28" s="6">
+        <v>0</v>
+      </c>
+      <c r="R28" s="7">
+        <v>0</v>
+      </c>
+      <c r="S28" s="9">
+        <v>0</v>
+      </c>
+      <c r="T28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U28" s="10">
+        <v>68405</v>
+      </c>
+      <c r="V28" s="11">
+        <v>11</v>
+      </c>
+      <c r="W28" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X28" s="12">
+        <v>0.36388890000000002</v>
+      </c>
+      <c r="Y28" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB28" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG28" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI28" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ28" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK28" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL28" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM28" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ28" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR28" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>1</v>
+      </c>
+      <c r="B29" s="2">
+        <v>2</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G29" s="5">
+        <v>1</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I29" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K29" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L29" s="6">
+        <v>35</v>
+      </c>
+      <c r="M29" s="7">
+        <v>13094.6</v>
+      </c>
+      <c r="N29" s="6">
+        <v>1</v>
+      </c>
+      <c r="O29" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P29" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q29" s="6">
+        <v>0</v>
+      </c>
+      <c r="R29" s="7">
+        <v>0</v>
+      </c>
+      <c r="S29" s="9">
+        <v>0</v>
+      </c>
+      <c r="T29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U29" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V29" s="11">
+        <v>11</v>
+      </c>
+      <c r="W29" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X29" s="12">
+        <v>0.37083329999999998</v>
+      </c>
+      <c r="Y29" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB29" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG29" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI29" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ29" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK29" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL29" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM29" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ29" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR29" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>1</v>
+      </c>
+      <c r="B30" s="2">
+        <v>2</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F30" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G30" s="5">
+        <v>2</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I30" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K30" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L30" s="6">
+        <v>36</v>
+      </c>
+      <c r="M30" s="7">
+        <v>13468.73</v>
+      </c>
+      <c r="N30" s="6">
+        <v>1</v>
+      </c>
+      <c r="O30" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P30" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q30" s="6">
+        <v>0</v>
+      </c>
+      <c r="R30" s="7">
+        <v>0</v>
+      </c>
+      <c r="S30" s="9">
+        <v>0</v>
+      </c>
+      <c r="T30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U30" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V30" s="11">
+        <v>11</v>
+      </c>
+      <c r="W30" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X30" s="12">
+        <v>0.3854167</v>
+      </c>
+      <c r="Y30" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB30" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG30" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI30" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ30" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK30" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL30" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM30" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ30" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR30" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>1</v>
+      </c>
+      <c r="B31" s="2">
+        <v>2</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G31" s="5">
+        <v>3</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I31" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J31" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K31" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L31" s="6">
+        <v>37</v>
+      </c>
+      <c r="M31" s="7">
+        <v>13842.86</v>
+      </c>
+      <c r="N31" s="6">
+        <v>1</v>
+      </c>
+      <c r="O31" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P31" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q31" s="6">
+        <v>0</v>
+      </c>
+      <c r="R31" s="7">
+        <v>0</v>
+      </c>
+      <c r="S31" s="9">
+        <v>0</v>
+      </c>
+      <c r="T31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U31" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V31" s="11">
+        <v>11</v>
+      </c>
+      <c r="W31" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X31" s="12">
+        <v>0.3854167</v>
+      </c>
+      <c r="Y31" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG31" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI31" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ31" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK31" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL31" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM31" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ31" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR31" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>1</v>
+      </c>
+      <c r="B32" s="2">
+        <v>2</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F32" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G32" s="5">
+        <v>4</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I32" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K32" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L32" s="6">
+        <v>38</v>
+      </c>
+      <c r="M32" s="7">
+        <v>14216.99</v>
+      </c>
+      <c r="N32" s="6">
+        <v>1</v>
+      </c>
+      <c r="O32" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P32" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q32" s="6">
+        <v>0</v>
+      </c>
+      <c r="R32" s="7">
+        <v>0</v>
+      </c>
+      <c r="S32" s="9">
+        <v>0</v>
+      </c>
+      <c r="T32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U32" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V32" s="11">
+        <v>11</v>
+      </c>
+      <c r="W32" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X32" s="12">
+        <v>0.3854167</v>
+      </c>
+      <c r="Y32" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB32" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG32" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI32" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ32" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK32" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL32" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM32" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ32" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR32" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>1</v>
+      </c>
+      <c r="B33" s="2">
+        <v>2</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G33" s="5">
+        <v>5</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L33" s="6">
+        <v>39</v>
+      </c>
+      <c r="M33" s="7">
+        <v>14591.13</v>
+      </c>
+      <c r="N33" s="6">
+        <v>1</v>
+      </c>
+      <c r="O33" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P33" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q33" s="6">
+        <v>0</v>
+      </c>
+      <c r="R33" s="7">
+        <v>0</v>
+      </c>
+      <c r="S33" s="9">
+        <v>0</v>
+      </c>
+      <c r="T33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U33" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V33" s="11">
+        <v>11</v>
+      </c>
+      <c r="W33" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X33" s="12">
+        <v>0.39166669999999998</v>
+      </c>
+      <c r="Y33" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB33" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG33" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI33" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK33" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL33" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM33" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR33" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>1</v>
+      </c>
+      <c r="B34" s="2">
+        <v>2</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G34" s="5">
+        <v>6</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L34" s="6">
+        <v>40</v>
+      </c>
+      <c r="M34" s="7">
+        <v>14965.26</v>
+      </c>
+      <c r="N34" s="6">
+        <v>1</v>
+      </c>
+      <c r="O34" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P34" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q34" s="6">
+        <v>0</v>
+      </c>
+      <c r="R34" s="7">
+        <v>0</v>
+      </c>
+      <c r="S34" s="9">
+        <v>0</v>
+      </c>
+      <c r="T34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U34" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V34" s="11">
+        <v>11</v>
+      </c>
+      <c r="W34" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X34" s="12">
+        <v>0.39166669999999998</v>
+      </c>
+      <c r="Y34" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB34" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG34" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI34" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK34" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL34" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM34" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR34" s="3" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2">
+        <v>2</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G35" s="5">
+        <v>7</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L35" s="6">
+        <v>41</v>
+      </c>
+      <c r="M35" s="7">
+        <v>15339.39</v>
+      </c>
+      <c r="N35" s="6">
+        <v>1</v>
+      </c>
+      <c r="O35" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P35" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q35" s="6">
+        <v>0</v>
+      </c>
+      <c r="R35" s="7">
+        <v>0</v>
+      </c>
+      <c r="S35" s="9">
+        <v>0</v>
+      </c>
+      <c r="T35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U35" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V35" s="11">
+        <v>11</v>
+      </c>
+      <c r="W35" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X35" s="12">
+        <v>0.39166669999999998</v>
+      </c>
+      <c r="Y35" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB35" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG35" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI35" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL35" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM35" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR35" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>1</v>
+      </c>
+      <c r="B36" s="2">
+        <v>2</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F36" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G36" s="5">
+        <v>8</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K36" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L36" s="6">
+        <v>42</v>
+      </c>
+      <c r="M36" s="7">
+        <v>15713.52</v>
+      </c>
+      <c r="N36" s="6">
+        <v>1</v>
+      </c>
+      <c r="O36" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P36" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q36" s="6">
+        <v>0</v>
+      </c>
+      <c r="R36" s="7">
+        <v>0</v>
+      </c>
+      <c r="S36" s="9">
+        <v>0</v>
+      </c>
+      <c r="T36" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U36" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V36" s="11">
+        <v>11</v>
+      </c>
+      <c r="W36" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X36" s="12">
+        <v>0.3986111</v>
+      </c>
+      <c r="Y36" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB36" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG36" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI36" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ36" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK36" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL36" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM36" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR36" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="37" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>1</v>
+      </c>
+      <c r="B37" s="2">
+        <v>2</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F37" s="4">
+        <v>46314</v>
+      </c>
+      <c r="G37" s="5">
+        <v>9</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L37" s="6">
+        <v>43</v>
+      </c>
+      <c r="M37" s="7">
+        <v>16087.65</v>
+      </c>
+      <c r="N37" s="6">
+        <v>1</v>
+      </c>
+      <c r="O37" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P37" s="8">
+        <v>374.13</v>
+      </c>
+      <c r="Q37" s="6">
+        <v>0</v>
+      </c>
+      <c r="R37" s="7">
+        <v>0</v>
+      </c>
+      <c r="S37" s="9">
+        <v>0</v>
+      </c>
+      <c r="T37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U37" s="10">
+        <v>68418</v>
+      </c>
+      <c r="V37" s="11">
+        <v>11</v>
+      </c>
+      <c r="W37" s="4">
+        <v>46314</v>
+      </c>
+      <c r="X37" s="12">
+        <v>0.3986111</v>
+      </c>
+      <c r="Y37" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB37" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG37" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI37" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ37" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK37" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL37" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM37" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR37" s="3" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 21/10/2026 11:58:57,20
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B30B092-9CDD-41F3-ACD9-FA7AF19F3C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE2100CB-61CD-4659-BE79-75E122875BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6722" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6992" uniqueCount="445">
   <si>
     <t>Sel</t>
   </si>
@@ -1213,6 +1213,51 @@
     <t>1881700005502</t>
   </si>
   <si>
+    <t>1881700005305</t>
+  </si>
+  <si>
+    <t>1881700005503</t>
+  </si>
+  <si>
+    <t>1881700005504</t>
+  </si>
+  <si>
+    <t>1881700005505</t>
+  </si>
+  <si>
+    <t>1881700005506</t>
+  </si>
+  <si>
+    <t>1881700005507</t>
+  </si>
+  <si>
+    <t>1881700005508</t>
+  </si>
+  <si>
+    <t>1881700005509</t>
+  </si>
+  <si>
+    <t>1881700005510</t>
+  </si>
+  <si>
+    <t>1881700005511</t>
+  </si>
+  <si>
+    <t>1881700005512</t>
+  </si>
+  <si>
+    <t>1881700005513</t>
+  </si>
+  <si>
+    <t>1881700005514</t>
+  </si>
+  <si>
+    <t>1881700005515</t>
+  </si>
+  <si>
+    <t>1881700005516</t>
+  </si>
+  <si>
     <t>10096354</t>
   </si>
   <si>
@@ -1885,7 +1930,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR372"/>
+  <dimension ref="A1:AR387"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -47858,10 +47903,10 @@
         <v>2</v>
       </c>
       <c r="C344" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D344" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E344" s="3" t="s">
         <v>46</v>
@@ -47870,7 +47915,7 @@
         <v>46316</v>
       </c>
       <c r="G344" s="5">
-        <v>1</v>
+        <v>976</v>
       </c>
       <c r="H344" s="3" t="s">
         <v>47</v>
@@ -47885,19 +47930,19 @@
         <v>50</v>
       </c>
       <c r="L344" s="6">
-        <v>19</v>
+        <v>574</v>
       </c>
       <c r="M344" s="7">
-        <v>6390.7</v>
+        <v>97872.34</v>
       </c>
       <c r="N344" s="6">
         <v>1</v>
       </c>
       <c r="O344" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P344" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q344" s="6">
         <v>0</v>
@@ -47912,7 +47957,7 @@
         <v>52</v>
       </c>
       <c r="U344" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V344" s="11">
         <v>11</v>
@@ -47921,7 +47966,7 @@
         <v>46316</v>
       </c>
       <c r="X344" s="12">
-        <v>0.3229167</v>
+        <v>0.47499999999999998</v>
       </c>
       <c r="Y344" s="10">
         <v>0</v>
@@ -47954,7 +47999,7 @@
         <v>53</v>
       </c>
       <c r="AI344" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ344" s="3" t="s">
         <v>52</v>
@@ -47981,7 +48026,7 @@
         <v>53</v>
       </c>
       <c r="AR344" s="3" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="345" spans="1:44" x14ac:dyDescent="0.3">
@@ -47992,10 +48037,10 @@
         <v>2</v>
       </c>
       <c r="C345" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D345" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E345" s="3" t="s">
         <v>46</v>
@@ -48004,7 +48049,7 @@
         <v>46316</v>
       </c>
       <c r="G345" s="5">
-        <v>2</v>
+        <v>977</v>
       </c>
       <c r="H345" s="3" t="s">
         <v>47</v>
@@ -48019,19 +48064,19 @@
         <v>50</v>
       </c>
       <c r="L345" s="6">
-        <v>20</v>
+        <v>575</v>
       </c>
       <c r="M345" s="7">
-        <v>6727.05</v>
+        <v>98042.85</v>
       </c>
       <c r="N345" s="6">
         <v>1</v>
       </c>
       <c r="O345" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P345" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q345" s="6">
         <v>0</v>
@@ -48046,7 +48091,7 @@
         <v>52</v>
       </c>
       <c r="U345" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V345" s="11">
         <v>11</v>
@@ -48055,7 +48100,7 @@
         <v>46316</v>
       </c>
       <c r="X345" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y345" s="10">
         <v>0</v>
@@ -48088,7 +48133,7 @@
         <v>53</v>
       </c>
       <c r="AI345" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ345" s="3" t="s">
         <v>52</v>
@@ -48115,7 +48160,7 @@
         <v>53</v>
       </c>
       <c r="AR345" s="3" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="346" spans="1:44" x14ac:dyDescent="0.3">
@@ -48126,10 +48171,10 @@
         <v>2</v>
       </c>
       <c r="C346" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D346" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E346" s="3" t="s">
         <v>46</v>
@@ -48138,7 +48183,7 @@
         <v>46316</v>
       </c>
       <c r="G346" s="5">
-        <v>3</v>
+        <v>978</v>
       </c>
       <c r="H346" s="3" t="s">
         <v>47</v>
@@ -48153,19 +48198,19 @@
         <v>50</v>
       </c>
       <c r="L346" s="6">
-        <v>21</v>
+        <v>576</v>
       </c>
       <c r="M346" s="7">
-        <v>7063.41</v>
+        <v>98213.36</v>
       </c>
       <c r="N346" s="6">
         <v>1</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P346" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q346" s="6">
         <v>0</v>
@@ -48180,7 +48225,7 @@
         <v>52</v>
       </c>
       <c r="U346" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V346" s="11">
         <v>11</v>
@@ -48189,7 +48234,7 @@
         <v>46316</v>
       </c>
       <c r="X346" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y346" s="10">
         <v>0</v>
@@ -48222,7 +48267,7 @@
         <v>53</v>
       </c>
       <c r="AI346" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ346" s="3" t="s">
         <v>52</v>
@@ -48249,7 +48294,7 @@
         <v>53</v>
       </c>
       <c r="AR346" s="3" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="347" spans="1:44" x14ac:dyDescent="0.3">
@@ -48260,10 +48305,10 @@
         <v>2</v>
       </c>
       <c r="C347" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D347" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E347" s="3" t="s">
         <v>46</v>
@@ -48272,7 +48317,7 @@
         <v>46316</v>
       </c>
       <c r="G347" s="5">
-        <v>4</v>
+        <v>979</v>
       </c>
       <c r="H347" s="3" t="s">
         <v>47</v>
@@ -48287,19 +48332,19 @@
         <v>50</v>
       </c>
       <c r="L347" s="6">
-        <v>22</v>
+        <v>577</v>
       </c>
       <c r="M347" s="7">
-        <v>7399.76</v>
+        <v>98383.87</v>
       </c>
       <c r="N347" s="6">
         <v>1</v>
       </c>
       <c r="O347" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P347" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q347" s="6">
         <v>0</v>
@@ -48314,7 +48359,7 @@
         <v>52</v>
       </c>
       <c r="U347" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V347" s="11">
         <v>11</v>
@@ -48323,7 +48368,7 @@
         <v>46316</v>
       </c>
       <c r="X347" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y347" s="10">
         <v>0</v>
@@ -48356,34 +48401,34 @@
         <v>53</v>
       </c>
       <c r="AI347" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ347" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK347" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL347" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM347" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN347" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO347" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP347" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ347" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR347" s="3" t="s">
         <v>400</v>
-      </c>
-      <c r="AJ347" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AK347" s="14">
-        <v>0</v>
-      </c>
-      <c r="AL347" s="10">
-        <v>0</v>
-      </c>
-      <c r="AM347" s="14">
-        <v>0</v>
-      </c>
-      <c r="AN347" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AO347" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AP347" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ347" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AR347" s="3" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="348" spans="1:44" x14ac:dyDescent="0.3">
@@ -48394,10 +48439,10 @@
         <v>2</v>
       </c>
       <c r="C348" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D348" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E348" s="3" t="s">
         <v>46</v>
@@ -48406,7 +48451,7 @@
         <v>46316</v>
       </c>
       <c r="G348" s="5">
-        <v>5</v>
+        <v>980</v>
       </c>
       <c r="H348" s="3" t="s">
         <v>47</v>
@@ -48421,19 +48466,19 @@
         <v>50</v>
       </c>
       <c r="L348" s="6">
-        <v>23</v>
+        <v>578</v>
       </c>
       <c r="M348" s="7">
-        <v>7736.11</v>
+        <v>98554.38</v>
       </c>
       <c r="N348" s="6">
         <v>1</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P348" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q348" s="6">
         <v>0</v>
@@ -48448,7 +48493,7 @@
         <v>52</v>
       </c>
       <c r="U348" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V348" s="11">
         <v>11</v>
@@ -48457,7 +48502,7 @@
         <v>46316</v>
       </c>
       <c r="X348" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y348" s="10">
         <v>0</v>
@@ -48490,7 +48535,7 @@
         <v>53</v>
       </c>
       <c r="AI348" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ348" s="3" t="s">
         <v>52</v>
@@ -48517,7 +48562,7 @@
         <v>53</v>
       </c>
       <c r="AR348" s="3" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="349" spans="1:44" x14ac:dyDescent="0.3">
@@ -48528,10 +48573,10 @@
         <v>2</v>
       </c>
       <c r="C349" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D349" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E349" s="3" t="s">
         <v>46</v>
@@ -48540,7 +48585,7 @@
         <v>46316</v>
       </c>
       <c r="G349" s="5">
-        <v>6</v>
+        <v>981</v>
       </c>
       <c r="H349" s="3" t="s">
         <v>47</v>
@@ -48555,19 +48600,19 @@
         <v>50</v>
       </c>
       <c r="L349" s="6">
-        <v>24</v>
+        <v>579</v>
       </c>
       <c r="M349" s="7">
-        <v>8072.46</v>
+        <v>98724.89</v>
       </c>
       <c r="N349" s="6">
         <v>1</v>
       </c>
       <c r="O349" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P349" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q349" s="6">
         <v>0</v>
@@ -48582,7 +48627,7 @@
         <v>52</v>
       </c>
       <c r="U349" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V349" s="11">
         <v>11</v>
@@ -48591,7 +48636,7 @@
         <v>46316</v>
       </c>
       <c r="X349" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y349" s="10">
         <v>0</v>
@@ -48624,7 +48669,7 @@
         <v>53</v>
       </c>
       <c r="AI349" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ349" s="3" t="s">
         <v>52</v>
@@ -48651,7 +48696,7 @@
         <v>53</v>
       </c>
       <c r="AR349" s="3" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
     </row>
     <row r="350" spans="1:44" x14ac:dyDescent="0.3">
@@ -48662,10 +48707,10 @@
         <v>2</v>
       </c>
       <c r="C350" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D350" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E350" s="3" t="s">
         <v>46</v>
@@ -48674,7 +48719,7 @@
         <v>46316</v>
       </c>
       <c r="G350" s="5">
-        <v>7</v>
+        <v>982</v>
       </c>
       <c r="H350" s="3" t="s">
         <v>47</v>
@@ -48689,19 +48734,19 @@
         <v>50</v>
       </c>
       <c r="L350" s="6">
-        <v>25</v>
+        <v>580</v>
       </c>
       <c r="M350" s="7">
-        <v>8408.82</v>
+        <v>98895.4</v>
       </c>
       <c r="N350" s="6">
         <v>1</v>
       </c>
       <c r="O350" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P350" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q350" s="6">
         <v>0</v>
@@ -48716,7 +48761,7 @@
         <v>52</v>
       </c>
       <c r="U350" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V350" s="11">
         <v>11</v>
@@ -48725,7 +48770,7 @@
         <v>46316</v>
       </c>
       <c r="X350" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y350" s="10">
         <v>0</v>
@@ -48758,7 +48803,7 @@
         <v>53</v>
       </c>
       <c r="AI350" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ350" s="3" t="s">
         <v>52</v>
@@ -48785,7 +48830,7 @@
         <v>53</v>
       </c>
       <c r="AR350" s="3" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="351" spans="1:44" x14ac:dyDescent="0.3">
@@ -48796,10 +48841,10 @@
         <v>2</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D351" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E351" s="3" t="s">
         <v>46</v>
@@ -48808,7 +48853,7 @@
         <v>46316</v>
       </c>
       <c r="G351" s="5">
-        <v>8</v>
+        <v>983</v>
       </c>
       <c r="H351" s="3" t="s">
         <v>47</v>
@@ -48823,19 +48868,19 @@
         <v>50</v>
       </c>
       <c r="L351" s="6">
-        <v>26</v>
+        <v>581</v>
       </c>
       <c r="M351" s="7">
-        <v>8745.17</v>
+        <v>99065.91</v>
       </c>
       <c r="N351" s="6">
         <v>1</v>
       </c>
       <c r="O351" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P351" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q351" s="6">
         <v>0</v>
@@ -48850,7 +48895,7 @@
         <v>52</v>
       </c>
       <c r="U351" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V351" s="11">
         <v>11</v>
@@ -48859,7 +48904,7 @@
         <v>46316</v>
       </c>
       <c r="X351" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y351" s="10">
         <v>0</v>
@@ -48892,7 +48937,7 @@
         <v>53</v>
       </c>
       <c r="AI351" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ351" s="3" t="s">
         <v>52</v>
@@ -48919,7 +48964,7 @@
         <v>53</v>
       </c>
       <c r="AR351" s="3" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
     </row>
     <row r="352" spans="1:44" x14ac:dyDescent="0.3">
@@ -48930,10 +48975,10 @@
         <v>2</v>
       </c>
       <c r="C352" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D352" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E352" s="3" t="s">
         <v>46</v>
@@ -48942,7 +48987,7 @@
         <v>46316</v>
       </c>
       <c r="G352" s="5">
-        <v>9</v>
+        <v>984</v>
       </c>
       <c r="H352" s="3" t="s">
         <v>47</v>
@@ -48957,19 +49002,19 @@
         <v>50</v>
       </c>
       <c r="L352" s="6">
-        <v>27</v>
+        <v>582</v>
       </c>
       <c r="M352" s="7">
-        <v>9081.52</v>
+        <v>99236.42</v>
       </c>
       <c r="N352" s="6">
         <v>1</v>
       </c>
       <c r="O352" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P352" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q352" s="6">
         <v>0</v>
@@ -48984,7 +49029,7 @@
         <v>52</v>
       </c>
       <c r="U352" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V352" s="11">
         <v>11</v>
@@ -48993,7 +49038,7 @@
         <v>46316</v>
       </c>
       <c r="X352" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y352" s="10">
         <v>0</v>
@@ -49026,7 +49071,7 @@
         <v>53</v>
       </c>
       <c r="AI352" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ352" s="3" t="s">
         <v>52</v>
@@ -49053,7 +49098,7 @@
         <v>53</v>
       </c>
       <c r="AR352" s="3" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="353" spans="1:44" x14ac:dyDescent="0.3">
@@ -49064,10 +49109,10 @@
         <v>2</v>
       </c>
       <c r="C353" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D353" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E353" s="3" t="s">
         <v>46</v>
@@ -49076,7 +49121,7 @@
         <v>46316</v>
       </c>
       <c r="G353" s="5">
-        <v>10</v>
+        <v>985</v>
       </c>
       <c r="H353" s="3" t="s">
         <v>47</v>
@@ -49091,19 +49136,19 @@
         <v>50</v>
       </c>
       <c r="L353" s="6">
-        <v>28</v>
+        <v>583</v>
       </c>
       <c r="M353" s="7">
-        <v>9417.8700000000008</v>
+        <v>99406.93</v>
       </c>
       <c r="N353" s="6">
         <v>1</v>
       </c>
       <c r="O353" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P353" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q353" s="6">
         <v>0</v>
@@ -49118,7 +49163,7 @@
         <v>52</v>
       </c>
       <c r="U353" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V353" s="11">
         <v>11</v>
@@ -49127,7 +49172,7 @@
         <v>46316</v>
       </c>
       <c r="X353" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y353" s="10">
         <v>0</v>
@@ -49160,7 +49205,7 @@
         <v>53</v>
       </c>
       <c r="AI353" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ353" s="3" t="s">
         <v>52</v>
@@ -49187,7 +49232,7 @@
         <v>53</v>
       </c>
       <c r="AR353" s="3" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="354" spans="1:44" x14ac:dyDescent="0.3">
@@ -49198,10 +49243,10 @@
         <v>2</v>
       </c>
       <c r="C354" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D354" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E354" s="3" t="s">
         <v>46</v>
@@ -49210,7 +49255,7 @@
         <v>46316</v>
       </c>
       <c r="G354" s="5">
-        <v>11</v>
+        <v>986</v>
       </c>
       <c r="H354" s="3" t="s">
         <v>47</v>
@@ -49225,19 +49270,19 @@
         <v>50</v>
       </c>
       <c r="L354" s="6">
-        <v>29</v>
+        <v>584</v>
       </c>
       <c r="M354" s="7">
-        <v>9754.23</v>
+        <v>99577.44</v>
       </c>
       <c r="N354" s="6">
         <v>1</v>
       </c>
       <c r="O354" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P354" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q354" s="6">
         <v>0</v>
@@ -49252,7 +49297,7 @@
         <v>52</v>
       </c>
       <c r="U354" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V354" s="11">
         <v>11</v>
@@ -49261,7 +49306,7 @@
         <v>46316</v>
       </c>
       <c r="X354" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y354" s="10">
         <v>0</v>
@@ -49294,7 +49339,7 @@
         <v>53</v>
       </c>
       <c r="AI354" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ354" s="3" t="s">
         <v>52</v>
@@ -49321,7 +49366,7 @@
         <v>53</v>
       </c>
       <c r="AR354" s="3" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="355" spans="1:44" x14ac:dyDescent="0.3">
@@ -49332,10 +49377,10 @@
         <v>2</v>
       </c>
       <c r="C355" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D355" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E355" s="3" t="s">
         <v>46</v>
@@ -49344,7 +49389,7 @@
         <v>46316</v>
       </c>
       <c r="G355" s="5">
-        <v>12</v>
+        <v>987</v>
       </c>
       <c r="H355" s="3" t="s">
         <v>47</v>
@@ -49359,19 +49404,19 @@
         <v>50</v>
       </c>
       <c r="L355" s="6">
-        <v>30</v>
+        <v>585</v>
       </c>
       <c r="M355" s="7">
-        <v>10090.58</v>
+        <v>99747.95</v>
       </c>
       <c r="N355" s="6">
         <v>1</v>
       </c>
       <c r="O355" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P355" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q355" s="6">
         <v>0</v>
@@ -49386,7 +49431,7 @@
         <v>52</v>
       </c>
       <c r="U355" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V355" s="11">
         <v>11</v>
@@ -49395,7 +49440,7 @@
         <v>46316</v>
       </c>
       <c r="X355" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y355" s="10">
         <v>0</v>
@@ -49428,7 +49473,7 @@
         <v>53</v>
       </c>
       <c r="AI355" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ355" s="3" t="s">
         <v>52</v>
@@ -49455,7 +49500,7 @@
         <v>53</v>
       </c>
       <c r="AR355" s="3" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="356" spans="1:44" x14ac:dyDescent="0.3">
@@ -49466,10 +49511,10 @@
         <v>2</v>
       </c>
       <c r="C356" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D356" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E356" s="3" t="s">
         <v>46</v>
@@ -49478,7 +49523,7 @@
         <v>46316</v>
       </c>
       <c r="G356" s="5">
-        <v>13</v>
+        <v>988</v>
       </c>
       <c r="H356" s="3" t="s">
         <v>47</v>
@@ -49493,19 +49538,19 @@
         <v>50</v>
       </c>
       <c r="L356" s="6">
-        <v>31</v>
+        <v>586</v>
       </c>
       <c r="M356" s="7">
-        <v>10426.93</v>
+        <v>99918.46</v>
       </c>
       <c r="N356" s="6">
         <v>1</v>
       </c>
       <c r="O356" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P356" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q356" s="6">
         <v>0</v>
@@ -49520,7 +49565,7 @@
         <v>52</v>
       </c>
       <c r="U356" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V356" s="11">
         <v>11</v>
@@ -49529,7 +49574,7 @@
         <v>46316</v>
       </c>
       <c r="X356" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y356" s="10">
         <v>0</v>
@@ -49562,7 +49607,7 @@
         <v>53</v>
       </c>
       <c r="AI356" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ356" s="3" t="s">
         <v>52</v>
@@ -49589,7 +49634,7 @@
         <v>53</v>
       </c>
       <c r="AR356" s="3" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="357" spans="1:44" x14ac:dyDescent="0.3">
@@ -49600,10 +49645,10 @@
         <v>2</v>
       </c>
       <c r="C357" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D357" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E357" s="3" t="s">
         <v>46</v>
@@ -49612,7 +49657,7 @@
         <v>46316</v>
       </c>
       <c r="G357" s="5">
-        <v>14</v>
+        <v>989</v>
       </c>
       <c r="H357" s="3" t="s">
         <v>47</v>
@@ -49627,19 +49672,19 @@
         <v>50</v>
       </c>
       <c r="L357" s="6">
-        <v>32</v>
+        <v>587</v>
       </c>
       <c r="M357" s="7">
-        <v>10763.28</v>
+        <v>100088.96000000001</v>
       </c>
       <c r="N357" s="6">
         <v>1</v>
       </c>
       <c r="O357" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P357" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q357" s="6">
         <v>0</v>
@@ -49654,7 +49699,7 @@
         <v>52</v>
       </c>
       <c r="U357" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V357" s="11">
         <v>11</v>
@@ -49663,7 +49708,7 @@
         <v>46316</v>
       </c>
       <c r="X357" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y357" s="10">
         <v>0</v>
@@ -49696,7 +49741,7 @@
         <v>53</v>
       </c>
       <c r="AI357" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ357" s="3" t="s">
         <v>52</v>
@@ -49723,7 +49768,7 @@
         <v>53</v>
       </c>
       <c r="AR357" s="3" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="358" spans="1:44" x14ac:dyDescent="0.3">
@@ -49734,10 +49779,10 @@
         <v>2</v>
       </c>
       <c r="C358" s="3" t="s">
-        <v>397</v>
+        <v>44</v>
       </c>
       <c r="D358" s="3" t="s">
-        <v>398</v>
+        <v>45</v>
       </c>
       <c r="E358" s="3" t="s">
         <v>46</v>
@@ -49746,7 +49791,7 @@
         <v>46316</v>
       </c>
       <c r="G358" s="5">
-        <v>15</v>
+        <v>990</v>
       </c>
       <c r="H358" s="3" t="s">
         <v>47</v>
@@ -49761,19 +49806,19 @@
         <v>50</v>
       </c>
       <c r="L358" s="6">
-        <v>33</v>
+        <v>588</v>
       </c>
       <c r="M358" s="7">
-        <v>11099.64</v>
+        <v>100259.47</v>
       </c>
       <c r="N358" s="6">
         <v>1</v>
       </c>
       <c r="O358" s="3" t="s">
-        <v>399</v>
+        <v>51</v>
       </c>
       <c r="P358" s="8">
-        <v>336.35</v>
+        <v>170.51</v>
       </c>
       <c r="Q358" s="6">
         <v>0</v>
@@ -49788,7 +49833,7 @@
         <v>52</v>
       </c>
       <c r="U358" s="10">
-        <v>68501</v>
+        <v>68459</v>
       </c>
       <c r="V358" s="11">
         <v>11</v>
@@ -49797,7 +49842,7 @@
         <v>46316</v>
       </c>
       <c r="X358" s="12">
-        <v>0.3229167</v>
+        <v>0.49652780000000002</v>
       </c>
       <c r="Y358" s="10">
         <v>0</v>
@@ -49830,7 +49875,7 @@
         <v>53</v>
       </c>
       <c r="AI358" s="3" t="s">
-        <v>400</v>
+        <v>54</v>
       </c>
       <c r="AJ358" s="3" t="s">
         <v>52</v>
@@ -49857,7 +49902,7 @@
         <v>53</v>
       </c>
       <c r="AR358" s="3" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="359" spans="1:44" x14ac:dyDescent="0.3">
@@ -49868,10 +49913,10 @@
         <v>2</v>
       </c>
       <c r="C359" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D359" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E359" s="3" t="s">
         <v>46</v>
@@ -49880,7 +49925,7 @@
         <v>46316</v>
       </c>
       <c r="G359" s="5">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="H359" s="3" t="s">
         <v>47</v>
@@ -49895,16 +49940,16 @@
         <v>50</v>
       </c>
       <c r="L359" s="6">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="M359" s="7">
-        <v>11435.99</v>
+        <v>6390.7</v>
       </c>
       <c r="N359" s="6">
         <v>1</v>
       </c>
       <c r="O359" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P359" s="8">
         <v>336.35</v>
@@ -49931,7 +49976,7 @@
         <v>46316</v>
       </c>
       <c r="X359" s="12">
-        <v>0.32986110000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y359" s="10">
         <v>0</v>
@@ -49964,7 +50009,7 @@
         <v>53</v>
       </c>
       <c r="AI359" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ359" s="3" t="s">
         <v>52</v>
@@ -50002,10 +50047,10 @@
         <v>2</v>
       </c>
       <c r="C360" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D360" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E360" s="3" t="s">
         <v>46</v>
@@ -50014,7 +50059,7 @@
         <v>46316</v>
       </c>
       <c r="G360" s="5">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="H360" s="3" t="s">
         <v>47</v>
@@ -50029,16 +50074,16 @@
         <v>50</v>
       </c>
       <c r="L360" s="6">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="M360" s="7">
-        <v>11772.34</v>
+        <v>6727.05</v>
       </c>
       <c r="N360" s="6">
         <v>1</v>
       </c>
       <c r="O360" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P360" s="8">
         <v>336.35</v>
@@ -50065,7 +50110,7 @@
         <v>46316</v>
       </c>
       <c r="X360" s="12">
-        <v>0.32986110000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y360" s="10">
         <v>0</v>
@@ -50098,7 +50143,7 @@
         <v>53</v>
       </c>
       <c r="AI360" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ360" s="3" t="s">
         <v>52</v>
@@ -50136,10 +50181,10 @@
         <v>2</v>
       </c>
       <c r="C361" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D361" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E361" s="3" t="s">
         <v>46</v>
@@ -50148,7 +50193,7 @@
         <v>46316</v>
       </c>
       <c r="G361" s="5">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H361" s="3" t="s">
         <v>47</v>
@@ -50163,16 +50208,16 @@
         <v>50</v>
       </c>
       <c r="L361" s="6">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="M361" s="7">
-        <v>12108.69</v>
+        <v>7063.41</v>
       </c>
       <c r="N361" s="6">
         <v>1</v>
       </c>
       <c r="O361" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P361" s="8">
         <v>336.35</v>
@@ -50199,7 +50244,7 @@
         <v>46316</v>
       </c>
       <c r="X361" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y361" s="10">
         <v>0</v>
@@ -50232,7 +50277,7 @@
         <v>53</v>
       </c>
       <c r="AI361" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ361" s="3" t="s">
         <v>52</v>
@@ -50270,10 +50315,10 @@
         <v>2</v>
       </c>
       <c r="C362" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D362" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E362" s="3" t="s">
         <v>46</v>
@@ -50282,7 +50327,7 @@
         <v>46316</v>
       </c>
       <c r="G362" s="5">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H362" s="3" t="s">
         <v>47</v>
@@ -50297,16 +50342,16 @@
         <v>50</v>
       </c>
       <c r="L362" s="6">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="M362" s="7">
-        <v>12445.05</v>
+        <v>7399.76</v>
       </c>
       <c r="N362" s="6">
         <v>1</v>
       </c>
       <c r="O362" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P362" s="8">
         <v>336.35</v>
@@ -50333,7 +50378,7 @@
         <v>46316</v>
       </c>
       <c r="X362" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y362" s="10">
         <v>0</v>
@@ -50366,7 +50411,7 @@
         <v>53</v>
       </c>
       <c r="AI362" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ362" s="3" t="s">
         <v>52</v>
@@ -50404,10 +50449,10 @@
         <v>2</v>
       </c>
       <c r="C363" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D363" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E363" s="3" t="s">
         <v>46</v>
@@ -50416,7 +50461,7 @@
         <v>46316</v>
       </c>
       <c r="G363" s="5">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H363" s="3" t="s">
         <v>47</v>
@@ -50431,16 +50476,16 @@
         <v>50</v>
       </c>
       <c r="L363" s="6">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="M363" s="7">
-        <v>12781.4</v>
+        <v>7736.11</v>
       </c>
       <c r="N363" s="6">
         <v>1</v>
       </c>
       <c r="O363" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P363" s="8">
         <v>336.35</v>
@@ -50467,7 +50512,7 @@
         <v>46316</v>
       </c>
       <c r="X363" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y363" s="10">
         <v>0</v>
@@ -50500,7 +50545,7 @@
         <v>53</v>
       </c>
       <c r="AI363" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ363" s="3" t="s">
         <v>52</v>
@@ -50538,10 +50583,10 @@
         <v>2</v>
       </c>
       <c r="C364" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D364" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E364" s="3" t="s">
         <v>46</v>
@@ -50550,7 +50595,7 @@
         <v>46316</v>
       </c>
       <c r="G364" s="5">
-        <v>21</v>
+        <v>6</v>
       </c>
       <c r="H364" s="3" t="s">
         <v>47</v>
@@ -50565,16 +50610,16 @@
         <v>50</v>
       </c>
       <c r="L364" s="6">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="M364" s="7">
-        <v>13117.75</v>
+        <v>8072.46</v>
       </c>
       <c r="N364" s="6">
         <v>1</v>
       </c>
       <c r="O364" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P364" s="8">
         <v>336.35</v>
@@ -50601,7 +50646,7 @@
         <v>46316</v>
       </c>
       <c r="X364" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y364" s="10">
         <v>0</v>
@@ -50634,7 +50679,7 @@
         <v>53</v>
       </c>
       <c r="AI364" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ364" s="3" t="s">
         <v>52</v>
@@ -50672,10 +50717,10 @@
         <v>2</v>
       </c>
       <c r="C365" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D365" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E365" s="3" t="s">
         <v>46</v>
@@ -50684,7 +50729,7 @@
         <v>46316</v>
       </c>
       <c r="G365" s="5">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="H365" s="3" t="s">
         <v>47</v>
@@ -50699,16 +50744,16 @@
         <v>50</v>
       </c>
       <c r="L365" s="6">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="M365" s="7">
-        <v>13454.11</v>
+        <v>8408.82</v>
       </c>
       <c r="N365" s="6">
         <v>1</v>
       </c>
       <c r="O365" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P365" s="8">
         <v>336.35</v>
@@ -50735,7 +50780,7 @@
         <v>46316</v>
       </c>
       <c r="X365" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y365" s="10">
         <v>0</v>
@@ -50768,7 +50813,7 @@
         <v>53</v>
       </c>
       <c r="AI365" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ365" s="3" t="s">
         <v>52</v>
@@ -50806,10 +50851,10 @@
         <v>2</v>
       </c>
       <c r="C366" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D366" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E366" s="3" t="s">
         <v>46</v>
@@ -50818,7 +50863,7 @@
         <v>46316</v>
       </c>
       <c r="G366" s="5">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="H366" s="3" t="s">
         <v>47</v>
@@ -50833,16 +50878,16 @@
         <v>50</v>
       </c>
       <c r="L366" s="6">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="M366" s="7">
-        <v>13790.46</v>
+        <v>8745.17</v>
       </c>
       <c r="N366" s="6">
         <v>1</v>
       </c>
       <c r="O366" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P366" s="8">
         <v>336.35</v>
@@ -50869,7 +50914,7 @@
         <v>46316</v>
       </c>
       <c r="X366" s="12">
-        <v>0.33680559999999998</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y366" s="10">
         <v>0</v>
@@ -50902,7 +50947,7 @@
         <v>53</v>
       </c>
       <c r="AI366" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ366" s="3" t="s">
         <v>52</v>
@@ -50940,10 +50985,10 @@
         <v>2</v>
       </c>
       <c r="C367" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D367" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E367" s="3" t="s">
         <v>46</v>
@@ -50952,7 +50997,7 @@
         <v>46316</v>
       </c>
       <c r="G367" s="5">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="H367" s="3" t="s">
         <v>47</v>
@@ -50967,16 +51012,16 @@
         <v>50</v>
       </c>
       <c r="L367" s="6">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="M367" s="7">
-        <v>14126.81</v>
+        <v>9081.52</v>
       </c>
       <c r="N367" s="6">
         <v>1</v>
       </c>
       <c r="O367" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P367" s="8">
         <v>336.35</v>
@@ -51003,7 +51048,7 @@
         <v>46316</v>
       </c>
       <c r="X367" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y367" s="10">
         <v>0</v>
@@ -51036,7 +51081,7 @@
         <v>53</v>
       </c>
       <c r="AI367" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ367" s="3" t="s">
         <v>52</v>
@@ -51074,10 +51119,10 @@
         <v>2</v>
       </c>
       <c r="C368" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D368" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E368" s="3" t="s">
         <v>46</v>
@@ -51086,7 +51131,7 @@
         <v>46316</v>
       </c>
       <c r="G368" s="5">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H368" s="3" t="s">
         <v>47</v>
@@ -51101,16 +51146,16 @@
         <v>50</v>
       </c>
       <c r="L368" s="6">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="M368" s="7">
-        <v>14463.16</v>
+        <v>9417.8700000000008</v>
       </c>
       <c r="N368" s="6">
         <v>1</v>
       </c>
       <c r="O368" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P368" s="8">
         <v>336.35</v>
@@ -51137,7 +51182,7 @@
         <v>46316</v>
       </c>
       <c r="X368" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y368" s="10">
         <v>0</v>
@@ -51170,7 +51215,7 @@
         <v>53</v>
       </c>
       <c r="AI368" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ368" s="3" t="s">
         <v>52</v>
@@ -51208,10 +51253,10 @@
         <v>2</v>
       </c>
       <c r="C369" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D369" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E369" s="3" t="s">
         <v>46</v>
@@ -51220,7 +51265,7 @@
         <v>46316</v>
       </c>
       <c r="G369" s="5">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="H369" s="3" t="s">
         <v>47</v>
@@ -51235,16 +51280,16 @@
         <v>50</v>
       </c>
       <c r="L369" s="6">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="M369" s="7">
-        <v>14799.52</v>
+        <v>9754.23</v>
       </c>
       <c r="N369" s="6">
         <v>1</v>
       </c>
       <c r="O369" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P369" s="8">
         <v>336.35</v>
@@ -51271,7 +51316,7 @@
         <v>46316</v>
       </c>
       <c r="X369" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y369" s="10">
         <v>0</v>
@@ -51304,7 +51349,7 @@
         <v>53</v>
       </c>
       <c r="AI369" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ369" s="3" t="s">
         <v>52</v>
@@ -51342,10 +51387,10 @@
         <v>2</v>
       </c>
       <c r="C370" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D370" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E370" s="3" t="s">
         <v>46</v>
@@ -51354,7 +51399,7 @@
         <v>46316</v>
       </c>
       <c r="G370" s="5">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="H370" s="3" t="s">
         <v>47</v>
@@ -51369,16 +51414,16 @@
         <v>50</v>
       </c>
       <c r="L370" s="6">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="M370" s="7">
-        <v>15135.87</v>
+        <v>10090.58</v>
       </c>
       <c r="N370" s="6">
         <v>1</v>
       </c>
       <c r="O370" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P370" s="8">
         <v>336.35</v>
@@ -51405,7 +51450,7 @@
         <v>46316</v>
       </c>
       <c r="X370" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y370" s="10">
         <v>0</v>
@@ -51438,7 +51483,7 @@
         <v>53</v>
       </c>
       <c r="AI370" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ370" s="3" t="s">
         <v>52</v>
@@ -51476,10 +51521,10 @@
         <v>2</v>
       </c>
       <c r="C371" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D371" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E371" s="3" t="s">
         <v>46</v>
@@ -51488,7 +51533,7 @@
         <v>46316</v>
       </c>
       <c r="G371" s="5">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="H371" s="3" t="s">
         <v>47</v>
@@ -51503,16 +51548,16 @@
         <v>50</v>
       </c>
       <c r="L371" s="6">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="M371" s="7">
-        <v>15472.22</v>
+        <v>10426.93</v>
       </c>
       <c r="N371" s="6">
         <v>1</v>
       </c>
       <c r="O371" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P371" s="8">
         <v>336.35</v>
@@ -51539,7 +51584,7 @@
         <v>46316</v>
       </c>
       <c r="X371" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y371" s="10">
         <v>0</v>
@@ -51572,7 +51617,7 @@
         <v>53</v>
       </c>
       <c r="AI371" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ371" s="3" t="s">
         <v>52</v>
@@ -51610,10 +51655,10 @@
         <v>2</v>
       </c>
       <c r="C372" s="3" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="D372" s="3" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="E372" s="3" t="s">
         <v>46</v>
@@ -51622,7 +51667,7 @@
         <v>46316</v>
       </c>
       <c r="G372" s="5">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="H372" s="3" t="s">
         <v>47</v>
@@ -51637,16 +51682,16 @@
         <v>50</v>
       </c>
       <c r="L372" s="6">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="M372" s="7">
-        <v>15808.57</v>
+        <v>10763.28</v>
       </c>
       <c r="N372" s="6">
         <v>1</v>
       </c>
       <c r="O372" s="3" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="P372" s="8">
         <v>336.35</v>
@@ -51673,7 +51718,7 @@
         <v>46316</v>
       </c>
       <c r="X372" s="12">
-        <v>0.33750000000000002</v>
+        <v>0.3229167</v>
       </c>
       <c r="Y372" s="10">
         <v>0</v>
@@ -51706,7 +51751,7 @@
         <v>53</v>
       </c>
       <c r="AI372" s="3" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="AJ372" s="3" t="s">
         <v>52</v>
@@ -51734,6 +51779,2016 @@
       </c>
       <c r="AR372" s="3" t="s">
         <v>429</v>
+      </c>
+    </row>
+    <row r="373" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A373" s="1">
+        <v>1</v>
+      </c>
+      <c r="B373" s="2">
+        <v>2</v>
+      </c>
+      <c r="C373" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D373" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E373" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F373" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G373" s="5">
+        <v>15</v>
+      </c>
+      <c r="H373" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I373" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J373" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K373" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L373" s="6">
+        <v>33</v>
+      </c>
+      <c r="M373" s="7">
+        <v>11099.64</v>
+      </c>
+      <c r="N373" s="6">
+        <v>1</v>
+      </c>
+      <c r="O373" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P373" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q373" s="6">
+        <v>0</v>
+      </c>
+      <c r="R373" s="7">
+        <v>0</v>
+      </c>
+      <c r="S373" s="9">
+        <v>0</v>
+      </c>
+      <c r="T373" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U373" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V373" s="11">
+        <v>11</v>
+      </c>
+      <c r="W373" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X373" s="12">
+        <v>0.3229167</v>
+      </c>
+      <c r="Y373" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB373" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG373" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI373" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ373" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK373" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL373" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM373" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ373" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR373" s="3" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="374" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A374" s="1">
+        <v>1</v>
+      </c>
+      <c r="B374" s="2">
+        <v>2</v>
+      </c>
+      <c r="C374" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D374" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E374" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F374" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G374" s="5">
+        <v>16</v>
+      </c>
+      <c r="H374" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I374" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J374" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K374" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L374" s="6">
+        <v>34</v>
+      </c>
+      <c r="M374" s="7">
+        <v>11435.99</v>
+      </c>
+      <c r="N374" s="6">
+        <v>1</v>
+      </c>
+      <c r="O374" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P374" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q374" s="6">
+        <v>0</v>
+      </c>
+      <c r="R374" s="7">
+        <v>0</v>
+      </c>
+      <c r="S374" s="9">
+        <v>0</v>
+      </c>
+      <c r="T374" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U374" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V374" s="11">
+        <v>11</v>
+      </c>
+      <c r="W374" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X374" s="12">
+        <v>0.32986110000000002</v>
+      </c>
+      <c r="Y374" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB374" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG374" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI374" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ374" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK374" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL374" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM374" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ374" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR374" s="3" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="375" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A375" s="1">
+        <v>1</v>
+      </c>
+      <c r="B375" s="2">
+        <v>2</v>
+      </c>
+      <c r="C375" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D375" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E375" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F375" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G375" s="5">
+        <v>17</v>
+      </c>
+      <c r="H375" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I375" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J375" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K375" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L375" s="6">
+        <v>35</v>
+      </c>
+      <c r="M375" s="7">
+        <v>11772.34</v>
+      </c>
+      <c r="N375" s="6">
+        <v>1</v>
+      </c>
+      <c r="O375" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P375" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q375" s="6">
+        <v>0</v>
+      </c>
+      <c r="R375" s="7">
+        <v>0</v>
+      </c>
+      <c r="S375" s="9">
+        <v>0</v>
+      </c>
+      <c r="T375" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U375" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V375" s="11">
+        <v>11</v>
+      </c>
+      <c r="W375" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X375" s="12">
+        <v>0.32986110000000002</v>
+      </c>
+      <c r="Y375" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB375" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG375" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI375" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ375" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK375" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL375" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM375" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ375" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR375" s="3" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="376" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A376" s="1">
+        <v>1</v>
+      </c>
+      <c r="B376" s="2">
+        <v>2</v>
+      </c>
+      <c r="C376" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D376" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E376" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F376" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G376" s="5">
+        <v>18</v>
+      </c>
+      <c r="H376" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I376" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J376" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K376" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L376" s="6">
+        <v>36</v>
+      </c>
+      <c r="M376" s="7">
+        <v>12108.69</v>
+      </c>
+      <c r="N376" s="6">
+        <v>1</v>
+      </c>
+      <c r="O376" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P376" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q376" s="6">
+        <v>0</v>
+      </c>
+      <c r="R376" s="7">
+        <v>0</v>
+      </c>
+      <c r="S376" s="9">
+        <v>0</v>
+      </c>
+      <c r="T376" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U376" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V376" s="11">
+        <v>11</v>
+      </c>
+      <c r="W376" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X376" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y376" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB376" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG376" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI376" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ376" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK376" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL376" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM376" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ376" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR376" s="3" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="377" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A377" s="1">
+        <v>1</v>
+      </c>
+      <c r="B377" s="2">
+        <v>2</v>
+      </c>
+      <c r="C377" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D377" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E377" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F377" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G377" s="5">
+        <v>19</v>
+      </c>
+      <c r="H377" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I377" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J377" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K377" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L377" s="6">
+        <v>37</v>
+      </c>
+      <c r="M377" s="7">
+        <v>12445.05</v>
+      </c>
+      <c r="N377" s="6">
+        <v>1</v>
+      </c>
+      <c r="O377" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P377" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q377" s="6">
+        <v>0</v>
+      </c>
+      <c r="R377" s="7">
+        <v>0</v>
+      </c>
+      <c r="S377" s="9">
+        <v>0</v>
+      </c>
+      <c r="T377" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U377" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V377" s="11">
+        <v>11</v>
+      </c>
+      <c r="W377" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X377" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y377" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB377" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG377" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI377" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ377" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK377" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL377" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM377" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ377" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR377" s="3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="378" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A378" s="1">
+        <v>1</v>
+      </c>
+      <c r="B378" s="2">
+        <v>2</v>
+      </c>
+      <c r="C378" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D378" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E378" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F378" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G378" s="5">
+        <v>20</v>
+      </c>
+      <c r="H378" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I378" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J378" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K378" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L378" s="6">
+        <v>38</v>
+      </c>
+      <c r="M378" s="7">
+        <v>12781.4</v>
+      </c>
+      <c r="N378" s="6">
+        <v>1</v>
+      </c>
+      <c r="O378" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P378" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q378" s="6">
+        <v>0</v>
+      </c>
+      <c r="R378" s="7">
+        <v>0</v>
+      </c>
+      <c r="S378" s="9">
+        <v>0</v>
+      </c>
+      <c r="T378" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U378" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V378" s="11">
+        <v>11</v>
+      </c>
+      <c r="W378" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X378" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y378" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB378" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG378" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI378" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ378" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK378" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL378" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM378" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ378" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR378" s="3" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="379" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A379" s="1">
+        <v>1</v>
+      </c>
+      <c r="B379" s="2">
+        <v>2</v>
+      </c>
+      <c r="C379" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D379" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E379" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F379" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G379" s="5">
+        <v>21</v>
+      </c>
+      <c r="H379" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I379" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J379" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K379" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L379" s="6">
+        <v>39</v>
+      </c>
+      <c r="M379" s="7">
+        <v>13117.75</v>
+      </c>
+      <c r="N379" s="6">
+        <v>1</v>
+      </c>
+      <c r="O379" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P379" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q379" s="6">
+        <v>0</v>
+      </c>
+      <c r="R379" s="7">
+        <v>0</v>
+      </c>
+      <c r="S379" s="9">
+        <v>0</v>
+      </c>
+      <c r="T379" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U379" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V379" s="11">
+        <v>11</v>
+      </c>
+      <c r="W379" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X379" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y379" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB379" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG379" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI379" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ379" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK379" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL379" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM379" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ379" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR379" s="3" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="380" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A380" s="1">
+        <v>1</v>
+      </c>
+      <c r="B380" s="2">
+        <v>2</v>
+      </c>
+      <c r="C380" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D380" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E380" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F380" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G380" s="5">
+        <v>22</v>
+      </c>
+      <c r="H380" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I380" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J380" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K380" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L380" s="6">
+        <v>40</v>
+      </c>
+      <c r="M380" s="7">
+        <v>13454.11</v>
+      </c>
+      <c r="N380" s="6">
+        <v>1</v>
+      </c>
+      <c r="O380" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P380" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q380" s="6">
+        <v>0</v>
+      </c>
+      <c r="R380" s="7">
+        <v>0</v>
+      </c>
+      <c r="S380" s="9">
+        <v>0</v>
+      </c>
+      <c r="T380" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U380" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V380" s="11">
+        <v>11</v>
+      </c>
+      <c r="W380" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X380" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y380" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB380" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG380" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI380" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ380" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK380" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL380" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM380" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ380" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR380" s="3" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="381" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A381" s="1">
+        <v>1</v>
+      </c>
+      <c r="B381" s="2">
+        <v>2</v>
+      </c>
+      <c r="C381" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D381" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E381" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F381" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G381" s="5">
+        <v>23</v>
+      </c>
+      <c r="H381" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I381" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J381" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K381" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L381" s="6">
+        <v>41</v>
+      </c>
+      <c r="M381" s="7">
+        <v>13790.46</v>
+      </c>
+      <c r="N381" s="6">
+        <v>1</v>
+      </c>
+      <c r="O381" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P381" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q381" s="6">
+        <v>0</v>
+      </c>
+      <c r="R381" s="7">
+        <v>0</v>
+      </c>
+      <c r="S381" s="9">
+        <v>0</v>
+      </c>
+      <c r="T381" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U381" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V381" s="11">
+        <v>11</v>
+      </c>
+      <c r="W381" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X381" s="12">
+        <v>0.33680559999999998</v>
+      </c>
+      <c r="Y381" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB381" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG381" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI381" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ381" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK381" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL381" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM381" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ381" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR381" s="3" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="382" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A382" s="1">
+        <v>1</v>
+      </c>
+      <c r="B382" s="2">
+        <v>2</v>
+      </c>
+      <c r="C382" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D382" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E382" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F382" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G382" s="5">
+        <v>24</v>
+      </c>
+      <c r="H382" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I382" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J382" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K382" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L382" s="6">
+        <v>42</v>
+      </c>
+      <c r="M382" s="7">
+        <v>14126.81</v>
+      </c>
+      <c r="N382" s="6">
+        <v>1</v>
+      </c>
+      <c r="O382" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P382" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q382" s="6">
+        <v>0</v>
+      </c>
+      <c r="R382" s="7">
+        <v>0</v>
+      </c>
+      <c r="S382" s="9">
+        <v>0</v>
+      </c>
+      <c r="T382" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U382" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V382" s="11">
+        <v>11</v>
+      </c>
+      <c r="W382" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X382" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y382" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB382" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG382" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI382" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ382" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK382" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL382" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM382" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ382" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR382" s="3" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="383" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A383" s="1">
+        <v>1</v>
+      </c>
+      <c r="B383" s="2">
+        <v>2</v>
+      </c>
+      <c r="C383" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D383" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E383" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F383" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G383" s="5">
+        <v>25</v>
+      </c>
+      <c r="H383" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I383" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J383" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K383" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L383" s="6">
+        <v>43</v>
+      </c>
+      <c r="M383" s="7">
+        <v>14463.16</v>
+      </c>
+      <c r="N383" s="6">
+        <v>1</v>
+      </c>
+      <c r="O383" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P383" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q383" s="6">
+        <v>0</v>
+      </c>
+      <c r="R383" s="7">
+        <v>0</v>
+      </c>
+      <c r="S383" s="9">
+        <v>0</v>
+      </c>
+      <c r="T383" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U383" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V383" s="11">
+        <v>11</v>
+      </c>
+      <c r="W383" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X383" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y383" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB383" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG383" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI383" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ383" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK383" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL383" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM383" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ383" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR383" s="3" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="384" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A384" s="1">
+        <v>1</v>
+      </c>
+      <c r="B384" s="2">
+        <v>2</v>
+      </c>
+      <c r="C384" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D384" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E384" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F384" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G384" s="5">
+        <v>26</v>
+      </c>
+      <c r="H384" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I384" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J384" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K384" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L384" s="6">
+        <v>44</v>
+      </c>
+      <c r="M384" s="7">
+        <v>14799.52</v>
+      </c>
+      <c r="N384" s="6">
+        <v>1</v>
+      </c>
+      <c r="O384" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P384" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q384" s="6">
+        <v>0</v>
+      </c>
+      <c r="R384" s="7">
+        <v>0</v>
+      </c>
+      <c r="S384" s="9">
+        <v>0</v>
+      </c>
+      <c r="T384" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U384" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V384" s="11">
+        <v>11</v>
+      </c>
+      <c r="W384" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X384" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y384" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB384" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG384" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI384" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ384" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK384" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL384" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM384" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ384" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR384" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="385" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A385" s="1">
+        <v>1</v>
+      </c>
+      <c r="B385" s="2">
+        <v>2</v>
+      </c>
+      <c r="C385" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D385" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E385" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F385" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G385" s="5">
+        <v>27</v>
+      </c>
+      <c r="H385" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I385" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J385" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K385" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L385" s="6">
+        <v>45</v>
+      </c>
+      <c r="M385" s="7">
+        <v>15135.87</v>
+      </c>
+      <c r="N385" s="6">
+        <v>1</v>
+      </c>
+      <c r="O385" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P385" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q385" s="6">
+        <v>0</v>
+      </c>
+      <c r="R385" s="7">
+        <v>0</v>
+      </c>
+      <c r="S385" s="9">
+        <v>0</v>
+      </c>
+      <c r="T385" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U385" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V385" s="11">
+        <v>11</v>
+      </c>
+      <c r="W385" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X385" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y385" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB385" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG385" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI385" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ385" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK385" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL385" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM385" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ385" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR385" s="3" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="386" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A386" s="1">
+        <v>1</v>
+      </c>
+      <c r="B386" s="2">
+        <v>2</v>
+      </c>
+      <c r="C386" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D386" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E386" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F386" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G386" s="5">
+        <v>28</v>
+      </c>
+      <c r="H386" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I386" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J386" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K386" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L386" s="6">
+        <v>46</v>
+      </c>
+      <c r="M386" s="7">
+        <v>15472.22</v>
+      </c>
+      <c r="N386" s="6">
+        <v>1</v>
+      </c>
+      <c r="O386" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P386" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q386" s="6">
+        <v>0</v>
+      </c>
+      <c r="R386" s="7">
+        <v>0</v>
+      </c>
+      <c r="S386" s="9">
+        <v>0</v>
+      </c>
+      <c r="T386" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U386" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V386" s="11">
+        <v>11</v>
+      </c>
+      <c r="W386" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X386" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y386" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB386" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG386" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI386" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ386" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK386" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL386" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM386" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ386" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR386" s="3" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="387" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A387" s="1">
+        <v>1</v>
+      </c>
+      <c r="B387" s="2">
+        <v>2</v>
+      </c>
+      <c r="C387" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="D387" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E387" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F387" s="4">
+        <v>46316</v>
+      </c>
+      <c r="G387" s="5">
+        <v>29</v>
+      </c>
+      <c r="H387" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I387" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J387" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K387" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L387" s="6">
+        <v>47</v>
+      </c>
+      <c r="M387" s="7">
+        <v>15808.57</v>
+      </c>
+      <c r="N387" s="6">
+        <v>1</v>
+      </c>
+      <c r="O387" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="P387" s="8">
+        <v>336.35</v>
+      </c>
+      <c r="Q387" s="6">
+        <v>0</v>
+      </c>
+      <c r="R387" s="7">
+        <v>0</v>
+      </c>
+      <c r="S387" s="9">
+        <v>0</v>
+      </c>
+      <c r="T387" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U387" s="10">
+        <v>68501</v>
+      </c>
+      <c r="V387" s="11">
+        <v>11</v>
+      </c>
+      <c r="W387" s="4">
+        <v>46316</v>
+      </c>
+      <c r="X387" s="12">
+        <v>0.33750000000000002</v>
+      </c>
+      <c r="Y387" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB387" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG387" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI387" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="AJ387" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK387" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL387" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM387" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ387" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR387" s="3" t="s">
+        <v>444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 22/10/2026  8:06:02,13
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{33273739-4B4E-4E2C-AE56-088A06DE5F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7C12364-4490-44CF-AB2B-BB89A3FE50BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="135">
   <si>
     <t>Sel</t>
   </si>
@@ -365,6 +365,66 @@
   </si>
   <si>
     <t>1858700158620</t>
+  </si>
+  <si>
+    <t>1858700158621</t>
+  </si>
+  <si>
+    <t>1858700158622</t>
+  </si>
+  <si>
+    <t>1858700158623</t>
+  </si>
+  <si>
+    <t>1858700158624</t>
+  </si>
+  <si>
+    <t>1858700158625</t>
+  </si>
+  <si>
+    <t>1858700158626</t>
+  </si>
+  <si>
+    <t>1858700158627</t>
+  </si>
+  <si>
+    <t>1858700158628</t>
+  </si>
+  <si>
+    <t>1858700158629</t>
+  </si>
+  <si>
+    <t>1858700158630</t>
+  </si>
+  <si>
+    <t>1858700158631</t>
+  </si>
+  <si>
+    <t>1858700158632</t>
+  </si>
+  <si>
+    <t>1858700158633</t>
+  </si>
+  <si>
+    <t>1858700158634</t>
+  </si>
+  <si>
+    <t>1858700158635</t>
+  </si>
+  <si>
+    <t>1858700158636</t>
+  </si>
+  <si>
+    <t>1858700158637</t>
+  </si>
+  <si>
+    <t>1858700158638</t>
+  </si>
+  <si>
+    <t>1858700158639</t>
+  </si>
+  <si>
+    <t>1858700158640</t>
   </si>
 </sst>
 </file>
@@ -940,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR61"/>
+  <dimension ref="A1:AR81"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -9115,6 +9175,2686 @@
       </c>
       <c r="AR61" s="3" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="62" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>1</v>
+      </c>
+      <c r="B62" s="2">
+        <v>2</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F62" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G62" s="5">
+        <v>61</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K62" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L62" s="6">
+        <v>5088</v>
+      </c>
+      <c r="M62" s="7">
+        <v>869772.92</v>
+      </c>
+      <c r="N62" s="6">
+        <v>1</v>
+      </c>
+      <c r="O62" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P62" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q62" s="6">
+        <v>0</v>
+      </c>
+      <c r="R62" s="7">
+        <v>0</v>
+      </c>
+      <c r="S62" s="9">
+        <v>0</v>
+      </c>
+      <c r="T62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U62" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V62" s="11">
+        <v>11</v>
+      </c>
+      <c r="W62" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X62" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y62" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB62" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG62" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI62" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ62" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL62" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM62" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ62" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR62" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="63" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>1</v>
+      </c>
+      <c r="B63" s="2">
+        <v>2</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F63" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G63" s="5">
+        <v>62</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K63" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L63" s="6">
+        <v>5089</v>
+      </c>
+      <c r="M63" s="7">
+        <v>869943.86</v>
+      </c>
+      <c r="N63" s="6">
+        <v>1</v>
+      </c>
+      <c r="O63" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P63" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q63" s="6">
+        <v>0</v>
+      </c>
+      <c r="R63" s="7">
+        <v>0</v>
+      </c>
+      <c r="S63" s="9">
+        <v>0</v>
+      </c>
+      <c r="T63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U63" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V63" s="11">
+        <v>11</v>
+      </c>
+      <c r="W63" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X63" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y63" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB63" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG63" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI63" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ63" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL63" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM63" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ63" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR63" s="3" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="64" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>1</v>
+      </c>
+      <c r="B64" s="2">
+        <v>2</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F64" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G64" s="5">
+        <v>63</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I64" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K64" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L64" s="6">
+        <v>5090</v>
+      </c>
+      <c r="M64" s="7">
+        <v>870114.81</v>
+      </c>
+      <c r="N64" s="6">
+        <v>1</v>
+      </c>
+      <c r="O64" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P64" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q64" s="6">
+        <v>0</v>
+      </c>
+      <c r="R64" s="7">
+        <v>0</v>
+      </c>
+      <c r="S64" s="9">
+        <v>0</v>
+      </c>
+      <c r="T64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U64" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V64" s="11">
+        <v>11</v>
+      </c>
+      <c r="W64" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X64" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y64" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB64" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG64" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI64" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ64" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL64" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM64" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ64" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR64" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="65" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>1</v>
+      </c>
+      <c r="B65" s="2">
+        <v>2</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F65" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G65" s="5">
+        <v>64</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I65" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K65" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L65" s="6">
+        <v>5091</v>
+      </c>
+      <c r="M65" s="7">
+        <v>870285.75</v>
+      </c>
+      <c r="N65" s="6">
+        <v>1</v>
+      </c>
+      <c r="O65" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P65" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q65" s="6">
+        <v>0</v>
+      </c>
+      <c r="R65" s="7">
+        <v>0</v>
+      </c>
+      <c r="S65" s="9">
+        <v>0</v>
+      </c>
+      <c r="T65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U65" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V65" s="11">
+        <v>11</v>
+      </c>
+      <c r="W65" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X65" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y65" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB65" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG65" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI65" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL65" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM65" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ65" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR65" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="66" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>1</v>
+      </c>
+      <c r="B66" s="2">
+        <v>2</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F66" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G66" s="5">
+        <v>65</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I66" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K66" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L66" s="6">
+        <v>5092</v>
+      </c>
+      <c r="M66" s="7">
+        <v>870456.7</v>
+      </c>
+      <c r="N66" s="6">
+        <v>1</v>
+      </c>
+      <c r="O66" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P66" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q66" s="6">
+        <v>0</v>
+      </c>
+      <c r="R66" s="7">
+        <v>0</v>
+      </c>
+      <c r="S66" s="9">
+        <v>0</v>
+      </c>
+      <c r="T66" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U66" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V66" s="11">
+        <v>11</v>
+      </c>
+      <c r="W66" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X66" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y66" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB66" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG66" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI66" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ66" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK66" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL66" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM66" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ66" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR66" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="67" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>1</v>
+      </c>
+      <c r="B67" s="2">
+        <v>2</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F67" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G67" s="5">
+        <v>66</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I67" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J67" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K67" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L67" s="6">
+        <v>5093</v>
+      </c>
+      <c r="M67" s="7">
+        <v>870627.65</v>
+      </c>
+      <c r="N67" s="6">
+        <v>1</v>
+      </c>
+      <c r="O67" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P67" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q67" s="6">
+        <v>0</v>
+      </c>
+      <c r="R67" s="7">
+        <v>0</v>
+      </c>
+      <c r="S67" s="9">
+        <v>0</v>
+      </c>
+      <c r="T67" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U67" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V67" s="11">
+        <v>11</v>
+      </c>
+      <c r="W67" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X67" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y67" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB67" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG67" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI67" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ67" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK67" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL67" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM67" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ67" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR67" s="3" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="68" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>1</v>
+      </c>
+      <c r="B68" s="2">
+        <v>2</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F68" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G68" s="5">
+        <v>67</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I68" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J68" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K68" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L68" s="6">
+        <v>5094</v>
+      </c>
+      <c r="M68" s="7">
+        <v>870798.59</v>
+      </c>
+      <c r="N68" s="6">
+        <v>1</v>
+      </c>
+      <c r="O68" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P68" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q68" s="6">
+        <v>0</v>
+      </c>
+      <c r="R68" s="7">
+        <v>0</v>
+      </c>
+      <c r="S68" s="9">
+        <v>0</v>
+      </c>
+      <c r="T68" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U68" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V68" s="11">
+        <v>11</v>
+      </c>
+      <c r="W68" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X68" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y68" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB68" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG68" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI68" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ68" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK68" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL68" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM68" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ68" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR68" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="69" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>1</v>
+      </c>
+      <c r="B69" s="2">
+        <v>2</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F69" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G69" s="5">
+        <v>68</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J69" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K69" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L69" s="6">
+        <v>5095</v>
+      </c>
+      <c r="M69" s="7">
+        <v>870969.54</v>
+      </c>
+      <c r="N69" s="6">
+        <v>1</v>
+      </c>
+      <c r="O69" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P69" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q69" s="6">
+        <v>0</v>
+      </c>
+      <c r="R69" s="7">
+        <v>0</v>
+      </c>
+      <c r="S69" s="9">
+        <v>0</v>
+      </c>
+      <c r="T69" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U69" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V69" s="11">
+        <v>11</v>
+      </c>
+      <c r="W69" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X69" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y69" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB69" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG69" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI69" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ69" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK69" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL69" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM69" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ69" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR69" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A70" s="1">
+        <v>1</v>
+      </c>
+      <c r="B70" s="2">
+        <v>2</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F70" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G70" s="5">
+        <v>69</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I70" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J70" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K70" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L70" s="6">
+        <v>5096</v>
+      </c>
+      <c r="M70" s="7">
+        <v>871140.48</v>
+      </c>
+      <c r="N70" s="6">
+        <v>1</v>
+      </c>
+      <c r="O70" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P70" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q70" s="6">
+        <v>0</v>
+      </c>
+      <c r="R70" s="7">
+        <v>0</v>
+      </c>
+      <c r="S70" s="9">
+        <v>0</v>
+      </c>
+      <c r="T70" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U70" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V70" s="11">
+        <v>11</v>
+      </c>
+      <c r="W70" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X70" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y70" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB70" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG70" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI70" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ70" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK70" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL70" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM70" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR70" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A71" s="1">
+        <v>1</v>
+      </c>
+      <c r="B71" s="2">
+        <v>2</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F71" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G71" s="5">
+        <v>70</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I71" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J71" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K71" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L71" s="6">
+        <v>5097</v>
+      </c>
+      <c r="M71" s="7">
+        <v>871311.43</v>
+      </c>
+      <c r="N71" s="6">
+        <v>1</v>
+      </c>
+      <c r="O71" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P71" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q71" s="6">
+        <v>0</v>
+      </c>
+      <c r="R71" s="7">
+        <v>0</v>
+      </c>
+      <c r="S71" s="9">
+        <v>0</v>
+      </c>
+      <c r="T71" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U71" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V71" s="11">
+        <v>11</v>
+      </c>
+      <c r="W71" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X71" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y71" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB71" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG71" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI71" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ71" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK71" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL71" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM71" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ71" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR71" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A72" s="1">
+        <v>1</v>
+      </c>
+      <c r="B72" s="2">
+        <v>2</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F72" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G72" s="5">
+        <v>71</v>
+      </c>
+      <c r="H72" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I72" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K72" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L72" s="6">
+        <v>5098</v>
+      </c>
+      <c r="M72" s="7">
+        <v>871482.38</v>
+      </c>
+      <c r="N72" s="6">
+        <v>1</v>
+      </c>
+      <c r="O72" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P72" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q72" s="6">
+        <v>0</v>
+      </c>
+      <c r="R72" s="7">
+        <v>0</v>
+      </c>
+      <c r="S72" s="9">
+        <v>0</v>
+      </c>
+      <c r="T72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U72" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V72" s="11">
+        <v>11</v>
+      </c>
+      <c r="W72" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X72" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y72" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB72" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG72" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI72" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ72" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL72" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM72" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ72" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR72" s="3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="73" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A73" s="1">
+        <v>1</v>
+      </c>
+      <c r="B73" s="2">
+        <v>2</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F73" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G73" s="5">
+        <v>72</v>
+      </c>
+      <c r="H73" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I73" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K73" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L73" s="6">
+        <v>5099</v>
+      </c>
+      <c r="M73" s="7">
+        <v>871653.32</v>
+      </c>
+      <c r="N73" s="6">
+        <v>1</v>
+      </c>
+      <c r="O73" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P73" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q73" s="6">
+        <v>0</v>
+      </c>
+      <c r="R73" s="7">
+        <v>0</v>
+      </c>
+      <c r="S73" s="9">
+        <v>0</v>
+      </c>
+      <c r="T73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U73" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V73" s="11">
+        <v>11</v>
+      </c>
+      <c r="W73" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X73" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y73" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB73" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG73" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI73" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ73" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL73" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM73" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ73" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR73" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="74" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A74" s="1">
+        <v>1</v>
+      </c>
+      <c r="B74" s="2">
+        <v>2</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F74" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G74" s="5">
+        <v>73</v>
+      </c>
+      <c r="H74" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I74" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K74" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L74" s="6">
+        <v>5100</v>
+      </c>
+      <c r="M74" s="7">
+        <v>871824.27</v>
+      </c>
+      <c r="N74" s="6">
+        <v>1</v>
+      </c>
+      <c r="O74" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P74" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q74" s="6">
+        <v>0</v>
+      </c>
+      <c r="R74" s="7">
+        <v>0</v>
+      </c>
+      <c r="S74" s="9">
+        <v>0</v>
+      </c>
+      <c r="T74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U74" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V74" s="11">
+        <v>11</v>
+      </c>
+      <c r="W74" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X74" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y74" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB74" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG74" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI74" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ74" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL74" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM74" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ74" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR74" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="75" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A75" s="1">
+        <v>1</v>
+      </c>
+      <c r="B75" s="2">
+        <v>2</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F75" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G75" s="5">
+        <v>74</v>
+      </c>
+      <c r="H75" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I75" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K75" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L75" s="6">
+        <v>5101</v>
+      </c>
+      <c r="M75" s="7">
+        <v>871995.21</v>
+      </c>
+      <c r="N75" s="6">
+        <v>1</v>
+      </c>
+      <c r="O75" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P75" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q75" s="6">
+        <v>0</v>
+      </c>
+      <c r="R75" s="7">
+        <v>0</v>
+      </c>
+      <c r="S75" s="9">
+        <v>0</v>
+      </c>
+      <c r="T75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U75" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V75" s="11">
+        <v>11</v>
+      </c>
+      <c r="W75" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X75" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y75" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB75" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG75" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI75" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ75" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL75" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM75" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ75" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR75" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="76" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A76" s="1">
+        <v>1</v>
+      </c>
+      <c r="B76" s="2">
+        <v>2</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F76" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G76" s="5">
+        <v>75</v>
+      </c>
+      <c r="H76" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I76" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J76" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K76" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L76" s="6">
+        <v>5102</v>
+      </c>
+      <c r="M76" s="7">
+        <v>872166.16</v>
+      </c>
+      <c r="N76" s="6">
+        <v>1</v>
+      </c>
+      <c r="O76" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P76" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q76" s="6">
+        <v>0</v>
+      </c>
+      <c r="R76" s="7">
+        <v>0</v>
+      </c>
+      <c r="S76" s="9">
+        <v>0</v>
+      </c>
+      <c r="T76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U76" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V76" s="11">
+        <v>11</v>
+      </c>
+      <c r="W76" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X76" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y76" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB76" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG76" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI76" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ76" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL76" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM76" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ76" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR76" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="77" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A77" s="1">
+        <v>1</v>
+      </c>
+      <c r="B77" s="2">
+        <v>2</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F77" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G77" s="5">
+        <v>76</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J77" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K77" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L77" s="6">
+        <v>5103</v>
+      </c>
+      <c r="M77" s="7">
+        <v>872337.11</v>
+      </c>
+      <c r="N77" s="6">
+        <v>1</v>
+      </c>
+      <c r="O77" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P77" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q77" s="6">
+        <v>0</v>
+      </c>
+      <c r="R77" s="7">
+        <v>0</v>
+      </c>
+      <c r="S77" s="9">
+        <v>0</v>
+      </c>
+      <c r="T77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U77" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V77" s="11">
+        <v>11</v>
+      </c>
+      <c r="W77" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X77" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y77" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB77" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG77" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI77" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ77" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL77" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM77" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ77" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR77" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="78" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A78" s="1">
+        <v>1</v>
+      </c>
+      <c r="B78" s="2">
+        <v>2</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F78" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G78" s="5">
+        <v>77</v>
+      </c>
+      <c r="H78" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I78" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J78" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K78" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L78" s="6">
+        <v>5104</v>
+      </c>
+      <c r="M78" s="7">
+        <v>872508.05</v>
+      </c>
+      <c r="N78" s="6">
+        <v>1</v>
+      </c>
+      <c r="O78" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P78" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q78" s="6">
+        <v>0</v>
+      </c>
+      <c r="R78" s="7">
+        <v>0</v>
+      </c>
+      <c r="S78" s="9">
+        <v>0</v>
+      </c>
+      <c r="T78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U78" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V78" s="11">
+        <v>11</v>
+      </c>
+      <c r="W78" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X78" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y78" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB78" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG78" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI78" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ78" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL78" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM78" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ78" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR78" s="3" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="79" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A79" s="1">
+        <v>1</v>
+      </c>
+      <c r="B79" s="2">
+        <v>2</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F79" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G79" s="5">
+        <v>78</v>
+      </c>
+      <c r="H79" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I79" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J79" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K79" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L79" s="6">
+        <v>5105</v>
+      </c>
+      <c r="M79" s="7">
+        <v>872679</v>
+      </c>
+      <c r="N79" s="6">
+        <v>1</v>
+      </c>
+      <c r="O79" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P79" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q79" s="6">
+        <v>0</v>
+      </c>
+      <c r="R79" s="7">
+        <v>0</v>
+      </c>
+      <c r="S79" s="9">
+        <v>0</v>
+      </c>
+      <c r="T79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U79" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V79" s="11">
+        <v>11</v>
+      </c>
+      <c r="W79" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X79" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y79" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB79" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG79" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI79" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ79" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL79" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM79" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ79" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR79" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="80" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A80" s="1">
+        <v>1</v>
+      </c>
+      <c r="B80" s="2">
+        <v>2</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F80" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G80" s="5">
+        <v>79</v>
+      </c>
+      <c r="H80" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I80" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J80" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K80" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L80" s="6">
+        <v>5106</v>
+      </c>
+      <c r="M80" s="7">
+        <v>872849.94</v>
+      </c>
+      <c r="N80" s="6">
+        <v>1</v>
+      </c>
+      <c r="O80" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P80" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q80" s="6">
+        <v>0</v>
+      </c>
+      <c r="R80" s="7">
+        <v>0</v>
+      </c>
+      <c r="S80" s="9">
+        <v>0</v>
+      </c>
+      <c r="T80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U80" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V80" s="11">
+        <v>11</v>
+      </c>
+      <c r="W80" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X80" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y80" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB80" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG80" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI80" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ80" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL80" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM80" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ80" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR80" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="81" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A81" s="1">
+        <v>1</v>
+      </c>
+      <c r="B81" s="2">
+        <v>2</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F81" s="4">
+        <v>46317</v>
+      </c>
+      <c r="G81" s="5">
+        <v>80</v>
+      </c>
+      <c r="H81" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I81" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J81" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K81" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L81" s="6">
+        <v>5107</v>
+      </c>
+      <c r="M81" s="7">
+        <v>873020.89</v>
+      </c>
+      <c r="N81" s="6">
+        <v>1</v>
+      </c>
+      <c r="O81" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P81" s="8">
+        <v>170.95</v>
+      </c>
+      <c r="Q81" s="6">
+        <v>0</v>
+      </c>
+      <c r="R81" s="7">
+        <v>0</v>
+      </c>
+      <c r="S81" s="9">
+        <v>0</v>
+      </c>
+      <c r="T81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U81" s="10">
+        <v>68458</v>
+      </c>
+      <c r="V81" s="11">
+        <v>11</v>
+      </c>
+      <c r="W81" s="4">
+        <v>46317</v>
+      </c>
+      <c r="X81" s="12">
+        <v>0.33472220000000003</v>
+      </c>
+      <c r="Y81" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB81" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG81" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI81" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ81" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL81" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM81" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ81" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR81" s="3" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 26/10/2026 14:25:37,96
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A34E3E53-0E04-4482-A1E1-8D3A59519369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98746A80-7EAE-447F-81D8-E6752E82E4EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12500" uniqueCount="756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12590" uniqueCount="761">
   <si>
     <t>Sel</t>
   </si>
@@ -1972,6 +1972,21 @@
     <t>1871400013444</t>
   </si>
   <si>
+    <t>1871400013445</t>
+  </si>
+  <si>
+    <t>1871400013446</t>
+  </si>
+  <si>
+    <t>1871400013447</t>
+  </si>
+  <si>
+    <t>1871400013448</t>
+  </si>
+  <si>
+    <t>1871400013449</t>
+  </si>
+  <si>
     <t>FORNO ELETRICO NARDELLI EMBUTIR 60L BLACK - NARDELLI EMBUTIR 60L BLACK - 220 V</t>
   </si>
   <si>
@@ -2863,7 +2878,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR693"/>
+  <dimension ref="A1:AR698"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -81669,7 +81684,7 @@
         <v>566</v>
       </c>
       <c r="D589" s="3" t="s">
-        <v>45</v>
+        <v>567</v>
       </c>
       <c r="E589" s="3" t="s">
         <v>46</v>
@@ -81678,7 +81693,7 @@
         <v>46321</v>
       </c>
       <c r="G589" s="5">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="H589" s="3" t="s">
         <v>47</v>
@@ -81693,19 +81708,19 @@
         <v>50</v>
       </c>
       <c r="L589" s="6">
-        <v>532</v>
+        <v>566</v>
       </c>
       <c r="M589" s="7">
-        <v>176390.14</v>
+        <v>190231.65</v>
       </c>
       <c r="N589" s="6">
         <v>1</v>
       </c>
       <c r="O589" s="3" t="s">
-        <v>650</v>
+        <v>568</v>
       </c>
       <c r="P589" s="8">
-        <v>331.56</v>
+        <v>336.1</v>
       </c>
       <c r="Q589" s="6">
         <v>0</v>
@@ -81720,7 +81735,7 @@
         <v>52</v>
       </c>
       <c r="U589" s="10">
-        <v>68570</v>
+        <v>68595</v>
       </c>
       <c r="V589" s="11">
         <v>11</v>
@@ -81729,7 +81744,7 @@
         <v>46321</v>
       </c>
       <c r="X589" s="12">
-        <v>0.3</v>
+        <v>0.59791669999999997</v>
       </c>
       <c r="Y589" s="10">
         <v>0</v>
@@ -81789,7 +81804,7 @@
         <v>53</v>
       </c>
       <c r="AR589" s="3" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="590" spans="1:44" x14ac:dyDescent="0.3">
@@ -81803,7 +81818,7 @@
         <v>566</v>
       </c>
       <c r="D590" s="3" t="s">
-        <v>45</v>
+        <v>567</v>
       </c>
       <c r="E590" s="3" t="s">
         <v>46</v>
@@ -81812,7 +81827,7 @@
         <v>46321</v>
       </c>
       <c r="G590" s="5">
-        <v>2</v>
+        <v>85</v>
       </c>
       <c r="H590" s="3" t="s">
         <v>47</v>
@@ -81827,19 +81842,19 @@
         <v>50</v>
       </c>
       <c r="L590" s="6">
-        <v>533</v>
+        <v>567</v>
       </c>
       <c r="M590" s="7">
-        <v>176721.7</v>
+        <v>190567.75</v>
       </c>
       <c r="N590" s="6">
         <v>1</v>
       </c>
       <c r="O590" s="3" t="s">
-        <v>650</v>
+        <v>568</v>
       </c>
       <c r="P590" s="8">
-        <v>331.56</v>
+        <v>336.1</v>
       </c>
       <c r="Q590" s="6">
         <v>0</v>
@@ -81854,7 +81869,7 @@
         <v>52</v>
       </c>
       <c r="U590" s="10">
-        <v>68570</v>
+        <v>68595</v>
       </c>
       <c r="V590" s="11">
         <v>11</v>
@@ -81863,7 +81878,7 @@
         <v>46321</v>
       </c>
       <c r="X590" s="12">
-        <v>0.3</v>
+        <v>0.59791669999999997</v>
       </c>
       <c r="Y590" s="10">
         <v>0</v>
@@ -81923,7 +81938,7 @@
         <v>53</v>
       </c>
       <c r="AR590" s="3" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="591" spans="1:44" x14ac:dyDescent="0.3">
@@ -81937,7 +81952,7 @@
         <v>566</v>
       </c>
       <c r="D591" s="3" t="s">
-        <v>45</v>
+        <v>567</v>
       </c>
       <c r="E591" s="3" t="s">
         <v>46</v>
@@ -81946,7 +81961,7 @@
         <v>46321</v>
       </c>
       <c r="G591" s="5">
-        <v>3</v>
+        <v>86</v>
       </c>
       <c r="H591" s="3" t="s">
         <v>47</v>
@@ -81961,19 +81976,19 @@
         <v>50</v>
       </c>
       <c r="L591" s="6">
-        <v>534</v>
+        <v>568</v>
       </c>
       <c r="M591" s="7">
-        <v>177053.26</v>
+        <v>190903.85</v>
       </c>
       <c r="N591" s="6">
         <v>1</v>
       </c>
       <c r="O591" s="3" t="s">
-        <v>650</v>
+        <v>568</v>
       </c>
       <c r="P591" s="8">
-        <v>331.56</v>
+        <v>336.1</v>
       </c>
       <c r="Q591" s="6">
         <v>0</v>
@@ -81988,7 +82003,7 @@
         <v>52</v>
       </c>
       <c r="U591" s="10">
-        <v>68570</v>
+        <v>68595</v>
       </c>
       <c r="V591" s="11">
         <v>11</v>
@@ -81997,7 +82012,7 @@
         <v>46321</v>
       </c>
       <c r="X591" s="12">
-        <v>0.3</v>
+        <v>0.59791669999999997</v>
       </c>
       <c r="Y591" s="10">
         <v>0</v>
@@ -82057,7 +82072,7 @@
         <v>53</v>
       </c>
       <c r="AR591" s="3" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="592" spans="1:44" x14ac:dyDescent="0.3">
@@ -82071,7 +82086,7 @@
         <v>566</v>
       </c>
       <c r="D592" s="3" t="s">
-        <v>45</v>
+        <v>567</v>
       </c>
       <c r="E592" s="3" t="s">
         <v>46</v>
@@ -82080,7 +82095,7 @@
         <v>46321</v>
       </c>
       <c r="G592" s="5">
-        <v>4</v>
+        <v>87</v>
       </c>
       <c r="H592" s="3" t="s">
         <v>47</v>
@@ -82095,19 +82110,19 @@
         <v>50</v>
       </c>
       <c r="L592" s="6">
-        <v>535</v>
+        <v>569</v>
       </c>
       <c r="M592" s="7">
-        <v>177384.82</v>
+        <v>191239.95</v>
       </c>
       <c r="N592" s="6">
         <v>1</v>
       </c>
       <c r="O592" s="3" t="s">
-        <v>650</v>
+        <v>568</v>
       </c>
       <c r="P592" s="8">
-        <v>331.56</v>
+        <v>336.1</v>
       </c>
       <c r="Q592" s="6">
         <v>0</v>
@@ -82122,7 +82137,7 @@
         <v>52</v>
       </c>
       <c r="U592" s="10">
-        <v>68570</v>
+        <v>68595</v>
       </c>
       <c r="V592" s="11">
         <v>11</v>
@@ -82131,7 +82146,7 @@
         <v>46321</v>
       </c>
       <c r="X592" s="12">
-        <v>0.3</v>
+        <v>0.59791669999999997</v>
       </c>
       <c r="Y592" s="10">
         <v>0</v>
@@ -82191,7 +82206,7 @@
         <v>53</v>
       </c>
       <c r="AR592" s="3" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="593" spans="1:44" x14ac:dyDescent="0.3">
@@ -82205,7 +82220,7 @@
         <v>566</v>
       </c>
       <c r="D593" s="3" t="s">
-        <v>45</v>
+        <v>567</v>
       </c>
       <c r="E593" s="3" t="s">
         <v>46</v>
@@ -82214,7 +82229,7 @@
         <v>46321</v>
       </c>
       <c r="G593" s="5">
-        <v>5</v>
+        <v>88</v>
       </c>
       <c r="H593" s="3" t="s">
         <v>47</v>
@@ -82229,19 +82244,19 @@
         <v>50</v>
       </c>
       <c r="L593" s="6">
-        <v>536</v>
+        <v>570</v>
       </c>
       <c r="M593" s="7">
-        <v>177716.38</v>
+        <v>191576.04</v>
       </c>
       <c r="N593" s="6">
         <v>1</v>
       </c>
       <c r="O593" s="3" t="s">
-        <v>650</v>
+        <v>568</v>
       </c>
       <c r="P593" s="8">
-        <v>331.56</v>
+        <v>336.1</v>
       </c>
       <c r="Q593" s="6">
         <v>0</v>
@@ -82256,7 +82271,7 @@
         <v>52</v>
       </c>
       <c r="U593" s="10">
-        <v>68570</v>
+        <v>68595</v>
       </c>
       <c r="V593" s="11">
         <v>11</v>
@@ -82265,7 +82280,7 @@
         <v>46321</v>
       </c>
       <c r="X593" s="12">
-        <v>0.30694440000000001</v>
+        <v>0.59791669999999997</v>
       </c>
       <c r="Y593" s="10">
         <v>0</v>
@@ -82325,7 +82340,7 @@
         <v>53</v>
       </c>
       <c r="AR593" s="3" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="594" spans="1:44" x14ac:dyDescent="0.3">
@@ -82348,7 +82363,7 @@
         <v>46321</v>
       </c>
       <c r="G594" s="5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H594" s="3" t="s">
         <v>47</v>
@@ -82363,16 +82378,16 @@
         <v>50</v>
       </c>
       <c r="L594" s="6">
-        <v>537</v>
+        <v>532</v>
       </c>
       <c r="M594" s="7">
-        <v>178047.94</v>
+        <v>176390.14</v>
       </c>
       <c r="N594" s="6">
         <v>1</v>
       </c>
       <c r="O594" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P594" s="8">
         <v>331.56</v>
@@ -82399,7 +82414,7 @@
         <v>46321</v>
       </c>
       <c r="X594" s="12">
-        <v>0.30694440000000001</v>
+        <v>0.3</v>
       </c>
       <c r="Y594" s="10">
         <v>0</v>
@@ -82482,7 +82497,7 @@
         <v>46321</v>
       </c>
       <c r="G595" s="5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H595" s="3" t="s">
         <v>47</v>
@@ -82497,16 +82512,16 @@
         <v>50</v>
       </c>
       <c r="L595" s="6">
-        <v>538</v>
+        <v>533</v>
       </c>
       <c r="M595" s="7">
-        <v>178379.5</v>
+        <v>176721.7</v>
       </c>
       <c r="N595" s="6">
         <v>1</v>
       </c>
       <c r="O595" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P595" s="8">
         <v>331.56</v>
@@ -82533,7 +82548,7 @@
         <v>46321</v>
       </c>
       <c r="X595" s="12">
-        <v>0.30694440000000001</v>
+        <v>0.3</v>
       </c>
       <c r="Y595" s="10">
         <v>0</v>
@@ -82616,7 +82631,7 @@
         <v>46321</v>
       </c>
       <c r="G596" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H596" s="3" t="s">
         <v>47</v>
@@ -82631,16 +82646,16 @@
         <v>50</v>
       </c>
       <c r="L596" s="6">
-        <v>539</v>
+        <v>534</v>
       </c>
       <c r="M596" s="7">
-        <v>178711.06</v>
+        <v>177053.26</v>
       </c>
       <c r="N596" s="6">
         <v>1</v>
       </c>
       <c r="O596" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P596" s="8">
         <v>331.56</v>
@@ -82667,7 +82682,7 @@
         <v>46321</v>
       </c>
       <c r="X596" s="12">
-        <v>0.30694440000000001</v>
+        <v>0.3</v>
       </c>
       <c r="Y596" s="10">
         <v>0</v>
@@ -82750,7 +82765,7 @@
         <v>46321</v>
       </c>
       <c r="G597" s="5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H597" s="3" t="s">
         <v>47</v>
@@ -82765,16 +82780,16 @@
         <v>50</v>
       </c>
       <c r="L597" s="6">
-        <v>540</v>
+        <v>535</v>
       </c>
       <c r="M597" s="7">
-        <v>179042.62</v>
+        <v>177384.82</v>
       </c>
       <c r="N597" s="6">
         <v>1</v>
       </c>
       <c r="O597" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P597" s="8">
         <v>331.56</v>
@@ -82801,7 +82816,7 @@
         <v>46321</v>
       </c>
       <c r="X597" s="12">
-        <v>0.31388890000000003</v>
+        <v>0.3</v>
       </c>
       <c r="Y597" s="10">
         <v>0</v>
@@ -82884,7 +82899,7 @@
         <v>46321</v>
       </c>
       <c r="G598" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H598" s="3" t="s">
         <v>47</v>
@@ -82899,16 +82914,16 @@
         <v>50</v>
       </c>
       <c r="L598" s="6">
-        <v>541</v>
+        <v>536</v>
       </c>
       <c r="M598" s="7">
-        <v>179374.18</v>
+        <v>177716.38</v>
       </c>
       <c r="N598" s="6">
         <v>1</v>
       </c>
       <c r="O598" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P598" s="8">
         <v>331.56</v>
@@ -82935,7 +82950,7 @@
         <v>46321</v>
       </c>
       <c r="X598" s="12">
-        <v>0.31388890000000003</v>
+        <v>0.30694440000000001</v>
       </c>
       <c r="Y598" s="10">
         <v>0</v>
@@ -83018,7 +83033,7 @@
         <v>46321</v>
       </c>
       <c r="G599" s="5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H599" s="3" t="s">
         <v>47</v>
@@ -83033,16 +83048,16 @@
         <v>50</v>
       </c>
       <c r="L599" s="6">
-        <v>542</v>
+        <v>537</v>
       </c>
       <c r="M599" s="7">
-        <v>179705.74</v>
+        <v>178047.94</v>
       </c>
       <c r="N599" s="6">
         <v>1</v>
       </c>
       <c r="O599" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P599" s="8">
         <v>331.56</v>
@@ -83069,7 +83084,7 @@
         <v>46321</v>
       </c>
       <c r="X599" s="12">
-        <v>0.31388890000000003</v>
+        <v>0.30694440000000001</v>
       </c>
       <c r="Y599" s="10">
         <v>0</v>
@@ -83152,7 +83167,7 @@
         <v>46321</v>
       </c>
       <c r="G600" s="5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H600" s="3" t="s">
         <v>47</v>
@@ -83167,16 +83182,16 @@
         <v>50</v>
       </c>
       <c r="L600" s="6">
-        <v>543</v>
+        <v>538</v>
       </c>
       <c r="M600" s="7">
-        <v>180037.3</v>
+        <v>178379.5</v>
       </c>
       <c r="N600" s="6">
         <v>1</v>
       </c>
       <c r="O600" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P600" s="8">
         <v>331.56</v>
@@ -83203,7 +83218,7 @@
         <v>46321</v>
       </c>
       <c r="X600" s="12">
-        <v>0.31388890000000003</v>
+        <v>0.30694440000000001</v>
       </c>
       <c r="Y600" s="10">
         <v>0</v>
@@ -83286,7 +83301,7 @@
         <v>46321</v>
       </c>
       <c r="G601" s="5">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H601" s="3" t="s">
         <v>47</v>
@@ -83301,16 +83316,16 @@
         <v>50</v>
       </c>
       <c r="L601" s="6">
-        <v>544</v>
+        <v>539</v>
       </c>
       <c r="M601" s="7">
-        <v>180368.86</v>
+        <v>178711.06</v>
       </c>
       <c r="N601" s="6">
         <v>1</v>
       </c>
       <c r="O601" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P601" s="8">
         <v>331.56</v>
@@ -83337,7 +83352,7 @@
         <v>46321</v>
       </c>
       <c r="X601" s="12">
-        <v>0.31388890000000003</v>
+        <v>0.30694440000000001</v>
       </c>
       <c r="Y601" s="10">
         <v>0</v>
@@ -83420,7 +83435,7 @@
         <v>46321</v>
       </c>
       <c r="G602" s="5">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H602" s="3" t="s">
         <v>47</v>
@@ -83435,16 +83450,16 @@
         <v>50</v>
       </c>
       <c r="L602" s="6">
-        <v>545</v>
+        <v>540</v>
       </c>
       <c r="M602" s="7">
-        <v>180700.42</v>
+        <v>179042.62</v>
       </c>
       <c r="N602" s="6">
         <v>1</v>
       </c>
       <c r="O602" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P602" s="8">
         <v>331.56</v>
@@ -83554,7 +83569,7 @@
         <v>46321</v>
       </c>
       <c r="G603" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H603" s="3" t="s">
         <v>47</v>
@@ -83569,16 +83584,16 @@
         <v>50</v>
       </c>
       <c r="L603" s="6">
-        <v>546</v>
+        <v>541</v>
       </c>
       <c r="M603" s="7">
-        <v>181031.98</v>
+        <v>179374.18</v>
       </c>
       <c r="N603" s="6">
         <v>1</v>
       </c>
       <c r="O603" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P603" s="8">
         <v>331.56</v>
@@ -83688,7 +83703,7 @@
         <v>46321</v>
       </c>
       <c r="G604" s="5">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H604" s="3" t="s">
         <v>47</v>
@@ -83703,16 +83718,16 @@
         <v>50</v>
       </c>
       <c r="L604" s="6">
-        <v>547</v>
+        <v>542</v>
       </c>
       <c r="M604" s="7">
-        <v>181363.54</v>
+        <v>179705.74</v>
       </c>
       <c r="N604" s="6">
         <v>1</v>
       </c>
       <c r="O604" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P604" s="8">
         <v>331.56</v>
@@ -83739,7 +83754,7 @@
         <v>46321</v>
       </c>
       <c r="X604" s="12">
-        <v>0.32152779999999997</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y604" s="10">
         <v>0</v>
@@ -83822,7 +83837,7 @@
         <v>46321</v>
       </c>
       <c r="G605" s="5">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H605" s="3" t="s">
         <v>47</v>
@@ -83837,16 +83852,16 @@
         <v>50</v>
       </c>
       <c r="L605" s="6">
-        <v>548</v>
+        <v>543</v>
       </c>
       <c r="M605" s="7">
-        <v>181695.1</v>
+        <v>180037.3</v>
       </c>
       <c r="N605" s="6">
         <v>1</v>
       </c>
       <c r="O605" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P605" s="8">
         <v>331.56</v>
@@ -83873,7 +83888,7 @@
         <v>46321</v>
       </c>
       <c r="X605" s="12">
-        <v>0.32152779999999997</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y605" s="10">
         <v>0</v>
@@ -83956,7 +83971,7 @@
         <v>46321</v>
       </c>
       <c r="G606" s="5">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H606" s="3" t="s">
         <v>47</v>
@@ -83971,16 +83986,16 @@
         <v>50</v>
       </c>
       <c r="L606" s="6">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="M606" s="7">
-        <v>182026.66</v>
+        <v>180368.86</v>
       </c>
       <c r="N606" s="6">
         <v>1</v>
       </c>
       <c r="O606" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P606" s="8">
         <v>331.56</v>
@@ -84007,7 +84022,7 @@
         <v>46321</v>
       </c>
       <c r="X606" s="12">
-        <v>0.32152779999999997</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y606" s="10">
         <v>0</v>
@@ -84090,7 +84105,7 @@
         <v>46321</v>
       </c>
       <c r="G607" s="5">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H607" s="3" t="s">
         <v>47</v>
@@ -84105,16 +84120,16 @@
         <v>50</v>
       </c>
       <c r="L607" s="6">
-        <v>550</v>
+        <v>545</v>
       </c>
       <c r="M607" s="7">
-        <v>182358.22</v>
+        <v>180700.42</v>
       </c>
       <c r="N607" s="6">
         <v>1</v>
       </c>
       <c r="O607" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P607" s="8">
         <v>331.56</v>
@@ -84141,7 +84156,7 @@
         <v>46321</v>
       </c>
       <c r="X607" s="12">
-        <v>0.32152779999999997</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y607" s="10">
         <v>0</v>
@@ -84224,7 +84239,7 @@
         <v>46321</v>
       </c>
       <c r="G608" s="5">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="H608" s="3" t="s">
         <v>47</v>
@@ -84239,16 +84254,16 @@
         <v>50</v>
       </c>
       <c r="L608" s="6">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="M608" s="7">
-        <v>182689.78</v>
+        <v>181031.98</v>
       </c>
       <c r="N608" s="6">
         <v>1</v>
       </c>
       <c r="O608" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P608" s="8">
         <v>331.56</v>
@@ -84275,7 +84290,7 @@
         <v>46321</v>
       </c>
       <c r="X608" s="12">
-        <v>0.34930559999999999</v>
+        <v>0.31388890000000003</v>
       </c>
       <c r="Y608" s="10">
         <v>0</v>
@@ -84358,7 +84373,7 @@
         <v>46321</v>
       </c>
       <c r="G609" s="5">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="H609" s="3" t="s">
         <v>47</v>
@@ -84373,16 +84388,16 @@
         <v>50</v>
       </c>
       <c r="L609" s="6">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="M609" s="7">
-        <v>183021.34</v>
+        <v>181363.54</v>
       </c>
       <c r="N609" s="6">
         <v>1</v>
       </c>
       <c r="O609" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P609" s="8">
         <v>331.56</v>
@@ -84409,7 +84424,7 @@
         <v>46321</v>
       </c>
       <c r="X609" s="12">
-        <v>0.34930559999999999</v>
+        <v>0.32152779999999997</v>
       </c>
       <c r="Y609" s="10">
         <v>0</v>
@@ -84492,7 +84507,7 @@
         <v>46321</v>
       </c>
       <c r="G610" s="5">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="H610" s="3" t="s">
         <v>47</v>
@@ -84507,16 +84522,16 @@
         <v>50</v>
       </c>
       <c r="L610" s="6">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="M610" s="7">
-        <v>183352.9</v>
+        <v>181695.1</v>
       </c>
       <c r="N610" s="6">
         <v>1</v>
       </c>
       <c r="O610" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P610" s="8">
         <v>331.56</v>
@@ -84543,7 +84558,7 @@
         <v>46321</v>
       </c>
       <c r="X610" s="12">
-        <v>0.34930559999999999</v>
+        <v>0.32152779999999997</v>
       </c>
       <c r="Y610" s="10">
         <v>0</v>
@@ -84626,7 +84641,7 @@
         <v>46321</v>
       </c>
       <c r="G611" s="5">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="H611" s="3" t="s">
         <v>47</v>
@@ -84641,16 +84656,16 @@
         <v>50</v>
       </c>
       <c r="L611" s="6">
-        <v>554</v>
+        <v>549</v>
       </c>
       <c r="M611" s="7">
-        <v>183684.46</v>
+        <v>182026.66</v>
       </c>
       <c r="N611" s="6">
         <v>1</v>
       </c>
       <c r="O611" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P611" s="8">
         <v>331.56</v>
@@ -84677,7 +84692,7 @@
         <v>46321</v>
       </c>
       <c r="X611" s="12">
-        <v>0.34930559999999999</v>
+        <v>0.32152779999999997</v>
       </c>
       <c r="Y611" s="10">
         <v>0</v>
@@ -84760,7 +84775,7 @@
         <v>46321</v>
       </c>
       <c r="G612" s="5">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="H612" s="3" t="s">
         <v>47</v>
@@ -84775,16 +84790,16 @@
         <v>50</v>
       </c>
       <c r="L612" s="6">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="M612" s="7">
-        <v>184016.02</v>
+        <v>182358.22</v>
       </c>
       <c r="N612" s="6">
         <v>1</v>
       </c>
       <c r="O612" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P612" s="8">
         <v>331.56</v>
@@ -84811,7 +84826,7 @@
         <v>46321</v>
       </c>
       <c r="X612" s="12">
-        <v>0.34930559999999999</v>
+        <v>0.32152779999999997</v>
       </c>
       <c r="Y612" s="10">
         <v>0</v>
@@ -84894,7 +84909,7 @@
         <v>46321</v>
       </c>
       <c r="G613" s="5">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H613" s="3" t="s">
         <v>47</v>
@@ -84909,16 +84924,16 @@
         <v>50</v>
       </c>
       <c r="L613" s="6">
-        <v>556</v>
+        <v>551</v>
       </c>
       <c r="M613" s="7">
-        <v>184347.58</v>
+        <v>182689.78</v>
       </c>
       <c r="N613" s="6">
         <v>1</v>
       </c>
       <c r="O613" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P613" s="8">
         <v>331.56</v>
@@ -85028,7 +85043,7 @@
         <v>46321</v>
       </c>
       <c r="G614" s="5">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H614" s="3" t="s">
         <v>47</v>
@@ -85043,16 +85058,16 @@
         <v>50</v>
       </c>
       <c r="L614" s="6">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="M614" s="7">
-        <v>184679.15</v>
+        <v>183021.34</v>
       </c>
       <c r="N614" s="6">
         <v>1</v>
       </c>
       <c r="O614" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P614" s="8">
         <v>331.56</v>
@@ -85162,7 +85177,7 @@
         <v>46321</v>
       </c>
       <c r="G615" s="5">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H615" s="3" t="s">
         <v>47</v>
@@ -85177,16 +85192,16 @@
         <v>50</v>
       </c>
       <c r="L615" s="6">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="M615" s="7">
-        <v>185010.71</v>
+        <v>183352.9</v>
       </c>
       <c r="N615" s="6">
         <v>1</v>
       </c>
       <c r="O615" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P615" s="8">
         <v>331.56</v>
@@ -85296,7 +85311,7 @@
         <v>46321</v>
       </c>
       <c r="G616" s="5">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H616" s="3" t="s">
         <v>47</v>
@@ -85311,16 +85326,16 @@
         <v>50</v>
       </c>
       <c r="L616" s="6">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="M616" s="7">
-        <v>185342.27</v>
+        <v>183684.46</v>
       </c>
       <c r="N616" s="6">
         <v>1</v>
       </c>
       <c r="O616" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P616" s="8">
         <v>331.56</v>
@@ -85430,7 +85445,7 @@
         <v>46321</v>
       </c>
       <c r="G617" s="5">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H617" s="3" t="s">
         <v>47</v>
@@ -85445,16 +85460,16 @@
         <v>50</v>
       </c>
       <c r="L617" s="6">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="M617" s="7">
-        <v>185673.83</v>
+        <v>184016.02</v>
       </c>
       <c r="N617" s="6">
         <v>1</v>
       </c>
       <c r="O617" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P617" s="8">
         <v>331.56</v>
@@ -85564,7 +85579,7 @@
         <v>46321</v>
       </c>
       <c r="G618" s="5">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H618" s="3" t="s">
         <v>47</v>
@@ -85579,16 +85594,16 @@
         <v>50</v>
       </c>
       <c r="L618" s="6">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="M618" s="7">
-        <v>186005.39</v>
+        <v>184347.58</v>
       </c>
       <c r="N618" s="6">
         <v>1</v>
       </c>
       <c r="O618" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P618" s="8">
         <v>331.56</v>
@@ -85698,7 +85713,7 @@
         <v>46321</v>
       </c>
       <c r="G619" s="5">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H619" s="3" t="s">
         <v>47</v>
@@ -85713,16 +85728,16 @@
         <v>50</v>
       </c>
       <c r="L619" s="6">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="M619" s="7">
-        <v>186336.95</v>
+        <v>184679.15</v>
       </c>
       <c r="N619" s="6">
         <v>1</v>
       </c>
       <c r="O619" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P619" s="8">
         <v>331.56</v>
@@ -85832,7 +85847,7 @@
         <v>46321</v>
       </c>
       <c r="G620" s="5">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="H620" s="3" t="s">
         <v>47</v>
@@ -85847,16 +85862,16 @@
         <v>50</v>
       </c>
       <c r="L620" s="6">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="M620" s="7">
-        <v>186668.51</v>
+        <v>185010.71</v>
       </c>
       <c r="N620" s="6">
         <v>1</v>
       </c>
       <c r="O620" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P620" s="8">
         <v>331.56</v>
@@ -85966,7 +85981,7 @@
         <v>46321</v>
       </c>
       <c r="G621" s="5">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H621" s="3" t="s">
         <v>47</v>
@@ -85981,16 +85996,16 @@
         <v>50</v>
       </c>
       <c r="L621" s="6">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="M621" s="7">
-        <v>187000.07</v>
+        <v>185342.27</v>
       </c>
       <c r="N621" s="6">
         <v>1</v>
       </c>
       <c r="O621" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P621" s="8">
         <v>331.56</v>
@@ -86100,7 +86115,7 @@
         <v>46321</v>
       </c>
       <c r="G622" s="5">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H622" s="3" t="s">
         <v>47</v>
@@ -86115,16 +86130,16 @@
         <v>50</v>
       </c>
       <c r="L622" s="6">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="M622" s="7">
-        <v>187331.63</v>
+        <v>185673.83</v>
       </c>
       <c r="N622" s="6">
         <v>1</v>
       </c>
       <c r="O622" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P622" s="8">
         <v>331.56</v>
@@ -86234,7 +86249,7 @@
         <v>46321</v>
       </c>
       <c r="G623" s="5">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H623" s="3" t="s">
         <v>47</v>
@@ -86249,16 +86264,16 @@
         <v>50</v>
       </c>
       <c r="L623" s="6">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="M623" s="7">
-        <v>187663.19</v>
+        <v>186005.39</v>
       </c>
       <c r="N623" s="6">
         <v>1</v>
       </c>
       <c r="O623" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P623" s="8">
         <v>331.56</v>
@@ -86368,7 +86383,7 @@
         <v>46321</v>
       </c>
       <c r="G624" s="5">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H624" s="3" t="s">
         <v>47</v>
@@ -86383,16 +86398,16 @@
         <v>50</v>
       </c>
       <c r="L624" s="6">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="M624" s="7">
-        <v>187994.75</v>
+        <v>186336.95</v>
       </c>
       <c r="N624" s="6">
         <v>1</v>
       </c>
       <c r="O624" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P624" s="8">
         <v>331.56</v>
@@ -86419,7 +86434,7 @@
         <v>46321</v>
       </c>
       <c r="X624" s="12">
-        <v>0.35555560000000003</v>
+        <v>0.34930559999999999</v>
       </c>
       <c r="Y624" s="10">
         <v>0</v>
@@ -86502,7 +86517,7 @@
         <v>46321</v>
       </c>
       <c r="G625" s="5">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H625" s="3" t="s">
         <v>47</v>
@@ -86517,16 +86532,16 @@
         <v>50</v>
       </c>
       <c r="L625" s="6">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="M625" s="7">
-        <v>188326.31</v>
+        <v>186668.51</v>
       </c>
       <c r="N625" s="6">
         <v>1</v>
       </c>
       <c r="O625" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P625" s="8">
         <v>331.56</v>
@@ -86553,7 +86568,7 @@
         <v>46321</v>
       </c>
       <c r="X625" s="12">
-        <v>0.35555560000000003</v>
+        <v>0.34930559999999999</v>
       </c>
       <c r="Y625" s="10">
         <v>0</v>
@@ -86636,7 +86651,7 @@
         <v>46321</v>
       </c>
       <c r="G626" s="5">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H626" s="3" t="s">
         <v>47</v>
@@ -86651,16 +86666,16 @@
         <v>50</v>
       </c>
       <c r="L626" s="6">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="M626" s="7">
-        <v>188657.87</v>
+        <v>187000.07</v>
       </c>
       <c r="N626" s="6">
         <v>1</v>
       </c>
       <c r="O626" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P626" s="8">
         <v>331.56</v>
@@ -86687,7 +86702,7 @@
         <v>46321</v>
       </c>
       <c r="X626" s="12">
-        <v>0.35555560000000003</v>
+        <v>0.34930559999999999</v>
       </c>
       <c r="Y626" s="10">
         <v>0</v>
@@ -86770,7 +86785,7 @@
         <v>46321</v>
       </c>
       <c r="G627" s="5">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="H627" s="3" t="s">
         <v>47</v>
@@ -86785,16 +86800,16 @@
         <v>50</v>
       </c>
       <c r="L627" s="6">
-        <v>570</v>
+        <v>565</v>
       </c>
       <c r="M627" s="7">
-        <v>188989.43</v>
+        <v>187331.63</v>
       </c>
       <c r="N627" s="6">
         <v>1</v>
       </c>
       <c r="O627" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P627" s="8">
         <v>331.56</v>
@@ -86821,7 +86836,7 @@
         <v>46321</v>
       </c>
       <c r="X627" s="12">
-        <v>0.35555560000000003</v>
+        <v>0.34930559999999999</v>
       </c>
       <c r="Y627" s="10">
         <v>0</v>
@@ -86904,7 +86919,7 @@
         <v>46321</v>
       </c>
       <c r="G628" s="5">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H628" s="3" t="s">
         <v>47</v>
@@ -86919,16 +86934,16 @@
         <v>50</v>
       </c>
       <c r="L628" s="6">
-        <v>571</v>
+        <v>566</v>
       </c>
       <c r="M628" s="7">
-        <v>189320.99</v>
+        <v>187663.19</v>
       </c>
       <c r="N628" s="6">
         <v>1</v>
       </c>
       <c r="O628" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P628" s="8">
         <v>331.56</v>
@@ -86955,7 +86970,7 @@
         <v>46321</v>
       </c>
       <c r="X628" s="12">
-        <v>0.36319439999999997</v>
+        <v>0.34930559999999999</v>
       </c>
       <c r="Y628" s="10">
         <v>0</v>
@@ -87038,7 +87053,7 @@
         <v>46321</v>
       </c>
       <c r="G629" s="5">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H629" s="3" t="s">
         <v>47</v>
@@ -87053,16 +87068,16 @@
         <v>50</v>
       </c>
       <c r="L629" s="6">
-        <v>572</v>
+        <v>567</v>
       </c>
       <c r="M629" s="7">
-        <v>189652.55</v>
+        <v>187994.75</v>
       </c>
       <c r="N629" s="6">
         <v>1</v>
       </c>
       <c r="O629" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P629" s="8">
         <v>331.56</v>
@@ -87089,7 +87104,7 @@
         <v>46321</v>
       </c>
       <c r="X629" s="12">
-        <v>0.36319439999999997</v>
+        <v>0.35555560000000003</v>
       </c>
       <c r="Y629" s="10">
         <v>0</v>
@@ -87172,7 +87187,7 @@
         <v>46321</v>
       </c>
       <c r="G630" s="5">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H630" s="3" t="s">
         <v>47</v>
@@ -87187,16 +87202,16 @@
         <v>50</v>
       </c>
       <c r="L630" s="6">
-        <v>573</v>
+        <v>568</v>
       </c>
       <c r="M630" s="7">
-        <v>189984.11</v>
+        <v>188326.31</v>
       </c>
       <c r="N630" s="6">
         <v>1</v>
       </c>
       <c r="O630" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P630" s="8">
         <v>331.56</v>
@@ -87223,7 +87238,7 @@
         <v>46321</v>
       </c>
       <c r="X630" s="12">
-        <v>0.36319439999999997</v>
+        <v>0.35555560000000003</v>
       </c>
       <c r="Y630" s="10">
         <v>0</v>
@@ -87306,7 +87321,7 @@
         <v>46321</v>
       </c>
       <c r="G631" s="5">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="H631" s="3" t="s">
         <v>47</v>
@@ -87321,16 +87336,16 @@
         <v>50</v>
       </c>
       <c r="L631" s="6">
-        <v>574</v>
+        <v>569</v>
       </c>
       <c r="M631" s="7">
-        <v>190315.67</v>
+        <v>188657.87</v>
       </c>
       <c r="N631" s="6">
         <v>1</v>
       </c>
       <c r="O631" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P631" s="8">
         <v>331.56</v>
@@ -87357,7 +87372,7 @@
         <v>46321</v>
       </c>
       <c r="X631" s="12">
-        <v>0.36319439999999997</v>
+        <v>0.35555560000000003</v>
       </c>
       <c r="Y631" s="10">
         <v>0</v>
@@ -87440,7 +87455,7 @@
         <v>46321</v>
       </c>
       <c r="G632" s="5">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="H632" s="3" t="s">
         <v>47</v>
@@ -87455,16 +87470,16 @@
         <v>50</v>
       </c>
       <c r="L632" s="6">
-        <v>575</v>
+        <v>570</v>
       </c>
       <c r="M632" s="7">
-        <v>190647.23</v>
+        <v>188989.43</v>
       </c>
       <c r="N632" s="6">
         <v>1</v>
       </c>
       <c r="O632" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P632" s="8">
         <v>331.56</v>
@@ -87491,7 +87506,7 @@
         <v>46321</v>
       </c>
       <c r="X632" s="12">
-        <v>0.36319439999999997</v>
+        <v>0.35555560000000003</v>
       </c>
       <c r="Y632" s="10">
         <v>0</v>
@@ -87574,7 +87589,7 @@
         <v>46321</v>
       </c>
       <c r="G633" s="5">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="H633" s="3" t="s">
         <v>47</v>
@@ -87589,16 +87604,16 @@
         <v>50</v>
       </c>
       <c r="L633" s="6">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="M633" s="7">
-        <v>190978.79</v>
+        <v>189320.99</v>
       </c>
       <c r="N633" s="6">
         <v>1</v>
       </c>
       <c r="O633" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P633" s="8">
         <v>331.56</v>
@@ -87708,7 +87723,7 @@
         <v>46321</v>
       </c>
       <c r="G634" s="5">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="H634" s="3" t="s">
         <v>47</v>
@@ -87723,16 +87738,16 @@
         <v>50</v>
       </c>
       <c r="L634" s="6">
-        <v>577</v>
+        <v>572</v>
       </c>
       <c r="M634" s="7">
-        <v>191310.35</v>
+        <v>189652.55</v>
       </c>
       <c r="N634" s="6">
         <v>1</v>
       </c>
       <c r="O634" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P634" s="8">
         <v>331.56</v>
@@ -87842,7 +87857,7 @@
         <v>46321</v>
       </c>
       <c r="G635" s="5">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="H635" s="3" t="s">
         <v>47</v>
@@ -87857,16 +87872,16 @@
         <v>50</v>
       </c>
       <c r="L635" s="6">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="M635" s="7">
-        <v>191641.91</v>
+        <v>189984.11</v>
       </c>
       <c r="N635" s="6">
         <v>1</v>
       </c>
       <c r="O635" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P635" s="8">
         <v>331.56</v>
@@ -87976,7 +87991,7 @@
         <v>46321</v>
       </c>
       <c r="G636" s="5">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="H636" s="3" t="s">
         <v>47</v>
@@ -87991,16 +88006,16 @@
         <v>50</v>
       </c>
       <c r="L636" s="6">
-        <v>579</v>
+        <v>574</v>
       </c>
       <c r="M636" s="7">
-        <v>191973.47</v>
+        <v>190315.67</v>
       </c>
       <c r="N636" s="6">
         <v>1</v>
       </c>
       <c r="O636" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P636" s="8">
         <v>331.56</v>
@@ -88110,7 +88125,7 @@
         <v>46321</v>
       </c>
       <c r="G637" s="5">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="H637" s="3" t="s">
         <v>47</v>
@@ -88125,16 +88140,16 @@
         <v>50</v>
       </c>
       <c r="L637" s="6">
-        <v>580</v>
+        <v>575</v>
       </c>
       <c r="M637" s="7">
-        <v>192305.03</v>
+        <v>190647.23</v>
       </c>
       <c r="N637" s="6">
         <v>1</v>
       </c>
       <c r="O637" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P637" s="8">
         <v>331.56</v>
@@ -88244,7 +88259,7 @@
         <v>46321</v>
       </c>
       <c r="G638" s="5">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="H638" s="3" t="s">
         <v>47</v>
@@ -88259,16 +88274,16 @@
         <v>50</v>
       </c>
       <c r="L638" s="6">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="M638" s="7">
-        <v>192636.59</v>
+        <v>190978.79</v>
       </c>
       <c r="N638" s="6">
         <v>1</v>
       </c>
       <c r="O638" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P638" s="8">
         <v>331.56</v>
@@ -88295,7 +88310,7 @@
         <v>46321</v>
       </c>
       <c r="X638" s="12">
-        <v>0.36875000000000002</v>
+        <v>0.36319439999999997</v>
       </c>
       <c r="Y638" s="10">
         <v>0</v>
@@ -88378,7 +88393,7 @@
         <v>46321</v>
       </c>
       <c r="G639" s="5">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H639" s="3" t="s">
         <v>47</v>
@@ -88393,16 +88408,16 @@
         <v>50</v>
       </c>
       <c r="L639" s="6">
-        <v>582</v>
+        <v>577</v>
       </c>
       <c r="M639" s="7">
-        <v>192968.16</v>
+        <v>191310.35</v>
       </c>
       <c r="N639" s="6">
         <v>1</v>
       </c>
       <c r="O639" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P639" s="8">
         <v>331.56</v>
@@ -88429,7 +88444,7 @@
         <v>46321</v>
       </c>
       <c r="X639" s="12">
-        <v>0.4034722</v>
+        <v>0.36319439999999997</v>
       </c>
       <c r="Y639" s="10">
         <v>0</v>
@@ -88512,7 +88527,7 @@
         <v>46321</v>
       </c>
       <c r="G640" s="5">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="H640" s="3" t="s">
         <v>47</v>
@@ -88527,16 +88542,16 @@
         <v>50</v>
       </c>
       <c r="L640" s="6">
-        <v>583</v>
+        <v>578</v>
       </c>
       <c r="M640" s="7">
-        <v>193299.72</v>
+        <v>191641.91</v>
       </c>
       <c r="N640" s="6">
         <v>1</v>
       </c>
       <c r="O640" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P640" s="8">
         <v>331.56</v>
@@ -88563,7 +88578,7 @@
         <v>46321</v>
       </c>
       <c r="X640" s="12">
-        <v>0.4034722</v>
+        <v>0.36319439999999997</v>
       </c>
       <c r="Y640" s="10">
         <v>0</v>
@@ -88646,7 +88661,7 @@
         <v>46321</v>
       </c>
       <c r="G641" s="5">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="H641" s="3" t="s">
         <v>47</v>
@@ -88661,16 +88676,16 @@
         <v>50</v>
       </c>
       <c r="L641" s="6">
-        <v>584</v>
+        <v>579</v>
       </c>
       <c r="M641" s="7">
-        <v>193631.28</v>
+        <v>191973.47</v>
       </c>
       <c r="N641" s="6">
         <v>1</v>
       </c>
       <c r="O641" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P641" s="8">
         <v>331.56</v>
@@ -88697,7 +88712,7 @@
         <v>46321</v>
       </c>
       <c r="X641" s="12">
-        <v>0.4034722</v>
+        <v>0.36319439999999997</v>
       </c>
       <c r="Y641" s="10">
         <v>0</v>
@@ -88780,7 +88795,7 @@
         <v>46321</v>
       </c>
       <c r="G642" s="5">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="H642" s="3" t="s">
         <v>47</v>
@@ -88795,16 +88810,16 @@
         <v>50</v>
       </c>
       <c r="L642" s="6">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="M642" s="7">
-        <v>193962.84</v>
+        <v>192305.03</v>
       </c>
       <c r="N642" s="6">
         <v>1</v>
       </c>
       <c r="O642" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P642" s="8">
         <v>331.56</v>
@@ -88831,7 +88846,7 @@
         <v>46321</v>
       </c>
       <c r="X642" s="12">
-        <v>0.4034722</v>
+        <v>0.36319439999999997</v>
       </c>
       <c r="Y642" s="10">
         <v>0</v>
@@ -88914,7 +88929,7 @@
         <v>46321</v>
       </c>
       <c r="G643" s="5">
-        <v>104</v>
+        <v>79</v>
       </c>
       <c r="H643" s="3" t="s">
         <v>47</v>
@@ -88929,16 +88944,16 @@
         <v>50</v>
       </c>
       <c r="L643" s="6">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="M643" s="7">
-        <v>194294.39999999999</v>
+        <v>192636.59</v>
       </c>
       <c r="N643" s="6">
         <v>1</v>
       </c>
       <c r="O643" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P643" s="8">
         <v>331.56</v>
@@ -88965,7 +88980,7 @@
         <v>46321</v>
       </c>
       <c r="X643" s="12">
-        <v>0.4034722</v>
+        <v>0.36875000000000002</v>
       </c>
       <c r="Y643" s="10">
         <v>0</v>
@@ -89048,7 +89063,7 @@
         <v>46321</v>
       </c>
       <c r="G644" s="5">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H644" s="3" t="s">
         <v>47</v>
@@ -89063,16 +89078,16 @@
         <v>50</v>
       </c>
       <c r="L644" s="6">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="M644" s="7">
-        <v>194625.96</v>
+        <v>192968.16</v>
       </c>
       <c r="N644" s="6">
         <v>1</v>
       </c>
       <c r="O644" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P644" s="8">
         <v>331.56</v>
@@ -89182,7 +89197,7 @@
         <v>46321</v>
       </c>
       <c r="G645" s="5">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="H645" s="3" t="s">
         <v>47</v>
@@ -89197,16 +89212,16 @@
         <v>50</v>
       </c>
       <c r="L645" s="6">
-        <v>588</v>
+        <v>583</v>
       </c>
       <c r="M645" s="7">
-        <v>194957.52</v>
+        <v>193299.72</v>
       </c>
       <c r="N645" s="6">
         <v>1</v>
       </c>
       <c r="O645" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P645" s="8">
         <v>331.56</v>
@@ -89316,7 +89331,7 @@
         <v>46321</v>
       </c>
       <c r="G646" s="5">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H646" s="3" t="s">
         <v>47</v>
@@ -89331,16 +89346,16 @@
         <v>50</v>
       </c>
       <c r="L646" s="6">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="M646" s="7">
-        <v>195289.08</v>
+        <v>193631.28</v>
       </c>
       <c r="N646" s="6">
         <v>1</v>
       </c>
       <c r="O646" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P646" s="8">
         <v>331.56</v>
@@ -89450,7 +89465,7 @@
         <v>46321</v>
       </c>
       <c r="G647" s="5">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="H647" s="3" t="s">
         <v>47</v>
@@ -89465,16 +89480,16 @@
         <v>50</v>
       </c>
       <c r="L647" s="6">
-        <v>590</v>
+        <v>585</v>
       </c>
       <c r="M647" s="7">
-        <v>195620.64</v>
+        <v>193962.84</v>
       </c>
       <c r="N647" s="6">
         <v>1</v>
       </c>
       <c r="O647" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P647" s="8">
         <v>331.56</v>
@@ -89584,7 +89599,7 @@
         <v>46321</v>
       </c>
       <c r="G648" s="5">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H648" s="3" t="s">
         <v>47</v>
@@ -89599,16 +89614,16 @@
         <v>50</v>
       </c>
       <c r="L648" s="6">
-        <v>591</v>
+        <v>586</v>
       </c>
       <c r="M648" s="7">
-        <v>195952.2</v>
+        <v>194294.39999999999</v>
       </c>
       <c r="N648" s="6">
         <v>1</v>
       </c>
       <c r="O648" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P648" s="8">
         <v>331.56</v>
@@ -89718,7 +89733,7 @@
         <v>46321</v>
       </c>
       <c r="G649" s="5">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H649" s="3" t="s">
         <v>47</v>
@@ -89733,16 +89748,16 @@
         <v>50</v>
       </c>
       <c r="L649" s="6">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="M649" s="7">
-        <v>196283.76</v>
+        <v>194625.96</v>
       </c>
       <c r="N649" s="6">
         <v>1</v>
       </c>
       <c r="O649" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P649" s="8">
         <v>331.56</v>
@@ -89852,7 +89867,7 @@
         <v>46321</v>
       </c>
       <c r="G650" s="5">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="H650" s="3" t="s">
         <v>47</v>
@@ -89867,16 +89882,16 @@
         <v>50</v>
       </c>
       <c r="L650" s="6">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="M650" s="7">
-        <v>196615.32</v>
+        <v>194957.52</v>
       </c>
       <c r="N650" s="6">
         <v>1</v>
       </c>
       <c r="O650" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P650" s="8">
         <v>331.56</v>
@@ -89986,7 +90001,7 @@
         <v>46321</v>
       </c>
       <c r="G651" s="5">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="H651" s="3" t="s">
         <v>47</v>
@@ -90001,16 +90016,16 @@
         <v>50</v>
       </c>
       <c r="L651" s="6">
-        <v>594</v>
+        <v>589</v>
       </c>
       <c r="M651" s="7">
-        <v>196946.88</v>
+        <v>195289.08</v>
       </c>
       <c r="N651" s="6">
         <v>1</v>
       </c>
       <c r="O651" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P651" s="8">
         <v>331.56</v>
@@ -90120,7 +90135,7 @@
         <v>46321</v>
       </c>
       <c r="G652" s="5">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H652" s="3" t="s">
         <v>47</v>
@@ -90135,16 +90150,16 @@
         <v>50</v>
       </c>
       <c r="L652" s="6">
-        <v>595</v>
+        <v>590</v>
       </c>
       <c r="M652" s="7">
-        <v>197278.44</v>
+        <v>195620.64</v>
       </c>
       <c r="N652" s="6">
         <v>1</v>
       </c>
       <c r="O652" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P652" s="8">
         <v>331.56</v>
@@ -90254,7 +90269,7 @@
         <v>46321</v>
       </c>
       <c r="G653" s="5">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="H653" s="3" t="s">
         <v>47</v>
@@ -90269,16 +90284,16 @@
         <v>50</v>
       </c>
       <c r="L653" s="6">
-        <v>596</v>
+        <v>591</v>
       </c>
       <c r="M653" s="7">
-        <v>197610</v>
+        <v>195952.2</v>
       </c>
       <c r="N653" s="6">
         <v>1</v>
       </c>
       <c r="O653" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P653" s="8">
         <v>331.56</v>
@@ -90388,7 +90403,7 @@
         <v>46321</v>
       </c>
       <c r="G654" s="5">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H654" s="3" t="s">
         <v>47</v>
@@ -90403,16 +90418,16 @@
         <v>50</v>
       </c>
       <c r="L654" s="6">
-        <v>597</v>
+        <v>592</v>
       </c>
       <c r="M654" s="7">
-        <v>197941.56</v>
+        <v>196283.76</v>
       </c>
       <c r="N654" s="6">
         <v>1</v>
       </c>
       <c r="O654" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P654" s="8">
         <v>331.56</v>
@@ -90439,7 +90454,7 @@
         <v>46321</v>
       </c>
       <c r="X654" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.4034722</v>
       </c>
       <c r="Y654" s="10">
         <v>0</v>
@@ -90522,7 +90537,7 @@
         <v>46321</v>
       </c>
       <c r="G655" s="5">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H655" s="3" t="s">
         <v>47</v>
@@ -90537,16 +90552,16 @@
         <v>50</v>
       </c>
       <c r="L655" s="6">
-        <v>598</v>
+        <v>593</v>
       </c>
       <c r="M655" s="7">
-        <v>198273.12</v>
+        <v>196615.32</v>
       </c>
       <c r="N655" s="6">
         <v>1</v>
       </c>
       <c r="O655" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P655" s="8">
         <v>331.56</v>
@@ -90573,7 +90588,7 @@
         <v>46321</v>
       </c>
       <c r="X655" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.4034722</v>
       </c>
       <c r="Y655" s="10">
         <v>0</v>
@@ -90656,7 +90671,7 @@
         <v>46321</v>
       </c>
       <c r="G656" s="5">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H656" s="3" t="s">
         <v>47</v>
@@ -90671,16 +90686,16 @@
         <v>50</v>
       </c>
       <c r="L656" s="6">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="M656" s="7">
-        <v>198604.68</v>
+        <v>196946.88</v>
       </c>
       <c r="N656" s="6">
         <v>1</v>
       </c>
       <c r="O656" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P656" s="8">
         <v>331.56</v>
@@ -90707,7 +90722,7 @@
         <v>46321</v>
       </c>
       <c r="X656" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.4034722</v>
       </c>
       <c r="Y656" s="10">
         <v>0</v>
@@ -90790,7 +90805,7 @@
         <v>46321</v>
       </c>
       <c r="G657" s="5">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H657" s="3" t="s">
         <v>47</v>
@@ -90805,16 +90820,16 @@
         <v>50</v>
       </c>
       <c r="L657" s="6">
-        <v>600</v>
+        <v>595</v>
       </c>
       <c r="M657" s="7">
-        <v>198936.24</v>
+        <v>197278.44</v>
       </c>
       <c r="N657" s="6">
         <v>1</v>
       </c>
       <c r="O657" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P657" s="8">
         <v>331.56</v>
@@ -90841,7 +90856,7 @@
         <v>46321</v>
       </c>
       <c r="X657" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.4034722</v>
       </c>
       <c r="Y657" s="10">
         <v>0</v>
@@ -90924,7 +90939,7 @@
         <v>46321</v>
       </c>
       <c r="G658" s="5">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="H658" s="3" t="s">
         <v>47</v>
@@ -90939,16 +90954,16 @@
         <v>50</v>
       </c>
       <c r="L658" s="6">
-        <v>601</v>
+        <v>596</v>
       </c>
       <c r="M658" s="7">
-        <v>199267.8</v>
+        <v>197610</v>
       </c>
       <c r="N658" s="6">
         <v>1</v>
       </c>
       <c r="O658" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P658" s="8">
         <v>331.56</v>
@@ -90975,7 +90990,7 @@
         <v>46321</v>
       </c>
       <c r="X658" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.4034722</v>
       </c>
       <c r="Y658" s="10">
         <v>0</v>
@@ -91058,7 +91073,7 @@
         <v>46321</v>
       </c>
       <c r="G659" s="5">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H659" s="3" t="s">
         <v>47</v>
@@ -91073,16 +91088,16 @@
         <v>50</v>
       </c>
       <c r="L659" s="6">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="M659" s="7">
-        <v>199599.35999999999</v>
+        <v>197941.56</v>
       </c>
       <c r="N659" s="6">
         <v>1</v>
       </c>
       <c r="O659" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P659" s="8">
         <v>331.56</v>
@@ -91192,7 +91207,7 @@
         <v>46321</v>
       </c>
       <c r="G660" s="5">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H660" s="3" t="s">
         <v>47</v>
@@ -91207,16 +91222,16 @@
         <v>50</v>
       </c>
       <c r="L660" s="6">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="M660" s="7">
-        <v>199930.92</v>
+        <v>198273.12</v>
       </c>
       <c r="N660" s="6">
         <v>1</v>
       </c>
       <c r="O660" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P660" s="8">
         <v>331.56</v>
@@ -91326,7 +91341,7 @@
         <v>46321</v>
       </c>
       <c r="G661" s="5">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H661" s="3" t="s">
         <v>47</v>
@@ -91341,16 +91356,16 @@
         <v>50</v>
       </c>
       <c r="L661" s="6">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="M661" s="7">
-        <v>200262.48</v>
+        <v>198604.68</v>
       </c>
       <c r="N661" s="6">
         <v>1</v>
       </c>
       <c r="O661" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P661" s="8">
         <v>331.56</v>
@@ -91460,7 +91475,7 @@
         <v>46321</v>
       </c>
       <c r="G662" s="5">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H662" s="3" t="s">
         <v>47</v>
@@ -91475,16 +91490,16 @@
         <v>50</v>
       </c>
       <c r="L662" s="6">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="M662" s="7">
-        <v>200594.04</v>
+        <v>198936.24</v>
       </c>
       <c r="N662" s="6">
         <v>1</v>
       </c>
       <c r="O662" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P662" s="8">
         <v>331.56</v>
@@ -91594,7 +91609,7 @@
         <v>46321</v>
       </c>
       <c r="G663" s="5">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H663" s="3" t="s">
         <v>47</v>
@@ -91609,16 +91624,16 @@
         <v>50</v>
       </c>
       <c r="L663" s="6">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="M663" s="7">
-        <v>200925.61</v>
+        <v>199267.8</v>
       </c>
       <c r="N663" s="6">
         <v>1</v>
       </c>
       <c r="O663" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P663" s="8">
         <v>331.56</v>
@@ -91728,7 +91743,7 @@
         <v>46321</v>
       </c>
       <c r="G664" s="5">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H664" s="3" t="s">
         <v>47</v>
@@ -91743,16 +91758,16 @@
         <v>50</v>
       </c>
       <c r="L664" s="6">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="M664" s="7">
-        <v>201257.17</v>
+        <v>199599.35999999999</v>
       </c>
       <c r="N664" s="6">
         <v>1</v>
       </c>
       <c r="O664" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P664" s="8">
         <v>331.56</v>
@@ -91779,7 +91794,7 @@
         <v>46321</v>
       </c>
       <c r="X664" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y664" s="10">
         <v>0</v>
@@ -91862,7 +91877,7 @@
         <v>46321</v>
       </c>
       <c r="G665" s="5">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="H665" s="3" t="s">
         <v>47</v>
@@ -91877,16 +91892,16 @@
         <v>50</v>
       </c>
       <c r="L665" s="6">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="M665" s="7">
-        <v>201588.73</v>
+        <v>199930.92</v>
       </c>
       <c r="N665" s="6">
         <v>1</v>
       </c>
       <c r="O665" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P665" s="8">
         <v>331.56</v>
@@ -91913,7 +91928,7 @@
         <v>46321</v>
       </c>
       <c r="X665" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y665" s="10">
         <v>0</v>
@@ -91996,7 +92011,7 @@
         <v>46321</v>
       </c>
       <c r="G666" s="5">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="H666" s="3" t="s">
         <v>47</v>
@@ -92011,16 +92026,16 @@
         <v>50</v>
       </c>
       <c r="L666" s="6">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="M666" s="7">
-        <v>201920.29</v>
+        <v>200262.48</v>
       </c>
       <c r="N666" s="6">
         <v>1</v>
       </c>
       <c r="O666" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P666" s="8">
         <v>331.56</v>
@@ -92047,7 +92062,7 @@
         <v>46321</v>
       </c>
       <c r="X666" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y666" s="10">
         <v>0</v>
@@ -92130,7 +92145,7 @@
         <v>46321</v>
       </c>
       <c r="G667" s="5">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="H667" s="3" t="s">
         <v>47</v>
@@ -92145,16 +92160,16 @@
         <v>50</v>
       </c>
       <c r="L667" s="6">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="M667" s="7">
-        <v>202251.85</v>
+        <v>200594.04</v>
       </c>
       <c r="N667" s="6">
         <v>1</v>
       </c>
       <c r="O667" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P667" s="8">
         <v>331.56</v>
@@ -92181,7 +92196,7 @@
         <v>46321</v>
       </c>
       <c r="X667" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y667" s="10">
         <v>0</v>
@@ -92264,7 +92279,7 @@
         <v>46321</v>
       </c>
       <c r="G668" s="5">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="H668" s="3" t="s">
         <v>47</v>
@@ -92279,16 +92294,16 @@
         <v>50</v>
       </c>
       <c r="L668" s="6">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="M668" s="7">
-        <v>202583.41</v>
+        <v>200925.61</v>
       </c>
       <c r="N668" s="6">
         <v>1</v>
       </c>
       <c r="O668" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P668" s="8">
         <v>331.56</v>
@@ -92315,7 +92330,7 @@
         <v>46321</v>
       </c>
       <c r="X668" s="12">
-        <v>0.4243056</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y668" s="10">
         <v>0</v>
@@ -92398,7 +92413,7 @@
         <v>46321</v>
       </c>
       <c r="G669" s="5">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="H669" s="3" t="s">
         <v>47</v>
@@ -92413,16 +92428,16 @@
         <v>50</v>
       </c>
       <c r="L669" s="6">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="M669" s="7">
-        <v>202914.97</v>
+        <v>201257.17</v>
       </c>
       <c r="N669" s="6">
         <v>1</v>
       </c>
       <c r="O669" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P669" s="8">
         <v>331.56</v>
@@ -92449,7 +92464,7 @@
         <v>46321</v>
       </c>
       <c r="X669" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y669" s="10">
         <v>0</v>
@@ -92532,7 +92547,7 @@
         <v>46321</v>
       </c>
       <c r="G670" s="5">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="H670" s="3" t="s">
         <v>47</v>
@@ -92547,16 +92562,16 @@
         <v>50</v>
       </c>
       <c r="L670" s="6">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="M670" s="7">
-        <v>203246.53</v>
+        <v>201588.73</v>
       </c>
       <c r="N670" s="6">
         <v>1</v>
       </c>
       <c r="O670" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P670" s="8">
         <v>331.56</v>
@@ -92583,7 +92598,7 @@
         <v>46321</v>
       </c>
       <c r="X670" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y670" s="10">
         <v>0</v>
@@ -92666,7 +92681,7 @@
         <v>46321</v>
       </c>
       <c r="G671" s="5">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="H671" s="3" t="s">
         <v>47</v>
@@ -92681,16 +92696,16 @@
         <v>50</v>
       </c>
       <c r="L671" s="6">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="M671" s="7">
-        <v>203578.09</v>
+        <v>201920.29</v>
       </c>
       <c r="N671" s="6">
         <v>1</v>
       </c>
       <c r="O671" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P671" s="8">
         <v>331.56</v>
@@ -92717,7 +92732,7 @@
         <v>46321</v>
       </c>
       <c r="X671" s="12">
-        <v>0.43194440000000001</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y671" s="10">
         <v>0</v>
@@ -92800,7 +92815,7 @@
         <v>46321</v>
       </c>
       <c r="G672" s="5">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="H672" s="3" t="s">
         <v>47</v>
@@ -92815,16 +92830,16 @@
         <v>50</v>
       </c>
       <c r="L672" s="6">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="M672" s="7">
-        <v>203909.65</v>
+        <v>202251.85</v>
       </c>
       <c r="N672" s="6">
         <v>1</v>
       </c>
       <c r="O672" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P672" s="8">
         <v>331.56</v>
@@ -92851,7 +92866,7 @@
         <v>46321</v>
       </c>
       <c r="X672" s="12">
-        <v>0.43194440000000001</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y672" s="10">
         <v>0</v>
@@ -92934,7 +92949,7 @@
         <v>46321</v>
       </c>
       <c r="G673" s="5">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="H673" s="3" t="s">
         <v>47</v>
@@ -92949,16 +92964,16 @@
         <v>50</v>
       </c>
       <c r="L673" s="6">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="M673" s="7">
-        <v>204241.21</v>
+        <v>202583.41</v>
       </c>
       <c r="N673" s="6">
         <v>1</v>
       </c>
       <c r="O673" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P673" s="8">
         <v>331.56</v>
@@ -92985,7 +93000,7 @@
         <v>46321</v>
       </c>
       <c r="X673" s="12">
-        <v>0.43194440000000001</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y673" s="10">
         <v>0</v>
@@ -93068,7 +93083,7 @@
         <v>46321</v>
       </c>
       <c r="G674" s="5">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H674" s="3" t="s">
         <v>47</v>
@@ -93083,16 +93098,16 @@
         <v>50</v>
       </c>
       <c r="L674" s="6">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="M674" s="7">
-        <v>204572.77</v>
+        <v>202914.97</v>
       </c>
       <c r="N674" s="6">
         <v>1</v>
       </c>
       <c r="O674" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P674" s="8">
         <v>331.56</v>
@@ -93119,7 +93134,7 @@
         <v>46321</v>
       </c>
       <c r="X674" s="12">
-        <v>0.43194440000000001</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y674" s="10">
         <v>0</v>
@@ -93202,7 +93217,7 @@
         <v>46321</v>
       </c>
       <c r="G675" s="5">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="H675" s="3" t="s">
         <v>47</v>
@@ -93217,16 +93232,16 @@
         <v>50</v>
       </c>
       <c r="L675" s="6">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="M675" s="7">
-        <v>204904.33</v>
+        <v>203246.53</v>
       </c>
       <c r="N675" s="6">
         <v>1</v>
       </c>
       <c r="O675" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P675" s="8">
         <v>331.56</v>
@@ -93253,7 +93268,7 @@
         <v>46321</v>
       </c>
       <c r="X675" s="12">
-        <v>0.43194440000000001</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y675" s="10">
         <v>0</v>
@@ -93336,7 +93351,7 @@
         <v>46321</v>
       </c>
       <c r="G676" s="5">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="H676" s="3" t="s">
         <v>47</v>
@@ -93351,16 +93366,16 @@
         <v>50</v>
       </c>
       <c r="L676" s="6">
-        <v>619</v>
+        <v>614</v>
       </c>
       <c r="M676" s="7">
-        <v>205235.89</v>
+        <v>203578.09</v>
       </c>
       <c r="N676" s="6">
         <v>1</v>
       </c>
       <c r="O676" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P676" s="8">
         <v>331.56</v>
@@ -93387,7 +93402,7 @@
         <v>46321</v>
       </c>
       <c r="X676" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43194440000000001</v>
       </c>
       <c r="Y676" s="10">
         <v>0</v>
@@ -93470,7 +93485,7 @@
         <v>46321</v>
       </c>
       <c r="G677" s="5">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="H677" s="3" t="s">
         <v>47</v>
@@ -93485,16 +93500,16 @@
         <v>50</v>
       </c>
       <c r="L677" s="6">
-        <v>620</v>
+        <v>615</v>
       </c>
       <c r="M677" s="7">
-        <v>205567.45</v>
+        <v>203909.65</v>
       </c>
       <c r="N677" s="6">
         <v>1</v>
       </c>
       <c r="O677" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P677" s="8">
         <v>331.56</v>
@@ -93521,7 +93536,7 @@
         <v>46321</v>
       </c>
       <c r="X677" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43194440000000001</v>
       </c>
       <c r="Y677" s="10">
         <v>0</v>
@@ -93604,7 +93619,7 @@
         <v>46321</v>
       </c>
       <c r="G678" s="5">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="H678" s="3" t="s">
         <v>47</v>
@@ -93619,16 +93634,16 @@
         <v>50</v>
       </c>
       <c r="L678" s="6">
-        <v>621</v>
+        <v>616</v>
       </c>
       <c r="M678" s="7">
-        <v>205899.01</v>
+        <v>204241.21</v>
       </c>
       <c r="N678" s="6">
         <v>1</v>
       </c>
       <c r="O678" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P678" s="8">
         <v>331.56</v>
@@ -93655,7 +93670,7 @@
         <v>46321</v>
       </c>
       <c r="X678" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43194440000000001</v>
       </c>
       <c r="Y678" s="10">
         <v>0</v>
@@ -93738,7 +93753,7 @@
         <v>46321</v>
       </c>
       <c r="G679" s="5">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="H679" s="3" t="s">
         <v>47</v>
@@ -93753,16 +93768,16 @@
         <v>50</v>
       </c>
       <c r="L679" s="6">
-        <v>622</v>
+        <v>617</v>
       </c>
       <c r="M679" s="7">
-        <v>206230.57</v>
+        <v>204572.77</v>
       </c>
       <c r="N679" s="6">
         <v>1</v>
       </c>
       <c r="O679" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P679" s="8">
         <v>331.56</v>
@@ -93789,7 +93804,7 @@
         <v>46321</v>
       </c>
       <c r="X679" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43194440000000001</v>
       </c>
       <c r="Y679" s="10">
         <v>0</v>
@@ -93872,7 +93887,7 @@
         <v>46321</v>
       </c>
       <c r="G680" s="5">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="H680" s="3" t="s">
         <v>47</v>
@@ -93887,16 +93902,16 @@
         <v>50</v>
       </c>
       <c r="L680" s="6">
-        <v>623</v>
+        <v>618</v>
       </c>
       <c r="M680" s="7">
-        <v>206562.13</v>
+        <v>204904.33</v>
       </c>
       <c r="N680" s="6">
         <v>1</v>
       </c>
       <c r="O680" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P680" s="8">
         <v>331.56</v>
@@ -93923,7 +93938,7 @@
         <v>46321</v>
       </c>
       <c r="X680" s="12">
-        <v>0.43819439999999998</v>
+        <v>0.43194440000000001</v>
       </c>
       <c r="Y680" s="10">
         <v>0</v>
@@ -94006,7 +94021,7 @@
         <v>46321</v>
       </c>
       <c r="G681" s="5">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="H681" s="3" t="s">
         <v>47</v>
@@ -94021,16 +94036,16 @@
         <v>50</v>
       </c>
       <c r="L681" s="6">
-        <v>624</v>
+        <v>619</v>
       </c>
       <c r="M681" s="7">
-        <v>206893.69</v>
+        <v>205235.89</v>
       </c>
       <c r="N681" s="6">
         <v>1</v>
       </c>
       <c r="O681" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P681" s="8">
         <v>331.56</v>
@@ -94057,7 +94072,7 @@
         <v>46321</v>
       </c>
       <c r="X681" s="12">
-        <v>0.44652779999999997</v>
+        <v>0.43819439999999998</v>
       </c>
       <c r="Y681" s="10">
         <v>0</v>
@@ -94140,7 +94155,7 @@
         <v>46321</v>
       </c>
       <c r="G682" s="5">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H682" s="3" t="s">
         <v>47</v>
@@ -94155,16 +94170,16 @@
         <v>50</v>
       </c>
       <c r="L682" s="6">
-        <v>625</v>
+        <v>620</v>
       </c>
       <c r="M682" s="7">
-        <v>207225.25</v>
+        <v>205567.45</v>
       </c>
       <c r="N682" s="6">
         <v>1</v>
       </c>
       <c r="O682" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P682" s="8">
         <v>331.56</v>
@@ -94191,7 +94206,7 @@
         <v>46321</v>
       </c>
       <c r="X682" s="12">
-        <v>0.44652779999999997</v>
+        <v>0.43819439999999998</v>
       </c>
       <c r="Y682" s="10">
         <v>0</v>
@@ -94274,7 +94289,7 @@
         <v>46321</v>
       </c>
       <c r="G683" s="5">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="H683" s="3" t="s">
         <v>47</v>
@@ -94289,16 +94304,16 @@
         <v>50</v>
       </c>
       <c r="L683" s="6">
-        <v>626</v>
+        <v>621</v>
       </c>
       <c r="M683" s="7">
-        <v>207556.81</v>
+        <v>205899.01</v>
       </c>
       <c r="N683" s="6">
         <v>1</v>
       </c>
       <c r="O683" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P683" s="8">
         <v>331.56</v>
@@ -94325,7 +94340,7 @@
         <v>46321</v>
       </c>
       <c r="X683" s="12">
-        <v>0.44652779999999997</v>
+        <v>0.43819439999999998</v>
       </c>
       <c r="Y683" s="10">
         <v>0</v>
@@ -94408,7 +94423,7 @@
         <v>46321</v>
       </c>
       <c r="G684" s="5">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H684" s="3" t="s">
         <v>47</v>
@@ -94423,16 +94438,16 @@
         <v>50</v>
       </c>
       <c r="L684" s="6">
-        <v>627</v>
+        <v>622</v>
       </c>
       <c r="M684" s="7">
-        <v>207888.37</v>
+        <v>206230.57</v>
       </c>
       <c r="N684" s="6">
         <v>1</v>
       </c>
       <c r="O684" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P684" s="8">
         <v>331.56</v>
@@ -94459,7 +94474,7 @@
         <v>46321</v>
       </c>
       <c r="X684" s="12">
-        <v>0.44652779999999997</v>
+        <v>0.43819439999999998</v>
       </c>
       <c r="Y684" s="10">
         <v>0</v>
@@ -94542,7 +94557,7 @@
         <v>46321</v>
       </c>
       <c r="G685" s="5">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="H685" s="3" t="s">
         <v>47</v>
@@ -94557,16 +94572,16 @@
         <v>50</v>
       </c>
       <c r="L685" s="6">
-        <v>628</v>
+        <v>623</v>
       </c>
       <c r="M685" s="7">
-        <v>208219.93</v>
+        <v>206562.13</v>
       </c>
       <c r="N685" s="6">
         <v>1</v>
       </c>
       <c r="O685" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P685" s="8">
         <v>331.56</v>
@@ -94593,7 +94608,7 @@
         <v>46321</v>
       </c>
       <c r="X685" s="12">
-        <v>0.44652779999999997</v>
+        <v>0.43819439999999998</v>
       </c>
       <c r="Y685" s="10">
         <v>0</v>
@@ -94676,7 +94691,7 @@
         <v>46321</v>
       </c>
       <c r="G686" s="5">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="H686" s="3" t="s">
         <v>47</v>
@@ -94691,16 +94706,16 @@
         <v>50</v>
       </c>
       <c r="L686" s="6">
-        <v>629</v>
+        <v>624</v>
       </c>
       <c r="M686" s="7">
-        <v>208551.49</v>
+        <v>206893.69</v>
       </c>
       <c r="N686" s="6">
         <v>1</v>
       </c>
       <c r="O686" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P686" s="8">
         <v>331.56</v>
@@ -94810,7 +94825,7 @@
         <v>46321</v>
       </c>
       <c r="G687" s="5">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="H687" s="3" t="s">
         <v>47</v>
@@ -94825,16 +94840,16 @@
         <v>50</v>
       </c>
       <c r="L687" s="6">
-        <v>630</v>
+        <v>625</v>
       </c>
       <c r="M687" s="7">
-        <v>208883.05</v>
+        <v>207225.25</v>
       </c>
       <c r="N687" s="6">
         <v>1</v>
       </c>
       <c r="O687" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P687" s="8">
         <v>331.56</v>
@@ -94944,7 +94959,7 @@
         <v>46321</v>
       </c>
       <c r="G688" s="5">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="H688" s="3" t="s">
         <v>47</v>
@@ -94959,16 +94974,16 @@
         <v>50</v>
       </c>
       <c r="L688" s="6">
-        <v>631</v>
+        <v>626</v>
       </c>
       <c r="M688" s="7">
-        <v>209214.62</v>
+        <v>207556.81</v>
       </c>
       <c r="N688" s="6">
         <v>1</v>
       </c>
       <c r="O688" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P688" s="8">
         <v>331.56</v>
@@ -95078,7 +95093,7 @@
         <v>46321</v>
       </c>
       <c r="G689" s="5">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="H689" s="3" t="s">
         <v>47</v>
@@ -95093,16 +95108,16 @@
         <v>50</v>
       </c>
       <c r="L689" s="6">
-        <v>632</v>
+        <v>627</v>
       </c>
       <c r="M689" s="7">
-        <v>209546.18</v>
+        <v>207888.37</v>
       </c>
       <c r="N689" s="6">
         <v>1</v>
       </c>
       <c r="O689" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P689" s="8">
         <v>331.56</v>
@@ -95129,7 +95144,7 @@
         <v>46321</v>
       </c>
       <c r="X689" s="12">
-        <v>0.45208330000000002</v>
+        <v>0.44652779999999997</v>
       </c>
       <c r="Y689" s="10">
         <v>0</v>
@@ -95212,7 +95227,7 @@
         <v>46321</v>
       </c>
       <c r="G690" s="5">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="H690" s="3" t="s">
         <v>47</v>
@@ -95227,16 +95242,16 @@
         <v>50</v>
       </c>
       <c r="L690" s="6">
-        <v>633</v>
+        <v>628</v>
       </c>
       <c r="M690" s="7">
-        <v>209877.74</v>
+        <v>208219.93</v>
       </c>
       <c r="N690" s="6">
         <v>1</v>
       </c>
       <c r="O690" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P690" s="8">
         <v>331.56</v>
@@ -95263,7 +95278,7 @@
         <v>46321</v>
       </c>
       <c r="X690" s="12">
-        <v>0.45208330000000002</v>
+        <v>0.44652779999999997</v>
       </c>
       <c r="Y690" s="10">
         <v>0</v>
@@ -95346,7 +95361,7 @@
         <v>46321</v>
       </c>
       <c r="G691" s="5">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="H691" s="3" t="s">
         <v>47</v>
@@ -95361,16 +95376,16 @@
         <v>50</v>
       </c>
       <c r="L691" s="6">
-        <v>634</v>
+        <v>629</v>
       </c>
       <c r="M691" s="7">
-        <v>210209.3</v>
+        <v>208551.49</v>
       </c>
       <c r="N691" s="6">
         <v>1</v>
       </c>
       <c r="O691" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P691" s="8">
         <v>331.56</v>
@@ -95397,7 +95412,7 @@
         <v>46321</v>
       </c>
       <c r="X691" s="12">
-        <v>0.45208330000000002</v>
+        <v>0.44652779999999997</v>
       </c>
       <c r="Y691" s="10">
         <v>0</v>
@@ -95480,7 +95495,7 @@
         <v>46321</v>
       </c>
       <c r="G692" s="5">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="H692" s="3" t="s">
         <v>47</v>
@@ -95495,16 +95510,16 @@
         <v>50</v>
       </c>
       <c r="L692" s="6">
-        <v>635</v>
+        <v>630</v>
       </c>
       <c r="M692" s="7">
-        <v>210540.86</v>
+        <v>208883.05</v>
       </c>
       <c r="N692" s="6">
         <v>1</v>
       </c>
       <c r="O692" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P692" s="8">
         <v>331.56</v>
@@ -95531,7 +95546,7 @@
         <v>46321</v>
       </c>
       <c r="X692" s="12">
-        <v>0.45208330000000002</v>
+        <v>0.44652779999999997</v>
       </c>
       <c r="Y692" s="10">
         <v>0</v>
@@ -95614,7 +95629,7 @@
         <v>46321</v>
       </c>
       <c r="G693" s="5">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="H693" s="3" t="s">
         <v>47</v>
@@ -95629,16 +95644,16 @@
         <v>50</v>
       </c>
       <c r="L693" s="6">
-        <v>636</v>
+        <v>631</v>
       </c>
       <c r="M693" s="7">
-        <v>210872.42</v>
+        <v>209214.62</v>
       </c>
       <c r="N693" s="6">
         <v>1</v>
       </c>
       <c r="O693" s="3" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="P693" s="8">
         <v>331.56</v>
@@ -95665,7 +95680,7 @@
         <v>46321</v>
       </c>
       <c r="X693" s="12">
-        <v>0.45208330000000002</v>
+        <v>0.44652779999999997</v>
       </c>
       <c r="Y693" s="10">
         <v>0</v>
@@ -95726,6 +95741,676 @@
       </c>
       <c r="AR693" s="3" t="s">
         <v>755</v>
+      </c>
+    </row>
+    <row r="694" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A694" s="1">
+        <v>1</v>
+      </c>
+      <c r="B694" s="2">
+        <v>2</v>
+      </c>
+      <c r="C694" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D694" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E694" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F694" s="4">
+        <v>46321</v>
+      </c>
+      <c r="G694" s="5">
+        <v>151</v>
+      </c>
+      <c r="H694" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I694" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J694" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K694" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L694" s="6">
+        <v>632</v>
+      </c>
+      <c r="M694" s="7">
+        <v>209546.18</v>
+      </c>
+      <c r="N694" s="6">
+        <v>1</v>
+      </c>
+      <c r="O694" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="P694" s="8">
+        <v>331.56</v>
+      </c>
+      <c r="Q694" s="6">
+        <v>0</v>
+      </c>
+      <c r="R694" s="7">
+        <v>0</v>
+      </c>
+      <c r="S694" s="9">
+        <v>0</v>
+      </c>
+      <c r="T694" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U694" s="10">
+        <v>68570</v>
+      </c>
+      <c r="V694" s="11">
+        <v>11</v>
+      </c>
+      <c r="W694" s="4">
+        <v>46321</v>
+      </c>
+      <c r="X694" s="12">
+        <v>0.45208330000000002</v>
+      </c>
+      <c r="Y694" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB694" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG694" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI694" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="AJ694" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK694" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL694" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM694" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ694" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR694" s="3" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="695" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A695" s="1">
+        <v>1</v>
+      </c>
+      <c r="B695" s="2">
+        <v>2</v>
+      </c>
+      <c r="C695" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D695" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E695" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F695" s="4">
+        <v>46321</v>
+      </c>
+      <c r="G695" s="5">
+        <v>152</v>
+      </c>
+      <c r="H695" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I695" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J695" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K695" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L695" s="6">
+        <v>633</v>
+      </c>
+      <c r="M695" s="7">
+        <v>209877.74</v>
+      </c>
+      <c r="N695" s="6">
+        <v>1</v>
+      </c>
+      <c r="O695" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="P695" s="8">
+        <v>331.56</v>
+      </c>
+      <c r="Q695" s="6">
+        <v>0</v>
+      </c>
+      <c r="R695" s="7">
+        <v>0</v>
+      </c>
+      <c r="S695" s="9">
+        <v>0</v>
+      </c>
+      <c r="T695" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U695" s="10">
+        <v>68570</v>
+      </c>
+      <c r="V695" s="11">
+        <v>11</v>
+      </c>
+      <c r="W695" s="4">
+        <v>46321</v>
+      </c>
+      <c r="X695" s="12">
+        <v>0.45208330000000002</v>
+      </c>
+      <c r="Y695" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB695" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG695" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI695" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="AJ695" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK695" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL695" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM695" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ695" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR695" s="3" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="696" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A696" s="1">
+        <v>1</v>
+      </c>
+      <c r="B696" s="2">
+        <v>2</v>
+      </c>
+      <c r="C696" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D696" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E696" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F696" s="4">
+        <v>46321</v>
+      </c>
+      <c r="G696" s="5">
+        <v>153</v>
+      </c>
+      <c r="H696" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I696" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J696" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K696" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L696" s="6">
+        <v>634</v>
+      </c>
+      <c r="M696" s="7">
+        <v>210209.3</v>
+      </c>
+      <c r="N696" s="6">
+        <v>1</v>
+      </c>
+      <c r="O696" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="P696" s="8">
+        <v>331.56</v>
+      </c>
+      <c r="Q696" s="6">
+        <v>0</v>
+      </c>
+      <c r="R696" s="7">
+        <v>0</v>
+      </c>
+      <c r="S696" s="9">
+        <v>0</v>
+      </c>
+      <c r="T696" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U696" s="10">
+        <v>68570</v>
+      </c>
+      <c r="V696" s="11">
+        <v>11</v>
+      </c>
+      <c r="W696" s="4">
+        <v>46321</v>
+      </c>
+      <c r="X696" s="12">
+        <v>0.45208330000000002</v>
+      </c>
+      <c r="Y696" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB696" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG696" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI696" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="AJ696" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK696" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL696" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM696" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ696" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR696" s="3" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="697" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A697" s="1">
+        <v>1</v>
+      </c>
+      <c r="B697" s="2">
+        <v>2</v>
+      </c>
+      <c r="C697" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D697" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E697" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F697" s="4">
+        <v>46321</v>
+      </c>
+      <c r="G697" s="5">
+        <v>154</v>
+      </c>
+      <c r="H697" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I697" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J697" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K697" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L697" s="6">
+        <v>635</v>
+      </c>
+      <c r="M697" s="7">
+        <v>210540.86</v>
+      </c>
+      <c r="N697" s="6">
+        <v>1</v>
+      </c>
+      <c r="O697" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="P697" s="8">
+        <v>331.56</v>
+      </c>
+      <c r="Q697" s="6">
+        <v>0</v>
+      </c>
+      <c r="R697" s="7">
+        <v>0</v>
+      </c>
+      <c r="S697" s="9">
+        <v>0</v>
+      </c>
+      <c r="T697" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U697" s="10">
+        <v>68570</v>
+      </c>
+      <c r="V697" s="11">
+        <v>11</v>
+      </c>
+      <c r="W697" s="4">
+        <v>46321</v>
+      </c>
+      <c r="X697" s="12">
+        <v>0.45208330000000002</v>
+      </c>
+      <c r="Y697" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB697" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG697" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI697" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="AJ697" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK697" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL697" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM697" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ697" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR697" s="3" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="698" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A698" s="1">
+        <v>1</v>
+      </c>
+      <c r="B698" s="2">
+        <v>2</v>
+      </c>
+      <c r="C698" s="3" t="s">
+        <v>566</v>
+      </c>
+      <c r="D698" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E698" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F698" s="4">
+        <v>46321</v>
+      </c>
+      <c r="G698" s="5">
+        <v>155</v>
+      </c>
+      <c r="H698" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I698" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J698" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K698" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L698" s="6">
+        <v>636</v>
+      </c>
+      <c r="M698" s="7">
+        <v>210872.42</v>
+      </c>
+      <c r="N698" s="6">
+        <v>1</v>
+      </c>
+      <c r="O698" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="P698" s="8">
+        <v>331.56</v>
+      </c>
+      <c r="Q698" s="6">
+        <v>0</v>
+      </c>
+      <c r="R698" s="7">
+        <v>0</v>
+      </c>
+      <c r="S698" s="9">
+        <v>0</v>
+      </c>
+      <c r="T698" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U698" s="10">
+        <v>68570</v>
+      </c>
+      <c r="V698" s="11">
+        <v>11</v>
+      </c>
+      <c r="W698" s="4">
+        <v>46321</v>
+      </c>
+      <c r="X698" s="12">
+        <v>0.45208330000000002</v>
+      </c>
+      <c r="Y698" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB698" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG698" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI698" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="AJ698" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK698" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL698" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM698" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ698" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR698" s="3" t="s">
+        <v>760</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizacao automatica 30/10/2026 11:11:28,70
</commit_message>
<xml_diff>
--- a/movimentos_estoque_dados.xlsx
+++ b/movimentos_estoque_dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jucieli\Desktop\automacao_senior\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EAC686F8-8269-4E53-87EC-182ED6511EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E27113E-720C-4480-B2D5-2ACA36361771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6362" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6452" uniqueCount="420">
   <si>
     <t>Sel</t>
   </si>
@@ -1018,6 +1018,21 @@
     <t>1871600010919</t>
   </si>
   <si>
+    <t>1871600010920</t>
+  </si>
+  <si>
+    <t>1871600010921</t>
+  </si>
+  <si>
+    <t>1871600010922</t>
+  </si>
+  <si>
+    <t>1871600010923</t>
+  </si>
+  <si>
+    <t>1871600010924</t>
+  </si>
+  <si>
     <t>10059364</t>
   </si>
   <si>
@@ -1840,7 +1855,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR352"/>
+  <dimension ref="A1:AR357"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -38299,10 +38314,10 @@
         <v>2</v>
       </c>
       <c r="C273" s="3" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D273" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="E273" s="3" t="s">
         <v>46</v>
@@ -38311,7 +38326,7 @@
         <v>46325</v>
       </c>
       <c r="G273" s="5">
-        <v>1</v>
+        <v>146</v>
       </c>
       <c r="H273" s="3" t="s">
         <v>47</v>
@@ -38326,19 +38341,19 @@
         <v>50</v>
       </c>
       <c r="L273" s="6">
-        <v>1</v>
+        <v>765</v>
       </c>
       <c r="M273" s="7">
-        <v>189.55</v>
+        <v>233808.5</v>
       </c>
       <c r="N273" s="6">
         <v>1</v>
       </c>
       <c r="O273" s="3" t="s">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="P273" s="8">
-        <v>189.55</v>
+        <v>305.63</v>
       </c>
       <c r="Q273" s="6">
         <v>0</v>
@@ -38353,7 +38368,7 @@
         <v>52</v>
       </c>
       <c r="U273" s="10">
-        <v>68729</v>
+        <v>68735</v>
       </c>
       <c r="V273" s="11">
         <v>11</v>
@@ -38362,7 +38377,7 @@
         <v>46325</v>
       </c>
       <c r="X273" s="12">
-        <v>0.3958333</v>
+        <v>0.45902779999999999</v>
       </c>
       <c r="Y273" s="10">
         <v>0</v>
@@ -38395,7 +38410,7 @@
         <v>53</v>
       </c>
       <c r="AI273" s="3" t="s">
-        <v>54</v>
+        <v>251</v>
       </c>
       <c r="AJ273" s="3" t="s">
         <v>52</v>
@@ -38422,7 +38437,7 @@
         <v>53</v>
       </c>
       <c r="AR273" s="3" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="274" spans="1:44" x14ac:dyDescent="0.3">
@@ -38433,10 +38448,10 @@
         <v>2</v>
       </c>
       <c r="C274" s="3" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D274" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="E274" s="3" t="s">
         <v>46</v>
@@ -38445,7 +38460,7 @@
         <v>46325</v>
       </c>
       <c r="G274" s="5">
-        <v>2</v>
+        <v>147</v>
       </c>
       <c r="H274" s="3" t="s">
         <v>47</v>
@@ -38460,19 +38475,19 @@
         <v>50</v>
       </c>
       <c r="L274" s="6">
-        <v>2</v>
+        <v>766</v>
       </c>
       <c r="M274" s="7">
-        <v>379.1</v>
+        <v>234114.13</v>
       </c>
       <c r="N274" s="6">
         <v>1</v>
       </c>
       <c r="O274" s="3" t="s">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="P274" s="8">
-        <v>189.55</v>
+        <v>305.63</v>
       </c>
       <c r="Q274" s="6">
         <v>0</v>
@@ -38487,7 +38502,7 @@
         <v>52</v>
       </c>
       <c r="U274" s="10">
-        <v>68729</v>
+        <v>68735</v>
       </c>
       <c r="V274" s="11">
         <v>11</v>
@@ -38496,7 +38511,7 @@
         <v>46325</v>
       </c>
       <c r="X274" s="12">
-        <v>0.3958333</v>
+        <v>0.45902779999999999</v>
       </c>
       <c r="Y274" s="10">
         <v>0</v>
@@ -38529,7 +38544,7 @@
         <v>53</v>
       </c>
       <c r="AI274" s="3" t="s">
-        <v>54</v>
+        <v>251</v>
       </c>
       <c r="AJ274" s="3" t="s">
         <v>52</v>
@@ -38556,7 +38571,7 @@
         <v>53</v>
       </c>
       <c r="AR274" s="3" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="275" spans="1:44" x14ac:dyDescent="0.3">
@@ -38567,10 +38582,10 @@
         <v>2</v>
       </c>
       <c r="C275" s="3" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="E275" s="3" t="s">
         <v>46</v>
@@ -38579,7 +38594,7 @@
         <v>46325</v>
       </c>
       <c r="G275" s="5">
-        <v>3</v>
+        <v>148</v>
       </c>
       <c r="H275" s="3" t="s">
         <v>47</v>
@@ -38594,19 +38609,19 @@
         <v>50</v>
       </c>
       <c r="L275" s="6">
-        <v>3</v>
+        <v>767</v>
       </c>
       <c r="M275" s="7">
-        <v>568.65</v>
+        <v>234419.76</v>
       </c>
       <c r="N275" s="6">
         <v>1</v>
       </c>
       <c r="O275" s="3" t="s">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="P275" s="8">
-        <v>189.55</v>
+        <v>305.63</v>
       </c>
       <c r="Q275" s="6">
         <v>0</v>
@@ -38621,7 +38636,7 @@
         <v>52</v>
       </c>
       <c r="U275" s="10">
-        <v>68729</v>
+        <v>68735</v>
       </c>
       <c r="V275" s="11">
         <v>11</v>
@@ -38630,7 +38645,7 @@
         <v>46325</v>
       </c>
       <c r="X275" s="12">
-        <v>0.3958333</v>
+        <v>0.45902779999999999</v>
       </c>
       <c r="Y275" s="10">
         <v>0</v>
@@ -38663,7 +38678,7 @@
         <v>53</v>
       </c>
       <c r="AI275" s="3" t="s">
-        <v>54</v>
+        <v>251</v>
       </c>
       <c r="AJ275" s="3" t="s">
         <v>52</v>
@@ -38690,7 +38705,7 @@
         <v>53</v>
       </c>
       <c r="AR275" s="3" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="276" spans="1:44" x14ac:dyDescent="0.3">
@@ -38701,10 +38716,10 @@
         <v>2</v>
       </c>
       <c r="C276" s="3" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D276" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="E276" s="3" t="s">
         <v>46</v>
@@ -38713,7 +38728,7 @@
         <v>46325</v>
       </c>
       <c r="G276" s="5">
-        <v>4</v>
+        <v>149</v>
       </c>
       <c r="H276" s="3" t="s">
         <v>47</v>
@@ -38728,19 +38743,19 @@
         <v>50</v>
       </c>
       <c r="L276" s="6">
-        <v>4</v>
+        <v>768</v>
       </c>
       <c r="M276" s="7">
-        <v>758.2</v>
+        <v>234725.39</v>
       </c>
       <c r="N276" s="6">
         <v>1</v>
       </c>
       <c r="O276" s="3" t="s">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="P276" s="8">
-        <v>189.55</v>
+        <v>305.63</v>
       </c>
       <c r="Q276" s="6">
         <v>0</v>
@@ -38755,7 +38770,7 @@
         <v>52</v>
       </c>
       <c r="U276" s="10">
-        <v>68729</v>
+        <v>68735</v>
       </c>
       <c r="V276" s="11">
         <v>11</v>
@@ -38764,7 +38779,7 @@
         <v>46325</v>
       </c>
       <c r="X276" s="12">
-        <v>0.3958333</v>
+        <v>0.45902779999999999</v>
       </c>
       <c r="Y276" s="10">
         <v>0</v>
@@ -38797,7 +38812,7 @@
         <v>53</v>
       </c>
       <c r="AI276" s="3" t="s">
-        <v>54</v>
+        <v>251</v>
       </c>
       <c r="AJ276" s="3" t="s">
         <v>52</v>
@@ -38824,7 +38839,7 @@
         <v>53</v>
       </c>
       <c r="AR276" s="3" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="277" spans="1:44" x14ac:dyDescent="0.3">
@@ -38835,10 +38850,10 @@
         <v>2</v>
       </c>
       <c r="C277" s="3" t="s">
-        <v>332</v>
+        <v>249</v>
       </c>
       <c r="D277" s="3" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="E277" s="3" t="s">
         <v>46</v>
@@ -38847,7 +38862,7 @@
         <v>46325</v>
       </c>
       <c r="G277" s="5">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="H277" s="3" t="s">
         <v>47</v>
@@ -38862,19 +38877,19 @@
         <v>50</v>
       </c>
       <c r="L277" s="6">
-        <v>5</v>
+        <v>769</v>
       </c>
       <c r="M277" s="7">
-        <v>947.75</v>
+        <v>235031.02</v>
       </c>
       <c r="N277" s="6">
         <v>1</v>
       </c>
       <c r="O277" s="3" t="s">
-        <v>333</v>
+        <v>250</v>
       </c>
       <c r="P277" s="8">
-        <v>189.55</v>
+        <v>305.63</v>
       </c>
       <c r="Q277" s="6">
         <v>0</v>
@@ -38889,7 +38904,7 @@
         <v>52</v>
       </c>
       <c r="U277" s="10">
-        <v>68729</v>
+        <v>68735</v>
       </c>
       <c r="V277" s="11">
         <v>11</v>
@@ -38898,7 +38913,7 @@
         <v>46325</v>
       </c>
       <c r="X277" s="12">
-        <v>0.3958333</v>
+        <v>0.45902779999999999</v>
       </c>
       <c r="Y277" s="10">
         <v>0</v>
@@ -38931,7 +38946,7 @@
         <v>53</v>
       </c>
       <c r="AI277" s="3" t="s">
-        <v>54</v>
+        <v>251</v>
       </c>
       <c r="AJ277" s="3" t="s">
         <v>52</v>
@@ -38958,7 +38973,7 @@
         <v>53</v>
       </c>
       <c r="AR277" s="3" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="278" spans="1:44" x14ac:dyDescent="0.3">
@@ -38969,7 +38984,7 @@
         <v>2</v>
       </c>
       <c r="C278" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D278" s="3" t="s">
         <v>45</v>
@@ -38981,7 +38996,7 @@
         <v>46325</v>
       </c>
       <c r="G278" s="5">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H278" s="3" t="s">
         <v>47</v>
@@ -38996,16 +39011,16 @@
         <v>50</v>
       </c>
       <c r="L278" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M278" s="7">
-        <v>1137.3</v>
+        <v>189.55</v>
       </c>
       <c r="N278" s="6">
         <v>1</v>
       </c>
       <c r="O278" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P278" s="8">
         <v>189.55</v>
@@ -39103,7 +39118,7 @@
         <v>2</v>
       </c>
       <c r="C279" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D279" s="3" t="s">
         <v>45</v>
@@ -39115,7 +39130,7 @@
         <v>46325</v>
       </c>
       <c r="G279" s="5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H279" s="3" t="s">
         <v>47</v>
@@ -39130,16 +39145,16 @@
         <v>50</v>
       </c>
       <c r="L279" s="6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="M279" s="7">
-        <v>1326.85</v>
+        <v>379.1</v>
       </c>
       <c r="N279" s="6">
         <v>1</v>
       </c>
       <c r="O279" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P279" s="8">
         <v>189.55</v>
@@ -39237,7 +39252,7 @@
         <v>2</v>
       </c>
       <c r="C280" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D280" s="3" t="s">
         <v>45</v>
@@ -39249,7 +39264,7 @@
         <v>46325</v>
       </c>
       <c r="G280" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H280" s="3" t="s">
         <v>47</v>
@@ -39264,16 +39279,16 @@
         <v>50</v>
       </c>
       <c r="L280" s="6">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M280" s="7">
-        <v>1516.4</v>
+        <v>568.65</v>
       </c>
       <c r="N280" s="6">
         <v>1</v>
       </c>
       <c r="O280" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P280" s="8">
         <v>189.55</v>
@@ -39300,7 +39315,7 @@
         <v>46325</v>
       </c>
       <c r="X280" s="12">
-        <v>0.39652779999999999</v>
+        <v>0.3958333</v>
       </c>
       <c r="Y280" s="10">
         <v>0</v>
@@ -39371,7 +39386,7 @@
         <v>2</v>
       </c>
       <c r="C281" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D281" s="3" t="s">
         <v>45</v>
@@ -39383,7 +39398,7 @@
         <v>46325</v>
       </c>
       <c r="G281" s="5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H281" s="3" t="s">
         <v>47</v>
@@ -39398,16 +39413,16 @@
         <v>50</v>
       </c>
       <c r="L281" s="6">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="M281" s="7">
-        <v>1705.95</v>
+        <v>758.2</v>
       </c>
       <c r="N281" s="6">
         <v>1</v>
       </c>
       <c r="O281" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P281" s="8">
         <v>189.55</v>
@@ -39434,7 +39449,7 @@
         <v>46325</v>
       </c>
       <c r="X281" s="12">
-        <v>0.39652779999999999</v>
+        <v>0.3958333</v>
       </c>
       <c r="Y281" s="10">
         <v>0</v>
@@ -39505,7 +39520,7 @@
         <v>2</v>
       </c>
       <c r="C282" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D282" s="3" t="s">
         <v>45</v>
@@ -39517,7 +39532,7 @@
         <v>46325</v>
       </c>
       <c r="G282" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H282" s="3" t="s">
         <v>47</v>
@@ -39532,16 +39547,16 @@
         <v>50</v>
       </c>
       <c r="L282" s="6">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M282" s="7">
-        <v>1895.5</v>
+        <v>947.75</v>
       </c>
       <c r="N282" s="6">
         <v>1</v>
       </c>
       <c r="O282" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P282" s="8">
         <v>189.55</v>
@@ -39568,7 +39583,7 @@
         <v>46325</v>
       </c>
       <c r="X282" s="12">
-        <v>0.39652779999999999</v>
+        <v>0.3958333</v>
       </c>
       <c r="Y282" s="10">
         <v>0</v>
@@ -39639,7 +39654,7 @@
         <v>2</v>
       </c>
       <c r="C283" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D283" s="3" t="s">
         <v>45</v>
@@ -39651,7 +39666,7 @@
         <v>46325</v>
       </c>
       <c r="G283" s="5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H283" s="3" t="s">
         <v>47</v>
@@ -39666,16 +39681,16 @@
         <v>50</v>
       </c>
       <c r="L283" s="6">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M283" s="7">
-        <v>2085.0500000000002</v>
+        <v>1137.3</v>
       </c>
       <c r="N283" s="6">
         <v>1</v>
       </c>
       <c r="O283" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P283" s="8">
         <v>189.55</v>
@@ -39702,7 +39717,7 @@
         <v>46325</v>
       </c>
       <c r="X283" s="12">
-        <v>0.39652779999999999</v>
+        <v>0.3958333</v>
       </c>
       <c r="Y283" s="10">
         <v>0</v>
@@ -39773,7 +39788,7 @@
         <v>2</v>
       </c>
       <c r="C284" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D284" s="3" t="s">
         <v>45</v>
@@ -39785,7 +39800,7 @@
         <v>46325</v>
       </c>
       <c r="G284" s="5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H284" s="3" t="s">
         <v>47</v>
@@ -39800,16 +39815,16 @@
         <v>50</v>
       </c>
       <c r="L284" s="6">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="M284" s="7">
-        <v>2274.6</v>
+        <v>1326.85</v>
       </c>
       <c r="N284" s="6">
         <v>1</v>
       </c>
       <c r="O284" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P284" s="8">
         <v>189.55</v>
@@ -39836,7 +39851,7 @@
         <v>46325</v>
       </c>
       <c r="X284" s="12">
-        <v>0.39652779999999999</v>
+        <v>0.3958333</v>
       </c>
       <c r="Y284" s="10">
         <v>0</v>
@@ -39907,7 +39922,7 @@
         <v>2</v>
       </c>
       <c r="C285" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D285" s="3" t="s">
         <v>45</v>
@@ -39919,7 +39934,7 @@
         <v>46325</v>
       </c>
       <c r="G285" s="5">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H285" s="3" t="s">
         <v>47</v>
@@ -39934,16 +39949,16 @@
         <v>50</v>
       </c>
       <c r="L285" s="6">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="M285" s="7">
-        <v>2464.15</v>
+        <v>1516.4</v>
       </c>
       <c r="N285" s="6">
         <v>1</v>
       </c>
       <c r="O285" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P285" s="8">
         <v>189.55</v>
@@ -40041,7 +40056,7 @@
         <v>2</v>
       </c>
       <c r="C286" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D286" s="3" t="s">
         <v>45</v>
@@ -40053,7 +40068,7 @@
         <v>46325</v>
       </c>
       <c r="G286" s="5">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H286" s="3" t="s">
         <v>47</v>
@@ -40068,16 +40083,16 @@
         <v>50</v>
       </c>
       <c r="L286" s="6">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M286" s="7">
-        <v>2653.7</v>
+        <v>1705.95</v>
       </c>
       <c r="N286" s="6">
         <v>1</v>
       </c>
       <c r="O286" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P286" s="8">
         <v>189.55</v>
@@ -40175,7 +40190,7 @@
         <v>2</v>
       </c>
       <c r="C287" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D287" s="3" t="s">
         <v>45</v>
@@ -40187,7 +40202,7 @@
         <v>46325</v>
       </c>
       <c r="G287" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H287" s="3" t="s">
         <v>47</v>
@@ -40202,16 +40217,16 @@
         <v>50</v>
       </c>
       <c r="L287" s="6">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M287" s="7">
-        <v>2843.25</v>
+        <v>1895.5</v>
       </c>
       <c r="N287" s="6">
         <v>1</v>
       </c>
       <c r="O287" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P287" s="8">
         <v>189.55</v>
@@ -40309,7 +40324,7 @@
         <v>2</v>
       </c>
       <c r="C288" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D288" s="3" t="s">
         <v>45</v>
@@ -40321,7 +40336,7 @@
         <v>46325</v>
       </c>
       <c r="G288" s="5">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H288" s="3" t="s">
         <v>47</v>
@@ -40336,16 +40351,16 @@
         <v>50</v>
       </c>
       <c r="L288" s="6">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="M288" s="7">
-        <v>3032.8</v>
+        <v>2085.0500000000002</v>
       </c>
       <c r="N288" s="6">
         <v>1</v>
       </c>
       <c r="O288" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P288" s="8">
         <v>189.55</v>
@@ -40443,7 +40458,7 @@
         <v>2</v>
       </c>
       <c r="C289" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D289" s="3" t="s">
         <v>45</v>
@@ -40455,7 +40470,7 @@
         <v>46325</v>
       </c>
       <c r="G289" s="5">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H289" s="3" t="s">
         <v>47</v>
@@ -40470,16 +40485,16 @@
         <v>50</v>
       </c>
       <c r="L289" s="6">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="M289" s="7">
-        <v>3222.35</v>
+        <v>2274.6</v>
       </c>
       <c r="N289" s="6">
         <v>1</v>
       </c>
       <c r="O289" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P289" s="8">
         <v>189.55</v>
@@ -40577,7 +40592,7 @@
         <v>2</v>
       </c>
       <c r="C290" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D290" s="3" t="s">
         <v>45</v>
@@ -40589,7 +40604,7 @@
         <v>46325</v>
       </c>
       <c r="G290" s="5">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H290" s="3" t="s">
         <v>47</v>
@@ -40604,16 +40619,16 @@
         <v>50</v>
       </c>
       <c r="L290" s="6">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M290" s="7">
-        <v>3411.9</v>
+        <v>2464.15</v>
       </c>
       <c r="N290" s="6">
         <v>1</v>
       </c>
       <c r="O290" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P290" s="8">
         <v>189.55</v>
@@ -40711,7 +40726,7 @@
         <v>2</v>
       </c>
       <c r="C291" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D291" s="3" t="s">
         <v>45</v>
@@ -40723,7 +40738,7 @@
         <v>46325</v>
       </c>
       <c r="G291" s="5">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H291" s="3" t="s">
         <v>47</v>
@@ -40738,16 +40753,16 @@
         <v>50</v>
       </c>
       <c r="L291" s="6">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="M291" s="7">
-        <v>3601.45</v>
+        <v>2653.7</v>
       </c>
       <c r="N291" s="6">
         <v>1</v>
       </c>
       <c r="O291" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P291" s="8">
         <v>189.55</v>
@@ -40845,7 +40860,7 @@
         <v>2</v>
       </c>
       <c r="C292" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D292" s="3" t="s">
         <v>45</v>
@@ -40857,7 +40872,7 @@
         <v>46325</v>
       </c>
       <c r="G292" s="5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H292" s="3" t="s">
         <v>47</v>
@@ -40872,16 +40887,16 @@
         <v>50</v>
       </c>
       <c r="L292" s="6">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M292" s="7">
-        <v>3791</v>
+        <v>2843.25</v>
       </c>
       <c r="N292" s="6">
         <v>1</v>
       </c>
       <c r="O292" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P292" s="8">
         <v>189.55</v>
@@ -40979,7 +40994,7 @@
         <v>2</v>
       </c>
       <c r="C293" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D293" s="3" t="s">
         <v>45</v>
@@ -40991,7 +41006,7 @@
         <v>46325</v>
       </c>
       <c r="G293" s="5">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H293" s="3" t="s">
         <v>47</v>
@@ -41006,16 +41021,16 @@
         <v>50</v>
       </c>
       <c r="L293" s="6">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M293" s="7">
-        <v>3980.55</v>
+        <v>3032.8</v>
       </c>
       <c r="N293" s="6">
         <v>1</v>
       </c>
       <c r="O293" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P293" s="8">
         <v>189.55</v>
@@ -41042,7 +41057,7 @@
         <v>46325</v>
       </c>
       <c r="X293" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39652779999999999</v>
       </c>
       <c r="Y293" s="10">
         <v>0</v>
@@ -41113,7 +41128,7 @@
         <v>2</v>
       </c>
       <c r="C294" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D294" s="3" t="s">
         <v>45</v>
@@ -41125,7 +41140,7 @@
         <v>46325</v>
       </c>
       <c r="G294" s="5">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H294" s="3" t="s">
         <v>47</v>
@@ -41140,16 +41155,16 @@
         <v>50</v>
       </c>
       <c r="L294" s="6">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="M294" s="7">
-        <v>4170.1000000000004</v>
+        <v>3222.35</v>
       </c>
       <c r="N294" s="6">
         <v>1</v>
       </c>
       <c r="O294" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P294" s="8">
         <v>189.55</v>
@@ -41176,7 +41191,7 @@
         <v>46325</v>
       </c>
       <c r="X294" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39652779999999999</v>
       </c>
       <c r="Y294" s="10">
         <v>0</v>
@@ -41247,7 +41262,7 @@
         <v>2</v>
       </c>
       <c r="C295" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D295" s="3" t="s">
         <v>45</v>
@@ -41259,7 +41274,7 @@
         <v>46325</v>
       </c>
       <c r="G295" s="5">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H295" s="3" t="s">
         <v>47</v>
@@ -41274,16 +41289,16 @@
         <v>50</v>
       </c>
       <c r="L295" s="6">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="M295" s="7">
-        <v>4359.6499999999996</v>
+        <v>3411.9</v>
       </c>
       <c r="N295" s="6">
         <v>1</v>
       </c>
       <c r="O295" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P295" s="8">
         <v>189.55</v>
@@ -41310,7 +41325,7 @@
         <v>46325</v>
       </c>
       <c r="X295" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39652779999999999</v>
       </c>
       <c r="Y295" s="10">
         <v>0</v>
@@ -41381,7 +41396,7 @@
         <v>2</v>
       </c>
       <c r="C296" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D296" s="3" t="s">
         <v>45</v>
@@ -41393,7 +41408,7 @@
         <v>46325</v>
       </c>
       <c r="G296" s="5">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="H296" s="3" t="s">
         <v>47</v>
@@ -41408,16 +41423,16 @@
         <v>50</v>
       </c>
       <c r="L296" s="6">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="M296" s="7">
-        <v>4549.2</v>
+        <v>3601.45</v>
       </c>
       <c r="N296" s="6">
         <v>1</v>
       </c>
       <c r="O296" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P296" s="8">
         <v>189.55</v>
@@ -41444,7 +41459,7 @@
         <v>46325</v>
       </c>
       <c r="X296" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39652779999999999</v>
       </c>
       <c r="Y296" s="10">
         <v>0</v>
@@ -41515,7 +41530,7 @@
         <v>2</v>
       </c>
       <c r="C297" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D297" s="3" t="s">
         <v>45</v>
@@ -41527,7 +41542,7 @@
         <v>46325</v>
       </c>
       <c r="G297" s="5">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="H297" s="3" t="s">
         <v>47</v>
@@ -41542,16 +41557,16 @@
         <v>50</v>
       </c>
       <c r="L297" s="6">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M297" s="7">
-        <v>4738.75</v>
+        <v>3791</v>
       </c>
       <c r="N297" s="6">
         <v>1</v>
       </c>
       <c r="O297" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P297" s="8">
         <v>189.55</v>
@@ -41578,7 +41593,7 @@
         <v>46325</v>
       </c>
       <c r="X297" s="12">
-        <v>0.41041670000000002</v>
+        <v>0.39652779999999999</v>
       </c>
       <c r="Y297" s="10">
         <v>0</v>
@@ -41649,7 +41664,7 @@
         <v>2</v>
       </c>
       <c r="C298" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D298" s="3" t="s">
         <v>45</v>
@@ -41661,7 +41676,7 @@
         <v>46325</v>
       </c>
       <c r="G298" s="5">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="H298" s="3" t="s">
         <v>47</v>
@@ -41676,16 +41691,16 @@
         <v>50</v>
       </c>
       <c r="L298" s="6">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="M298" s="7">
-        <v>4928.3</v>
+        <v>3980.55</v>
       </c>
       <c r="N298" s="6">
         <v>1</v>
       </c>
       <c r="O298" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P298" s="8">
         <v>189.55</v>
@@ -41783,7 +41798,7 @@
         <v>2</v>
       </c>
       <c r="C299" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D299" s="3" t="s">
         <v>45</v>
@@ -41795,7 +41810,7 @@
         <v>46325</v>
       </c>
       <c r="G299" s="5">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H299" s="3" t="s">
         <v>47</v>
@@ -41810,16 +41825,16 @@
         <v>50</v>
       </c>
       <c r="L299" s="6">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="M299" s="7">
-        <v>5117.8500000000004</v>
+        <v>4170.1000000000004</v>
       </c>
       <c r="N299" s="6">
         <v>1</v>
       </c>
       <c r="O299" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P299" s="8">
         <v>189.55</v>
@@ -41917,7 +41932,7 @@
         <v>2</v>
       </c>
       <c r="C300" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D300" s="3" t="s">
         <v>45</v>
@@ -41929,7 +41944,7 @@
         <v>46325</v>
       </c>
       <c r="G300" s="5">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="H300" s="3" t="s">
         <v>47</v>
@@ -41944,16 +41959,16 @@
         <v>50</v>
       </c>
       <c r="L300" s="6">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M300" s="7">
-        <v>5307.4</v>
+        <v>4359.6499999999996</v>
       </c>
       <c r="N300" s="6">
         <v>1</v>
       </c>
       <c r="O300" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P300" s="8">
         <v>189.55</v>
@@ -42051,7 +42066,7 @@
         <v>2</v>
       </c>
       <c r="C301" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D301" s="3" t="s">
         <v>45</v>
@@ -42063,7 +42078,7 @@
         <v>46325</v>
       </c>
       <c r="G301" s="5">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H301" s="3" t="s">
         <v>47</v>
@@ -42078,16 +42093,16 @@
         <v>50</v>
       </c>
       <c r="L301" s="6">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="M301" s="7">
-        <v>5496.95</v>
+        <v>4549.2</v>
       </c>
       <c r="N301" s="6">
         <v>1</v>
       </c>
       <c r="O301" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P301" s="8">
         <v>189.55</v>
@@ -42185,7 +42200,7 @@
         <v>2</v>
       </c>
       <c r="C302" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D302" s="3" t="s">
         <v>45</v>
@@ -42197,7 +42212,7 @@
         <v>46325</v>
       </c>
       <c r="G302" s="5">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H302" s="3" t="s">
         <v>47</v>
@@ -42212,16 +42227,16 @@
         <v>50</v>
       </c>
       <c r="L302" s="6">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="M302" s="7">
-        <v>5686.5</v>
+        <v>4738.75</v>
       </c>
       <c r="N302" s="6">
         <v>1</v>
       </c>
       <c r="O302" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P302" s="8">
         <v>189.55</v>
@@ -42319,7 +42334,7 @@
         <v>2</v>
       </c>
       <c r="C303" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D303" s="3" t="s">
         <v>45</v>
@@ -42331,7 +42346,7 @@
         <v>46325</v>
       </c>
       <c r="G303" s="5">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H303" s="3" t="s">
         <v>47</v>
@@ -42346,16 +42361,16 @@
         <v>50</v>
       </c>
       <c r="L303" s="6">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="M303" s="7">
-        <v>5876.05</v>
+        <v>4928.3</v>
       </c>
       <c r="N303" s="6">
         <v>1</v>
       </c>
       <c r="O303" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P303" s="8">
         <v>189.55</v>
@@ -42453,7 +42468,7 @@
         <v>2</v>
       </c>
       <c r="C304" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D304" s="3" t="s">
         <v>45</v>
@@ -42465,7 +42480,7 @@
         <v>46325</v>
       </c>
       <c r="G304" s="5">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="H304" s="3" t="s">
         <v>47</v>
@@ -42480,16 +42495,16 @@
         <v>50</v>
       </c>
       <c r="L304" s="6">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="M304" s="7">
-        <v>6065.6</v>
+        <v>5117.8500000000004</v>
       </c>
       <c r="N304" s="6">
         <v>1</v>
       </c>
       <c r="O304" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P304" s="8">
         <v>189.55</v>
@@ -42587,7 +42602,7 @@
         <v>2</v>
       </c>
       <c r="C305" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D305" s="3" t="s">
         <v>45</v>
@@ -42599,7 +42614,7 @@
         <v>46325</v>
       </c>
       <c r="G305" s="5">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="H305" s="3" t="s">
         <v>47</v>
@@ -42614,16 +42629,16 @@
         <v>50</v>
       </c>
       <c r="L305" s="6">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M305" s="7">
-        <v>6255.15</v>
+        <v>5307.4</v>
       </c>
       <c r="N305" s="6">
         <v>1</v>
       </c>
       <c r="O305" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P305" s="8">
         <v>189.55</v>
@@ -42721,7 +42736,7 @@
         <v>2</v>
       </c>
       <c r="C306" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D306" s="3" t="s">
         <v>45</v>
@@ -42733,7 +42748,7 @@
         <v>46325</v>
       </c>
       <c r="G306" s="5">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="H306" s="3" t="s">
         <v>47</v>
@@ -42748,16 +42763,16 @@
         <v>50</v>
       </c>
       <c r="L306" s="6">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="M306" s="7">
-        <v>6444.7</v>
+        <v>5496.95</v>
       </c>
       <c r="N306" s="6">
         <v>1</v>
       </c>
       <c r="O306" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P306" s="8">
         <v>189.55</v>
@@ -42855,7 +42870,7 @@
         <v>2</v>
       </c>
       <c r="C307" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D307" s="3" t="s">
         <v>45</v>
@@ -42867,7 +42882,7 @@
         <v>46325</v>
       </c>
       <c r="G307" s="5">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H307" s="3" t="s">
         <v>47</v>
@@ -42882,16 +42897,16 @@
         <v>50</v>
       </c>
       <c r="L307" s="6">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="M307" s="7">
-        <v>6634.25</v>
+        <v>5686.5</v>
       </c>
       <c r="N307" s="6">
         <v>1</v>
       </c>
       <c r="O307" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P307" s="8">
         <v>189.55</v>
@@ -42989,7 +43004,7 @@
         <v>2</v>
       </c>
       <c r="C308" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D308" s="3" t="s">
         <v>45</v>
@@ -43001,7 +43016,7 @@
         <v>46325</v>
       </c>
       <c r="G308" s="5">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H308" s="3" t="s">
         <v>47</v>
@@ -43016,16 +43031,16 @@
         <v>50</v>
       </c>
       <c r="L308" s="6">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="M308" s="7">
-        <v>6823.8</v>
+        <v>5876.05</v>
       </c>
       <c r="N308" s="6">
         <v>1</v>
       </c>
       <c r="O308" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P308" s="8">
         <v>189.55</v>
@@ -43123,7 +43138,7 @@
         <v>2</v>
       </c>
       <c r="C309" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D309" s="3" t="s">
         <v>45</v>
@@ -43135,7 +43150,7 @@
         <v>46325</v>
       </c>
       <c r="G309" s="5">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="H309" s="3" t="s">
         <v>47</v>
@@ -43150,16 +43165,16 @@
         <v>50</v>
       </c>
       <c r="L309" s="6">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="M309" s="7">
-        <v>7013.35</v>
+        <v>6065.6</v>
       </c>
       <c r="N309" s="6">
         <v>1</v>
       </c>
       <c r="O309" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P309" s="8">
         <v>189.55</v>
@@ -43257,7 +43272,7 @@
         <v>2</v>
       </c>
       <c r="C310" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D310" s="3" t="s">
         <v>45</v>
@@ -43269,7 +43284,7 @@
         <v>46325</v>
       </c>
       <c r="G310" s="5">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="H310" s="3" t="s">
         <v>47</v>
@@ -43284,16 +43299,16 @@
         <v>50</v>
       </c>
       <c r="L310" s="6">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="M310" s="7">
-        <v>7202.9</v>
+        <v>6255.15</v>
       </c>
       <c r="N310" s="6">
         <v>1</v>
       </c>
       <c r="O310" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P310" s="8">
         <v>189.55</v>
@@ -43391,7 +43406,7 @@
         <v>2</v>
       </c>
       <c r="C311" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D311" s="3" t="s">
         <v>45</v>
@@ -43403,7 +43418,7 @@
         <v>46325</v>
       </c>
       <c r="G311" s="5">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H311" s="3" t="s">
         <v>47</v>
@@ -43418,16 +43433,16 @@
         <v>50</v>
       </c>
       <c r="L311" s="6">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="M311" s="7">
-        <v>7392.45</v>
+        <v>6444.7</v>
       </c>
       <c r="N311" s="6">
         <v>1</v>
       </c>
       <c r="O311" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P311" s="8">
         <v>189.55</v>
@@ -43525,7 +43540,7 @@
         <v>2</v>
       </c>
       <c r="C312" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D312" s="3" t="s">
         <v>45</v>
@@ -43537,7 +43552,7 @@
         <v>46325</v>
       </c>
       <c r="G312" s="5">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="H312" s="3" t="s">
         <v>47</v>
@@ -43552,16 +43567,16 @@
         <v>50</v>
       </c>
       <c r="L312" s="6">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="M312" s="7">
-        <v>7582</v>
+        <v>6634.25</v>
       </c>
       <c r="N312" s="6">
         <v>1</v>
       </c>
       <c r="O312" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P312" s="8">
         <v>189.55</v>
@@ -43659,7 +43674,7 @@
         <v>2</v>
       </c>
       <c r="C313" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D313" s="3" t="s">
         <v>45</v>
@@ -43671,7 +43686,7 @@
         <v>46325</v>
       </c>
       <c r="G313" s="5">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="H313" s="3" t="s">
         <v>47</v>
@@ -43686,16 +43701,16 @@
         <v>50</v>
       </c>
       <c r="L313" s="6">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="M313" s="7">
-        <v>7771.55</v>
+        <v>6823.8</v>
       </c>
       <c r="N313" s="6">
         <v>1</v>
       </c>
       <c r="O313" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P313" s="8">
         <v>189.55</v>
@@ -43793,7 +43808,7 @@
         <v>2</v>
       </c>
       <c r="C314" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D314" s="3" t="s">
         <v>45</v>
@@ -43805,7 +43820,7 @@
         <v>46325</v>
       </c>
       <c r="G314" s="5">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="H314" s="3" t="s">
         <v>47</v>
@@ -43820,16 +43835,16 @@
         <v>50</v>
       </c>
       <c r="L314" s="6">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="M314" s="7">
-        <v>7961.1</v>
+        <v>7013.35</v>
       </c>
       <c r="N314" s="6">
         <v>1</v>
       </c>
       <c r="O314" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P314" s="8">
         <v>189.55</v>
@@ -43927,7 +43942,7 @@
         <v>2</v>
       </c>
       <c r="C315" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D315" s="3" t="s">
         <v>45</v>
@@ -43939,7 +43954,7 @@
         <v>46325</v>
       </c>
       <c r="G315" s="5">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H315" s="3" t="s">
         <v>47</v>
@@ -43954,16 +43969,16 @@
         <v>50</v>
       </c>
       <c r="L315" s="6">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="M315" s="7">
-        <v>8150.65</v>
+        <v>7202.9</v>
       </c>
       <c r="N315" s="6">
         <v>1</v>
       </c>
       <c r="O315" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P315" s="8">
         <v>189.55</v>
@@ -43990,7 +44005,7 @@
         <v>46325</v>
       </c>
       <c r="X315" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y315" s="10">
         <v>0</v>
@@ -44061,7 +44076,7 @@
         <v>2</v>
       </c>
       <c r="C316" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D316" s="3" t="s">
         <v>45</v>
@@ -44073,7 +44088,7 @@
         <v>46325</v>
       </c>
       <c r="G316" s="5">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H316" s="3" t="s">
         <v>47</v>
@@ -44088,16 +44103,16 @@
         <v>50</v>
       </c>
       <c r="L316" s="6">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="M316" s="7">
-        <v>8340.2000000000007</v>
+        <v>7392.45</v>
       </c>
       <c r="N316" s="6">
         <v>1</v>
       </c>
       <c r="O316" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P316" s="8">
         <v>189.55</v>
@@ -44124,7 +44139,7 @@
         <v>46325</v>
       </c>
       <c r="X316" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y316" s="10">
         <v>0</v>
@@ -44195,7 +44210,7 @@
         <v>2</v>
       </c>
       <c r="C317" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D317" s="3" t="s">
         <v>45</v>
@@ -44207,7 +44222,7 @@
         <v>46325</v>
       </c>
       <c r="G317" s="5">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H317" s="3" t="s">
         <v>47</v>
@@ -44222,16 +44237,16 @@
         <v>50</v>
       </c>
       <c r="L317" s="6">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="M317" s="7">
-        <v>8529.75</v>
+        <v>7582</v>
       </c>
       <c r="N317" s="6">
         <v>1</v>
       </c>
       <c r="O317" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P317" s="8">
         <v>189.55</v>
@@ -44258,7 +44273,7 @@
         <v>46325</v>
       </c>
       <c r="X317" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y317" s="10">
         <v>0</v>
@@ -44329,7 +44344,7 @@
         <v>2</v>
       </c>
       <c r="C318" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D318" s="3" t="s">
         <v>45</v>
@@ -44341,7 +44356,7 @@
         <v>46325</v>
       </c>
       <c r="G318" s="5">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="H318" s="3" t="s">
         <v>47</v>
@@ -44356,16 +44371,16 @@
         <v>50</v>
       </c>
       <c r="L318" s="6">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="M318" s="7">
-        <v>8719.2999999999993</v>
+        <v>7771.55</v>
       </c>
       <c r="N318" s="6">
         <v>1</v>
       </c>
       <c r="O318" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P318" s="8">
         <v>189.55</v>
@@ -44392,7 +44407,7 @@
         <v>46325</v>
       </c>
       <c r="X318" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y318" s="10">
         <v>0</v>
@@ -44463,7 +44478,7 @@
         <v>2</v>
       </c>
       <c r="C319" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D319" s="3" t="s">
         <v>45</v>
@@ -44475,7 +44490,7 @@
         <v>46325</v>
       </c>
       <c r="G319" s="5">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="H319" s="3" t="s">
         <v>47</v>
@@ -44490,16 +44505,16 @@
         <v>50</v>
       </c>
       <c r="L319" s="6">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="M319" s="7">
-        <v>8908.85</v>
+        <v>7961.1</v>
       </c>
       <c r="N319" s="6">
         <v>1</v>
       </c>
       <c r="O319" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P319" s="8">
         <v>189.55</v>
@@ -44526,7 +44541,7 @@
         <v>46325</v>
       </c>
       <c r="X319" s="12">
-        <v>0.41736109999999998</v>
+        <v>0.41041670000000002</v>
       </c>
       <c r="Y319" s="10">
         <v>0</v>
@@ -44597,7 +44612,7 @@
         <v>2</v>
       </c>
       <c r="C320" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D320" s="3" t="s">
         <v>45</v>
@@ -44609,7 +44624,7 @@
         <v>46325</v>
       </c>
       <c r="G320" s="5">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="H320" s="3" t="s">
         <v>47</v>
@@ -44624,16 +44639,16 @@
         <v>50</v>
       </c>
       <c r="L320" s="6">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="M320" s="7">
-        <v>9098.4</v>
+        <v>8150.65</v>
       </c>
       <c r="N320" s="6">
         <v>1</v>
       </c>
       <c r="O320" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P320" s="8">
         <v>189.55</v>
@@ -44731,7 +44746,7 @@
         <v>2</v>
       </c>
       <c r="C321" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D321" s="3" t="s">
         <v>45</v>
@@ -44743,7 +44758,7 @@
         <v>46325</v>
       </c>
       <c r="G321" s="5">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="H321" s="3" t="s">
         <v>47</v>
@@ -44758,16 +44773,16 @@
         <v>50</v>
       </c>
       <c r="L321" s="6">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="M321" s="7">
-        <v>9287.9500000000007</v>
+        <v>8340.2000000000007</v>
       </c>
       <c r="N321" s="6">
         <v>1</v>
       </c>
       <c r="O321" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P321" s="8">
         <v>189.55</v>
@@ -44865,7 +44880,7 @@
         <v>2</v>
       </c>
       <c r="C322" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D322" s="3" t="s">
         <v>45</v>
@@ -44877,7 +44892,7 @@
         <v>46325</v>
       </c>
       <c r="G322" s="5">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="H322" s="3" t="s">
         <v>47</v>
@@ -44892,16 +44907,16 @@
         <v>50</v>
       </c>
       <c r="L322" s="6">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="M322" s="7">
-        <v>9477.5</v>
+        <v>8529.75</v>
       </c>
       <c r="N322" s="6">
         <v>1</v>
       </c>
       <c r="O322" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P322" s="8">
         <v>189.55</v>
@@ -44928,7 +44943,7 @@
         <v>46325</v>
       </c>
       <c r="X322" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y322" s="10">
         <v>0</v>
@@ -44999,7 +45014,7 @@
         <v>2</v>
       </c>
       <c r="C323" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D323" s="3" t="s">
         <v>45</v>
@@ -45011,7 +45026,7 @@
         <v>46325</v>
       </c>
       <c r="G323" s="5">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H323" s="3" t="s">
         <v>47</v>
@@ -45026,16 +45041,16 @@
         <v>50</v>
       </c>
       <c r="L323" s="6">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="M323" s="7">
-        <v>9667.0499999999993</v>
+        <v>8719.2999999999993</v>
       </c>
       <c r="N323" s="6">
         <v>1</v>
       </c>
       <c r="O323" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P323" s="8">
         <v>189.55</v>
@@ -45062,7 +45077,7 @@
         <v>46325</v>
       </c>
       <c r="X323" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y323" s="10">
         <v>0</v>
@@ -45133,7 +45148,7 @@
         <v>2</v>
       </c>
       <c r="C324" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D324" s="3" t="s">
         <v>45</v>
@@ -45145,7 +45160,7 @@
         <v>46325</v>
       </c>
       <c r="G324" s="5">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="H324" s="3" t="s">
         <v>47</v>
@@ -45160,16 +45175,16 @@
         <v>50</v>
       </c>
       <c r="L324" s="6">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="M324" s="7">
-        <v>9856.6</v>
+        <v>8908.85</v>
       </c>
       <c r="N324" s="6">
         <v>1</v>
       </c>
       <c r="O324" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P324" s="8">
         <v>189.55</v>
@@ -45196,7 +45211,7 @@
         <v>46325</v>
       </c>
       <c r="X324" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y324" s="10">
         <v>0</v>
@@ -45267,7 +45282,7 @@
         <v>2</v>
       </c>
       <c r="C325" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D325" s="3" t="s">
         <v>45</v>
@@ -45279,7 +45294,7 @@
         <v>46325</v>
       </c>
       <c r="G325" s="5">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H325" s="3" t="s">
         <v>47</v>
@@ -45294,16 +45309,16 @@
         <v>50</v>
       </c>
       <c r="L325" s="6">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="M325" s="7">
-        <v>10046.15</v>
+        <v>9098.4</v>
       </c>
       <c r="N325" s="6">
         <v>1</v>
       </c>
       <c r="O325" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P325" s="8">
         <v>189.55</v>
@@ -45330,7 +45345,7 @@
         <v>46325</v>
       </c>
       <c r="X325" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y325" s="10">
         <v>0</v>
@@ -45401,7 +45416,7 @@
         <v>2</v>
       </c>
       <c r="C326" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D326" s="3" t="s">
         <v>45</v>
@@ -45413,7 +45428,7 @@
         <v>46325</v>
       </c>
       <c r="G326" s="5">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="H326" s="3" t="s">
         <v>47</v>
@@ -45428,16 +45443,16 @@
         <v>50</v>
       </c>
       <c r="L326" s="6">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M326" s="7">
-        <v>10235.700000000001</v>
+        <v>9287.9500000000007</v>
       </c>
       <c r="N326" s="6">
         <v>1</v>
       </c>
       <c r="O326" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P326" s="8">
         <v>189.55</v>
@@ -45464,7 +45479,7 @@
         <v>46325</v>
       </c>
       <c r="X326" s="12">
-        <v>0.4243056</v>
+        <v>0.41736109999999998</v>
       </c>
       <c r="Y326" s="10">
         <v>0</v>
@@ -45535,7 +45550,7 @@
         <v>2</v>
       </c>
       <c r="C327" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D327" s="3" t="s">
         <v>45</v>
@@ -45547,7 +45562,7 @@
         <v>46325</v>
       </c>
       <c r="G327" s="5">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="H327" s="3" t="s">
         <v>47</v>
@@ -45562,16 +45577,16 @@
         <v>50</v>
       </c>
       <c r="L327" s="6">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="M327" s="7">
-        <v>10425.25</v>
+        <v>9477.5</v>
       </c>
       <c r="N327" s="6">
         <v>1</v>
       </c>
       <c r="O327" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P327" s="8">
         <v>189.55</v>
@@ -45669,7 +45684,7 @@
         <v>2</v>
       </c>
       <c r="C328" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D328" s="3" t="s">
         <v>45</v>
@@ -45681,7 +45696,7 @@
         <v>46325</v>
       </c>
       <c r="G328" s="5">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H328" s="3" t="s">
         <v>47</v>
@@ -45696,16 +45711,16 @@
         <v>50</v>
       </c>
       <c r="L328" s="6">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="M328" s="7">
-        <v>10614.8</v>
+        <v>9667.0499999999993</v>
       </c>
       <c r="N328" s="6">
         <v>1</v>
       </c>
       <c r="O328" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P328" s="8">
         <v>189.55</v>
@@ -45803,7 +45818,7 @@
         <v>2</v>
       </c>
       <c r="C329" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D329" s="3" t="s">
         <v>45</v>
@@ -45815,7 +45830,7 @@
         <v>46325</v>
       </c>
       <c r="G329" s="5">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="H329" s="3" t="s">
         <v>47</v>
@@ -45830,16 +45845,16 @@
         <v>50</v>
       </c>
       <c r="L329" s="6">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M329" s="7">
-        <v>10804.35</v>
+        <v>9856.6</v>
       </c>
       <c r="N329" s="6">
         <v>1</v>
       </c>
       <c r="O329" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P329" s="8">
         <v>189.55</v>
@@ -45937,7 +45952,7 @@
         <v>2</v>
       </c>
       <c r="C330" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D330" s="3" t="s">
         <v>45</v>
@@ -45949,7 +45964,7 @@
         <v>46325</v>
       </c>
       <c r="G330" s="5">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H330" s="3" t="s">
         <v>47</v>
@@ -45964,16 +45979,16 @@
         <v>50</v>
       </c>
       <c r="L330" s="6">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="M330" s="7">
-        <v>10993.9</v>
+        <v>10046.15</v>
       </c>
       <c r="N330" s="6">
         <v>1</v>
       </c>
       <c r="O330" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P330" s="8">
         <v>189.55</v>
@@ -46071,7 +46086,7 @@
         <v>2</v>
       </c>
       <c r="C331" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D331" s="3" t="s">
         <v>45</v>
@@ -46083,7 +46098,7 @@
         <v>46325</v>
       </c>
       <c r="G331" s="5">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H331" s="3" t="s">
         <v>47</v>
@@ -46098,16 +46113,16 @@
         <v>50</v>
       </c>
       <c r="L331" s="6">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="M331" s="7">
-        <v>11183.45</v>
+        <v>10235.700000000001</v>
       </c>
       <c r="N331" s="6">
         <v>1</v>
       </c>
       <c r="O331" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P331" s="8">
         <v>189.55</v>
@@ -46205,7 +46220,7 @@
         <v>2</v>
       </c>
       <c r="C332" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D332" s="3" t="s">
         <v>45</v>
@@ -46217,7 +46232,7 @@
         <v>46325</v>
       </c>
       <c r="G332" s="5">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="H332" s="3" t="s">
         <v>47</v>
@@ -46232,16 +46247,16 @@
         <v>50</v>
       </c>
       <c r="L332" s="6">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="M332" s="7">
-        <v>11373</v>
+        <v>10425.25</v>
       </c>
       <c r="N332" s="6">
         <v>1</v>
       </c>
       <c r="O332" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="P332" s="8">
         <v>189.55</v>
@@ -46339,10 +46354,10 @@
         <v>2</v>
       </c>
       <c r="C333" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D333" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E333" s="3" t="s">
         <v>46</v>
@@ -46351,7 +46366,7 @@
         <v>46325</v>
       </c>
       <c r="G333" s="5">
-        <v>2</v>
+        <v>57</v>
       </c>
       <c r="H333" s="3" t="s">
         <v>47</v>
@@ -46366,19 +46381,19 @@
         <v>50</v>
       </c>
       <c r="L333" s="6">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="M333" s="7">
-        <v>10149.84</v>
+        <v>10614.8</v>
       </c>
       <c r="N333" s="6">
         <v>1</v>
       </c>
       <c r="O333" s="3" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="P333" s="8">
-        <v>187.96</v>
+        <v>189.55</v>
       </c>
       <c r="Q333" s="6">
         <v>0</v>
@@ -46393,7 +46408,7 @@
         <v>52</v>
       </c>
       <c r="U333" s="10">
-        <v>68776</v>
+        <v>68729</v>
       </c>
       <c r="V333" s="11">
         <v>11</v>
@@ -46402,7 +46417,7 @@
         <v>46325</v>
       </c>
       <c r="X333" s="12">
-        <v>0.37638890000000003</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y333" s="10">
         <v>0</v>
@@ -46462,7 +46477,7 @@
         <v>53</v>
       </c>
       <c r="AR333" s="3" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="334" spans="1:44" x14ac:dyDescent="0.3">
@@ -46473,10 +46488,10 @@
         <v>2</v>
       </c>
       <c r="C334" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D334" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E334" s="3" t="s">
         <v>46</v>
@@ -46485,7 +46500,7 @@
         <v>46325</v>
       </c>
       <c r="G334" s="5">
-        <v>3</v>
+        <v>58</v>
       </c>
       <c r="H334" s="3" t="s">
         <v>47</v>
@@ -46500,19 +46515,19 @@
         <v>50</v>
       </c>
       <c r="L334" s="6">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="M334" s="7">
-        <v>10337.799999999999</v>
+        <v>10804.35</v>
       </c>
       <c r="N334" s="6">
         <v>1</v>
       </c>
       <c r="O334" s="3" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="P334" s="8">
-        <v>187.96</v>
+        <v>189.55</v>
       </c>
       <c r="Q334" s="6">
         <v>0</v>
@@ -46527,7 +46542,7 @@
         <v>52</v>
       </c>
       <c r="U334" s="10">
-        <v>68776</v>
+        <v>68729</v>
       </c>
       <c r="V334" s="11">
         <v>11</v>
@@ -46536,7 +46551,7 @@
         <v>46325</v>
       </c>
       <c r="X334" s="12">
-        <v>0.37638890000000003</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y334" s="10">
         <v>0</v>
@@ -46596,7 +46611,7 @@
         <v>53</v>
       </c>
       <c r="AR334" s="3" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="335" spans="1:44" x14ac:dyDescent="0.3">
@@ -46607,10 +46622,10 @@
         <v>2</v>
       </c>
       <c r="C335" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D335" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E335" s="3" t="s">
         <v>46</v>
@@ -46619,7 +46634,7 @@
         <v>46325</v>
       </c>
       <c r="G335" s="5">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="H335" s="3" t="s">
         <v>47</v>
@@ -46634,19 +46649,19 @@
         <v>50</v>
       </c>
       <c r="L335" s="6">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M335" s="7">
-        <v>10525.76</v>
+        <v>10993.9</v>
       </c>
       <c r="N335" s="6">
         <v>1</v>
       </c>
       <c r="O335" s="3" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="P335" s="8">
-        <v>187.96</v>
+        <v>189.55</v>
       </c>
       <c r="Q335" s="6">
         <v>0</v>
@@ -46661,7 +46676,7 @@
         <v>52</v>
       </c>
       <c r="U335" s="10">
-        <v>68776</v>
+        <v>68729</v>
       </c>
       <c r="V335" s="11">
         <v>11</v>
@@ -46670,7 +46685,7 @@
         <v>46325</v>
       </c>
       <c r="X335" s="12">
-        <v>0.37638890000000003</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y335" s="10">
         <v>0</v>
@@ -46730,7 +46745,7 @@
         <v>53</v>
       </c>
       <c r="AR335" s="3" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="336" spans="1:44" x14ac:dyDescent="0.3">
@@ -46741,10 +46756,10 @@
         <v>2</v>
       </c>
       <c r="C336" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D336" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E336" s="3" t="s">
         <v>46</v>
@@ -46753,7 +46768,7 @@
         <v>46325</v>
       </c>
       <c r="G336" s="5">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="H336" s="3" t="s">
         <v>47</v>
@@ -46768,19 +46783,19 @@
         <v>50</v>
       </c>
       <c r="L336" s="6">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M336" s="7">
-        <v>10713.72</v>
+        <v>11183.45</v>
       </c>
       <c r="N336" s="6">
         <v>1</v>
       </c>
       <c r="O336" s="3" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="P336" s="8">
-        <v>187.96</v>
+        <v>189.55</v>
       </c>
       <c r="Q336" s="6">
         <v>0</v>
@@ -46795,7 +46810,7 @@
         <v>52</v>
       </c>
       <c r="U336" s="10">
-        <v>68776</v>
+        <v>68729</v>
       </c>
       <c r="V336" s="11">
         <v>11</v>
@@ -46804,7 +46819,7 @@
         <v>46325</v>
       </c>
       <c r="X336" s="12">
-        <v>0.37638890000000003</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y336" s="10">
         <v>0</v>
@@ -46864,7 +46879,7 @@
         <v>53</v>
       </c>
       <c r="AR336" s="3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="337" spans="1:44" x14ac:dyDescent="0.3">
@@ -46875,10 +46890,10 @@
         <v>2</v>
       </c>
       <c r="C337" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D337" s="3" t="s">
-        <v>89</v>
+        <v>45</v>
       </c>
       <c r="E337" s="3" t="s">
         <v>46</v>
@@ -46887,7 +46902,7 @@
         <v>46325</v>
       </c>
       <c r="G337" s="5">
-        <v>6</v>
+        <v>61</v>
       </c>
       <c r="H337" s="3" t="s">
         <v>47</v>
@@ -46902,19 +46917,19 @@
         <v>50</v>
       </c>
       <c r="L337" s="6">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="M337" s="7">
-        <v>10901.68</v>
+        <v>11373</v>
       </c>
       <c r="N337" s="6">
         <v>1</v>
       </c>
       <c r="O337" s="3" t="s">
-        <v>394</v>
+        <v>338</v>
       </c>
       <c r="P337" s="8">
-        <v>187.96</v>
+        <v>189.55</v>
       </c>
       <c r="Q337" s="6">
         <v>0</v>
@@ -46929,7 +46944,7 @@
         <v>52</v>
       </c>
       <c r="U337" s="10">
-        <v>68776</v>
+        <v>68729</v>
       </c>
       <c r="V337" s="11">
         <v>11</v>
@@ -46938,7 +46953,7 @@
         <v>46325</v>
       </c>
       <c r="X337" s="12">
-        <v>0.37638890000000003</v>
+        <v>0.4243056</v>
       </c>
       <c r="Y337" s="10">
         <v>0</v>
@@ -46998,7 +47013,7 @@
         <v>53</v>
       </c>
       <c r="AR337" s="3" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="338" spans="1:44" x14ac:dyDescent="0.3">
@@ -47009,7 +47024,7 @@
         <v>2</v>
       </c>
       <c r="C338" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D338" s="3" t="s">
         <v>89</v>
@@ -47021,7 +47036,7 @@
         <v>46325</v>
       </c>
       <c r="G338" s="5">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="H338" s="3" t="s">
         <v>47</v>
@@ -47036,16 +47051,16 @@
         <v>50</v>
       </c>
       <c r="L338" s="6">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="M338" s="7">
-        <v>11089.64</v>
+        <v>10149.84</v>
       </c>
       <c r="N338" s="6">
         <v>1</v>
       </c>
       <c r="O338" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P338" s="8">
         <v>187.96</v>
@@ -47143,7 +47158,7 @@
         <v>2</v>
       </c>
       <c r="C339" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D339" s="3" t="s">
         <v>89</v>
@@ -47155,7 +47170,7 @@
         <v>46325</v>
       </c>
       <c r="G339" s="5">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H339" s="3" t="s">
         <v>47</v>
@@ -47170,16 +47185,16 @@
         <v>50</v>
       </c>
       <c r="L339" s="6">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="M339" s="7">
-        <v>11277.6</v>
+        <v>10337.799999999999</v>
       </c>
       <c r="N339" s="6">
         <v>1</v>
       </c>
       <c r="O339" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P339" s="8">
         <v>187.96</v>
@@ -47277,7 +47292,7 @@
         <v>2</v>
       </c>
       <c r="C340" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D340" s="3" t="s">
         <v>89</v>
@@ -47289,7 +47304,7 @@
         <v>46325</v>
       </c>
       <c r="G340" s="5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H340" s="3" t="s">
         <v>47</v>
@@ -47304,16 +47319,16 @@
         <v>50</v>
       </c>
       <c r="L340" s="6">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M340" s="7">
-        <v>11465.56</v>
+        <v>10525.76</v>
       </c>
       <c r="N340" s="6">
         <v>1</v>
       </c>
       <c r="O340" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P340" s="8">
         <v>187.96</v>
@@ -47411,7 +47426,7 @@
         <v>2</v>
       </c>
       <c r="C341" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D341" s="3" t="s">
         <v>89</v>
@@ -47423,7 +47438,7 @@
         <v>46325</v>
       </c>
       <c r="G341" s="5">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H341" s="3" t="s">
         <v>47</v>
@@ -47438,16 +47453,16 @@
         <v>50</v>
       </c>
       <c r="L341" s="6">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="M341" s="7">
-        <v>11653.52</v>
+        <v>10713.72</v>
       </c>
       <c r="N341" s="6">
         <v>1</v>
       </c>
       <c r="O341" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P341" s="8">
         <v>187.96</v>
@@ -47545,7 +47560,7 @@
         <v>2</v>
       </c>
       <c r="C342" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D342" s="3" t="s">
         <v>89</v>
@@ -47557,7 +47572,7 @@
         <v>46325</v>
       </c>
       <c r="G342" s="5">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="H342" s="3" t="s">
         <v>47</v>
@@ -47572,16 +47587,16 @@
         <v>50</v>
       </c>
       <c r="L342" s="6">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="M342" s="7">
-        <v>11841.48</v>
+        <v>10901.68</v>
       </c>
       <c r="N342" s="6">
         <v>1</v>
       </c>
       <c r="O342" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P342" s="8">
         <v>187.96</v>
@@ -47679,7 +47694,7 @@
         <v>2</v>
       </c>
       <c r="C343" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D343" s="3" t="s">
         <v>89</v>
@@ -47691,7 +47706,7 @@
         <v>46325</v>
       </c>
       <c r="G343" s="5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="H343" s="3" t="s">
         <v>47</v>
@@ -47706,16 +47721,16 @@
         <v>50</v>
       </c>
       <c r="L343" s="6">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="M343" s="7">
-        <v>12029.44</v>
+        <v>11089.64</v>
       </c>
       <c r="N343" s="6">
         <v>1</v>
       </c>
       <c r="O343" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P343" s="8">
         <v>187.96</v>
@@ -47813,7 +47828,7 @@
         <v>2</v>
       </c>
       <c r="C344" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D344" s="3" t="s">
         <v>89</v>
@@ -47825,7 +47840,7 @@
         <v>46325</v>
       </c>
       <c r="G344" s="5">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H344" s="3" t="s">
         <v>47</v>
@@ -47840,16 +47855,16 @@
         <v>50</v>
       </c>
       <c r="L344" s="6">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M344" s="7">
-        <v>12217.4</v>
+        <v>11277.6</v>
       </c>
       <c r="N344" s="6">
         <v>1</v>
       </c>
       <c r="O344" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P344" s="8">
         <v>187.96</v>
@@ -47947,7 +47962,7 @@
         <v>2</v>
       </c>
       <c r="C345" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D345" s="3" t="s">
         <v>89</v>
@@ -47959,7 +47974,7 @@
         <v>46325</v>
       </c>
       <c r="G345" s="5">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="H345" s="3" t="s">
         <v>47</v>
@@ -47974,16 +47989,16 @@
         <v>50</v>
       </c>
       <c r="L345" s="6">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="M345" s="7">
-        <v>12405.36</v>
+        <v>11465.56</v>
       </c>
       <c r="N345" s="6">
         <v>1</v>
       </c>
       <c r="O345" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P345" s="8">
         <v>187.96</v>
@@ -48081,7 +48096,7 @@
         <v>2</v>
       </c>
       <c r="C346" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D346" s="3" t="s">
         <v>89</v>
@@ -48093,7 +48108,7 @@
         <v>46325</v>
       </c>
       <c r="G346" s="5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="H346" s="3" t="s">
         <v>47</v>
@@ -48108,16 +48123,16 @@
         <v>50</v>
       </c>
       <c r="L346" s="6">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="M346" s="7">
-        <v>12593.32</v>
+        <v>11653.52</v>
       </c>
       <c r="N346" s="6">
         <v>1</v>
       </c>
       <c r="O346" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P346" s="8">
         <v>187.96</v>
@@ -48215,7 +48230,7 @@
         <v>2</v>
       </c>
       <c r="C347" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D347" s="3" t="s">
         <v>89</v>
@@ -48227,7 +48242,7 @@
         <v>46325</v>
       </c>
       <c r="G347" s="5">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H347" s="3" t="s">
         <v>47</v>
@@ -48242,16 +48257,16 @@
         <v>50</v>
       </c>
       <c r="L347" s="6">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="M347" s="7">
-        <v>12781.28</v>
+        <v>11841.48</v>
       </c>
       <c r="N347" s="6">
         <v>1</v>
       </c>
       <c r="O347" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P347" s="8">
         <v>187.96</v>
@@ -48278,7 +48293,7 @@
         <v>46325</v>
       </c>
       <c r="X347" s="12">
-        <v>0.38333329999999999</v>
+        <v>0.37638890000000003</v>
       </c>
       <c r="Y347" s="10">
         <v>0</v>
@@ -48349,7 +48364,7 @@
         <v>2</v>
       </c>
       <c r="C348" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D348" s="3" t="s">
         <v>89</v>
@@ -48361,7 +48376,7 @@
         <v>46325</v>
       </c>
       <c r="G348" s="5">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H348" s="3" t="s">
         <v>47</v>
@@ -48376,16 +48391,16 @@
         <v>50</v>
       </c>
       <c r="L348" s="6">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="M348" s="7">
-        <v>12969.24</v>
+        <v>12029.44</v>
       </c>
       <c r="N348" s="6">
         <v>1</v>
       </c>
       <c r="O348" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P348" s="8">
         <v>187.96</v>
@@ -48412,7 +48427,7 @@
         <v>46325</v>
       </c>
       <c r="X348" s="12">
-        <v>0.38333329999999999</v>
+        <v>0.37638890000000003</v>
       </c>
       <c r="Y348" s="10">
         <v>0</v>
@@ -48483,7 +48498,7 @@
         <v>2</v>
       </c>
       <c r="C349" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D349" s="3" t="s">
         <v>89</v>
@@ -48495,7 +48510,7 @@
         <v>46325</v>
       </c>
       <c r="G349" s="5">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H349" s="3" t="s">
         <v>47</v>
@@ -48510,16 +48525,16 @@
         <v>50</v>
       </c>
       <c r="L349" s="6">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="M349" s="7">
-        <v>13157.2</v>
+        <v>12217.4</v>
       </c>
       <c r="N349" s="6">
         <v>1</v>
       </c>
       <c r="O349" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P349" s="8">
         <v>187.96</v>
@@ -48546,7 +48561,7 @@
         <v>46325</v>
       </c>
       <c r="X349" s="12">
-        <v>0.38333329999999999</v>
+        <v>0.37638890000000003</v>
       </c>
       <c r="Y349" s="10">
         <v>0</v>
@@ -48617,7 +48632,7 @@
         <v>2</v>
       </c>
       <c r="C350" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D350" s="3" t="s">
         <v>89</v>
@@ -48629,7 +48644,7 @@
         <v>46325</v>
       </c>
       <c r="G350" s="5">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="H350" s="3" t="s">
         <v>47</v>
@@ -48644,16 +48659,16 @@
         <v>50</v>
       </c>
       <c r="L350" s="6">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="M350" s="7">
-        <v>13345.16</v>
+        <v>12405.36</v>
       </c>
       <c r="N350" s="6">
         <v>1</v>
       </c>
       <c r="O350" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P350" s="8">
         <v>187.96</v>
@@ -48680,7 +48695,7 @@
         <v>46325</v>
       </c>
       <c r="X350" s="12">
-        <v>0.38333329999999999</v>
+        <v>0.37638890000000003</v>
       </c>
       <c r="Y350" s="10">
         <v>0</v>
@@ -48751,7 +48766,7 @@
         <v>2</v>
       </c>
       <c r="C351" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D351" s="3" t="s">
         <v>89</v>
@@ -48763,7 +48778,7 @@
         <v>46325</v>
       </c>
       <c r="G351" s="5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="H351" s="3" t="s">
         <v>47</v>
@@ -48778,16 +48793,16 @@
         <v>50</v>
       </c>
       <c r="L351" s="6">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="M351" s="7">
-        <v>13533.12</v>
+        <v>12593.32</v>
       </c>
       <c r="N351" s="6">
         <v>1</v>
       </c>
       <c r="O351" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P351" s="8">
         <v>187.96</v>
@@ -48814,7 +48829,7 @@
         <v>46325</v>
       </c>
       <c r="X351" s="12">
-        <v>0.38333329999999999</v>
+        <v>0.37638890000000003</v>
       </c>
       <c r="Y351" s="10">
         <v>0</v>
@@ -48885,7 +48900,7 @@
         <v>2</v>
       </c>
       <c r="C352" s="3" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D352" s="3" t="s">
         <v>89</v>
@@ -48897,7 +48912,7 @@
         <v>46325</v>
       </c>
       <c r="G352" s="5">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H352" s="3" t="s">
         <v>47</v>
@@ -48912,16 +48927,16 @@
         <v>50</v>
       </c>
       <c r="L352" s="6">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M352" s="7">
-        <v>13721.08</v>
+        <v>12781.28</v>
       </c>
       <c r="N352" s="6">
         <v>1</v>
       </c>
       <c r="O352" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="P352" s="8">
         <v>187.96</v>
@@ -49009,6 +49024,676 @@
       </c>
       <c r="AR352" s="3" t="s">
         <v>414</v>
+      </c>
+    </row>
+    <row r="353" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A353" s="1">
+        <v>1</v>
+      </c>
+      <c r="B353" s="2">
+        <v>2</v>
+      </c>
+      <c r="C353" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D353" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E353" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F353" s="4">
+        <v>46325</v>
+      </c>
+      <c r="G353" s="5">
+        <v>17</v>
+      </c>
+      <c r="H353" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I353" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J353" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K353" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L353" s="6">
+        <v>69</v>
+      </c>
+      <c r="M353" s="7">
+        <v>12969.24</v>
+      </c>
+      <c r="N353" s="6">
+        <v>1</v>
+      </c>
+      <c r="O353" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="P353" s="8">
+        <v>187.96</v>
+      </c>
+      <c r="Q353" s="6">
+        <v>0</v>
+      </c>
+      <c r="R353" s="7">
+        <v>0</v>
+      </c>
+      <c r="S353" s="9">
+        <v>0</v>
+      </c>
+      <c r="T353" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U353" s="10">
+        <v>68776</v>
+      </c>
+      <c r="V353" s="11">
+        <v>11</v>
+      </c>
+      <c r="W353" s="4">
+        <v>46325</v>
+      </c>
+      <c r="X353" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y353" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB353" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG353" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI353" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ353" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK353" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL353" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM353" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ353" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR353" s="3" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="354" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A354" s="1">
+        <v>1</v>
+      </c>
+      <c r="B354" s="2">
+        <v>2</v>
+      </c>
+      <c r="C354" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D354" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E354" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F354" s="4">
+        <v>46325</v>
+      </c>
+      <c r="G354" s="5">
+        <v>18</v>
+      </c>
+      <c r="H354" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I354" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J354" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K354" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L354" s="6">
+        <v>70</v>
+      </c>
+      <c r="M354" s="7">
+        <v>13157.2</v>
+      </c>
+      <c r="N354" s="6">
+        <v>1</v>
+      </c>
+      <c r="O354" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="P354" s="8">
+        <v>187.96</v>
+      </c>
+      <c r="Q354" s="6">
+        <v>0</v>
+      </c>
+      <c r="R354" s="7">
+        <v>0</v>
+      </c>
+      <c r="S354" s="9">
+        <v>0</v>
+      </c>
+      <c r="T354" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U354" s="10">
+        <v>68776</v>
+      </c>
+      <c r="V354" s="11">
+        <v>11</v>
+      </c>
+      <c r="W354" s="4">
+        <v>46325</v>
+      </c>
+      <c r="X354" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y354" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB354" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG354" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI354" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ354" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK354" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL354" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM354" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ354" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR354" s="3" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="355" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A355" s="1">
+        <v>1</v>
+      </c>
+      <c r="B355" s="2">
+        <v>2</v>
+      </c>
+      <c r="C355" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D355" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E355" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F355" s="4">
+        <v>46325</v>
+      </c>
+      <c r="G355" s="5">
+        <v>19</v>
+      </c>
+      <c r="H355" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I355" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J355" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K355" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L355" s="6">
+        <v>71</v>
+      </c>
+      <c r="M355" s="7">
+        <v>13345.16</v>
+      </c>
+      <c r="N355" s="6">
+        <v>1</v>
+      </c>
+      <c r="O355" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="P355" s="8">
+        <v>187.96</v>
+      </c>
+      <c r="Q355" s="6">
+        <v>0</v>
+      </c>
+      <c r="R355" s="7">
+        <v>0</v>
+      </c>
+      <c r="S355" s="9">
+        <v>0</v>
+      </c>
+      <c r="T355" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U355" s="10">
+        <v>68776</v>
+      </c>
+      <c r="V355" s="11">
+        <v>11</v>
+      </c>
+      <c r="W355" s="4">
+        <v>46325</v>
+      </c>
+      <c r="X355" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y355" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB355" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG355" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI355" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ355" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK355" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL355" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM355" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ355" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR355" s="3" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="356" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A356" s="1">
+        <v>1</v>
+      </c>
+      <c r="B356" s="2">
+        <v>2</v>
+      </c>
+      <c r="C356" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D356" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E356" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F356" s="4">
+        <v>46325</v>
+      </c>
+      <c r="G356" s="5">
+        <v>20</v>
+      </c>
+      <c r="H356" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I356" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J356" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K356" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L356" s="6">
+        <v>72</v>
+      </c>
+      <c r="M356" s="7">
+        <v>13533.12</v>
+      </c>
+      <c r="N356" s="6">
+        <v>1</v>
+      </c>
+      <c r="O356" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="P356" s="8">
+        <v>187.96</v>
+      </c>
+      <c r="Q356" s="6">
+        <v>0</v>
+      </c>
+      <c r="R356" s="7">
+        <v>0</v>
+      </c>
+      <c r="S356" s="9">
+        <v>0</v>
+      </c>
+      <c r="T356" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U356" s="10">
+        <v>68776</v>
+      </c>
+      <c r="V356" s="11">
+        <v>11</v>
+      </c>
+      <c r="W356" s="4">
+        <v>46325</v>
+      </c>
+      <c r="X356" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y356" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB356" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG356" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI356" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ356" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL356" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM356" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ356" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR356" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="357" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A357" s="1">
+        <v>1</v>
+      </c>
+      <c r="B357" s="2">
+        <v>2</v>
+      </c>
+      <c r="C357" s="3" t="s">
+        <v>337</v>
+      </c>
+      <c r="D357" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E357" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F357" s="4">
+        <v>46325</v>
+      </c>
+      <c r="G357" s="5">
+        <v>21</v>
+      </c>
+      <c r="H357" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I357" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="J357" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K357" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L357" s="6">
+        <v>73</v>
+      </c>
+      <c r="M357" s="7">
+        <v>13721.08</v>
+      </c>
+      <c r="N357" s="6">
+        <v>1</v>
+      </c>
+      <c r="O357" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="P357" s="8">
+        <v>187.96</v>
+      </c>
+      <c r="Q357" s="6">
+        <v>0</v>
+      </c>
+      <c r="R357" s="7">
+        <v>0</v>
+      </c>
+      <c r="S357" s="9">
+        <v>0</v>
+      </c>
+      <c r="T357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="U357" s="10">
+        <v>68776</v>
+      </c>
+      <c r="V357" s="11">
+        <v>11</v>
+      </c>
+      <c r="W357" s="4">
+        <v>46325</v>
+      </c>
+      <c r="X357" s="12">
+        <v>0.38333329999999999</v>
+      </c>
+      <c r="Y357" s="10">
+        <v>0</v>
+      </c>
+      <c r="Z357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AA357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AB357" s="13">
+        <v>0</v>
+      </c>
+      <c r="AC357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AD357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AE357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AF357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AG357" s="5">
+        <v>0</v>
+      </c>
+      <c r="AH357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI357" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AJ357" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="AK357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AL357" s="10">
+        <v>0</v>
+      </c>
+      <c r="AM357" s="14">
+        <v>0</v>
+      </c>
+      <c r="AN357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AO357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AP357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AQ357" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="AR357" s="3" t="s">
+        <v>419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>